<commit_message>
- apply fen standard to store to database - change fen storage from localstorage to db - absolute path for backend import - refactor game functions - implement game action buttons
</commit_message>
<xml_diff>
--- a/tools/languages.xlsx
+++ b/tools/languages.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/macbook/projects/hieunm/xiangqi/Tools/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{24C1AFBA-3AF9-2C49-AC72-E3C8A74393EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE7EE2C6-BCB0-804D-8121-32BDDF94284C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="15880" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,16 +16,11 @@
     <sheet name="languages" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="0" iterateDelta="1E-4"/>
-  <extLst>
-    <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
-      <loext:extCalcPr stringRefSyntax="ExcelA1"/>
-    </ext>
-  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="498" uniqueCount="418">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="525" uniqueCount="443">
   <si>
     <t>Key</t>
   </si>
@@ -327,6 +322,15 @@
     <t>Đóng</t>
   </si>
   <si>
+    <t>settings.change-password</t>
+  </si>
+  <si>
+    <t>Change password</t>
+  </si>
+  <si>
+    <t>Đổi mật khẩu</t>
+  </si>
+  <si>
     <t>popup.alert.title</t>
   </si>
   <si>
@@ -396,36 +400,42 @@
     <t>Thoát phòng</t>
   </si>
   <si>
+    <t>room.actions.confirm-leave</t>
+  </si>
+  <si>
+    <t>Are you sure you want to leave room?</t>
+  </si>
+  <si>
+    <t>Bạn có chắc muốn rời bàn chơi?</t>
+  </si>
+  <si>
+    <t>room.info.waiting-user</t>
+  </si>
+  <si>
+    <t>Waiting player…</t>
+  </si>
+  <si>
+    <t>Đang chờ người chơi…</t>
+  </si>
+  <si>
+    <t>game.general.captured</t>
+  </si>
+  <si>
     <t>General has been captured. Room over</t>
   </si>
   <si>
     <t>Tướng đã bị bắt. Game kết thúc</t>
   </si>
   <si>
+    <t>game.general.in-check</t>
+  </si>
+  <si>
     <t>Your general is under attack</t>
   </si>
   <si>
     <t>Tướng của bạn đang bị chiếu</t>
   </si>
   <si>
-    <t>room.actions.confirm-leave</t>
-  </si>
-  <si>
-    <t>Are you sure you want to leave room?</t>
-  </si>
-  <si>
-    <t>Bạn có chắc muốn rời bàn chơi?</t>
-  </si>
-  <si>
-    <t>room.info.waiting-user</t>
-  </si>
-  <si>
-    <t>Waiting player…</t>
-  </si>
-  <si>
-    <t>Đang chờ người chơi…</t>
-  </si>
-  <si>
     <t>login.page.title</t>
   </si>
   <si>
@@ -1122,6 +1132,15 @@
     <t>Thiếu cookie token làm mới</t>
   </si>
   <si>
+    <t>refresh-token.messages.mismatch-or-expired</t>
+  </si>
+  <si>
+    <t>Refresh token mismatch or expired</t>
+  </si>
+  <si>
+    <t>Thiếu refresh token hoặc đã hết hạn</t>
+  </si>
+  <si>
     <t>refresh-token.messages.success</t>
   </si>
   <si>
@@ -1257,28 +1276,79 @@
     <t>Token hợp lệ</t>
   </si>
   <si>
-    <t>refresh-token.messages.mismatch-or-expired</t>
-  </si>
-  <si>
-    <t>Refresh token mismatch or expired</t>
-  </si>
-  <si>
-    <t>Thiếu refresh token hoặc đã hết hạn</t>
-  </si>
-  <si>
-    <t>settings.change-password</t>
-  </si>
-  <si>
-    <t>Change password</t>
-  </si>
-  <si>
-    <t>Đổi mật khẩu</t>
-  </si>
-  <si>
-    <t>game.general.in-check</t>
-  </si>
-  <si>
-    <t>game.general.captured</t>
+    <t>room.actions.confirm-surrender</t>
+  </si>
+  <si>
+    <t>Are you sure you want to surrender?</t>
+  </si>
+  <si>
+    <t>Bạn có chắc chắn muốn đầu hàng không?</t>
+  </si>
+  <si>
+    <t>surrender.messages.game-already-finished</t>
+  </si>
+  <si>
+    <t>Game is already finished</t>
+  </si>
+  <si>
+    <t>Trò chơi đã kết thúc</t>
+  </si>
+  <si>
+    <t>surrender.messages.game-history-not-found</t>
+  </si>
+  <si>
+    <t>Game history not found</t>
+  </si>
+  <si>
+    <t>Không tìm thấy lịch sử trò chơi</t>
+  </si>
+  <si>
+    <t>surrender.messages.game-not-found</t>
+  </si>
+  <si>
+    <t>Game not found</t>
+  </si>
+  <si>
+    <t>Không tìm thấy trò chơi</t>
+  </si>
+  <si>
+    <t>surrender.messages.internal-server-error</t>
+  </si>
+  <si>
+    <t>surrender.messages.invalid-game-id</t>
+  </si>
+  <si>
+    <t>Invalid game ID</t>
+  </si>
+  <si>
+    <t>ID trò chơi không hợp lệ</t>
+  </si>
+  <si>
+    <t>surrender.messages.invalid-surrender-player</t>
+  </si>
+  <si>
+    <t>You are not a player in this game</t>
+  </si>
+  <si>
+    <t>Bạn không phải là người chơi trong trò chơi này</t>
+  </si>
+  <si>
+    <t>surrender.messages.opponent-not-found</t>
+  </si>
+  <si>
+    <t>Opponent not found</t>
+  </si>
+  <si>
+    <t>Không tìm thấy đối thủ</t>
+  </si>
+  <si>
+    <t>surrender.messages.success</t>
+  </si>
+  <si>
+    <t>Surrendered</t>
+  </si>
+  <si>
+    <t>Đã đầu hàng</t>
   </si>
 </sst>
 </file>
@@ -1938,13 +2008,13 @@
     </row>
     <row r="39" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A39" s="3" t="s">
-        <v>413</v>
+        <v>100</v>
       </c>
       <c r="B39" s="4" t="s">
-        <v>414</v>
+        <v>101</v>
       </c>
       <c r="C39" s="4" t="s">
-        <v>415</v>
+        <v>102</v>
       </c>
     </row>
     <row r="40" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
@@ -1954,112 +2024,112 @@
     </row>
     <row r="41" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" s="3" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="B41" s="4" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="C41" s="4" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
     </row>
     <row r="42" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" s="3" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="B42" s="4" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="C42" s="4" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
     </row>
     <row r="43" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="3" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="B43" s="4" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="C43" s="4" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
     </row>
     <row r="44" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A44" s="3" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="B44" s="4" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="C44" s="4" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
     </row>
     <row r="45" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A45" s="3" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="B45" s="4" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="C45" s="4" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
     </row>
     <row r="46" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A46" s="3" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="B46" s="4" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="C46" s="4" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
     </row>
     <row r="47" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A47" s="3" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="B47" s="4" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="C47" s="4" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
     </row>
     <row r="48" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A48" s="3" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="B48" s="4" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="C48" s="4" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
     </row>
     <row r="49" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A49" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="B49" s="4" t="s">
         <v>127</v>
       </c>
-      <c r="B49" s="4" t="s">
+      <c r="C49" s="4" t="s">
         <v>128</v>
-      </c>
-      <c r="C49" s="4" t="s">
-        <v>129</v>
       </c>
     </row>
     <row r="50" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A50" s="3" t="s">
+        <v>129</v>
+      </c>
+      <c r="B50" s="4" t="s">
         <v>130</v>
       </c>
-      <c r="B50" s="4" t="s">
+      <c r="C50" s="4" t="s">
         <v>131</v>
-      </c>
-      <c r="C50" s="4" t="s">
-        <v>132</v>
       </c>
     </row>
     <row r="51" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
@@ -2069,24 +2139,24 @@
     </row>
     <row r="52" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A52" s="3" t="s">
-        <v>417</v>
+        <v>132</v>
       </c>
       <c r="B52" s="4" t="s">
-        <v>123</v>
+        <v>133</v>
       </c>
       <c r="C52" s="4" t="s">
-        <v>124</v>
+        <v>134</v>
       </c>
     </row>
     <row r="53" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A53" s="3" t="s">
-        <v>416</v>
+        <v>135</v>
       </c>
       <c r="B53" s="4" t="s">
-        <v>125</v>
+        <v>136</v>
       </c>
       <c r="C53" s="4" t="s">
-        <v>126</v>
+        <v>137</v>
       </c>
     </row>
     <row r="54" spans="1:3" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
@@ -2096,145 +2166,145 @@
     </row>
     <row r="55" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A55" s="3" t="s">
-        <v>133</v>
+        <v>138</v>
       </c>
       <c r="B55" s="4" t="s">
-        <v>134</v>
+        <v>139</v>
       </c>
       <c r="C55" s="4" t="s">
-        <v>135</v>
+        <v>140</v>
       </c>
     </row>
     <row r="56" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A56" s="3" t="s">
-        <v>136</v>
+        <v>141</v>
       </c>
       <c r="B56" s="4" t="s">
-        <v>134</v>
+        <v>139</v>
       </c>
       <c r="C56" s="4" t="s">
-        <v>135</v>
+        <v>140</v>
       </c>
     </row>
     <row r="57" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A57" s="3" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="B57" s="4" t="s">
-        <v>138</v>
+        <v>143</v>
       </c>
       <c r="C57" s="4" t="s">
-        <v>139</v>
+        <v>144</v>
       </c>
     </row>
     <row r="58" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A58" s="3" t="s">
-        <v>140</v>
+        <v>145</v>
       </c>
       <c r="B58" s="4" t="s">
-        <v>138</v>
+        <v>143</v>
       </c>
       <c r="C58" s="4" t="s">
-        <v>139</v>
+        <v>144</v>
       </c>
     </row>
     <row r="59" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A59" s="3" t="s">
-        <v>141</v>
+        <v>146</v>
       </c>
       <c r="B59" s="4" t="s">
-        <v>142</v>
+        <v>147</v>
       </c>
       <c r="C59" s="4" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
     </row>
     <row r="60" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A60" s="3" t="s">
-        <v>144</v>
+        <v>149</v>
       </c>
       <c r="B60" s="4" t="s">
-        <v>142</v>
+        <v>147</v>
       </c>
       <c r="C60" s="4" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
     </row>
     <row r="61" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A61" s="3" t="s">
-        <v>145</v>
+        <v>150</v>
       </c>
       <c r="B61" s="4" t="s">
-        <v>146</v>
+        <v>151</v>
       </c>
       <c r="C61" s="4" t="s">
-        <v>147</v>
+        <v>152</v>
       </c>
     </row>
     <row r="62" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A62" s="3" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="B62" s="4" t="s">
-        <v>149</v>
+        <v>154</v>
       </c>
       <c r="C62" s="4" t="s">
-        <v>150</v>
+        <v>155</v>
       </c>
     </row>
     <row r="63" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A63" s="3" t="s">
-        <v>151</v>
+        <v>156</v>
       </c>
       <c r="B63" s="4" t="s">
-        <v>152</v>
+        <v>157</v>
       </c>
       <c r="C63" s="4" t="s">
-        <v>153</v>
+        <v>158</v>
       </c>
     </row>
     <row r="64" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A64" s="3" t="s">
-        <v>154</v>
+        <v>159</v>
       </c>
       <c r="B64" s="4" t="s">
-        <v>155</v>
+        <v>160</v>
       </c>
       <c r="C64" s="4" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
     </row>
     <row r="65" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A65" s="3" t="s">
-        <v>157</v>
+        <v>162</v>
       </c>
       <c r="B65" s="4" t="s">
-        <v>158</v>
+        <v>163</v>
       </c>
       <c r="C65" s="4" t="s">
-        <v>159</v>
+        <v>164</v>
       </c>
     </row>
     <row r="66" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A66" s="3" t="s">
-        <v>160</v>
+        <v>165</v>
       </c>
       <c r="B66" s="4" t="s">
-        <v>161</v>
+        <v>166</v>
       </c>
       <c r="C66" s="4" t="s">
-        <v>162</v>
+        <v>167</v>
       </c>
     </row>
     <row r="67" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A67" s="3" t="s">
-        <v>163</v>
+        <v>168</v>
       </c>
       <c r="B67" s="4" t="s">
-        <v>134</v>
+        <v>139</v>
       </c>
       <c r="C67" s="4" t="s">
-        <v>135</v>
+        <v>140</v>
       </c>
     </row>
     <row r="68" spans="1:3" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
@@ -2244,321 +2314,322 @@
     </row>
     <row r="69" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A69" s="3" t="s">
-        <v>164</v>
+        <v>169</v>
       </c>
       <c r="B69" s="4" t="s">
-        <v>165</v>
+        <v>170</v>
       </c>
       <c r="C69" s="4" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
     </row>
     <row r="70" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A70" s="3" t="s">
-        <v>167</v>
+        <v>172</v>
       </c>
       <c r="B70" s="4" t="s">
-        <v>168</v>
+        <v>173</v>
       </c>
       <c r="C70" s="4" t="s">
-        <v>169</v>
+        <v>174</v>
       </c>
     </row>
     <row r="71" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A71" s="3" t="s">
-        <v>170</v>
+        <v>175</v>
       </c>
       <c r="B71" s="4" t="s">
-        <v>171</v>
+        <v>176</v>
       </c>
       <c r="C71" s="4" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
     </row>
     <row r="72" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A72" s="3" t="s">
-        <v>173</v>
+        <v>178</v>
       </c>
       <c r="B72" s="4" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="C72" s="4" t="s">
-        <v>175</v>
-      </c>
-    </row>
+        <v>180</v>
+      </c>
+    </row>
+    <row r="73" spans="1:3" ht="16" x14ac:dyDescent="0.2"/>
     <row r="74" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A74" s="3" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="B74" s="4" t="s">
-        <v>177</v>
+        <v>182</v>
       </c>
       <c r="C74" s="4" t="s">
-        <v>178</v>
+        <v>183</v>
       </c>
     </row>
     <row r="75" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A75" s="3" t="s">
-        <v>179</v>
+        <v>184</v>
       </c>
       <c r="B75" s="4" t="s">
-        <v>180</v>
+        <v>185</v>
       </c>
       <c r="C75" s="4" t="s">
-        <v>181</v>
+        <v>186</v>
       </c>
     </row>
     <row r="76" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A76" s="3" t="s">
-        <v>182</v>
+        <v>187</v>
       </c>
       <c r="B76" s="4" t="s">
-        <v>180</v>
+        <v>185</v>
       </c>
       <c r="C76" s="4" t="s">
-        <v>181</v>
+        <v>186</v>
       </c>
     </row>
     <row r="77" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A77" s="3" t="s">
-        <v>183</v>
+        <v>188</v>
       </c>
       <c r="B77" s="4" t="s">
-        <v>184</v>
+        <v>189</v>
       </c>
       <c r="C77" s="4" t="s">
-        <v>185</v>
+        <v>190</v>
       </c>
     </row>
     <row r="78" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A78" s="3" t="s">
-        <v>186</v>
+        <v>191</v>
       </c>
       <c r="B78" s="4" t="s">
-        <v>184</v>
+        <v>189</v>
       </c>
       <c r="C78" s="4" t="s">
-        <v>185</v>
+        <v>190</v>
       </c>
     </row>
     <row r="79" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A79" s="3" t="s">
-        <v>187</v>
+        <v>192</v>
       </c>
       <c r="B79" s="4" t="s">
-        <v>188</v>
+        <v>193</v>
       </c>
       <c r="C79" s="4" t="s">
-        <v>189</v>
+        <v>194</v>
       </c>
     </row>
     <row r="80" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A80" s="3" t="s">
-        <v>190</v>
+        <v>195</v>
       </c>
       <c r="B80" s="4" t="s">
-        <v>191</v>
+        <v>196</v>
       </c>
       <c r="C80" s="4" t="s">
-        <v>191</v>
+        <v>196</v>
       </c>
     </row>
     <row r="81" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A81" s="3" t="s">
-        <v>192</v>
+        <v>197</v>
       </c>
       <c r="B81" s="4" t="s">
-        <v>191</v>
+        <v>196</v>
       </c>
       <c r="C81" s="4" t="s">
-        <v>191</v>
+        <v>196</v>
       </c>
     </row>
     <row r="82" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A82" s="3" t="s">
-        <v>193</v>
+        <v>198</v>
       </c>
       <c r="B82" s="4" t="s">
-        <v>194</v>
+        <v>199</v>
       </c>
       <c r="C82" s="4" t="s">
-        <v>195</v>
+        <v>200</v>
       </c>
     </row>
     <row r="83" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A83" s="3" t="s">
-        <v>196</v>
+        <v>201</v>
       </c>
       <c r="B83" s="4" t="s">
-        <v>161</v>
+        <v>166</v>
       </c>
       <c r="C83" s="4" t="s">
-        <v>162</v>
+        <v>167</v>
       </c>
     </row>
     <row r="84" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A84" s="3" t="s">
-        <v>197</v>
+        <v>202</v>
       </c>
       <c r="B84" s="4" t="s">
-        <v>198</v>
+        <v>203</v>
       </c>
       <c r="C84" s="4" t="s">
-        <v>199</v>
+        <v>204</v>
       </c>
     </row>
     <row r="85" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A85" s="3" t="s">
-        <v>200</v>
+        <v>205</v>
       </c>
       <c r="B85" s="4" t="s">
-        <v>161</v>
+        <v>166</v>
       </c>
       <c r="C85" s="4" t="s">
-        <v>162</v>
+        <v>167</v>
       </c>
     </row>
     <row r="86" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A86" s="3" t="s">
-        <v>201</v>
+        <v>206</v>
       </c>
       <c r="B86" s="4" t="s">
-        <v>202</v>
+        <v>207</v>
       </c>
       <c r="C86" s="4" t="s">
-        <v>203</v>
+        <v>208</v>
       </c>
     </row>
     <row r="87" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A87" s="3" t="s">
-        <v>204</v>
+        <v>209</v>
       </c>
       <c r="B87" s="4" t="s">
-        <v>205</v>
+        <v>210</v>
       </c>
       <c r="C87" s="4" t="s">
-        <v>206</v>
+        <v>211</v>
       </c>
     </row>
     <row r="88" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A88" s="3" t="s">
-        <v>207</v>
+        <v>212</v>
       </c>
       <c r="B88" s="4" t="s">
-        <v>208</v>
+        <v>213</v>
       </c>
       <c r="C88" s="4" t="s">
-        <v>209</v>
+        <v>214</v>
       </c>
     </row>
     <row r="89" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A89" s="3" t="s">
-        <v>210</v>
+        <v>215</v>
       </c>
       <c r="B89" s="4" t="s">
-        <v>211</v>
+        <v>216</v>
       </c>
       <c r="C89" s="4" t="s">
-        <v>212</v>
+        <v>217</v>
       </c>
     </row>
     <row r="90" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A90" s="3" t="s">
-        <v>213</v>
+        <v>218</v>
       </c>
       <c r="B90" s="4" t="s">
-        <v>161</v>
+        <v>166</v>
       </c>
       <c r="C90" s="4" t="s">
-        <v>162</v>
+        <v>167</v>
       </c>
     </row>
     <row r="91" spans="1:3" ht="54" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A91" s="3" t="s">
-        <v>214</v>
+        <v>219</v>
       </c>
       <c r="B91" s="4" t="s">
-        <v>215</v>
+        <v>220</v>
       </c>
       <c r="C91" s="4" t="s">
-        <v>216</v>
+        <v>221</v>
       </c>
     </row>
     <row r="92" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A92" s="3" t="s">
-        <v>217</v>
+        <v>222</v>
       </c>
       <c r="B92" s="4" t="s">
-        <v>152</v>
+        <v>157</v>
       </c>
       <c r="C92" s="4" t="s">
-        <v>153</v>
+        <v>158</v>
       </c>
     </row>
     <row r="93" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A93" s="3" t="s">
-        <v>218</v>
+        <v>223</v>
       </c>
       <c r="B93" s="4" t="s">
-        <v>142</v>
+        <v>147</v>
       </c>
       <c r="C93" s="4" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
     </row>
     <row r="94" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A94" s="3" t="s">
-        <v>219</v>
+        <v>224</v>
       </c>
       <c r="B94" s="4" t="s">
-        <v>142</v>
+        <v>147</v>
       </c>
       <c r="C94" s="4" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
     </row>
     <row r="95" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A95" s="3" t="s">
-        <v>220</v>
+        <v>225</v>
       </c>
       <c r="B95" s="4" t="s">
-        <v>149</v>
+        <v>154</v>
       </c>
       <c r="C95" s="4" t="s">
-        <v>150</v>
+        <v>155</v>
       </c>
     </row>
     <row r="96" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A96" s="3" t="s">
-        <v>221</v>
+        <v>226</v>
       </c>
       <c r="B96" s="4" t="s">
-        <v>222</v>
+        <v>227</v>
       </c>
       <c r="C96" s="4" t="s">
-        <v>223</v>
+        <v>228</v>
       </c>
     </row>
     <row r="97" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A97" s="3" t="s">
-        <v>224</v>
+        <v>229</v>
       </c>
       <c r="B97" s="4" t="s">
-        <v>138</v>
+        <v>143</v>
       </c>
       <c r="C97" s="4" t="s">
-        <v>139</v>
+        <v>144</v>
       </c>
     </row>
     <row r="98" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A98" s="3" t="s">
-        <v>225</v>
+        <v>230</v>
       </c>
       <c r="B98" s="4" t="s">
-        <v>138</v>
+        <v>143</v>
       </c>
       <c r="C98" s="4" t="s">
-        <v>139</v>
+        <v>144</v>
       </c>
     </row>
     <row r="99" spans="1:3" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
@@ -2568,68 +2639,68 @@
     </row>
     <row r="100" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A100" s="3" t="s">
-        <v>226</v>
+        <v>231</v>
       </c>
       <c r="B100" s="4" t="s">
-        <v>227</v>
+        <v>232</v>
       </c>
       <c r="C100" s="4" t="s">
-        <v>159</v>
+        <v>164</v>
       </c>
     </row>
     <row r="101" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A101" s="3" t="s">
-        <v>228</v>
+        <v>233</v>
       </c>
       <c r="B101" s="4" t="s">
-        <v>227</v>
+        <v>232</v>
       </c>
       <c r="C101" s="4" t="s">
-        <v>159</v>
+        <v>164</v>
       </c>
     </row>
     <row r="102" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A102" s="3" t="s">
-        <v>229</v>
+        <v>234</v>
       </c>
       <c r="B102" s="4" t="s">
-        <v>194</v>
+        <v>199</v>
       </c>
       <c r="C102" s="4" t="s">
-        <v>195</v>
+        <v>200</v>
       </c>
     </row>
     <row r="103" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A103" s="3" t="s">
-        <v>230</v>
+        <v>235</v>
       </c>
       <c r="B103" s="4" t="s">
-        <v>158</v>
+        <v>163</v>
       </c>
       <c r="C103" s="4" t="s">
-        <v>159</v>
+        <v>164</v>
       </c>
     </row>
     <row r="104" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A104" s="4" t="s">
-        <v>231</v>
+        <v>236</v>
       </c>
       <c r="B104" s="4" t="s">
-        <v>232</v>
+        <v>237</v>
       </c>
       <c r="C104" s="4" t="s">
-        <v>233</v>
+        <v>238</v>
       </c>
     </row>
     <row r="105" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A105" s="4" t="s">
-        <v>234</v>
+        <v>239</v>
       </c>
       <c r="B105" s="4" t="s">
-        <v>235</v>
+        <v>240</v>
       </c>
       <c r="C105" s="4" t="s">
-        <v>236</v>
+        <v>241</v>
       </c>
     </row>
     <row r="106" spans="1:3" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
@@ -2639,90 +2710,90 @@
     </row>
     <row r="107" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A107" s="4" t="s">
-        <v>237</v>
+        <v>242</v>
       </c>
       <c r="B107" s="4" t="s">
-        <v>238</v>
+        <v>243</v>
       </c>
       <c r="C107" s="4" t="s">
-        <v>239</v>
+        <v>244</v>
       </c>
     </row>
     <row r="108" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A108" s="4" t="s">
-        <v>240</v>
+        <v>245</v>
       </c>
       <c r="B108" s="4" t="s">
-        <v>241</v>
+        <v>246</v>
       </c>
       <c r="C108" s="4" t="s">
-        <v>242</v>
+        <v>247</v>
       </c>
     </row>
     <row r="109" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A109" s="4" t="s">
+        <v>248</v>
+      </c>
+      <c r="B109" s="4" t="s">
         <v>243</v>
       </c>
-      <c r="B109" s="4" t="s">
-        <v>238</v>
-      </c>
       <c r="C109" s="4" t="s">
-        <v>239</v>
+        <v>244</v>
       </c>
     </row>
     <row r="110" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A110" s="4" t="s">
-        <v>244</v>
+        <v>249</v>
       </c>
       <c r="B110" s="4" t="s">
-        <v>245</v>
+        <v>250</v>
       </c>
       <c r="C110" s="4" t="s">
-        <v>246</v>
+        <v>251</v>
       </c>
     </row>
     <row r="111" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A111" s="4" t="s">
-        <v>247</v>
+        <v>252</v>
       </c>
       <c r="B111" s="4" t="s">
-        <v>248</v>
+        <v>253</v>
       </c>
       <c r="C111" s="4" t="s">
-        <v>249</v>
+        <v>254</v>
       </c>
     </row>
     <row r="112" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A112" s="4" t="s">
-        <v>250</v>
+        <v>255</v>
       </c>
       <c r="B112" s="4" t="s">
-        <v>251</v>
+        <v>256</v>
       </c>
       <c r="C112" s="4" t="s">
-        <v>252</v>
+        <v>257</v>
       </c>
     </row>
     <row r="113" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A113" s="4" t="s">
-        <v>253</v>
+        <v>258</v>
       </c>
       <c r="B113" s="4" t="s">
-        <v>194</v>
+        <v>199</v>
       </c>
       <c r="C113" s="4" t="s">
-        <v>254</v>
+        <v>259</v>
       </c>
     </row>
     <row r="114" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A114" s="4" t="s">
-        <v>255</v>
+        <v>260</v>
       </c>
       <c r="B114" s="4" t="s">
-        <v>256</v>
+        <v>261</v>
       </c>
       <c r="C114" s="4" t="s">
-        <v>239</v>
+        <v>244</v>
       </c>
     </row>
     <row r="115" spans="1:3" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
@@ -2730,686 +2801,686 @@
       <c r="B115" s="4"/>
       <c r="C115" s="4"/>
     </row>
-    <row r="116" spans="1:3" ht="36" x14ac:dyDescent="0.2">
+    <row r="116" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A116" s="4" t="s">
-        <v>257</v>
+        <v>262</v>
       </c>
       <c r="B116" s="4" t="s">
-        <v>258</v>
+        <v>263</v>
       </c>
       <c r="C116" s="4" t="s">
-        <v>259</v>
-      </c>
-    </row>
-    <row r="117" spans="1:3" ht="36" x14ac:dyDescent="0.2">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="117" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A117" s="4" t="s">
-        <v>260</v>
+        <v>265</v>
       </c>
       <c r="B117" s="4" t="s">
-        <v>261</v>
+        <v>266</v>
       </c>
       <c r="C117" s="4" t="s">
-        <v>262</v>
-      </c>
-    </row>
-    <row r="118" spans="1:3" ht="18" x14ac:dyDescent="0.2">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="118" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A118" s="4" t="s">
-        <v>263</v>
+        <v>268</v>
       </c>
       <c r="B118" s="4" t="s">
-        <v>264</v>
+        <v>269</v>
       </c>
       <c r="C118" s="4" t="s">
-        <v>265</v>
-      </c>
-    </row>
-    <row r="119" spans="1:3" ht="18" x14ac:dyDescent="0.2">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="119" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A119" s="4" t="s">
-        <v>266</v>
+        <v>271</v>
       </c>
       <c r="B119" s="4" t="s">
-        <v>267</v>
+        <v>272</v>
       </c>
       <c r="C119" s="4" t="s">
-        <v>268</v>
-      </c>
-    </row>
-    <row r="120" spans="1:3" ht="18" x14ac:dyDescent="0.2">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="120" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A120" s="4" t="s">
-        <v>269</v>
+        <v>274</v>
       </c>
       <c r="B120" s="4" t="s">
-        <v>270</v>
+        <v>275</v>
       </c>
       <c r="C120" s="4" t="s">
-        <v>271</v>
-      </c>
-    </row>
-    <row r="121" spans="1:3" ht="36" x14ac:dyDescent="0.2">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="121" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A121" s="4" t="s">
-        <v>272</v>
+        <v>277</v>
       </c>
       <c r="B121" s="4" t="s">
-        <v>273</v>
+        <v>278</v>
       </c>
       <c r="C121" s="4" t="s">
-        <v>274</v>
-      </c>
-    </row>
-    <row r="122" spans="1:3" ht="36" x14ac:dyDescent="0.2">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="122" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A122" s="4" t="s">
-        <v>275</v>
+        <v>280</v>
       </c>
       <c r="B122" s="4" t="s">
-        <v>276</v>
+        <v>281</v>
       </c>
       <c r="C122" s="4" t="s">
-        <v>277</v>
-      </c>
-    </row>
-    <row r="123" spans="1:3" ht="18" x14ac:dyDescent="0.2">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="123" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A123" s="4" t="s">
-        <v>278</v>
+        <v>283</v>
       </c>
       <c r="B123" s="4" t="s">
-        <v>279</v>
+        <v>284</v>
       </c>
       <c r="C123" s="4" t="s">
-        <v>280</v>
-      </c>
-    </row>
-    <row r="124" spans="1:3" ht="36" x14ac:dyDescent="0.2">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="124" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A124" s="4" t="s">
-        <v>281</v>
+        <v>286</v>
       </c>
       <c r="B124" s="4" t="s">
-        <v>282</v>
+        <v>287</v>
       </c>
       <c r="C124" s="4" t="s">
-        <v>283</v>
-      </c>
-    </row>
-    <row r="125" spans="1:3" ht="18" x14ac:dyDescent="0.2">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="125" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A125" s="4" t="s">
-        <v>284</v>
+        <v>289</v>
       </c>
       <c r="B125" s="4" t="s">
-        <v>285</v>
+        <v>290</v>
       </c>
       <c r="C125" s="4" t="s">
-        <v>286</v>
-      </c>
-    </row>
-    <row r="126" spans="1:3" ht="36" x14ac:dyDescent="0.2">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="126" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A126" s="4" t="s">
-        <v>287</v>
+        <v>292</v>
       </c>
       <c r="B126" s="4" t="s">
-        <v>288</v>
+        <v>293</v>
       </c>
       <c r="C126" s="4" t="s">
-        <v>289</v>
-      </c>
-    </row>
-    <row r="127" spans="1:3" ht="36" x14ac:dyDescent="0.2">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="127" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A127" s="4" t="s">
-        <v>290</v>
+        <v>295</v>
       </c>
       <c r="B127" s="4" t="s">
-        <v>291</v>
+        <v>296</v>
       </c>
       <c r="C127" s="4" t="s">
-        <v>292</v>
-      </c>
-    </row>
-    <row r="128" spans="1:3" ht="18" x14ac:dyDescent="0.2">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="128" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A128" s="4" t="s">
-        <v>293</v>
+        <v>298</v>
       </c>
       <c r="B128" s="4" t="s">
-        <v>294</v>
+        <v>299</v>
       </c>
       <c r="C128" s="4" t="s">
-        <v>295</v>
-      </c>
-    </row>
-    <row r="129" spans="1:3" ht="18" x14ac:dyDescent="0.2">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="129" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A129" s="4" t="s">
-        <v>296</v>
+        <v>301</v>
       </c>
       <c r="B129" s="4" t="s">
-        <v>297</v>
+        <v>302</v>
       </c>
       <c r="C129" s="4" t="s">
-        <v>298</v>
-      </c>
-    </row>
-    <row r="130" spans="1:3" ht="18" x14ac:dyDescent="0.2">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="130" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A130" s="4" t="s">
-        <v>299</v>
+        <v>304</v>
       </c>
       <c r="B130" s="4" t="s">
-        <v>300</v>
+        <v>305</v>
       </c>
       <c r="C130" s="4" t="s">
-        <v>301</v>
-      </c>
-    </row>
-    <row r="131" spans="1:3" ht="18" x14ac:dyDescent="0.2">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="131" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A131" s="4" t="s">
+        <v>307</v>
+      </c>
+      <c r="B131" s="4" t="s">
+        <v>308</v>
+      </c>
+      <c r="C131" s="4" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="132" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A132" s="4" t="s">
+        <v>310</v>
+      </c>
+      <c r="B132" s="4" t="s">
+        <v>311</v>
+      </c>
+      <c r="C132" s="4" t="s">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="133" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A133" s="4" t="s">
+        <v>313</v>
+      </c>
+      <c r="B133" s="4" t="s">
+        <v>314</v>
+      </c>
+      <c r="C133" s="4" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="134" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A134" s="4" t="s">
+        <v>316</v>
+      </c>
+      <c r="B134" s="4" t="s">
         <v>302</v>
       </c>
-      <c r="B131" s="4" t="s">
+      <c r="C134" s="4" t="s">
         <v>303</v>
       </c>
-      <c r="C131" s="4" t="s">
-        <v>304</v>
-      </c>
-    </row>
-    <row r="132" spans="1:3" ht="18" x14ac:dyDescent="0.2">
-      <c r="A132" s="4" t="s">
-        <v>305</v>
-      </c>
-      <c r="B132" s="4" t="s">
-        <v>306</v>
-      </c>
-      <c r="C132" s="4" t="s">
-        <v>307</v>
-      </c>
-    </row>
-    <row r="133" spans="1:3" ht="36" x14ac:dyDescent="0.2">
-      <c r="A133" s="4" t="s">
-        <v>308</v>
-      </c>
-      <c r="B133" s="4" t="s">
-        <v>309</v>
-      </c>
-      <c r="C133" s="4" t="s">
-        <v>310</v>
-      </c>
-    </row>
-    <row r="134" spans="1:3" ht="36" x14ac:dyDescent="0.2">
-      <c r="A134" s="4" t="s">
-        <v>311</v>
-      </c>
-      <c r="B134" s="4" t="s">
-        <v>297</v>
-      </c>
-      <c r="C134" s="4" t="s">
-        <v>298</v>
-      </c>
-    </row>
-    <row r="135" spans="1:3" ht="36" x14ac:dyDescent="0.2">
+    </row>
+    <row r="135" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A135" s="4" t="s">
-        <v>312</v>
+        <v>317</v>
       </c>
       <c r="B135" s="4" t="s">
-        <v>188</v>
+        <v>193</v>
       </c>
       <c r="C135" s="4" t="s">
-        <v>189</v>
-      </c>
-    </row>
-    <row r="136" spans="1:3" ht="18" x14ac:dyDescent="0.2">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="136" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A136" s="4" t="s">
-        <v>313</v>
+        <v>318</v>
       </c>
       <c r="B136" s="4" t="s">
-        <v>314</v>
+        <v>319</v>
       </c>
       <c r="C136" s="4" t="s">
-        <v>315</v>
-      </c>
-    </row>
-    <row r="137" spans="1:3" ht="18" x14ac:dyDescent="0.2">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="137" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A137" s="4" t="s">
-        <v>316</v>
+        <v>321</v>
       </c>
       <c r="B137" s="4" t="s">
-        <v>317</v>
+        <v>322</v>
       </c>
       <c r="C137" s="4" t="s">
-        <v>318</v>
-      </c>
-    </row>
-    <row r="138" spans="1:3" ht="18" x14ac:dyDescent="0.2">
+        <v>323</v>
+      </c>
+    </row>
+    <row r="138" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A138" s="4" t="s">
-        <v>319</v>
+        <v>324</v>
       </c>
       <c r="B138" s="4" t="s">
-        <v>297</v>
+        <v>302</v>
       </c>
       <c r="C138" s="4" t="s">
-        <v>298</v>
-      </c>
-    </row>
-    <row r="139" spans="1:3" ht="36" x14ac:dyDescent="0.2">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="139" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A139" s="4" t="s">
-        <v>320</v>
+        <v>325</v>
       </c>
       <c r="B139" s="4" t="s">
-        <v>321</v>
+        <v>326</v>
       </c>
       <c r="C139" s="4" t="s">
-        <v>322</v>
-      </c>
-    </row>
-    <row r="140" spans="1:3" ht="18" x14ac:dyDescent="0.2">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="140" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A140" s="4" t="s">
-        <v>323</v>
+        <v>328</v>
       </c>
       <c r="B140" s="4" t="s">
-        <v>324</v>
+        <v>329</v>
       </c>
       <c r="C140" s="4" t="s">
-        <v>325</v>
-      </c>
-    </row>
-    <row r="141" spans="1:3" ht="18" x14ac:dyDescent="0.2">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="141" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A141" s="4" t="s">
+        <v>331</v>
+      </c>
+      <c r="B141" s="4" t="s">
+        <v>332</v>
+      </c>
+      <c r="C141" s="4" t="s">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="142" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A142" s="4" t="s">
+        <v>334</v>
+      </c>
+      <c r="B142" s="4" t="s">
+        <v>302</v>
+      </c>
+      <c r="C142" s="4" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="143" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A143" s="4" t="s">
+        <v>335</v>
+      </c>
+      <c r="B143" s="4" t="s">
         <v>326</v>
       </c>
-      <c r="B141" s="4" t="s">
+      <c r="C143" s="4" t="s">
         <v>327</v>
       </c>
-      <c r="C141" s="4" t="s">
-        <v>328</v>
-      </c>
-    </row>
-    <row r="142" spans="1:3" ht="18" x14ac:dyDescent="0.2">
-      <c r="A142" s="4" t="s">
+    </row>
+    <row r="144" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A144" s="4" t="s">
+        <v>336</v>
+      </c>
+      <c r="B144" s="4" t="s">
+        <v>337</v>
+      </c>
+      <c r="C144" s="4" t="s">
+        <v>338</v>
+      </c>
+    </row>
+    <row r="145" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A145" s="4" t="s">
+        <v>339</v>
+      </c>
+      <c r="B145" s="4" t="s">
+        <v>340</v>
+      </c>
+      <c r="C145" s="4" t="s">
+        <v>341</v>
+      </c>
+    </row>
+    <row r="146" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A146" s="4" t="s">
+        <v>342</v>
+      </c>
+      <c r="B146" s="4" t="s">
+        <v>302</v>
+      </c>
+      <c r="C146" s="4" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="147" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A147" s="4" t="s">
+        <v>343</v>
+      </c>
+      <c r="B147" s="4" t="s">
+        <v>344</v>
+      </c>
+      <c r="C147" s="4" t="s">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="148" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A148" s="4" t="s">
+        <v>346</v>
+      </c>
+      <c r="B148" s="4" t="s">
         <v>329</v>
       </c>
-      <c r="B142" s="4" t="s">
-        <v>297</v>
-      </c>
-      <c r="C142" s="4" t="s">
-        <v>298</v>
-      </c>
-    </row>
-    <row r="143" spans="1:3" ht="36" x14ac:dyDescent="0.2">
-      <c r="A143" s="4" t="s">
+      <c r="C148" s="4" t="s">
         <v>330</v>
       </c>
-      <c r="B143" s="4" t="s">
-        <v>321</v>
-      </c>
-      <c r="C143" s="4" t="s">
-        <v>322</v>
-      </c>
-    </row>
-    <row r="144" spans="1:3" ht="18" x14ac:dyDescent="0.2">
-      <c r="A144" s="4" t="s">
-        <v>331</v>
-      </c>
-      <c r="B144" s="4" t="s">
-        <v>332</v>
-      </c>
-      <c r="C144" s="4" t="s">
-        <v>333</v>
-      </c>
-    </row>
-    <row r="145" spans="1:3" ht="18" x14ac:dyDescent="0.2">
-      <c r="A145" s="4" t="s">
-        <v>334</v>
-      </c>
-      <c r="B145" s="4" t="s">
-        <v>335</v>
-      </c>
-      <c r="C145" s="4" t="s">
-        <v>336</v>
-      </c>
-    </row>
-    <row r="146" spans="1:3" ht="18" x14ac:dyDescent="0.2">
-      <c r="A146" s="4" t="s">
-        <v>337</v>
-      </c>
-      <c r="B146" s="4" t="s">
-        <v>297</v>
-      </c>
-      <c r="C146" s="4" t="s">
-        <v>298</v>
-      </c>
-    </row>
-    <row r="147" spans="1:3" ht="18" x14ac:dyDescent="0.2">
-      <c r="A147" s="4" t="s">
-        <v>338</v>
-      </c>
-      <c r="B147" s="4" t="s">
-        <v>339</v>
-      </c>
-      <c r="C147" s="4" t="s">
-        <v>340</v>
-      </c>
-    </row>
-    <row r="148" spans="1:3" ht="18" x14ac:dyDescent="0.2">
-      <c r="A148" s="4" t="s">
-        <v>341</v>
-      </c>
-      <c r="B148" s="4" t="s">
-        <v>324</v>
-      </c>
-      <c r="C148" s="4" t="s">
-        <v>325</v>
-      </c>
-    </row>
-    <row r="149" spans="1:3" ht="18" x14ac:dyDescent="0.2">
+    </row>
+    <row r="149" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A149" s="4" t="s">
-        <v>342</v>
+        <v>347</v>
       </c>
       <c r="B149" s="4" t="s">
-        <v>343</v>
+        <v>348</v>
       </c>
       <c r="C149" s="4" t="s">
-        <v>344</v>
-      </c>
-    </row>
-    <row r="150" spans="1:3" ht="36" x14ac:dyDescent="0.2">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="150" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A150" s="4" t="s">
-        <v>345</v>
+        <v>350</v>
       </c>
       <c r="B150" s="4" t="s">
-        <v>346</v>
+        <v>351</v>
       </c>
       <c r="C150" s="4" t="s">
-        <v>347</v>
-      </c>
-    </row>
-    <row r="151" spans="1:3" ht="18" x14ac:dyDescent="0.2">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="151" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A151" s="4" t="s">
-        <v>348</v>
+        <v>353</v>
       </c>
       <c r="B151" s="4" t="s">
-        <v>297</v>
+        <v>302</v>
       </c>
       <c r="C151" s="4" t="s">
-        <v>298</v>
-      </c>
-    </row>
-    <row r="152" spans="1:3" ht="18" x14ac:dyDescent="0.2">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="152" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A152" s="4" t="s">
-        <v>349</v>
+        <v>354</v>
       </c>
       <c r="B152" s="4" t="s">
-        <v>350</v>
+        <v>355</v>
       </c>
       <c r="C152" s="4" t="s">
-        <v>351</v>
-      </c>
-    </row>
-    <row r="153" spans="1:3" ht="18" x14ac:dyDescent="0.2">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="153" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A153" s="4" t="s">
-        <v>352</v>
+        <v>357</v>
       </c>
       <c r="B153" s="4" t="s">
-        <v>353</v>
+        <v>358</v>
       </c>
       <c r="C153" s="4" t="s">
-        <v>354</v>
-      </c>
-    </row>
-    <row r="154" spans="1:3" ht="18" x14ac:dyDescent="0.2">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="154" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A154" s="4" t="s">
-        <v>355</v>
+        <v>360</v>
       </c>
       <c r="B154" s="4" t="s">
-        <v>356</v>
+        <v>361</v>
       </c>
       <c r="C154" s="4" t="s">
-        <v>357</v>
-      </c>
-    </row>
-    <row r="155" spans="1:3" ht="18" x14ac:dyDescent="0.2">
+        <v>362</v>
+      </c>
+    </row>
+    <row r="155" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A155" s="4" t="s">
-        <v>358</v>
+        <v>363</v>
       </c>
       <c r="B155" s="4" t="s">
-        <v>297</v>
+        <v>302</v>
       </c>
       <c r="C155" s="4" t="s">
-        <v>298</v>
-      </c>
-    </row>
-    <row r="156" spans="1:3" ht="18" x14ac:dyDescent="0.2">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="156" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A156" s="4" t="s">
-        <v>359</v>
+        <v>364</v>
       </c>
       <c r="B156" s="4" t="s">
-        <v>360</v>
+        <v>365</v>
       </c>
       <c r="C156" s="4" t="s">
-        <v>361</v>
-      </c>
-    </row>
-    <row r="157" spans="1:3" ht="36" x14ac:dyDescent="0.2">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="157" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A157" s="4" t="s">
-        <v>362</v>
+        <v>367</v>
       </c>
       <c r="B157" s="4" t="s">
-        <v>363</v>
+        <v>368</v>
       </c>
       <c r="C157" s="4" t="s">
-        <v>364</v>
-      </c>
-    </row>
-    <row r="158" spans="1:3" ht="36" x14ac:dyDescent="0.2">
+        <v>369</v>
+      </c>
+    </row>
+    <row r="158" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A158" s="4" t="s">
+        <v>370</v>
+      </c>
+      <c r="B158" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="C158" s="4" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="159" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A159" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="B159" s="4" t="s">
+        <v>374</v>
+      </c>
+      <c r="C159" s="4" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="160" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A160" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="B160" s="4" t="s">
+        <v>377</v>
+      </c>
+      <c r="C160" s="4" t="s">
+        <v>378</v>
+      </c>
+    </row>
+    <row r="161" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A161" s="4" t="s">
+        <v>379</v>
+      </c>
+      <c r="B161" s="4" t="s">
+        <v>302</v>
+      </c>
+      <c r="C161" s="4" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="162" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A162" s="4" t="s">
+        <v>380</v>
+      </c>
+      <c r="B162" s="4" t="s">
+        <v>381</v>
+      </c>
+      <c r="C162" s="4" t="s">
+        <v>382</v>
+      </c>
+    </row>
+    <row r="163" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A163" s="4" t="s">
+        <v>383</v>
+      </c>
+      <c r="B163" s="4" t="s">
+        <v>384</v>
+      </c>
+      <c r="C163" s="4" t="s">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="164" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A164" s="4" t="s">
+        <v>386</v>
+      </c>
+      <c r="B164" s="4" t="s">
+        <v>387</v>
+      </c>
+      <c r="C164" s="4" t="s">
+        <v>388</v>
+      </c>
+    </row>
+    <row r="165" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A165" s="4" t="s">
+        <v>389</v>
+      </c>
+      <c r="B165" s="4" t="s">
+        <v>302</v>
+      </c>
+      <c r="C165" s="4" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="166" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A166" s="4" t="s">
+        <v>390</v>
+      </c>
+      <c r="B166" s="4" t="s">
+        <v>253</v>
+      </c>
+      <c r="C166" s="4" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="167" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A167" s="4" t="s">
+        <v>391</v>
+      </c>
+      <c r="B167" s="4" t="s">
+        <v>392</v>
+      </c>
+      <c r="C167" s="4" t="s">
+        <v>393</v>
+      </c>
+    </row>
+    <row r="168" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A168" s="4" t="s">
+        <v>394</v>
+      </c>
+      <c r="B168" s="4" t="s">
+        <v>395</v>
+      </c>
+      <c r="C168" s="4" t="s">
+        <v>396</v>
+      </c>
+    </row>
+    <row r="169" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A169" s="4" t="s">
+        <v>397</v>
+      </c>
+      <c r="B169" s="4" t="s">
+        <v>398</v>
+      </c>
+      <c r="C169" s="4" t="s">
+        <v>399</v>
+      </c>
+    </row>
+    <row r="170" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A170" s="4" t="s">
+        <v>400</v>
+      </c>
+      <c r="B170" s="4" t="s">
+        <v>401</v>
+      </c>
+      <c r="C170" s="4" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="171" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A171" s="4" t="s">
+        <v>403</v>
+      </c>
+      <c r="B171" s="4" t="s">
+        <v>404</v>
+      </c>
+      <c r="C171" s="4" t="s">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="172" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A172" s="4" t="s">
+        <v>406</v>
+      </c>
+      <c r="B172" s="4" t="s">
+        <v>302</v>
+      </c>
+      <c r="C172" s="4" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="173" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A173" s="4" t="s">
+        <v>407</v>
+      </c>
+      <c r="B173" s="4" t="s">
+        <v>326</v>
+      </c>
+      <c r="C173" s="4" t="s">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="174" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A174" s="4" t="s">
+        <v>408</v>
+      </c>
+      <c r="B174" s="4" t="s">
+        <v>409</v>
+      </c>
+      <c r="C174" s="4" t="s">
         <v>410</v>
       </c>
-      <c r="B158" s="4" t="s">
+    </row>
+    <row r="175" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A175" s="4" t="s">
         <v>411</v>
       </c>
-      <c r="C158" s="4" t="s">
+      <c r="B175" s="4" t="s">
+        <v>329</v>
+      </c>
+      <c r="C175" s="4" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="176" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A176" s="4" t="s">
         <v>412</v>
       </c>
-    </row>
-    <row r="159" spans="1:3" ht="18" x14ac:dyDescent="0.2">
-      <c r="A159" s="4" t="s">
-        <v>365</v>
-      </c>
-      <c r="B159" s="4" t="s">
-        <v>366</v>
-      </c>
-      <c r="C159" s="4" t="s">
-        <v>367</v>
-      </c>
-    </row>
-    <row r="160" spans="1:3" ht="18" x14ac:dyDescent="0.2">
-      <c r="A160" s="4" t="s">
-        <v>368</v>
-      </c>
-      <c r="B160" s="4" t="s">
-        <v>369</v>
-      </c>
-      <c r="C160" s="4" t="s">
-        <v>370</v>
-      </c>
-    </row>
-    <row r="161" spans="1:3" ht="18" x14ac:dyDescent="0.2">
-      <c r="A161" s="4" t="s">
-        <v>371</v>
-      </c>
-      <c r="B161" s="4" t="s">
-        <v>297</v>
-      </c>
-      <c r="C161" s="4" t="s">
-        <v>298</v>
-      </c>
-    </row>
-    <row r="162" spans="1:3" ht="36" x14ac:dyDescent="0.2">
-      <c r="A162" s="4" t="s">
-        <v>372</v>
-      </c>
-      <c r="B162" s="4" t="s">
-        <v>373</v>
-      </c>
-      <c r="C162" s="4" t="s">
-        <v>374</v>
-      </c>
-    </row>
-    <row r="163" spans="1:3" ht="18" x14ac:dyDescent="0.2">
-      <c r="A163" s="4" t="s">
-        <v>375</v>
-      </c>
-      <c r="B163" s="4" t="s">
-        <v>376</v>
-      </c>
-      <c r="C163" s="4" t="s">
-        <v>377</v>
-      </c>
-    </row>
-    <row r="164" spans="1:3" ht="18" x14ac:dyDescent="0.2">
-      <c r="A164" s="4" t="s">
-        <v>378</v>
-      </c>
-      <c r="B164" s="4" t="s">
-        <v>379</v>
-      </c>
-      <c r="C164" s="4" t="s">
-        <v>380</v>
-      </c>
-    </row>
-    <row r="165" spans="1:3" ht="36" x14ac:dyDescent="0.2">
-      <c r="A165" s="4" t="s">
-        <v>381</v>
-      </c>
-      <c r="B165" s="4" t="s">
-        <v>297</v>
-      </c>
-      <c r="C165" s="4" t="s">
-        <v>298</v>
-      </c>
-    </row>
-    <row r="166" spans="1:3" ht="36" x14ac:dyDescent="0.2">
-      <c r="A166" s="4" t="s">
-        <v>382</v>
-      </c>
-      <c r="B166" s="4" t="s">
-        <v>248</v>
-      </c>
-      <c r="C166" s="4" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="167" spans="1:3" ht="18" x14ac:dyDescent="0.2">
-      <c r="A167" s="4" t="s">
-        <v>383</v>
-      </c>
-      <c r="B167" s="4" t="s">
-        <v>384</v>
-      </c>
-      <c r="C167" s="4" t="s">
-        <v>385</v>
-      </c>
-    </row>
-    <row r="168" spans="1:3" ht="36" x14ac:dyDescent="0.2">
-      <c r="A168" s="4" t="s">
-        <v>386</v>
-      </c>
-      <c r="B168" s="4" t="s">
-        <v>387</v>
-      </c>
-      <c r="C168" s="4" t="s">
-        <v>388</v>
-      </c>
-    </row>
-    <row r="169" spans="1:3" ht="36" x14ac:dyDescent="0.2">
-      <c r="A169" s="4" t="s">
-        <v>389</v>
-      </c>
-      <c r="B169" s="4" t="s">
-        <v>390</v>
-      </c>
-      <c r="C169" s="4" t="s">
-        <v>391</v>
-      </c>
-    </row>
-    <row r="170" spans="1:3" ht="18" x14ac:dyDescent="0.2">
-      <c r="A170" s="4" t="s">
-        <v>392</v>
-      </c>
-      <c r="B170" s="4" t="s">
-        <v>393</v>
-      </c>
-      <c r="C170" s="4" t="s">
-        <v>394</v>
-      </c>
-    </row>
-    <row r="171" spans="1:3" ht="18" x14ac:dyDescent="0.2">
-      <c r="A171" s="4" t="s">
-        <v>395</v>
-      </c>
-      <c r="B171" s="4" t="s">
-        <v>396</v>
-      </c>
-      <c r="C171" s="4" t="s">
-        <v>397</v>
-      </c>
-    </row>
-    <row r="172" spans="1:3" ht="36" x14ac:dyDescent="0.2">
-      <c r="A172" s="4" t="s">
-        <v>398</v>
-      </c>
-      <c r="B172" s="4" t="s">
-        <v>297</v>
-      </c>
-      <c r="C172" s="4" t="s">
-        <v>298</v>
-      </c>
-    </row>
-    <row r="173" spans="1:3" ht="36" x14ac:dyDescent="0.2">
-      <c r="A173" s="4" t="s">
-        <v>399</v>
-      </c>
-      <c r="B173" s="4" t="s">
-        <v>321</v>
-      </c>
-      <c r="C173" s="4" t="s">
-        <v>322</v>
-      </c>
-    </row>
-    <row r="174" spans="1:3" ht="18" x14ac:dyDescent="0.2">
-      <c r="A174" s="4" t="s">
-        <v>400</v>
-      </c>
-      <c r="B174" s="4" t="s">
-        <v>401</v>
-      </c>
-      <c r="C174" s="4" t="s">
-        <v>402</v>
-      </c>
-    </row>
-    <row r="175" spans="1:3" ht="18" x14ac:dyDescent="0.2">
-      <c r="A175" s="4" t="s">
-        <v>403</v>
-      </c>
-      <c r="B175" s="4" t="s">
-        <v>324</v>
-      </c>
-      <c r="C175" s="4" t="s">
-        <v>325</v>
-      </c>
-    </row>
-    <row r="176" spans="1:3" ht="18" x14ac:dyDescent="0.2">
-      <c r="A176" s="4" t="s">
-        <v>404</v>
-      </c>
       <c r="B176" s="4" t="s">
-        <v>405</v>
+        <v>413</v>
       </c>
       <c r="C176" s="4" t="s">
-        <v>406</v>
-      </c>
-    </row>
-    <row r="177" spans="1:3" ht="18" x14ac:dyDescent="0.2">
+        <v>414</v>
+      </c>
+    </row>
+    <row r="177" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A177" s="4" t="s">
-        <v>407</v>
+        <v>415</v>
       </c>
       <c r="B177" s="4" t="s">
-        <v>408</v>
+        <v>416</v>
       </c>
       <c r="C177" s="4" t="s">
-        <v>409</v>
+        <v>417</v>
       </c>
     </row>
     <row r="178" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3417,62 +3488,116 @@
       <c r="B178" s="4"/>
       <c r="C178" s="4"/>
     </row>
-    <row r="179" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A179" s="4"/>
-      <c r="B179" s="4"/>
-      <c r="C179" s="4"/>
-    </row>
-    <row r="180" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A180" s="4"/>
-      <c r="B180" s="4"/>
-      <c r="C180" s="4"/>
-    </row>
-    <row r="181" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A181" s="4"/>
-      <c r="B181" s="4"/>
-      <c r="C181" s="4"/>
-    </row>
-    <row r="182" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A182" s="4"/>
-      <c r="B182" s="4"/>
-      <c r="C182" s="4"/>
-    </row>
-    <row r="183" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A183" s="4"/>
-      <c r="B183" s="4"/>
-      <c r="C183" s="4"/>
-    </row>
-    <row r="184" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A184" s="4"/>
-      <c r="B184" s="4"/>
-      <c r="C184" s="4"/>
-    </row>
-    <row r="185" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A185" s="4"/>
-      <c r="B185" s="4"/>
-      <c r="C185" s="4"/>
-    </row>
-    <row r="186" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A186" s="4"/>
-      <c r="B186" s="4"/>
-      <c r="C186" s="4"/>
-    </row>
-    <row r="187" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A187" s="4"/>
-      <c r="B187" s="4"/>
-      <c r="C187" s="4"/>
-    </row>
-    <row r="188" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="179" spans="1:3" ht="18" x14ac:dyDescent="0.2">
+      <c r="A179" s="4" t="s">
+        <v>418</v>
+      </c>
+      <c r="B179" s="4" t="s">
+        <v>419</v>
+      </c>
+      <c r="C179" s="4" t="s">
+        <v>420</v>
+      </c>
+    </row>
+    <row r="180" spans="1:3" ht="18" x14ac:dyDescent="0.2">
+      <c r="A180" s="4" t="s">
+        <v>421</v>
+      </c>
+      <c r="B180" s="4" t="s">
+        <v>422</v>
+      </c>
+      <c r="C180" s="4" t="s">
+        <v>423</v>
+      </c>
+    </row>
+    <row r="181" spans="1:3" ht="36" x14ac:dyDescent="0.2">
+      <c r="A181" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="B181" s="4" t="s">
+        <v>425</v>
+      </c>
+      <c r="C181" s="4" t="s">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="182" spans="1:3" ht="18" x14ac:dyDescent="0.2">
+      <c r="A182" s="4" t="s">
+        <v>427</v>
+      </c>
+      <c r="B182" s="4" t="s">
+        <v>428</v>
+      </c>
+      <c r="C182" s="4" t="s">
+        <v>429</v>
+      </c>
+    </row>
+    <row r="183" spans="1:3" ht="18" x14ac:dyDescent="0.2">
+      <c r="A183" s="4" t="s">
+        <v>430</v>
+      </c>
+      <c r="B183" s="4" t="s">
+        <v>302</v>
+      </c>
+      <c r="C183" s="4" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="184" spans="1:3" ht="18" x14ac:dyDescent="0.2">
+      <c r="A184" s="4" t="s">
+        <v>431</v>
+      </c>
+      <c r="B184" s="4" t="s">
+        <v>432</v>
+      </c>
+      <c r="C184" s="4" t="s">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="185" spans="1:3" ht="36" x14ac:dyDescent="0.2">
+      <c r="A185" s="4" t="s">
+        <v>434</v>
+      </c>
+      <c r="B185" s="4" t="s">
+        <v>435</v>
+      </c>
+      <c r="C185" s="4" t="s">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="186" spans="1:3" ht="18" x14ac:dyDescent="0.2">
+      <c r="A186" s="4" t="s">
+        <v>437</v>
+      </c>
+      <c r="B186" s="4" t="s">
+        <v>438</v>
+      </c>
+      <c r="C186" s="4" t="s">
+        <v>439</v>
+      </c>
+    </row>
+    <row r="187" spans="1:3" ht="18" x14ac:dyDescent="0.2">
+      <c r="A187" s="4" t="s">
+        <v>440</v>
+      </c>
+      <c r="B187" s="4" t="s">
+        <v>441</v>
+      </c>
+      <c r="C187" s="4" t="s">
+        <v>442</v>
+      </c>
+    </row>
+    <row r="188" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="A188" s="4"/>
       <c r="B188" s="4"/>
       <c r="C188" s="4"/>
     </row>
-    <row r="189" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="189" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="A189" s="4"/>
       <c r="B189" s="4"/>
       <c r="C189" s="4"/>
     </row>
-    <row r="190" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="190" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="A190" s="4"/>
       <c r="B190" s="4"/>
       <c r="C190" s="4"/>
@@ -3747,6 +3872,15 @@
       <c r="B244" s="4"/>
       <c r="C244" s="4"/>
     </row>
+    <row r="245" spans="1:3" ht="16" x14ac:dyDescent="0.2"/>
+    <row r="246" spans="1:3" ht="16" x14ac:dyDescent="0.2"/>
+    <row r="247" spans="1:3" ht="16" x14ac:dyDescent="0.2"/>
+    <row r="248" spans="1:3" ht="16" x14ac:dyDescent="0.2"/>
+    <row r="249" spans="1:3" ht="16" x14ac:dyDescent="0.2"/>
+    <row r="250" spans="1:3" ht="16" x14ac:dyDescent="0.2"/>
+    <row r="251" spans="1:3" ht="16" x14ac:dyDescent="0.2"/>
+    <row r="252" spans="1:3" ht="16" x14ac:dyDescent="0.2"/>
+    <row r="253" spans="1:3" ht="16" x14ac:dyDescent="0.2"/>
     <row r="1048118" ht="12.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="1048119" ht="12.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="1048120" ht="12.75" customHeight="1" x14ac:dyDescent="0.2"/>

</xml_diff>

<commit_message>
- add protected route and handle validate token here - add draw game action - fix logic visible / enable 4 game buttons - game page layout: move player info card to the left, action button to the right on desktop mode - responsive for mobile with new game page layout - setup socket.io for to manage game real time, use for move piece first
</commit_message>
<xml_diff>
--- a/tools/languages.xlsx
+++ b/tools/languages.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10503"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/macbook/projects/hieunm/xiangqi/Tools/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\xiangqi\tools\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE7EE2C6-BCB0-804D-8121-32BDDF94284C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16BD24EA-3C6B-4918-999A-F39828FF7C84}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="15880" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="languages" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="525" uniqueCount="443">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="531" uniqueCount="449">
   <si>
     <t>Key</t>
   </si>
@@ -1349,6 +1349,24 @@
   </si>
   <si>
     <t>Đã đầu hàng</t>
+  </si>
+  <si>
+    <t>room.actions.draw</t>
+  </si>
+  <si>
+    <t>Draw</t>
+  </si>
+  <si>
+    <t>Hòa</t>
+  </si>
+  <si>
+    <t>room.actions.confirm-draw</t>
+  </si>
+  <si>
+    <t>Are you sure you want to draw?</t>
+  </si>
+  <si>
+    <t>Bạn có chắc chắn muốn hòa không?</t>
   </si>
 </sst>
 </file>
@@ -1598,15 +1616,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C1048121"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:C1048123"/>
+  <sheetFormatPr defaultColWidth="11.5" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="40.6640625" style="1" customWidth="1"/>
-    <col min="2" max="2" width="41.6640625" style="2" customWidth="1"/>
-    <col min="3" max="3" width="42.1640625" style="2" customWidth="1"/>
+    <col min="1" max="1" width="40.625" style="1" customWidth="1"/>
+    <col min="2" max="2" width="41.625" style="2" customWidth="1"/>
+    <col min="3" max="3" width="42.125" style="2" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -1617,7 +1635,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>3</v>
       </c>
@@ -1628,7 +1646,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:3" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>6</v>
       </c>
@@ -1639,7 +1657,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:3" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>9</v>
       </c>
@@ -1650,7 +1668,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:3" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
         <v>12</v>
       </c>
@@ -1661,7 +1679,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:3" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
         <v>15</v>
       </c>
@@ -1672,7 +1690,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:3" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
         <v>18</v>
       </c>
@@ -1683,12 +1701,12 @@
         <v>20</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:3" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="3"/>
       <c r="B8" s="4"/>
       <c r="C8" s="3"/>
     </row>
-    <row r="9" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
         <v>21</v>
       </c>
@@ -1699,7 +1717,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="10" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
         <v>24</v>
       </c>
@@ -1710,7 +1728,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
         <v>27</v>
       </c>
@@ -1721,7 +1739,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="12" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
         <v>30</v>
       </c>
@@ -1732,7 +1750,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
         <v>33</v>
       </c>
@@ -1743,7 +1761,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
         <v>36</v>
       </c>
@@ -1754,7 +1772,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
         <v>37</v>
       </c>
@@ -1765,7 +1783,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
         <v>40</v>
       </c>
@@ -1776,7 +1794,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="17" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
         <v>43</v>
       </c>
@@ -1787,7 +1805,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="18" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
         <v>46</v>
       </c>
@@ -1798,12 +1816,12 @@
         <v>48</v>
       </c>
     </row>
-    <row r="19" spans="1:3" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:3" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="3"/>
       <c r="B19" s="4"/>
       <c r="C19" s="4"/>
     </row>
-    <row r="20" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
         <v>49</v>
       </c>
@@ -1814,7 +1832,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="21" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="3" t="s">
         <v>52</v>
       </c>
@@ -1825,7 +1843,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="22" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="3" t="s">
         <v>55</v>
       </c>
@@ -1836,7 +1854,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="23" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="3" t="s">
         <v>58</v>
       </c>
@@ -1847,7 +1865,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="24" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="3" t="s">
         <v>61</v>
       </c>
@@ -1858,7 +1876,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="25" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="3" t="s">
         <v>64</v>
       </c>
@@ -1869,7 +1887,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="26" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="3" t="s">
         <v>67</v>
       </c>
@@ -1880,7 +1898,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="27" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="3" t="s">
         <v>70</v>
       </c>
@@ -1891,7 +1909,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="28" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="3" t="s">
         <v>73</v>
       </c>
@@ -1902,7 +1920,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="29" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="3" t="s">
         <v>76</v>
       </c>
@@ -1913,7 +1931,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="30" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="3" t="s">
         <v>79</v>
       </c>
@@ -1924,7 +1942,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="31" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="3" t="s">
         <v>82</v>
       </c>
@@ -1935,7 +1953,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="32" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="3" t="s">
         <v>85</v>
       </c>
@@ -1946,7 +1964,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="33" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="3" t="s">
         <v>88</v>
       </c>
@@ -1957,12 +1975,12 @@
         <v>89</v>
       </c>
     </row>
-    <row r="34" spans="1:3" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:3" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="3"/>
       <c r="B34" s="4"/>
       <c r="C34" s="4"/>
     </row>
-    <row r="35" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="3" t="s">
         <v>90</v>
       </c>
@@ -1973,7 +1991,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="36" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="3" t="s">
         <v>91</v>
       </c>
@@ -1984,7 +2002,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="37" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="3" t="s">
         <v>94</v>
       </c>
@@ -1995,7 +2013,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="38" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="3" t="s">
         <v>97</v>
       </c>
@@ -2006,7 +2024,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="39" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="3" t="s">
         <v>100</v>
       </c>
@@ -2017,12 +2035,12 @@
         <v>102</v>
       </c>
     </row>
-    <row r="40" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="3"/>
       <c r="B40" s="4"/>
       <c r="C40" s="4"/>
     </row>
-    <row r="41" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="3" t="s">
         <v>103</v>
       </c>
@@ -2033,7 +2051,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="42" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="3" t="s">
         <v>106</v>
       </c>
@@ -2044,7 +2062,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="43" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="3" t="s">
         <v>109</v>
       </c>
@@ -2055,7 +2073,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="44" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="3" t="s">
         <v>111</v>
       </c>
@@ -2066,7 +2084,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="45" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="3" t="s">
         <v>114</v>
       </c>
@@ -2077,7 +2095,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="46" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="3" t="s">
         <v>117</v>
       </c>
@@ -2088,7 +2106,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="47" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="3" t="s">
         <v>120</v>
       </c>
@@ -2099,7 +2117,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="48" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="3" t="s">
         <v>123</v>
       </c>
@@ -2110,7 +2128,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="49" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="3" t="s">
         <v>126</v>
       </c>
@@ -2121,7 +2139,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="50" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="3" t="s">
         <v>129</v>
       </c>
@@ -2132,12 +2150,12 @@
         <v>131</v>
       </c>
     </row>
-    <row r="51" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" s="3"/>
       <c r="B51" s="4"/>
       <c r="C51" s="4"/>
     </row>
-    <row r="52" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A52" s="3" t="s">
         <v>132</v>
       </c>
@@ -2148,7 +2166,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="53" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A53" s="3" t="s">
         <v>135</v>
       </c>
@@ -2159,12 +2177,12 @@
         <v>137</v>
       </c>
     </row>
-    <row r="54" spans="1:3" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:3" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A54" s="3"/>
       <c r="B54" s="4"/>
       <c r="C54" s="4"/>
     </row>
-    <row r="55" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A55" s="3" t="s">
         <v>138</v>
       </c>
@@ -2175,7 +2193,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="56" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56" s="3" t="s">
         <v>141</v>
       </c>
@@ -2186,7 +2204,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="57" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A57" s="3" t="s">
         <v>142</v>
       </c>
@@ -2197,7 +2215,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="58" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A58" s="3" t="s">
         <v>145</v>
       </c>
@@ -2208,7 +2226,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="59" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A59" s="3" t="s">
         <v>146</v>
       </c>
@@ -2219,7 +2237,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="60" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A60" s="3" t="s">
         <v>149</v>
       </c>
@@ -2230,7 +2248,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="61" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A61" s="3" t="s">
         <v>150</v>
       </c>
@@ -2241,7 +2259,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="62" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A62" s="3" t="s">
         <v>153</v>
       </c>
@@ -2252,7 +2270,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="63" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A63" s="3" t="s">
         <v>156</v>
       </c>
@@ -2263,7 +2281,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="64" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A64" s="3" t="s">
         <v>159</v>
       </c>
@@ -2274,7 +2292,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="65" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A65" s="3" t="s">
         <v>162</v>
       </c>
@@ -2285,7 +2303,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="66" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A66" s="3" t="s">
         <v>165</v>
       </c>
@@ -2296,7 +2314,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="67" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A67" s="3" t="s">
         <v>168</v>
       </c>
@@ -2307,12 +2325,12 @@
         <v>140</v>
       </c>
     </row>
-    <row r="68" spans="1:3" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:3" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A68" s="3"/>
       <c r="B68" s="4"/>
       <c r="C68" s="4"/>
     </row>
-    <row r="69" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A69" s="3" t="s">
         <v>169</v>
       </c>
@@ -2323,7 +2341,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="70" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A70" s="3" t="s">
         <v>172</v>
       </c>
@@ -2334,7 +2352,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="71" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A71" s="3" t="s">
         <v>175</v>
       </c>
@@ -2345,7 +2363,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="72" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A72" s="3" t="s">
         <v>178</v>
       </c>
@@ -2356,8 +2374,8 @@
         <v>180</v>
       </c>
     </row>
-    <row r="73" spans="1:3" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="74" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:3" ht="15.95" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="74" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A74" s="3" t="s">
         <v>181</v>
       </c>
@@ -2368,7 +2386,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="75" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A75" s="3" t="s">
         <v>184</v>
       </c>
@@ -2379,7 +2397,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="76" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A76" s="3" t="s">
         <v>187</v>
       </c>
@@ -2390,7 +2408,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="77" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A77" s="3" t="s">
         <v>188</v>
       </c>
@@ -2401,7 +2419,7 @@
         <v>190</v>
       </c>
     </row>
-    <row r="78" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A78" s="3" t="s">
         <v>191</v>
       </c>
@@ -2412,7 +2430,7 @@
         <v>190</v>
       </c>
     </row>
-    <row r="79" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A79" s="3" t="s">
         <v>192</v>
       </c>
@@ -2423,7 +2441,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="80" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A80" s="3" t="s">
         <v>195</v>
       </c>
@@ -2434,7 +2452,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="81" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A81" s="3" t="s">
         <v>197</v>
       </c>
@@ -2445,7 +2463,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="82" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A82" s="3" t="s">
         <v>198</v>
       </c>
@@ -2456,7 +2474,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="83" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="83" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A83" s="3" t="s">
         <v>201</v>
       </c>
@@ -2467,7 +2485,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="84" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A84" s="3" t="s">
         <v>202</v>
       </c>
@@ -2478,7 +2496,7 @@
         <v>204</v>
       </c>
     </row>
-    <row r="85" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="85" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A85" s="3" t="s">
         <v>205</v>
       </c>
@@ -2489,7 +2507,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="86" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="86" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A86" s="3" t="s">
         <v>206</v>
       </c>
@@ -2500,7 +2518,7 @@
         <v>208</v>
       </c>
     </row>
-    <row r="87" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="87" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A87" s="3" t="s">
         <v>209</v>
       </c>
@@ -2511,7 +2529,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="88" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="88" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A88" s="3" t="s">
         <v>212</v>
       </c>
@@ -2522,7 +2540,7 @@
         <v>214</v>
       </c>
     </row>
-    <row r="89" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="89" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A89" s="3" t="s">
         <v>215</v>
       </c>
@@ -2533,7 +2551,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="90" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="90" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A90" s="3" t="s">
         <v>218</v>
       </c>
@@ -2544,7 +2562,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="91" spans="1:3" ht="54" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="91" spans="1:3" ht="54" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A91" s="3" t="s">
         <v>219</v>
       </c>
@@ -2555,7 +2573,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="92" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="92" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A92" s="3" t="s">
         <v>222</v>
       </c>
@@ -2566,7 +2584,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="93" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="93" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A93" s="3" t="s">
         <v>223</v>
       </c>
@@ -2577,7 +2595,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="94" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="94" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A94" s="3" t="s">
         <v>224</v>
       </c>
@@ -2588,7 +2606,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="95" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="95" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A95" s="3" t="s">
         <v>225</v>
       </c>
@@ -2599,7 +2617,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="96" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="96" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A96" s="3" t="s">
         <v>226</v>
       </c>
@@ -2610,7 +2628,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="97" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="97" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A97" s="3" t="s">
         <v>229</v>
       </c>
@@ -2621,7 +2639,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="98" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="98" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A98" s="3" t="s">
         <v>230</v>
       </c>
@@ -2632,12 +2650,12 @@
         <v>144</v>
       </c>
     </row>
-    <row r="99" spans="1:3" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="99" spans="1:3" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A99" s="3"/>
       <c r="B99" s="4"/>
       <c r="C99" s="4"/>
     </row>
-    <row r="100" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="100" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A100" s="3" t="s">
         <v>231</v>
       </c>
@@ -2648,7 +2666,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="101" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="101" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A101" s="3" t="s">
         <v>233</v>
       </c>
@@ -2659,7 +2677,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="102" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="102" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A102" s="3" t="s">
         <v>234</v>
       </c>
@@ -2670,7 +2688,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="103" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="103" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A103" s="3" t="s">
         <v>235</v>
       </c>
@@ -2681,7 +2699,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="104" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="104" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A104" s="4" t="s">
         <v>236</v>
       </c>
@@ -2692,7 +2710,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="105" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="105" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A105" s="4" t="s">
         <v>239</v>
       </c>
@@ -2703,12 +2721,12 @@
         <v>241</v>
       </c>
     </row>
-    <row r="106" spans="1:3" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="106" spans="1:3" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A106" s="4"/>
       <c r="B106" s="4"/>
       <c r="C106" s="4"/>
     </row>
-    <row r="107" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="107" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A107" s="4" t="s">
         <v>242</v>
       </c>
@@ -2719,7 +2737,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="108" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="108" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A108" s="4" t="s">
         <v>245</v>
       </c>
@@ -2730,7 +2748,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="109" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="109" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A109" s="4" t="s">
         <v>248</v>
       </c>
@@ -2741,7 +2759,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="110" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="110" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A110" s="4" t="s">
         <v>249</v>
       </c>
@@ -2752,7 +2770,7 @@
         <v>251</v>
       </c>
     </row>
-    <row r="111" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="111" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A111" s="4" t="s">
         <v>252</v>
       </c>
@@ -2763,7 +2781,7 @@
         <v>254</v>
       </c>
     </row>
-    <row r="112" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="112" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A112" s="4" t="s">
         <v>255</v>
       </c>
@@ -2774,7 +2792,7 @@
         <v>257</v>
       </c>
     </row>
-    <row r="113" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="113" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A113" s="4" t="s">
         <v>258</v>
       </c>
@@ -2785,7 +2803,7 @@
         <v>259</v>
       </c>
     </row>
-    <row r="114" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="114" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A114" s="4" t="s">
         <v>260</v>
       </c>
@@ -2796,12 +2814,12 @@
         <v>244</v>
       </c>
     </row>
-    <row r="115" spans="1:3" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="115" spans="1:3" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A115" s="4"/>
       <c r="B115" s="4"/>
       <c r="C115" s="4"/>
     </row>
-    <row r="116" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="116" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A116" s="4" t="s">
         <v>262</v>
       </c>
@@ -2812,7 +2830,7 @@
         <v>264</v>
       </c>
     </row>
-    <row r="117" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="117" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A117" s="4" t="s">
         <v>265</v>
       </c>
@@ -2823,7 +2841,7 @@
         <v>267</v>
       </c>
     </row>
-    <row r="118" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="118" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A118" s="4" t="s">
         <v>268</v>
       </c>
@@ -2834,7 +2852,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="119" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="119" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A119" s="4" t="s">
         <v>271</v>
       </c>
@@ -2845,7 +2863,7 @@
         <v>273</v>
       </c>
     </row>
-    <row r="120" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="120" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A120" s="4" t="s">
         <v>274</v>
       </c>
@@ -2856,7 +2874,7 @@
         <v>276</v>
       </c>
     </row>
-    <row r="121" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="121" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A121" s="4" t="s">
         <v>277</v>
       </c>
@@ -2867,7 +2885,7 @@
         <v>279</v>
       </c>
     </row>
-    <row r="122" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="122" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A122" s="4" t="s">
         <v>280</v>
       </c>
@@ -2878,7 +2896,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="123" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="123" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A123" s="4" t="s">
         <v>283</v>
       </c>
@@ -2889,7 +2907,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="124" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="124" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A124" s="4" t="s">
         <v>286</v>
       </c>
@@ -2900,7 +2918,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="125" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="125" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A125" s="4" t="s">
         <v>289</v>
       </c>
@@ -2911,7 +2929,7 @@
         <v>291</v>
       </c>
     </row>
-    <row r="126" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="126" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A126" s="4" t="s">
         <v>292</v>
       </c>
@@ -2922,7 +2940,7 @@
         <v>294</v>
       </c>
     </row>
-    <row r="127" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="127" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A127" s="4" t="s">
         <v>295</v>
       </c>
@@ -2933,7 +2951,7 @@
         <v>297</v>
       </c>
     </row>
-    <row r="128" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="128" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A128" s="4" t="s">
         <v>298</v>
       </c>
@@ -2944,7 +2962,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="129" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="129" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A129" s="4" t="s">
         <v>301</v>
       </c>
@@ -2955,7 +2973,7 @@
         <v>303</v>
       </c>
     </row>
-    <row r="130" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="130" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A130" s="4" t="s">
         <v>304</v>
       </c>
@@ -2966,7 +2984,7 @@
         <v>306</v>
       </c>
     </row>
-    <row r="131" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="131" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A131" s="4" t="s">
         <v>307</v>
       </c>
@@ -2977,7 +2995,7 @@
         <v>309</v>
       </c>
     </row>
-    <row r="132" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="132" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A132" s="4" t="s">
         <v>310</v>
       </c>
@@ -2988,7 +3006,7 @@
         <v>312</v>
       </c>
     </row>
-    <row r="133" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="133" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A133" s="4" t="s">
         <v>313</v>
       </c>
@@ -2999,7 +3017,7 @@
         <v>315</v>
       </c>
     </row>
-    <row r="134" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="134" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A134" s="4" t="s">
         <v>316</v>
       </c>
@@ -3010,7 +3028,7 @@
         <v>303</v>
       </c>
     </row>
-    <row r="135" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="135" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A135" s="4" t="s">
         <v>317</v>
       </c>
@@ -3021,7 +3039,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="136" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="136" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A136" s="4" t="s">
         <v>318</v>
       </c>
@@ -3032,7 +3050,7 @@
         <v>320</v>
       </c>
     </row>
-    <row r="137" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="137" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A137" s="4" t="s">
         <v>321</v>
       </c>
@@ -3043,7 +3061,7 @@
         <v>323</v>
       </c>
     </row>
-    <row r="138" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="138" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A138" s="4" t="s">
         <v>324</v>
       </c>
@@ -3054,7 +3072,7 @@
         <v>303</v>
       </c>
     </row>
-    <row r="139" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="139" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A139" s="4" t="s">
         <v>325</v>
       </c>
@@ -3065,7 +3083,7 @@
         <v>327</v>
       </c>
     </row>
-    <row r="140" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="140" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A140" s="4" t="s">
         <v>328</v>
       </c>
@@ -3076,7 +3094,7 @@
         <v>330</v>
       </c>
     </row>
-    <row r="141" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="141" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A141" s="4" t="s">
         <v>331</v>
       </c>
@@ -3087,7 +3105,7 @@
         <v>333</v>
       </c>
     </row>
-    <row r="142" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="142" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A142" s="4" t="s">
         <v>334</v>
       </c>
@@ -3098,7 +3116,7 @@
         <v>303</v>
       </c>
     </row>
-    <row r="143" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="143" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A143" s="4" t="s">
         <v>335</v>
       </c>
@@ -3109,7 +3127,7 @@
         <v>327</v>
       </c>
     </row>
-    <row r="144" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="144" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A144" s="4" t="s">
         <v>336</v>
       </c>
@@ -3120,7 +3138,7 @@
         <v>338</v>
       </c>
     </row>
-    <row r="145" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="145" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A145" s="4" t="s">
         <v>339</v>
       </c>
@@ -3131,7 +3149,7 @@
         <v>341</v>
       </c>
     </row>
-    <row r="146" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="146" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A146" s="4" t="s">
         <v>342</v>
       </c>
@@ -3142,7 +3160,7 @@
         <v>303</v>
       </c>
     </row>
-    <row r="147" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="147" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A147" s="4" t="s">
         <v>343</v>
       </c>
@@ -3153,7 +3171,7 @@
         <v>345</v>
       </c>
     </row>
-    <row r="148" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="148" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A148" s="4" t="s">
         <v>346</v>
       </c>
@@ -3164,7 +3182,7 @@
         <v>330</v>
       </c>
     </row>
-    <row r="149" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="149" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A149" s="4" t="s">
         <v>347</v>
       </c>
@@ -3175,7 +3193,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="150" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="150" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A150" s="4" t="s">
         <v>350</v>
       </c>
@@ -3186,7 +3204,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="151" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="151" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A151" s="4" t="s">
         <v>353</v>
       </c>
@@ -3197,7 +3215,7 @@
         <v>303</v>
       </c>
     </row>
-    <row r="152" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="152" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A152" s="4" t="s">
         <v>354</v>
       </c>
@@ -3208,7 +3226,7 @@
         <v>356</v>
       </c>
     </row>
-    <row r="153" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="153" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A153" s="4" t="s">
         <v>357</v>
       </c>
@@ -3219,7 +3237,7 @@
         <v>359</v>
       </c>
     </row>
-    <row r="154" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="154" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A154" s="4" t="s">
         <v>360</v>
       </c>
@@ -3230,7 +3248,7 @@
         <v>362</v>
       </c>
     </row>
-    <row r="155" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="155" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A155" s="4" t="s">
         <v>363</v>
       </c>
@@ -3241,7 +3259,7 @@
         <v>303</v>
       </c>
     </row>
-    <row r="156" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="156" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A156" s="4" t="s">
         <v>364</v>
       </c>
@@ -3252,7 +3270,7 @@
         <v>366</v>
       </c>
     </row>
-    <row r="157" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="157" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A157" s="4" t="s">
         <v>367</v>
       </c>
@@ -3263,7 +3281,7 @@
         <v>369</v>
       </c>
     </row>
-    <row r="158" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="158" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A158" s="4" t="s">
         <v>370</v>
       </c>
@@ -3274,7 +3292,7 @@
         <v>372</v>
       </c>
     </row>
-    <row r="159" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="159" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A159" s="4" t="s">
         <v>373</v>
       </c>
@@ -3285,7 +3303,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="160" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="160" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A160" s="4" t="s">
         <v>376</v>
       </c>
@@ -3296,7 +3314,7 @@
         <v>378</v>
       </c>
     </row>
-    <row r="161" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="161" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A161" s="4" t="s">
         <v>379</v>
       </c>
@@ -3307,7 +3325,7 @@
         <v>303</v>
       </c>
     </row>
-    <row r="162" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="162" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A162" s="4" t="s">
         <v>380</v>
       </c>
@@ -3318,7 +3336,7 @@
         <v>382</v>
       </c>
     </row>
-    <row r="163" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="163" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A163" s="4" t="s">
         <v>383</v>
       </c>
@@ -3329,7 +3347,7 @@
         <v>385</v>
       </c>
     </row>
-    <row r="164" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="164" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A164" s="4" t="s">
         <v>386</v>
       </c>
@@ -3340,7 +3358,7 @@
         <v>388</v>
       </c>
     </row>
-    <row r="165" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="165" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A165" s="4" t="s">
         <v>389</v>
       </c>
@@ -3351,7 +3369,7 @@
         <v>303</v>
       </c>
     </row>
-    <row r="166" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="166" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A166" s="4" t="s">
         <v>390</v>
       </c>
@@ -3362,7 +3380,7 @@
         <v>254</v>
       </c>
     </row>
-    <row r="167" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="167" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A167" s="4" t="s">
         <v>391</v>
       </c>
@@ -3373,7 +3391,7 @@
         <v>393</v>
       </c>
     </row>
-    <row r="168" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="168" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A168" s="4" t="s">
         <v>394</v>
       </c>
@@ -3384,7 +3402,7 @@
         <v>396</v>
       </c>
     </row>
-    <row r="169" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="169" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A169" s="4" t="s">
         <v>397</v>
       </c>
@@ -3395,7 +3413,7 @@
         <v>399</v>
       </c>
     </row>
-    <row r="170" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="170" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A170" s="4" t="s">
         <v>400</v>
       </c>
@@ -3406,7 +3424,7 @@
         <v>402</v>
       </c>
     </row>
-    <row r="171" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="171" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A171" s="4" t="s">
         <v>403</v>
       </c>
@@ -3417,7 +3435,7 @@
         <v>405</v>
       </c>
     </row>
-    <row r="172" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="172" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A172" s="4" t="s">
         <v>406</v>
       </c>
@@ -3428,7 +3446,7 @@
         <v>303</v>
       </c>
     </row>
-    <row r="173" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="173" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A173" s="4" t="s">
         <v>407</v>
       </c>
@@ -3439,7 +3457,7 @@
         <v>327</v>
       </c>
     </row>
-    <row r="174" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="174" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A174" s="4" t="s">
         <v>408</v>
       </c>
@@ -3450,7 +3468,7 @@
         <v>410</v>
       </c>
     </row>
-    <row r="175" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="175" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A175" s="4" t="s">
         <v>411</v>
       </c>
@@ -3461,7 +3479,7 @@
         <v>330</v>
       </c>
     </row>
-    <row r="176" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="176" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A176" s="4" t="s">
         <v>412</v>
       </c>
@@ -3472,7 +3490,7 @@
         <v>414</v>
       </c>
     </row>
-    <row r="177" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="177" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A177" s="4" t="s">
         <v>415</v>
       </c>
@@ -3483,12 +3501,12 @@
         <v>417</v>
       </c>
     </row>
-    <row r="178" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="178" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A178" s="4"/>
       <c r="B178" s="4"/>
       <c r="C178" s="4"/>
     </row>
-    <row r="179" spans="1:3" ht="18" x14ac:dyDescent="0.2">
+    <row r="179" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A179" s="4" t="s">
         <v>418</v>
       </c>
@@ -3499,392 +3517,406 @@
         <v>420</v>
       </c>
     </row>
-    <row r="180" spans="1:3" ht="18" x14ac:dyDescent="0.2">
+    <row r="180" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A180" s="4" t="s">
+        <v>443</v>
+      </c>
+      <c r="B180" s="4" t="s">
+        <v>444</v>
+      </c>
+      <c r="C180" s="4" t="s">
+        <v>445</v>
+      </c>
+    </row>
+    <row r="181" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A181" s="4" t="s">
+        <v>446</v>
+      </c>
+      <c r="B181" s="4" t="s">
+        <v>447</v>
+      </c>
+      <c r="C181" s="4" t="s">
+        <v>448</v>
+      </c>
+    </row>
+    <row r="182" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A182" s="4" t="s">
         <v>421</v>
       </c>
-      <c r="B180" s="4" t="s">
+      <c r="B182" s="4" t="s">
         <v>422</v>
       </c>
-      <c r="C180" s="4" t="s">
+      <c r="C182" s="4" t="s">
         <v>423</v>
       </c>
     </row>
-    <row r="181" spans="1:3" ht="36" x14ac:dyDescent="0.2">
-      <c r="A181" s="4" t="s">
+    <row r="183" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A183" s="4" t="s">
         <v>424</v>
       </c>
-      <c r="B181" s="4" t="s">
+      <c r="B183" s="4" t="s">
         <v>425</v>
       </c>
-      <c r="C181" s="4" t="s">
+      <c r="C183" s="4" t="s">
         <v>426</v>
       </c>
     </row>
-    <row r="182" spans="1:3" ht="18" x14ac:dyDescent="0.2">
-      <c r="A182" s="4" t="s">
+    <row r="184" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A184" s="4" t="s">
         <v>427</v>
       </c>
-      <c r="B182" s="4" t="s">
+      <c r="B184" s="4" t="s">
         <v>428</v>
       </c>
-      <c r="C182" s="4" t="s">
+      <c r="C184" s="4" t="s">
         <v>429</v>
       </c>
     </row>
-    <row r="183" spans="1:3" ht="18" x14ac:dyDescent="0.2">
-      <c r="A183" s="4" t="s">
+    <row r="185" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A185" s="4" t="s">
         <v>430</v>
       </c>
-      <c r="B183" s="4" t="s">
+      <c r="B185" s="4" t="s">
         <v>302</v>
       </c>
-      <c r="C183" s="4" t="s">
+      <c r="C185" s="4" t="s">
         <v>303</v>
       </c>
     </row>
-    <row r="184" spans="1:3" ht="18" x14ac:dyDescent="0.2">
-      <c r="A184" s="4" t="s">
+    <row r="186" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A186" s="4" t="s">
         <v>431</v>
       </c>
-      <c r="B184" s="4" t="s">
+      <c r="B186" s="4" t="s">
         <v>432</v>
       </c>
-      <c r="C184" s="4" t="s">
+      <c r="C186" s="4" t="s">
         <v>433</v>
       </c>
     </row>
-    <row r="185" spans="1:3" ht="36" x14ac:dyDescent="0.2">
-      <c r="A185" s="4" t="s">
+    <row r="187" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A187" s="4" t="s">
         <v>434</v>
       </c>
-      <c r="B185" s="4" t="s">
+      <c r="B187" s="4" t="s">
         <v>435</v>
       </c>
-      <c r="C185" s="4" t="s">
+      <c r="C187" s="4" t="s">
         <v>436</v>
       </c>
     </row>
-    <row r="186" spans="1:3" ht="18" x14ac:dyDescent="0.2">
-      <c r="A186" s="4" t="s">
+    <row r="188" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A188" s="4" t="s">
         <v>437</v>
       </c>
-      <c r="B186" s="4" t="s">
+      <c r="B188" s="4" t="s">
         <v>438</v>
       </c>
-      <c r="C186" s="4" t="s">
+      <c r="C188" s="4" t="s">
         <v>439</v>
       </c>
     </row>
-    <row r="187" spans="1:3" ht="18" x14ac:dyDescent="0.2">
-      <c r="A187" s="4" t="s">
+    <row r="189" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A189" s="4" t="s">
         <v>440</v>
       </c>
-      <c r="B187" s="4" t="s">
+      <c r="B189" s="4" t="s">
         <v>441</v>
       </c>
-      <c r="C187" s="4" t="s">
+      <c r="C189" s="4" t="s">
         <v>442</v>
       </c>
     </row>
-    <row r="188" spans="1:3" ht="17" x14ac:dyDescent="0.2">
-      <c r="A188" s="4"/>
-      <c r="B188" s="4"/>
-      <c r="C188" s="4"/>
-    </row>
-    <row r="189" spans="1:3" ht="17" x14ac:dyDescent="0.2">
-      <c r="A189" s="4"/>
-      <c r="B189" s="4"/>
-      <c r="C189" s="4"/>
-    </row>
-    <row r="190" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+    <row r="190" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A190" s="4"/>
       <c r="B190" s="4"/>
       <c r="C190" s="4"/>
     </row>
-    <row r="191" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A191" s="4"/>
-      <c r="B191" s="4"/>
-      <c r="C191" s="4"/>
-    </row>
-    <row r="192" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A192" s="4"/>
-      <c r="B192" s="4"/>
-      <c r="C192" s="4"/>
-    </row>
-    <row r="193" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="191" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="192" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="193" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A193" s="4"/>
       <c r="B193" s="4"/>
       <c r="C193" s="4"/>
     </row>
-    <row r="194" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="194" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A194" s="4"/>
       <c r="B194" s="4"/>
       <c r="C194" s="4"/>
     </row>
-    <row r="195" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="195" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A195" s="4"/>
       <c r="B195" s="4"/>
       <c r="C195" s="4"/>
     </row>
-    <row r="196" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="196" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A196" s="4"/>
       <c r="B196" s="4"/>
       <c r="C196" s="4"/>
     </row>
-    <row r="197" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="197" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A197" s="4"/>
       <c r="B197" s="4"/>
       <c r="C197" s="4"/>
     </row>
-    <row r="198" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="198" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A198" s="4"/>
       <c r="B198" s="4"/>
       <c r="C198" s="4"/>
     </row>
-    <row r="199" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="199" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A199" s="4"/>
       <c r="B199" s="4"/>
       <c r="C199" s="4"/>
     </row>
-    <row r="200" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="200" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A200" s="4"/>
       <c r="B200" s="4"/>
       <c r="C200" s="4"/>
     </row>
-    <row r="201" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="201" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A201" s="4"/>
       <c r="B201" s="4"/>
       <c r="C201" s="4"/>
     </row>
-    <row r="202" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="202" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A202" s="4"/>
       <c r="B202" s="4"/>
       <c r="C202" s="4"/>
     </row>
-    <row r="203" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="203" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A203" s="4"/>
       <c r="B203" s="4"/>
       <c r="C203" s="4"/>
     </row>
-    <row r="204" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="204" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A204" s="4"/>
       <c r="B204" s="4"/>
       <c r="C204" s="4"/>
     </row>
-    <row r="205" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="205" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A205" s="4"/>
       <c r="B205" s="4"/>
       <c r="C205" s="4"/>
     </row>
-    <row r="206" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="206" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A206" s="4"/>
       <c r="B206" s="4"/>
       <c r="C206" s="4"/>
     </row>
-    <row r="207" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="207" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A207" s="4"/>
       <c r="B207" s="4"/>
       <c r="C207" s="4"/>
     </row>
-    <row r="208" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="208" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A208" s="4"/>
       <c r="B208" s="4"/>
       <c r="C208" s="4"/>
     </row>
-    <row r="209" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="209" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A209" s="4"/>
       <c r="B209" s="4"/>
       <c r="C209" s="4"/>
     </row>
-    <row r="210" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="210" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A210" s="4"/>
       <c r="B210" s="4"/>
       <c r="C210" s="4"/>
     </row>
-    <row r="211" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="211" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A211" s="4"/>
       <c r="B211" s="4"/>
       <c r="C211" s="4"/>
     </row>
-    <row r="212" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="212" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A212" s="4"/>
       <c r="B212" s="4"/>
       <c r="C212" s="4"/>
     </row>
-    <row r="213" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="213" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A213" s="4"/>
       <c r="B213" s="4"/>
       <c r="C213" s="4"/>
     </row>
-    <row r="214" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="214" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A214" s="4"/>
       <c r="B214" s="4"/>
       <c r="C214" s="4"/>
     </row>
-    <row r="215" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="215" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A215" s="4"/>
       <c r="B215" s="4"/>
       <c r="C215" s="4"/>
     </row>
-    <row r="216" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="216" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A216" s="4"/>
       <c r="B216" s="4"/>
       <c r="C216" s="4"/>
     </row>
-    <row r="217" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="217" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A217" s="4"/>
       <c r="B217" s="4"/>
       <c r="C217" s="4"/>
     </row>
-    <row r="218" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="218" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A218" s="4"/>
       <c r="B218" s="4"/>
       <c r="C218" s="4"/>
     </row>
-    <row r="219" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="219" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A219" s="4"/>
       <c r="B219" s="4"/>
       <c r="C219" s="4"/>
     </row>
-    <row r="220" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="220" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A220" s="4"/>
       <c r="B220" s="4"/>
       <c r="C220" s="4"/>
     </row>
-    <row r="221" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="221" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A221" s="4"/>
       <c r="B221" s="4"/>
       <c r="C221" s="4"/>
     </row>
-    <row r="222" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="222" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A222" s="4"/>
       <c r="B222" s="4"/>
       <c r="C222" s="4"/>
     </row>
-    <row r="223" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="223" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A223" s="4"/>
       <c r="B223" s="4"/>
       <c r="C223" s="4"/>
     </row>
-    <row r="224" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="224" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A224" s="4"/>
       <c r="B224" s="4"/>
       <c r="C224" s="4"/>
     </row>
-    <row r="225" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="225" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A225" s="4"/>
       <c r="B225" s="4"/>
       <c r="C225" s="4"/>
     </row>
-    <row r="226" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="226" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A226" s="4"/>
       <c r="B226" s="4"/>
       <c r="C226" s="4"/>
     </row>
-    <row r="227" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="227" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A227" s="4"/>
       <c r="B227" s="4"/>
       <c r="C227" s="4"/>
     </row>
-    <row r="228" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="228" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A228" s="4"/>
       <c r="B228" s="4"/>
       <c r="C228" s="4"/>
     </row>
-    <row r="229" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="229" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A229" s="4"/>
       <c r="B229" s="4"/>
       <c r="C229" s="4"/>
     </row>
-    <row r="230" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="230" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A230" s="4"/>
       <c r="B230" s="4"/>
       <c r="C230" s="4"/>
     </row>
-    <row r="231" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="231" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A231" s="4"/>
       <c r="B231" s="4"/>
       <c r="C231" s="4"/>
     </row>
-    <row r="232" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="232" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A232" s="4"/>
       <c r="B232" s="4"/>
       <c r="C232" s="4"/>
     </row>
-    <row r="233" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="233" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A233" s="4"/>
       <c r="B233" s="4"/>
       <c r="C233" s="4"/>
     </row>
-    <row r="234" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="234" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A234" s="4"/>
       <c r="B234" s="4"/>
       <c r="C234" s="4"/>
     </row>
-    <row r="235" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="235" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A235" s="4"/>
       <c r="B235" s="4"/>
       <c r="C235" s="4"/>
     </row>
-    <row r="236" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="236" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A236" s="4"/>
       <c r="B236" s="4"/>
       <c r="C236" s="4"/>
     </row>
-    <row r="237" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="237" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A237" s="4"/>
       <c r="B237" s="4"/>
       <c r="C237" s="4"/>
     </row>
-    <row r="238" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="238" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A238" s="4"/>
       <c r="B238" s="4"/>
       <c r="C238" s="4"/>
     </row>
-    <row r="239" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="239" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A239" s="4"/>
       <c r="B239" s="4"/>
       <c r="C239" s="4"/>
     </row>
-    <row r="240" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="240" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A240" s="4"/>
       <c r="B240" s="4"/>
       <c r="C240" s="4"/>
     </row>
-    <row r="241" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="241" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A241" s="4"/>
       <c r="B241" s="4"/>
       <c r="C241" s="4"/>
     </row>
-    <row r="242" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="242" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A242" s="4"/>
       <c r="B242" s="4"/>
       <c r="C242" s="4"/>
     </row>
-    <row r="243" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="243" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A243" s="4"/>
       <c r="B243" s="4"/>
       <c r="C243" s="4"/>
     </row>
-    <row r="244" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="244" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A244" s="4"/>
       <c r="B244" s="4"/>
       <c r="C244" s="4"/>
     </row>
-    <row r="245" spans="1:3" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="246" spans="1:3" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="247" spans="1:3" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="248" spans="1:3" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="249" spans="1:3" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="250" spans="1:3" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="251" spans="1:3" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="252" spans="1:3" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="253" spans="1:3" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="1048118" ht="12.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="1048119" ht="12.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="1048120" ht="12.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="1048121" ht="12.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="245" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A245" s="4"/>
+      <c r="B245" s="4"/>
+      <c r="C245" s="4"/>
+    </row>
+    <row r="246" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A246" s="4"/>
+      <c r="B246" s="4"/>
+      <c r="C246" s="4"/>
+    </row>
+    <row r="247" spans="1:3" ht="15.95" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="248" spans="1:3" ht="15.95" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="249" spans="1:3" ht="15.95" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="250" spans="1:3" ht="15.95" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="251" spans="1:3" ht="15.95" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="252" spans="1:3" ht="15.95" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="253" spans="1:3" ht="15.95" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="254" spans="1:3" ht="15.95" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="255" spans="1:3" ht="15.95" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="1048120" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="1048121" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="1048122" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="1048123" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
- play with bot mode - play sound when interaction happens - change behavior on leave room, start game, create room - change in game behavior: can only control assigned team, highlight piece has moved
</commit_message>
<xml_diff>
--- a/tools/languages.xlsx
+++ b/tools/languages.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10517"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\xiangqi\Tools\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/macbook/projects/hieunm/xiangqi/Tools/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81A2B38B-B4E7-4F7D-8910-6323141D19CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9BB9B2B3-C6FB-3049-A7FA-075D073916E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="15840" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="languages" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="564" uniqueCount="471">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="570" uniqueCount="477">
   <si>
     <t>Key</t>
   </si>
@@ -1433,6 +1433,24 @@
   </si>
   <si>
     <t>Trang cá nhân</t>
+  </si>
+  <si>
+    <t>dashboard.popup.pve-mode</t>
+  </si>
+  <si>
+    <t>PVE mode</t>
+  </si>
+  <si>
+    <t>Chơi với máy</t>
+  </si>
+  <si>
+    <t>menu.expired</t>
+  </si>
+  <si>
+    <t>Set expired</t>
+  </si>
+  <si>
+    <t>Hết hạn token</t>
   </si>
 </sst>
 </file>
@@ -1670,14 +1688,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C188"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:C190"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="40" customWidth="1"/>
     <col min="2" max="3" width="50" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1688,7 +1706,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
@@ -1699,7 +1717,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>6</v>
       </c>
@@ -1710,7 +1728,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
         <v>9</v>
       </c>
@@ -1721,7 +1739,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
         <v>12</v>
       </c>
@@ -1732,7 +1750,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
         <v>15</v>
       </c>
@@ -1743,7 +1761,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
         <v>18</v>
       </c>
@@ -1754,7 +1772,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
         <v>21</v>
       </c>
@@ -1765,7 +1783,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
         <v>24</v>
       </c>
@@ -1776,7 +1794,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="10" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
         <v>27</v>
       </c>
@@ -1787,7 +1805,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="1" t="s">
         <v>30</v>
       </c>
@@ -1798,7 +1816,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="12" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="1" t="s">
         <v>33</v>
       </c>
@@ -1809,7 +1827,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="1" t="s">
         <v>36</v>
       </c>
@@ -1820,7 +1838,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="1" t="s">
         <v>468</v>
       </c>
@@ -1831,669 +1849,669 @@
         <v>470</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="1" t="s">
+        <v>474</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>475</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>476</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A16" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="B15" s="1" t="s">
+      <c r="B16" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="C15" s="1" t="s">
+      <c r="C16" s="1" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="1" t="s">
+    <row r="17" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A17" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="B16" s="1" t="s">
+      <c r="B17" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="C16" s="1" t="s">
+      <c r="C17" s="1" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="17" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="1" t="s">
+    <row r="18" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A18" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="B17" s="1" t="s">
+      <c r="B18" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="C17" s="1" t="s">
+      <c r="C18" s="1" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="18" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="1" t="s">
+    <row r="19" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A19" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="B18" s="1" t="s">
+      <c r="B19" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="C18" s="1" t="s">
+      <c r="C19" s="1" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="19" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="1" t="s">
+    <row r="20" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A20" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="B19" s="1" t="s">
+      <c r="B20" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="C19" s="1" t="s">
+      <c r="C20" s="1" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="20" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="1" t="s">
+    <row r="21" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A21" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="B20" s="1" t="s">
+      <c r="B21" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="C20" s="1" t="s">
+      <c r="C21" s="1" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="21" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="1" t="s">
+    <row r="22" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A22" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="B21" s="1" t="s">
+      <c r="B22" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="C21" s="1" t="s">
+      <c r="C22" s="1" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="22" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="1" t="s">
+    <row r="23" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A23" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="B22" s="1" t="s">
+      <c r="B23" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="C22" s="1" t="s">
+      <c r="C23" s="1" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="23" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="1" t="s">
+    <row r="24" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A24" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="B23" s="1" t="s">
+      <c r="B24" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="C23" s="1" t="s">
+      <c r="C24" s="1" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="24" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="1" t="s">
+    <row r="25" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A25" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="B24" s="1" t="s">
+      <c r="B25" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="C24" s="1" t="s">
+      <c r="C25" s="1" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="25" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="1" t="s">
+    <row r="26" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A26" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="B25" s="1" t="s">
+      <c r="B26" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="C25" s="1" t="s">
+      <c r="C26" s="1" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="26" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="1" t="s">
+    <row r="27" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A27" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="B26" s="1" t="s">
+      <c r="B27" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="C26" s="1" t="s">
+      <c r="C27" s="1" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="27" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="1" t="s">
+    <row r="28" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A28" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="B27" s="1" t="s">
+      <c r="B28" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="C27" s="1" t="s">
+      <c r="C28" s="1" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="28" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="1" t="s">
+    <row r="29" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A29" s="1" t="s">
+        <v>471</v>
+      </c>
+      <c r="B29" s="1" t="s">
+        <v>472</v>
+      </c>
+      <c r="C29" s="1" t="s">
+        <v>473</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A30" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="B28" s="1" t="s">
+      <c r="B30" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="C28" s="1" t="s">
+      <c r="C30" s="1" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="29" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="1" t="s">
+    <row r="31" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A31" s="1" t="s">
         <v>79</v>
       </c>
-      <c r="B29" s="1" t="s">
+      <c r="B31" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="C29" s="1" t="s">
+      <c r="C31" s="1" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="30" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="1" t="s">
+    <row r="32" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A32" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="B30" s="1" t="s">
+      <c r="B32" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C30" s="1" t="s">
+      <c r="C32" s="1" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="31" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="1" t="s">
+    <row r="33" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A33" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="B31" s="1" t="s">
+      <c r="B33" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="C31" s="1" t="s">
+      <c r="C33" s="1" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="32" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="1" t="s">
+    <row r="34" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A34" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="B32" s="1" t="s">
+      <c r="B34" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="C32" s="1" t="s">
+      <c r="C34" s="1" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="33" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="1" t="s">
+    <row r="35" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A35" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="B33" s="1" t="s">
+      <c r="B35" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="C33" s="1" t="s">
+      <c r="C35" s="1" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="34" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="1" t="s">
+    <row r="36" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A36" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="B34" s="1" t="s">
+      <c r="B36" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="C34" s="1" t="s">
+      <c r="C36" s="1" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="35" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="1" t="s">
+    <row r="37" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A37" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="B35" s="1" t="s">
+      <c r="B37" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="C35" s="1" t="s">
+      <c r="C37" s="1" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="36" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="1" t="s">
+    <row r="38" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A38" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="B36" s="1" t="s">
+      <c r="B38" s="1" t="s">
         <v>98</v>
       </c>
-      <c r="C36" s="1" t="s">
+      <c r="C38" s="1" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="37" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="1" t="s">
+    <row r="39" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A39" s="1" t="s">
         <v>100</v>
       </c>
-      <c r="B37" s="1" t="s">
+      <c r="B39" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="C37" s="1" t="s">
+      <c r="C39" s="1" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="38" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="1" t="s">
+    <row r="40" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A40" s="1" t="s">
         <v>103</v>
       </c>
-      <c r="B38" s="1" t="s">
+      <c r="B40" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="C38" s="1" t="s">
+      <c r="C40" s="1" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="39" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="1" t="s">
+    <row r="41" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A41" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="B39" s="1" t="s">
+      <c r="B41" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="C39" s="1" t="s">
+      <c r="C41" s="1" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="40" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="1" t="s">
+    <row r="42" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A42" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="B40" s="1" t="s">
+      <c r="B42" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="C40" s="1" t="s">
+      <c r="C42" s="1" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="41" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="1" t="s">
+    <row r="43" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A43" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="B41" s="1" t="s">
+      <c r="B43" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="C41" s="1" t="s">
+      <c r="C43" s="1" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="42" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="1" t="s">
+    <row r="44" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A44" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="B42" s="1" t="s">
+      <c r="B44" s="1" t="s">
         <v>115</v>
       </c>
-      <c r="C42" s="1" t="s">
+      <c r="C44" s="1" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="43" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="1" t="s">
+    <row r="45" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A45" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="B43" s="1" t="s">
+      <c r="B45" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="C43" s="1" t="s">
+      <c r="C45" s="1" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="44" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="1" t="s">
+    <row r="46" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A46" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="B44" s="1" t="s">
+      <c r="B46" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="C44" s="1" t="s">
+      <c r="C46" s="1" t="s">
         <v>122</v>
       </c>
     </row>
-    <row r="45" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="1" t="s">
+    <row r="47" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A47" s="1" t="s">
         <v>123</v>
       </c>
-      <c r="B45" s="1" t="s">
+      <c r="B47" s="1" t="s">
         <v>124</v>
       </c>
-      <c r="C45" s="1" t="s">
+      <c r="C47" s="1" t="s">
         <v>125</v>
       </c>
     </row>
-    <row r="46" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A46" s="1" t="s">
+    <row r="48" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A48" s="1" t="s">
         <v>126</v>
       </c>
-      <c r="B46" s="1" t="s">
+      <c r="B48" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="C46" s="1" t="s">
+      <c r="C48" s="1" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="47" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="1" t="s">
+    <row r="49" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A49" s="1" t="s">
         <v>129</v>
       </c>
-      <c r="B47" s="1" t="s">
+      <c r="B49" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="C47" s="1" t="s">
+      <c r="C49" s="1" t="s">
         <v>131</v>
       </c>
     </row>
-    <row r="48" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="1" t="s">
+    <row r="50" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A50" s="1" t="s">
         <v>132</v>
       </c>
-      <c r="B48" s="1" t="s">
+      <c r="B50" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="C48" s="1" t="s">
+      <c r="C50" s="1" t="s">
         <v>131</v>
       </c>
     </row>
-    <row r="49" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="1" t="s">
+    <row r="51" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A51" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="B49" s="1" t="s">
+      <c r="B51" s="1" t="s">
         <v>134</v>
       </c>
-      <c r="C49" s="1" t="s">
+      <c r="C51" s="1" t="s">
         <v>135</v>
       </c>
     </row>
-    <row r="50" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A50" s="1" t="s">
+    <row r="52" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A52" s="1" t="s">
         <v>136</v>
       </c>
-      <c r="B50" s="1" t="s">
+      <c r="B52" s="1" t="s">
         <v>134</v>
       </c>
-      <c r="C50" s="1" t="s">
+      <c r="C52" s="1" t="s">
         <v>135</v>
       </c>
     </row>
-    <row r="51" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A51" s="1" t="s">
+    <row r="53" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A53" s="1" t="s">
         <v>137</v>
       </c>
-      <c r="B51" s="1" t="s">
+      <c r="B53" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="C51" s="1" t="s">
+      <c r="C53" s="1" t="s">
         <v>139</v>
       </c>
     </row>
-    <row r="52" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A52" s="1" t="s">
+    <row r="54" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A54" s="1" t="s">
         <v>140</v>
       </c>
-      <c r="B52" s="1" t="s">
+      <c r="B54" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="C52" s="1" t="s">
+      <c r="C54" s="1" t="s">
         <v>139</v>
       </c>
     </row>
-    <row r="53" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A53" s="1" t="s">
+    <row r="55" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A55" s="1" t="s">
         <v>141</v>
       </c>
-      <c r="B53" s="1" t="s">
+      <c r="B55" s="1" t="s">
         <v>142</v>
       </c>
-      <c r="C53" s="1" t="s">
+      <c r="C55" s="1" t="s">
         <v>143</v>
       </c>
     </row>
-    <row r="54" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A54" s="1" t="s">
+    <row r="56" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A56" s="1" t="s">
         <v>144</v>
       </c>
-      <c r="B54" s="1" t="s">
+      <c r="B56" s="1" t="s">
         <v>145</v>
       </c>
-      <c r="C54" s="1" t="s">
+      <c r="C56" s="1" t="s">
         <v>146</v>
       </c>
     </row>
-    <row r="55" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A55" s="1" t="s">
+    <row r="57" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A57" s="1" t="s">
         <v>147</v>
       </c>
-      <c r="B55" s="1" t="s">
+      <c r="B57" s="1" t="s">
         <v>148</v>
       </c>
-      <c r="C55" s="1" t="s">
+      <c r="C57" s="1" t="s">
         <v>149</v>
       </c>
     </row>
-    <row r="56" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A56" s="1" t="s">
+    <row r="58" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A58" s="1" t="s">
         <v>150</v>
       </c>
-      <c r="B56" s="1" t="s">
+      <c r="B58" s="1" t="s">
         <v>151</v>
       </c>
-      <c r="C56" s="1" t="s">
+      <c r="C58" s="1" t="s">
         <v>152</v>
       </c>
     </row>
-    <row r="57" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A57" s="1" t="s">
+    <row r="59" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A59" s="1" t="s">
         <v>153</v>
       </c>
-      <c r="B57" s="1" t="s">
+      <c r="B59" s="1" t="s">
         <v>154</v>
       </c>
-      <c r="C57" s="1" t="s">
+      <c r="C59" s="1" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="58" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A58" s="1" t="s">
+    <row r="60" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A60" s="1" t="s">
         <v>156</v>
       </c>
-      <c r="B58" s="1" t="s">
+      <c r="B60" s="1" t="s">
         <v>157</v>
       </c>
-      <c r="C58" s="1" t="s">
+      <c r="C60" s="1" t="s">
         <v>158</v>
       </c>
     </row>
-    <row r="59" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A59" s="1" t="s">
+    <row r="61" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A61" s="1" t="s">
         <v>159</v>
       </c>
-      <c r="B59" s="1" t="s">
+      <c r="B61" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="C59" s="1" t="s">
+      <c r="C61" s="1" t="s">
         <v>131</v>
       </c>
     </row>
-    <row r="60" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A60" s="1" t="s">
+    <row r="62" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A62" s="1" t="s">
         <v>160</v>
       </c>
-      <c r="B60" s="1" t="s">
+      <c r="B62" s="1" t="s">
         <v>161</v>
       </c>
-      <c r="C60" s="1" t="s">
+      <c r="C62" s="1" t="s">
         <v>162</v>
       </c>
     </row>
-    <row r="61" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A61" s="1" t="s">
+    <row r="63" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A63" s="1" t="s">
         <v>163</v>
       </c>
-      <c r="B61" s="1" t="s">
+      <c r="B63" s="1" t="s">
         <v>164</v>
       </c>
-      <c r="C61" s="1" t="s">
+      <c r="C63" s="1" t="s">
         <v>165</v>
       </c>
     </row>
-    <row r="62" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A62" s="1" t="s">
+    <row r="64" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A64" s="1" t="s">
         <v>166</v>
       </c>
-      <c r="B62" s="1" t="s">
+      <c r="B64" s="1" t="s">
         <v>167</v>
       </c>
-      <c r="C62" s="1" t="s">
+      <c r="C64" s="1" t="s">
         <v>168</v>
       </c>
     </row>
-    <row r="63" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A63" s="1" t="s">
+    <row r="65" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A65" s="1" t="s">
         <v>169</v>
       </c>
-      <c r="B63" s="1" t="s">
+      <c r="B65" s="1" t="s">
         <v>170</v>
       </c>
-      <c r="C63" s="1" t="s">
+      <c r="C65" s="1" t="s">
         <v>171</v>
       </c>
     </row>
-    <row r="64" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A64" s="1" t="s">
+    <row r="66" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A66" s="1" t="s">
         <v>172</v>
       </c>
-      <c r="B64" s="1" t="s">
+      <c r="B66" s="1" t="s">
         <v>173</v>
       </c>
-      <c r="C64" s="1" t="s">
+      <c r="C66" s="1" t="s">
         <v>174</v>
       </c>
     </row>
-    <row r="65" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A65" s="1" t="s">
+    <row r="67" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A67" s="1" t="s">
         <v>175</v>
       </c>
-      <c r="B65" s="1" t="s">
+      <c r="B67" s="1" t="s">
         <v>176</v>
       </c>
-      <c r="C65" s="1" t="s">
+      <c r="C67" s="1" t="s">
         <v>177</v>
       </c>
     </row>
-    <row r="66" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A66" s="1" t="s">
+    <row r="68" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A68" s="1" t="s">
         <v>178</v>
       </c>
-      <c r="B66" s="1" t="s">
+      <c r="B68" s="1" t="s">
         <v>176</v>
       </c>
-      <c r="C66" s="1" t="s">
+      <c r="C68" s="1" t="s">
         <v>177</v>
       </c>
     </row>
-    <row r="67" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A67" s="1" t="s">
+    <row r="69" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A69" s="1" t="s">
         <v>179</v>
       </c>
-      <c r="B67" s="1" t="s">
+      <c r="B69" s="1" t="s">
         <v>180</v>
       </c>
-      <c r="C67" s="1" t="s">
+      <c r="C69" s="1" t="s">
         <v>181</v>
       </c>
     </row>
-    <row r="68" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A68" s="1" t="s">
+    <row r="70" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A70" s="1" t="s">
         <v>182</v>
       </c>
-      <c r="B68" s="1" t="s">
+      <c r="B70" s="1" t="s">
         <v>180</v>
       </c>
-      <c r="C68" s="1" t="s">
+      <c r="C70" s="1" t="s">
         <v>181</v>
       </c>
     </row>
-    <row r="69" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A69" s="1" t="s">
+    <row r="71" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A71" s="1" t="s">
         <v>183</v>
       </c>
-      <c r="B69" s="1" t="s">
+      <c r="B71" s="1" t="s">
         <v>184</v>
       </c>
-      <c r="C69" s="1" t="s">
+      <c r="C71" s="1" t="s">
         <v>185</v>
       </c>
     </row>
-    <row r="70" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A70" s="1" t="s">
+    <row r="72" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A72" s="1" t="s">
         <v>186</v>
       </c>
-      <c r="B70" s="1" t="s">
+      <c r="B72" s="1" t="s">
         <v>187</v>
       </c>
-      <c r="C70" s="1" t="s">
+      <c r="C72" s="1" t="s">
         <v>187</v>
       </c>
     </row>
-    <row r="71" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A71" s="1" t="s">
+    <row r="73" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A73" s="1" t="s">
         <v>188</v>
       </c>
-      <c r="B71" s="1" t="s">
+      <c r="B73" s="1" t="s">
         <v>187</v>
       </c>
-      <c r="C71" s="1" t="s">
+      <c r="C73" s="1" t="s">
         <v>187</v>
       </c>
     </row>
-    <row r="72" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A72" s="1" t="s">
+    <row r="74" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A74" s="1" t="s">
         <v>189</v>
       </c>
-      <c r="B72" s="1" t="s">
+      <c r="B74" s="1" t="s">
         <v>190</v>
       </c>
-      <c r="C72" s="1" t="s">
+      <c r="C74" s="1" t="s">
         <v>191</v>
       </c>
     </row>
-    <row r="73" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A73" s="1" t="s">
+    <row r="75" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A75" s="1" t="s">
         <v>192</v>
-      </c>
-      <c r="B73" s="1" t="s">
-        <v>157</v>
-      </c>
-      <c r="C73" s="1" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="74" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A74" s="1" t="s">
-        <v>193</v>
-      </c>
-      <c r="B74" s="1" t="s">
-        <v>194</v>
-      </c>
-      <c r="C74" s="1" t="s">
-        <v>195</v>
-      </c>
-    </row>
-    <row r="75" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A75" s="1" t="s">
-        <v>196</v>
       </c>
       <c r="B75" s="1" t="s">
         <v>157</v>
@@ -2502,240 +2520,240 @@
         <v>158</v>
       </c>
     </row>
-    <row r="76" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A76" s="1" t="s">
+        <v>193</v>
+      </c>
+      <c r="B76" s="1" t="s">
+        <v>194</v>
+      </c>
+      <c r="C76" s="1" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="77" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A77" s="1" t="s">
+        <v>196</v>
+      </c>
+      <c r="B77" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="C77" s="1" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="78" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A78" s="1" t="s">
         <v>197</v>
       </c>
-      <c r="B76" s="1" t="s">
+      <c r="B78" s="1" t="s">
         <v>198</v>
       </c>
-      <c r="C76" s="1" t="s">
+      <c r="C78" s="1" t="s">
         <v>199</v>
       </c>
     </row>
-    <row r="77" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A77" s="1" t="s">
+    <row r="79" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A79" s="1" t="s">
         <v>200</v>
       </c>
-      <c r="B77" s="1" t="s">
+      <c r="B79" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="C77" s="1" t="s">
+      <c r="C79" s="1" t="s">
         <v>202</v>
       </c>
     </row>
-    <row r="78" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A78" s="1" t="s">
+    <row r="80" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A80" s="1" t="s">
         <v>203</v>
       </c>
-      <c r="B78" s="1" t="s">
+      <c r="B80" s="1" t="s">
         <v>204</v>
       </c>
-      <c r="C78" s="1" t="s">
+      <c r="C80" s="1" t="s">
         <v>205</v>
       </c>
     </row>
-    <row r="79" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A79" s="1" t="s">
+    <row r="81" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A81" s="1" t="s">
         <v>206</v>
       </c>
-      <c r="B79" s="1" t="s">
+      <c r="B81" s="1" t="s">
         <v>207</v>
       </c>
-      <c r="C79" s="1" t="s">
+      <c r="C81" s="1" t="s">
         <v>208</v>
       </c>
     </row>
-    <row r="80" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A80" s="1" t="s">
+    <row r="82" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A82" s="1" t="s">
         <v>209</v>
       </c>
-      <c r="B80" s="1" t="s">
+      <c r="B82" s="1" t="s">
         <v>157</v>
       </c>
-      <c r="C80" s="1" t="s">
+      <c r="C82" s="1" t="s">
         <v>158</v>
       </c>
     </row>
-    <row r="81" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A81" s="1" t="s">
+    <row r="83" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A83" s="1" t="s">
         <v>210</v>
       </c>
-      <c r="B81" s="1" t="s">
+      <c r="B83" s="1" t="s">
         <v>211</v>
       </c>
-      <c r="C81" s="1" t="s">
+      <c r="C83" s="1" t="s">
         <v>212</v>
       </c>
     </row>
-    <row r="82" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A82" s="1" t="s">
+    <row r="84" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A84" s="1" t="s">
         <v>213</v>
       </c>
-      <c r="B82" s="1" t="s">
+      <c r="B84" s="1" t="s">
         <v>148</v>
       </c>
-      <c r="C82" s="1" t="s">
+      <c r="C84" s="1" t="s">
         <v>149</v>
       </c>
     </row>
-    <row r="83" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A83" s="1" t="s">
+    <row r="85" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A85" s="1" t="s">
         <v>214</v>
       </c>
-      <c r="B83" s="1" t="s">
+      <c r="B85" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="C83" s="1" t="s">
+      <c r="C85" s="1" t="s">
         <v>139</v>
       </c>
     </row>
-    <row r="84" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A84" s="1" t="s">
+    <row r="86" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A86" s="1" t="s">
         <v>215</v>
       </c>
-      <c r="B84" s="1" t="s">
+      <c r="B86" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="C84" s="1" t="s">
+      <c r="C86" s="1" t="s">
         <v>139</v>
       </c>
     </row>
-    <row r="85" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A85" s="1" t="s">
+    <row r="87" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A87" s="1" t="s">
         <v>216</v>
       </c>
-      <c r="B85" s="1" t="s">
+      <c r="B87" s="1" t="s">
         <v>145</v>
       </c>
-      <c r="C85" s="1" t="s">
+      <c r="C87" s="1" t="s">
         <v>146</v>
       </c>
     </row>
-    <row r="86" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A86" s="1" t="s">
+    <row r="88" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A88" s="1" t="s">
         <v>217</v>
       </c>
-      <c r="B86" s="1" t="s">
+      <c r="B88" s="1" t="s">
         <v>218</v>
       </c>
-      <c r="C86" s="1" t="s">
+      <c r="C88" s="1" t="s">
         <v>219</v>
       </c>
     </row>
-    <row r="87" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A87" s="1" t="s">
+    <row r="89" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A89" s="1" t="s">
         <v>220</v>
       </c>
-      <c r="B87" s="1" t="s">
+      <c r="B89" s="1" t="s">
         <v>134</v>
       </c>
-      <c r="C87" s="1" t="s">
+      <c r="C89" s="1" t="s">
         <v>135</v>
       </c>
     </row>
-    <row r="88" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A88" s="1" t="s">
+    <row r="90" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A90" s="1" t="s">
         <v>221</v>
       </c>
-      <c r="B88" s="1" t="s">
+      <c r="B90" s="1" t="s">
         <v>134</v>
       </c>
-      <c r="C88" s="1" t="s">
+      <c r="C90" s="1" t="s">
         <v>135</v>
       </c>
     </row>
-    <row r="89" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A89" s="1" t="s">
+    <row r="91" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A91" s="1" t="s">
         <v>222</v>
       </c>
-      <c r="B89" s="1" t="s">
+      <c r="B91" s="1" t="s">
         <v>223</v>
       </c>
-      <c r="C89" s="1" t="s">
+      <c r="C91" s="1" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="90" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A90" s="1" t="s">
+    <row r="92" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A92" s="1" t="s">
         <v>224</v>
       </c>
-      <c r="B90" s="1" t="s">
+      <c r="B92" s="1" t="s">
         <v>223</v>
-      </c>
-      <c r="C90" s="1" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="91" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A91" s="1" t="s">
-        <v>225</v>
-      </c>
-      <c r="B91" s="1" t="s">
-        <v>190</v>
-      </c>
-      <c r="C91" s="1" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="92" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A92" s="1" t="s">
-        <v>226</v>
-      </c>
-      <c r="B92" s="1" t="s">
-        <v>154</v>
       </c>
       <c r="C92" s="1" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="93" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A93" s="1" t="s">
+        <v>225</v>
+      </c>
+      <c r="B93" s="1" t="s">
+        <v>190</v>
+      </c>
+      <c r="C93" s="1" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="94" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A94" s="1" t="s">
+        <v>226</v>
+      </c>
+      <c r="B94" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="C94" s="1" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="95" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A95" s="1" t="s">
         <v>227</v>
       </c>
-      <c r="B93" s="1" t="s">
+      <c r="B95" s="1" t="s">
         <v>228</v>
       </c>
-      <c r="C93" s="1" t="s">
+      <c r="C95" s="1" t="s">
         <v>229</v>
       </c>
     </row>
-    <row r="94" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A94" s="1" t="s">
+    <row r="96" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A96" s="1" t="s">
         <v>230</v>
       </c>
-      <c r="B94" s="1" t="s">
+      <c r="B96" s="1" t="s">
         <v>231</v>
       </c>
-      <c r="C94" s="1" t="s">
+      <c r="C96" s="1" t="s">
         <v>232</v>
       </c>
     </row>
-    <row r="95" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A95" s="1" t="s">
+    <row r="97" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A97" s="1" t="s">
         <v>233</v>
-      </c>
-      <c r="B95" s="1" t="s">
-        <v>234</v>
-      </c>
-      <c r="C95" s="1" t="s">
-        <v>235</v>
-      </c>
-    </row>
-    <row r="96" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A96" s="1" t="s">
-        <v>236</v>
-      </c>
-      <c r="B96" s="1" t="s">
-        <v>237</v>
-      </c>
-      <c r="C96" s="1" t="s">
-        <v>238</v>
-      </c>
-    </row>
-    <row r="97" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A97" s="1" t="s">
-        <v>239</v>
       </c>
       <c r="B97" s="1" t="s">
         <v>234</v>
@@ -2744,1004 +2762,1026 @@
         <v>235</v>
       </c>
     </row>
-    <row r="98" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A98" s="1" t="s">
+        <v>236</v>
+      </c>
+      <c r="B98" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="C98" s="1" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="99" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A99" s="1" t="s">
+        <v>239</v>
+      </c>
+      <c r="B99" s="1" t="s">
+        <v>234</v>
+      </c>
+      <c r="C99" s="1" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="100" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A100" s="1" t="s">
         <v>240</v>
       </c>
-      <c r="B98" s="1" t="s">
+      <c r="B100" s="1" t="s">
         <v>241</v>
       </c>
-      <c r="C98" s="1" t="s">
+      <c r="C100" s="1" t="s">
         <v>242</v>
       </c>
     </row>
-    <row r="99" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A99" s="1" t="s">
+    <row r="101" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A101" s="1" t="s">
         <v>243</v>
       </c>
-      <c r="B99" s="1" t="s">
+      <c r="B101" s="1" t="s">
         <v>244</v>
       </c>
-      <c r="C99" s="1" t="s">
+      <c r="C101" s="1" t="s">
         <v>245</v>
       </c>
     </row>
-    <row r="100" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A100" s="1" t="s">
+    <row r="102" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A102" s="1" t="s">
         <v>246</v>
       </c>
-      <c r="B100" s="1" t="s">
+      <c r="B102" s="1" t="s">
         <v>247</v>
       </c>
-      <c r="C100" s="1" t="s">
+      <c r="C102" s="1" t="s">
         <v>248</v>
       </c>
     </row>
-    <row r="101" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A101" s="1" t="s">
+    <row r="103" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A103" s="1" t="s">
         <v>249</v>
       </c>
-      <c r="B101" s="1" t="s">
+      <c r="B103" s="1" t="s">
         <v>190</v>
       </c>
-      <c r="C101" s="1" t="s">
+      <c r="C103" s="1" t="s">
         <v>250</v>
       </c>
     </row>
-    <row r="102" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A102" s="1" t="s">
+    <row r="104" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A104" s="1" t="s">
         <v>251</v>
       </c>
-      <c r="B102" s="1" t="s">
+      <c r="B104" s="1" t="s">
         <v>252</v>
       </c>
-      <c r="C102" s="1" t="s">
+      <c r="C104" s="1" t="s">
         <v>235</v>
       </c>
     </row>
-    <row r="103" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A103" s="1" t="s">
+    <row r="105" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A105" s="1" t="s">
         <v>253</v>
       </c>
-      <c r="B103" s="1" t="s">
+      <c r="B105" s="1" t="s">
         <v>254</v>
       </c>
-      <c r="C103" s="1" t="s">
+      <c r="C105" s="1" t="s">
         <v>255</v>
       </c>
     </row>
-    <row r="104" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A104" s="1" t="s">
+    <row r="106" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A106" s="1" t="s">
         <v>256</v>
       </c>
-      <c r="B104" s="1" t="s">
+      <c r="B106" s="1" t="s">
         <v>257</v>
       </c>
-      <c r="C104" s="1" t="s">
+      <c r="C106" s="1" t="s">
         <v>258</v>
       </c>
     </row>
-    <row r="105" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A105" s="1" t="s">
+    <row r="107" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A107" s="1" t="s">
         <v>259</v>
       </c>
-      <c r="B105" s="1" t="s">
+      <c r="B107" s="1" t="s">
         <v>260</v>
       </c>
-      <c r="C105" s="1" t="s">
+      <c r="C107" s="1" t="s">
         <v>261</v>
       </c>
     </row>
-    <row r="106" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A106" s="1" t="s">
+    <row r="108" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A108" s="1" t="s">
         <v>262</v>
       </c>
-      <c r="B106" s="1" t="s">
+      <c r="B108" s="1" t="s">
         <v>263</v>
       </c>
-      <c r="C106" s="1" t="s">
+      <c r="C108" s="1" t="s">
         <v>264</v>
       </c>
     </row>
-    <row r="107" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A107" s="1" t="s">
+    <row r="109" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A109" s="1" t="s">
         <v>265</v>
       </c>
-      <c r="B107" s="1" t="s">
+      <c r="B109" s="1" t="s">
         <v>266</v>
       </c>
-      <c r="C107" s="1" t="s">
+      <c r="C109" s="1" t="s">
         <v>267</v>
       </c>
     </row>
-    <row r="108" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A108" s="1" t="s">
+    <row r="110" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A110" s="1" t="s">
         <v>268</v>
       </c>
-      <c r="B108" s="1" t="s">
+      <c r="B110" s="1" t="s">
         <v>269</v>
       </c>
-      <c r="C108" s="1" t="s">
+      <c r="C110" s="1" t="s">
         <v>270</v>
       </c>
     </row>
-    <row r="109" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A109" s="1" t="s">
+    <row r="111" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A111" s="1" t="s">
         <v>271</v>
       </c>
-      <c r="B109" s="1" t="s">
+      <c r="B111" s="1" t="s">
         <v>272</v>
       </c>
-      <c r="C109" s="1" t="s">
+      <c r="C111" s="1" t="s">
         <v>273</v>
       </c>
     </row>
-    <row r="110" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A110" s="1" t="s">
+    <row r="112" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A112" s="1" t="s">
         <v>274</v>
       </c>
-      <c r="B110" s="1" t="s">
+      <c r="B112" s="1" t="s">
         <v>275</v>
       </c>
-      <c r="C110" s="1" t="s">
+      <c r="C112" s="1" t="s">
         <v>276</v>
       </c>
     </row>
-    <row r="111" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A111" s="1" t="s">
+    <row r="113" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A113" s="1" t="s">
         <v>277</v>
       </c>
-      <c r="B111" s="1" t="s">
+      <c r="B113" s="1" t="s">
         <v>278</v>
       </c>
-      <c r="C111" s="1" t="s">
+      <c r="C113" s="1" t="s">
         <v>279</v>
       </c>
     </row>
-    <row r="112" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A112" s="1" t="s">
+    <row r="114" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A114" s="1" t="s">
         <v>280</v>
       </c>
-      <c r="B112" s="1" t="s">
+      <c r="B114" s="1" t="s">
         <v>281</v>
       </c>
-      <c r="C112" s="1" t="s">
+      <c r="C114" s="1" t="s">
         <v>282</v>
       </c>
     </row>
-    <row r="113" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A113" s="1" t="s">
+    <row r="115" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A115" s="1" t="s">
         <v>283</v>
       </c>
-      <c r="B113" s="1" t="s">
+      <c r="B115" s="1" t="s">
         <v>284</v>
       </c>
-      <c r="C113" s="1" t="s">
+      <c r="C115" s="1" t="s">
         <v>285</v>
       </c>
     </row>
-    <row r="114" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A114" s="1" t="s">
+    <row r="116" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A116" s="1" t="s">
         <v>286</v>
       </c>
-      <c r="B114" s="1" t="s">
+      <c r="B116" s="1" t="s">
         <v>287</v>
       </c>
-      <c r="C114" s="1" t="s">
+      <c r="C116" s="1" t="s">
         <v>288</v>
       </c>
     </row>
-    <row r="115" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A115" s="1" t="s">
+    <row r="117" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A117" s="1" t="s">
         <v>289</v>
       </c>
-      <c r="B115" s="1" t="s">
+      <c r="B117" s="1" t="s">
         <v>290</v>
       </c>
-      <c r="C115" s="1" t="s">
+      <c r="C117" s="1" t="s">
         <v>291</v>
       </c>
     </row>
-    <row r="116" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A116" s="1" t="s">
+    <row r="118" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A118" s="1" t="s">
         <v>292</v>
       </c>
-      <c r="B116" s="1" t="s">
+      <c r="B118" s="1" t="s">
         <v>293</v>
       </c>
-      <c r="C116" s="1" t="s">
+      <c r="C118" s="1" t="s">
         <v>294</v>
       </c>
     </row>
-    <row r="117" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A117" s="1" t="s">
+    <row r="119" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A119" s="1" t="s">
         <v>295</v>
       </c>
-      <c r="B117" s="1" t="s">
+      <c r="B119" s="1" t="s">
         <v>296</v>
       </c>
-      <c r="C117" s="1" t="s">
+      <c r="C119" s="1" t="s">
         <v>297</v>
       </c>
     </row>
-    <row r="118" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A118" s="1" t="s">
+    <row r="120" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A120" s="1" t="s">
         <v>298</v>
       </c>
-      <c r="B118" s="1" t="s">
+      <c r="B120" s="1" t="s">
         <v>299</v>
       </c>
-      <c r="C118" s="1" t="s">
+      <c r="C120" s="1" t="s">
         <v>300</v>
       </c>
     </row>
-    <row r="119" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A119" s="1" t="s">
+    <row r="121" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A121" s="1" t="s">
         <v>301</v>
       </c>
-      <c r="B119" s="1" t="s">
+      <c r="B121" s="1" t="s">
         <v>302</v>
       </c>
-      <c r="C119" s="1" t="s">
+      <c r="C121" s="1" t="s">
         <v>303</v>
       </c>
     </row>
-    <row r="120" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A120" s="1" t="s">
+    <row r="122" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A122" s="1" t="s">
         <v>304</v>
       </c>
-      <c r="B120" s="1" t="s">
+      <c r="B122" s="1" t="s">
         <v>305</v>
       </c>
-      <c r="C120" s="1" t="s">
+      <c r="C122" s="1" t="s">
         <v>306</v>
       </c>
     </row>
-    <row r="121" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A121" s="1" t="s">
+    <row r="123" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A123" s="1" t="s">
         <v>307</v>
       </c>
-      <c r="B121" s="1" t="s">
+      <c r="B123" s="1" t="s">
         <v>293</v>
       </c>
-      <c r="C121" s="1" t="s">
+      <c r="C123" s="1" t="s">
         <v>294</v>
       </c>
     </row>
-    <row r="122" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A122" s="1" t="s">
+    <row r="124" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A124" s="1" t="s">
         <v>308</v>
       </c>
-      <c r="B122" s="1" t="s">
+      <c r="B124" s="1" t="s">
         <v>184</v>
       </c>
-      <c r="C122" s="1" t="s">
+      <c r="C124" s="1" t="s">
         <v>185</v>
       </c>
     </row>
-    <row r="123" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A123" s="1" t="s">
+    <row r="125" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A125" s="1" t="s">
         <v>309</v>
       </c>
-      <c r="B123" s="1" t="s">
+      <c r="B125" s="1" t="s">
         <v>310</v>
       </c>
-      <c r="C123" s="1" t="s">
+      <c r="C125" s="1" t="s">
         <v>311</v>
       </c>
     </row>
-    <row r="124" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A124" s="1" t="s">
+    <row r="126" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A126" s="1" t="s">
         <v>312</v>
       </c>
-      <c r="B124" s="1" t="s">
+      <c r="B126" s="1" t="s">
         <v>313</v>
       </c>
-      <c r="C124" s="1" t="s">
+      <c r="C126" s="1" t="s">
         <v>314</v>
       </c>
     </row>
-    <row r="125" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A125" s="1" t="s">
+    <row r="127" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A127" s="1" t="s">
         <v>315</v>
       </c>
-      <c r="B125" s="1" t="s">
+      <c r="B127" s="1" t="s">
         <v>293</v>
       </c>
-      <c r="C125" s="1" t="s">
+      <c r="C127" s="1" t="s">
         <v>294</v>
       </c>
     </row>
-    <row r="126" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A126" s="1" t="s">
+    <row r="128" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A128" s="1" t="s">
         <v>316</v>
       </c>
-      <c r="B126" s="1" t="s">
+      <c r="B128" s="1" t="s">
         <v>317</v>
       </c>
-      <c r="C126" s="1" t="s">
+      <c r="C128" s="1" t="s">
         <v>318</v>
       </c>
     </row>
-    <row r="127" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A127" s="1" t="s">
+    <row r="129" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A129" s="1" t="s">
         <v>319</v>
       </c>
-      <c r="B127" s="1" t="s">
+      <c r="B129" s="1" t="s">
         <v>320</v>
       </c>
-      <c r="C127" s="1" t="s">
+      <c r="C129" s="1" t="s">
         <v>321</v>
       </c>
     </row>
-    <row r="128" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A128" s="1" t="s">
+    <row r="130" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A130" s="1" t="s">
         <v>322</v>
       </c>
-      <c r="B128" s="1" t="s">
+      <c r="B130" s="1" t="s">
         <v>323</v>
       </c>
-      <c r="C128" s="1" t="s">
+      <c r="C130" s="1" t="s">
         <v>324</v>
       </c>
     </row>
-    <row r="129" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A129" s="1" t="s">
+    <row r="131" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A131" s="1" t="s">
         <v>325</v>
       </c>
-      <c r="B129" s="1" t="s">
+      <c r="B131" s="1" t="s">
         <v>293</v>
       </c>
-      <c r="C129" s="1" t="s">
+      <c r="C131" s="1" t="s">
         <v>294</v>
       </c>
     </row>
-    <row r="130" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A130" s="1" t="s">
+    <row r="132" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A132" s="1" t="s">
         <v>326</v>
       </c>
-      <c r="B130" s="1" t="s">
+      <c r="B132" s="1" t="s">
         <v>317</v>
       </c>
-      <c r="C130" s="1" t="s">
+      <c r="C132" s="1" t="s">
         <v>318</v>
       </c>
     </row>
-    <row r="131" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A131" s="1" t="s">
+    <row r="133" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A133" s="1" t="s">
         <v>327</v>
       </c>
-      <c r="B131" s="1" t="s">
+      <c r="B133" s="1" t="s">
         <v>328</v>
       </c>
-      <c r="C131" s="1" t="s">
+      <c r="C133" s="1" t="s">
         <v>329</v>
       </c>
     </row>
-    <row r="132" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A132" s="1" t="s">
+    <row r="134" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A134" s="1" t="s">
         <v>330</v>
       </c>
-      <c r="B132" s="1" t="s">
+      <c r="B134" s="1" t="s">
         <v>331</v>
       </c>
-      <c r="C132" s="1" t="s">
+      <c r="C134" s="1" t="s">
         <v>332</v>
       </c>
     </row>
-    <row r="133" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A133" s="1" t="s">
+    <row r="135" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A135" s="1" t="s">
         <v>333</v>
       </c>
-      <c r="B133" s="1" t="s">
+      <c r="B135" s="1" t="s">
         <v>293</v>
       </c>
-      <c r="C133" s="1" t="s">
+      <c r="C135" s="1" t="s">
         <v>294</v>
       </c>
     </row>
-    <row r="134" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A134" s="1" t="s">
+    <row r="136" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A136" s="1" t="s">
         <v>334</v>
       </c>
-      <c r="B134" s="1" t="s">
+      <c r="B136" s="1" t="s">
         <v>335</v>
       </c>
-      <c r="C134" s="1" t="s">
+      <c r="C136" s="1" t="s">
         <v>336</v>
       </c>
     </row>
-    <row r="135" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A135" s="1" t="s">
+    <row r="137" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A137" s="1" t="s">
         <v>337</v>
       </c>
-      <c r="B135" s="1" t="s">
+      <c r="B137" s="1" t="s">
         <v>320</v>
       </c>
-      <c r="C135" s="1" t="s">
+      <c r="C137" s="1" t="s">
         <v>321</v>
       </c>
     </row>
-    <row r="136" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A136" s="1" t="s">
+    <row r="138" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A138" s="1" t="s">
         <v>338</v>
       </c>
-      <c r="B136" s="1" t="s">
+      <c r="B138" s="1" t="s">
         <v>339</v>
       </c>
-      <c r="C136" s="1" t="s">
+      <c r="C138" s="1" t="s">
         <v>340</v>
       </c>
     </row>
-    <row r="137" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A137" s="1" t="s">
+    <row r="139" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A139" s="1" t="s">
         <v>341</v>
       </c>
-      <c r="B137" s="1" t="s">
+      <c r="B139" s="1" t="s">
         <v>342</v>
       </c>
-      <c r="C137" s="1" t="s">
+      <c r="C139" s="1" t="s">
         <v>343</v>
       </c>
     </row>
-    <row r="138" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A138" s="1" t="s">
+    <row r="140" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A140" s="1" t="s">
         <v>344</v>
       </c>
-      <c r="B138" s="1" t="s">
+      <c r="B140" s="1" t="s">
         <v>293</v>
       </c>
-      <c r="C138" s="1" t="s">
+      <c r="C140" s="1" t="s">
         <v>294</v>
       </c>
     </row>
-    <row r="139" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A139" s="1" t="s">
+    <row r="141" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A141" s="1" t="s">
         <v>345</v>
       </c>
-      <c r="B139" s="1" t="s">
+      <c r="B141" s="1" t="s">
         <v>346</v>
       </c>
-      <c r="C139" s="1" t="s">
+      <c r="C141" s="1" t="s">
         <v>347</v>
       </c>
     </row>
-    <row r="140" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A140" s="1" t="s">
+    <row r="142" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A142" s="1" t="s">
         <v>348</v>
       </c>
-      <c r="B140" s="1" t="s">
+      <c r="B142" s="1" t="s">
         <v>349</v>
       </c>
-      <c r="C140" s="1" t="s">
+      <c r="C142" s="1" t="s">
         <v>350</v>
       </c>
     </row>
-    <row r="141" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A141" s="1" t="s">
+    <row r="143" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A143" s="1" t="s">
         <v>351</v>
       </c>
-      <c r="B141" s="1" t="s">
+      <c r="B143" s="1" t="s">
         <v>352</v>
       </c>
-      <c r="C141" s="1" t="s">
+      <c r="C143" s="1" t="s">
         <v>353</v>
       </c>
     </row>
-    <row r="142" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A142" s="1" t="s">
+    <row r="144" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A144" s="1" t="s">
         <v>354</v>
       </c>
-      <c r="B142" s="1" t="s">
+      <c r="B144" s="1" t="s">
         <v>293</v>
       </c>
-      <c r="C142" s="1" t="s">
+      <c r="C144" s="1" t="s">
         <v>294</v>
       </c>
     </row>
-    <row r="143" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A143" s="1" t="s">
+    <row r="145" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A145" s="1" t="s">
         <v>355</v>
       </c>
-      <c r="B143" s="1" t="s">
+      <c r="B145" s="1" t="s">
         <v>356</v>
       </c>
-      <c r="C143" s="1" t="s">
+      <c r="C145" s="1" t="s">
         <v>357</v>
       </c>
     </row>
-    <row r="144" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A144" s="1" t="s">
+    <row r="146" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A146" s="1" t="s">
         <v>358</v>
       </c>
-      <c r="B144" s="1" t="s">
+      <c r="B146" s="1" t="s">
         <v>359</v>
       </c>
-      <c r="C144" s="1" t="s">
+      <c r="C146" s="1" t="s">
         <v>360</v>
       </c>
     </row>
-    <row r="145" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A145" s="1" t="s">
+    <row r="147" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A147" s="1" t="s">
         <v>361</v>
       </c>
-      <c r="B145" s="1" t="s">
+      <c r="B147" s="1" t="s">
         <v>362</v>
       </c>
-      <c r="C145" s="1" t="s">
+      <c r="C147" s="1" t="s">
         <v>363</v>
       </c>
     </row>
-    <row r="146" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A146" s="1" t="s">
+    <row r="148" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A148" s="1" t="s">
         <v>364</v>
       </c>
-      <c r="B146" s="1" t="s">
+      <c r="B148" s="1" t="s">
         <v>365</v>
       </c>
-      <c r="C146" s="1" t="s">
+      <c r="C148" s="1" t="s">
         <v>366</v>
       </c>
     </row>
-    <row r="147" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A147" s="1" t="s">
+    <row r="149" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A149" s="1" t="s">
         <v>367</v>
       </c>
-      <c r="B147" s="1" t="s">
+      <c r="B149" s="1" t="s">
         <v>368</v>
       </c>
-      <c r="C147" s="1" t="s">
+      <c r="C149" s="1" t="s">
         <v>369</v>
       </c>
     </row>
-    <row r="148" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A148" s="1" t="s">
+    <row r="150" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A150" s="1" t="s">
         <v>370</v>
       </c>
-      <c r="B148" s="1" t="s">
+      <c r="B150" s="1" t="s">
         <v>293</v>
       </c>
-      <c r="C148" s="1" t="s">
+      <c r="C150" s="1" t="s">
         <v>294</v>
       </c>
     </row>
-    <row r="149" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A149" s="1" t="s">
+    <row r="151" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A151" s="1" t="s">
         <v>371</v>
       </c>
-      <c r="B149" s="1" t="s">
+      <c r="B151" s="1" t="s">
         <v>372</v>
       </c>
-      <c r="C149" s="1" t="s">
+      <c r="C151" s="1" t="s">
         <v>373</v>
       </c>
     </row>
-    <row r="150" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A150" s="1" t="s">
+    <row r="152" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A152" s="1" t="s">
         <v>374</v>
       </c>
-      <c r="B150" s="1" t="s">
+      <c r="B152" s="1" t="s">
         <v>375</v>
       </c>
-      <c r="C150" s="1" t="s">
+      <c r="C152" s="1" t="s">
         <v>376</v>
       </c>
     </row>
-    <row r="151" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A151" s="1" t="s">
+    <row r="153" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A153" s="1" t="s">
         <v>377</v>
       </c>
-      <c r="B151" s="1" t="s">
+      <c r="B153" s="1" t="s">
         <v>378</v>
       </c>
-      <c r="C151" s="1" t="s">
+      <c r="C153" s="1" t="s">
         <v>379</v>
       </c>
     </row>
-    <row r="152" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A152" s="1" t="s">
+    <row r="154" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A154" s="1" t="s">
         <v>380</v>
       </c>
-      <c r="B152" s="1" t="s">
+      <c r="B154" s="1" t="s">
         <v>293</v>
       </c>
-      <c r="C152" s="1" t="s">
+      <c r="C154" s="1" t="s">
         <v>294</v>
       </c>
     </row>
-    <row r="153" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A153" s="1" t="s">
+    <row r="155" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A155" s="1" t="s">
         <v>381</v>
       </c>
-      <c r="B153" s="1" t="s">
+      <c r="B155" s="1" t="s">
         <v>244</v>
       </c>
-      <c r="C153" s="1" t="s">
+      <c r="C155" s="1" t="s">
         <v>245</v>
       </c>
     </row>
-    <row r="154" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A154" s="1" t="s">
+    <row r="156" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A156" s="1" t="s">
         <v>382</v>
       </c>
-      <c r="B154" s="1" t="s">
+      <c r="B156" s="1" t="s">
         <v>383</v>
       </c>
-      <c r="C154" s="1" t="s">
+      <c r="C156" s="1" t="s">
         <v>384</v>
       </c>
     </row>
-    <row r="155" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A155" s="1" t="s">
+    <row r="157" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A157" s="1" t="s">
         <v>385</v>
       </c>
-      <c r="B155" s="1" t="s">
+      <c r="B157" s="1" t="s">
         <v>386</v>
       </c>
-      <c r="C155" s="1" t="s">
+      <c r="C157" s="1" t="s">
         <v>387</v>
       </c>
     </row>
-    <row r="156" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A156" s="1" t="s">
+    <row r="158" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A158" s="1" t="s">
         <v>388</v>
       </c>
-      <c r="B156" s="1" t="s">
+      <c r="B158" s="1" t="s">
         <v>389</v>
       </c>
-      <c r="C156" s="1" t="s">
+      <c r="C158" s="1" t="s">
         <v>390</v>
       </c>
     </row>
-    <row r="157" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A157" s="1" t="s">
+    <row r="159" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A159" s="1" t="s">
         <v>391</v>
       </c>
-      <c r="B157" s="1" t="s">
+      <c r="B159" s="1" t="s">
         <v>392</v>
       </c>
-      <c r="C157" s="1" t="s">
+      <c r="C159" s="1" t="s">
         <v>393</v>
       </c>
     </row>
-    <row r="158" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A158" s="1" t="s">
+    <row r="160" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A160" s="1" t="s">
         <v>394</v>
       </c>
-      <c r="B158" s="1" t="s">
+      <c r="B160" s="1" t="s">
         <v>395</v>
       </c>
-      <c r="C158" s="1" t="s">
+      <c r="C160" s="1" t="s">
         <v>396</v>
       </c>
     </row>
-    <row r="159" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A159" s="1" t="s">
+    <row r="161" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A161" s="1" t="s">
         <v>397</v>
       </c>
-      <c r="B159" s="1" t="s">
+      <c r="B161" s="1" t="s">
         <v>293</v>
       </c>
-      <c r="C159" s="1" t="s">
+      <c r="C161" s="1" t="s">
         <v>294</v>
       </c>
     </row>
-    <row r="160" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A160" s="1" t="s">
+    <row r="162" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A162" s="1" t="s">
         <v>398</v>
       </c>
-      <c r="B160" s="1" t="s">
+      <c r="B162" s="1" t="s">
         <v>317</v>
       </c>
-      <c r="C160" s="1" t="s">
+      <c r="C162" s="1" t="s">
         <v>318</v>
       </c>
     </row>
-    <row r="161" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A161" s="1" t="s">
+    <row r="163" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A163" s="1" t="s">
         <v>399</v>
       </c>
-      <c r="B161" s="1" t="s">
+      <c r="B163" s="1" t="s">
         <v>400</v>
       </c>
-      <c r="C161" s="1" t="s">
+      <c r="C163" s="1" t="s">
         <v>401</v>
       </c>
     </row>
-    <row r="162" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A162" s="1" t="s">
+    <row r="164" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A164" s="1" t="s">
         <v>402</v>
       </c>
-      <c r="B162" s="1" t="s">
+      <c r="B164" s="1" t="s">
         <v>320</v>
       </c>
-      <c r="C162" s="1" t="s">
+      <c r="C164" s="1" t="s">
         <v>321</v>
       </c>
     </row>
-    <row r="163" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A163" s="1" t="s">
+    <row r="165" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A165" s="1" t="s">
         <v>403</v>
       </c>
-      <c r="B163" s="1" t="s">
+      <c r="B165" s="1" t="s">
         <v>404</v>
       </c>
-      <c r="C163" s="1" t="s">
+      <c r="C165" s="1" t="s">
         <v>405</v>
       </c>
     </row>
-    <row r="164" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A164" s="1" t="s">
+    <row r="166" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A166" s="1" t="s">
         <v>406</v>
       </c>
-      <c r="B164" s="1" t="s">
+      <c r="B166" s="1" t="s">
         <v>407</v>
       </c>
-      <c r="C164" s="1" t="s">
+      <c r="C166" s="1" t="s">
         <v>408</v>
       </c>
     </row>
-    <row r="165" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A165" s="1" t="s">
+    <row r="167" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A167" s="1" t="s">
         <v>409</v>
       </c>
-      <c r="B165" s="1" t="s">
+      <c r="B167" s="1" t="s">
         <v>410</v>
       </c>
-      <c r="C165" s="1" t="s">
+      <c r="C167" s="1" t="s">
         <v>411</v>
       </c>
     </row>
-    <row r="166" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A166" s="1" t="s">
+    <row r="168" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A168" s="1" t="s">
         <v>412</v>
       </c>
-      <c r="B166" s="1" t="s">
+      <c r="B168" s="1" t="s">
         <v>413</v>
       </c>
-      <c r="C166" s="1" t="s">
+      <c r="C168" s="1" t="s">
         <v>414</v>
       </c>
     </row>
-    <row r="167" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A167" s="1" t="s">
+    <row r="169" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A169" s="1" t="s">
         <v>415</v>
       </c>
-      <c r="B167" s="1" t="s">
+      <c r="B169" s="1" t="s">
         <v>416</v>
       </c>
-      <c r="C167" s="1" t="s">
+      <c r="C169" s="1" t="s">
         <v>417</v>
       </c>
     </row>
-    <row r="168" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A168" s="1" t="s">
+    <row r="170" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A170" s="1" t="s">
         <v>418</v>
       </c>
-      <c r="B168" s="1" t="s">
+      <c r="B170" s="1" t="s">
         <v>419</v>
       </c>
-      <c r="C168" s="1" t="s">
+      <c r="C170" s="1" t="s">
         <v>420</v>
       </c>
     </row>
-    <row r="169" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A169" s="1" t="s">
+    <row r="171" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A171" s="1" t="s">
         <v>421</v>
       </c>
-      <c r="B169" s="1" t="s">
+      <c r="B171" s="1" t="s">
         <v>422</v>
       </c>
-      <c r="C169" s="1" t="s">
+      <c r="C171" s="1" t="s">
         <v>423</v>
       </c>
     </row>
-    <row r="170" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A170" s="1" t="s">
+    <row r="172" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A172" s="1" t="s">
         <v>424</v>
       </c>
-      <c r="B170" s="1" t="s">
+      <c r="B172" s="1" t="s">
         <v>425</v>
       </c>
-      <c r="C170" s="1" t="s">
+      <c r="C172" s="1" t="s">
         <v>426</v>
       </c>
     </row>
-    <row r="171" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A171" s="1" t="s">
+    <row r="173" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A173" s="1" t="s">
         <v>427</v>
       </c>
-      <c r="B171" s="1" t="s">
+      <c r="B173" s="1" t="s">
         <v>428</v>
       </c>
-      <c r="C171" s="1" t="s">
+      <c r="C173" s="1" t="s">
         <v>429</v>
       </c>
     </row>
-    <row r="172" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A172" s="1" t="s">
+    <row r="174" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A174" s="1" t="s">
         <v>430</v>
       </c>
-      <c r="B172" s="1" t="s">
+      <c r="B174" s="1" t="s">
         <v>431</v>
       </c>
-      <c r="C172" s="1" t="s">
+      <c r="C174" s="1" t="s">
         <v>432</v>
       </c>
     </row>
-    <row r="173" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A173" s="1" t="s">
+    <row r="175" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A175" s="1" t="s">
         <v>433</v>
       </c>
-      <c r="B173" s="1" t="s">
+      <c r="B175" s="1" t="s">
         <v>434</v>
       </c>
-      <c r="C173" s="1" t="s">
+      <c r="C175" s="1" t="s">
         <v>435</v>
       </c>
     </row>
-    <row r="174" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A174" s="1" t="s">
+    <row r="176" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A176" s="1" t="s">
         <v>436</v>
       </c>
-      <c r="B174" s="1" t="s">
+      <c r="B176" s="1" t="s">
         <v>437</v>
       </c>
-      <c r="C174" s="1" t="s">
+      <c r="C176" s="1" t="s">
         <v>438</v>
       </c>
     </row>
-    <row r="175" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A175" s="1" t="s">
+    <row r="177" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A177" s="1" t="s">
         <v>439</v>
       </c>
-      <c r="B175" s="1" t="s">
+      <c r="B177" s="1" t="s">
         <v>440</v>
       </c>
-      <c r="C175" s="1" t="s">
+      <c r="C177" s="1" t="s">
         <v>441</v>
       </c>
     </row>
-    <row r="176" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A176" s="1" t="s">
+    <row r="178" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A178" s="1" t="s">
         <v>442</v>
       </c>
-      <c r="B176" s="1" t="s">
+      <c r="B178" s="1" t="s">
         <v>443</v>
       </c>
-      <c r="C176" s="1" t="s">
+      <c r="C178" s="1" t="s">
         <v>444</v>
       </c>
     </row>
-    <row r="177" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A177" s="1" t="s">
+    <row r="179" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A179" s="1" t="s">
         <v>445</v>
       </c>
-      <c r="B177" s="1" t="s">
+      <c r="B179" s="1" t="s">
         <v>446</v>
       </c>
-      <c r="C177" s="1" t="s">
+      <c r="C179" s="1" t="s">
         <v>447</v>
       </c>
     </row>
-    <row r="178" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A178" s="1" t="s">
+    <row r="180" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A180" s="1" t="s">
         <v>448</v>
       </c>
-      <c r="B178" s="1" t="s">
+      <c r="B180" s="1" t="s">
         <v>449</v>
       </c>
-      <c r="C178" s="1" t="s">
+      <c r="C180" s="1" t="s">
         <v>432</v>
       </c>
     </row>
-    <row r="179" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A179" s="1" t="s">
+    <row r="181" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A181" s="1" t="s">
         <v>450</v>
       </c>
-      <c r="B179" s="1" t="s">
+      <c r="B181" s="1" t="s">
         <v>293</v>
       </c>
-      <c r="C179" s="1" t="s">
+      <c r="C181" s="1" t="s">
         <v>294</v>
       </c>
     </row>
-    <row r="180" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A180" s="1" t="s">
+    <row r="182" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A182" s="1" t="s">
         <v>451</v>
       </c>
-      <c r="B180" s="1" t="s">
+      <c r="B182" s="1" t="s">
         <v>446</v>
       </c>
-      <c r="C180" s="1" t="s">
+      <c r="C182" s="1" t="s">
         <v>447</v>
       </c>
     </row>
-    <row r="181" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A181" s="1" t="s">
+    <row r="183" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A183" s="1" t="s">
         <v>452</v>
       </c>
-      <c r="B181" s="1" t="s">
+      <c r="B183" s="1" t="s">
         <v>443</v>
       </c>
-      <c r="C181" s="1" t="s">
+      <c r="C183" s="1" t="s">
         <v>444</v>
       </c>
     </row>
-    <row r="182" spans="1:3" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A182" s="1" t="s">
+    <row r="184" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A184" s="1" t="s">
         <v>453</v>
       </c>
-      <c r="B182" s="1" t="s">
+      <c r="B184" s="1" t="s">
         <v>437</v>
       </c>
-      <c r="C182" s="1" t="s">
+      <c r="C184" s="1" t="s">
         <v>438</v>
       </c>
     </row>
-    <row r="183" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A183" t="s">
+    <row r="185" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A185" t="s">
         <v>454</v>
       </c>
-      <c r="B183" t="s">
+      <c r="B185" t="s">
         <v>293</v>
       </c>
-      <c r="C183" t="s">
+      <c r="C185" t="s">
         <v>294</v>
       </c>
     </row>
-    <row r="184" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A184" t="s">
+    <row r="186" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A186" t="s">
         <v>455</v>
       </c>
-      <c r="B184" t="s">
+      <c r="B186" t="s">
         <v>434</v>
       </c>
-      <c r="C184" t="s">
+      <c r="C186" t="s">
         <v>435</v>
       </c>
     </row>
-    <row r="185" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A185" t="s">
+    <row r="187" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A187" t="s">
         <v>456</v>
       </c>
-      <c r="B185" t="s">
+      <c r="B187" t="s">
         <v>457</v>
       </c>
-      <c r="C185" t="s">
+      <c r="C187" t="s">
         <v>458</v>
       </c>
     </row>
-    <row r="186" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A186" t="s">
+    <row r="188" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A188" t="s">
         <v>459</v>
       </c>
-      <c r="B186" t="s">
+      <c r="B188" t="s">
         <v>460</v>
       </c>
-      <c r="C186" t="s">
+      <c r="C188" t="s">
         <v>461</v>
       </c>
     </row>
-    <row r="187" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A187" t="s">
+    <row r="189" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A189" t="s">
         <v>462</v>
       </c>
-      <c r="B187" t="s">
+      <c r="B189" t="s">
         <v>463</v>
       </c>
-      <c r="C187" t="s">
+      <c r="C189" t="s">
         <v>464</v>
       </c>
     </row>
-    <row r="188" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A188" t="s">
+    <row r="190" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A190" t="s">
         <v>465</v>
       </c>
-      <c r="B188" t="s">
+      <c r="B190" t="s">
         <v>466</v>
       </c>
-      <c r="C188" t="s">
+      <c r="C190" t="s">
         <v>467</v>
       </c>
     </row>

</xml_diff>

<commit_message>
- start game and leave game with socket - play sound on socket emitted - add redis password - simplify piece array - join room popup - room setting popup for room host - popup profile with buttons to interact with user
</commit_message>
<xml_diff>
--- a/tools/languages.xlsx
+++ b/tools/languages.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/macbook/projects/hieunm/xiangqi/Tools/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9BB9B2B3-C6FB-3049-A7FA-075D073916E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E57FDA59-661A-3745-9248-53AB46318061}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="15840" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="570" uniqueCount="477">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="603" uniqueCount="505">
   <si>
     <t>Key</t>
   </si>
@@ -133,6 +133,24 @@
     <t>menu.home</t>
   </si>
   <si>
+    <t>menu.profile</t>
+  </si>
+  <si>
+    <t>Profile</t>
+  </si>
+  <si>
+    <t>Trang cá nhân</t>
+  </si>
+  <si>
+    <t>menu.expired</t>
+  </si>
+  <si>
+    <t>Set expired</t>
+  </si>
+  <si>
+    <t>Hết hạn token</t>
+  </si>
+  <si>
     <t>menu.logout</t>
   </si>
   <si>
@@ -250,6 +268,15 @@
     <t>Đỏ tiên</t>
   </si>
   <si>
+    <t>dashboard.popup.pve-mode</t>
+  </si>
+  <si>
+    <t>PVE mode</t>
+  </si>
+  <si>
+    <t>Chơi với máy</t>
+  </si>
+  <si>
     <t>dashboard.popup.bet-amount</t>
   </si>
   <si>
@@ -1321,6 +1348,81 @@
     <t>Hòa cờ thành công</t>
   </si>
   <si>
+    <t>room.actions.settings</t>
+  </si>
+  <si>
+    <t>Room settings</t>
+  </si>
+  <si>
+    <t>Cài đặt phòng</t>
+  </si>
+  <si>
+    <t>room.settings.title</t>
+  </si>
+  <si>
+    <t>Room Settings</t>
+  </si>
+  <si>
+    <t>room.settings.room-name</t>
+  </si>
+  <si>
+    <t>Room name</t>
+  </si>
+  <si>
+    <t>Tên phòng</t>
+  </si>
+  <si>
+    <t>room.settings.save</t>
+  </si>
+  <si>
+    <t>Save</t>
+  </si>
+  <si>
+    <t>Lưu</t>
+  </si>
+  <si>
+    <t>update-room.messages.success</t>
+  </si>
+  <si>
+    <t>Room updated successfully</t>
+  </si>
+  <si>
+    <t>Cập nhật phòng thành công</t>
+  </si>
+  <si>
+    <t>update-room.messages.internal-server-error</t>
+  </si>
+  <si>
+    <t>update-room.messages.invalid-room-id</t>
+  </si>
+  <si>
+    <t>Invalid room ID</t>
+  </si>
+  <si>
+    <t>ID phòng không hợp lệ</t>
+  </si>
+  <si>
+    <t>update-room.messages.name-required</t>
+  </si>
+  <si>
+    <t>Room name is required</t>
+  </si>
+  <si>
+    <t>Tên phòng không được để trống</t>
+  </si>
+  <si>
+    <t>update-room.messages.room-not-found</t>
+  </si>
+  <si>
+    <t>update-room.messages.forbidden</t>
+  </si>
+  <si>
+    <t>You are not the host of this room</t>
+  </si>
+  <si>
+    <t>Bạn không phải chủ phòng</t>
+  </si>
+  <si>
     <t>draw-game.messages.invalid-game-id</t>
   </si>
   <si>
@@ -1426,31 +1528,13 @@
     <t>Token hợp lệ</t>
   </si>
   <si>
-    <t>menu.profile</t>
-  </si>
-  <si>
-    <t>Profile</t>
-  </si>
-  <si>
-    <t>Trang cá nhân</t>
-  </si>
-  <si>
-    <t>dashboard.popup.pve-mode</t>
-  </si>
-  <si>
-    <t>PVE mode</t>
-  </si>
-  <si>
-    <t>Chơi với máy</t>
-  </si>
-  <si>
-    <t>menu.expired</t>
-  </si>
-  <si>
-    <t>Set expired</t>
-  </si>
-  <si>
-    <t>Hết hạn token</t>
+    <t>dashboard.popup.join-room</t>
+  </si>
+  <si>
+    <t>Join room</t>
+  </si>
+  <si>
+    <t>Vào phòng</t>
   </si>
 </sst>
 </file>
@@ -1688,7 +1772,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C190"/>
+  <dimension ref="A1:C201"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="40" customWidth="1"/>
@@ -1840,1949 +1924,2070 @@
     </row>
     <row r="14" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="1" t="s">
-        <v>468</v>
+        <v>37</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>469</v>
+        <v>38</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>470</v>
+        <v>39</v>
       </c>
     </row>
     <row r="15" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="1" t="s">
-        <v>474</v>
+        <v>40</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>475</v>
+        <v>41</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>476</v>
+        <v>42</v>
       </c>
     </row>
     <row r="16" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="1" t="s">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>38</v>
+        <v>44</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>39</v>
+        <v>45</v>
       </c>
     </row>
     <row r="17" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="1" t="s">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>42</v>
+        <v>48</v>
       </c>
     </row>
     <row r="18" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="1" t="s">
-        <v>43</v>
+        <v>49</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>44</v>
+        <v>50</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
     </row>
     <row r="19" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="1" t="s">
-        <v>46</v>
+        <v>52</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>48</v>
+        <v>54</v>
       </c>
     </row>
     <row r="20" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="1" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>50</v>
+        <v>56</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>51</v>
+        <v>57</v>
       </c>
     </row>
     <row r="21" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="1" t="s">
-        <v>52</v>
+        <v>58</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>54</v>
+        <v>60</v>
       </c>
     </row>
     <row r="22" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="1" t="s">
-        <v>55</v>
+        <v>61</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>56</v>
+        <v>62</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>57</v>
+        <v>63</v>
       </c>
     </row>
     <row r="23" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="1" t="s">
-        <v>58</v>
+        <v>64</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>60</v>
+        <v>66</v>
       </c>
     </row>
     <row r="24" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="1" t="s">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>63</v>
+        <v>69</v>
       </c>
     </row>
     <row r="25" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="1" t="s">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
     </row>
     <row r="26" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="1" t="s">
-        <v>67</v>
+        <v>73</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>69</v>
+        <v>75</v>
       </c>
     </row>
     <row r="27" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="1" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>71</v>
+        <v>77</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>72</v>
+        <v>78</v>
       </c>
     </row>
     <row r="28" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="1" t="s">
-        <v>73</v>
+        <v>79</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>74</v>
+        <v>80</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>75</v>
+        <v>81</v>
       </c>
     </row>
     <row r="29" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="1" t="s">
-        <v>471</v>
+        <v>82</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>472</v>
+        <v>83</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>473</v>
+        <v>84</v>
       </c>
     </row>
     <row r="30" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="1" t="s">
-        <v>76</v>
+        <v>85</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>77</v>
+        <v>86</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>78</v>
+        <v>87</v>
       </c>
     </row>
     <row r="31" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="1" t="s">
-        <v>79</v>
+        <v>88</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>80</v>
+        <v>89</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>81</v>
+        <v>90</v>
       </c>
     </row>
     <row r="32" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="1" t="s">
-        <v>82</v>
+        <v>91</v>
       </c>
       <c r="B32" s="1" t="s">
         <v>4</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>83</v>
+        <v>92</v>
       </c>
     </row>
     <row r="33" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="1" t="s">
-        <v>84</v>
+        <v>502</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>31</v>
+        <v>503</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>32</v>
+        <v>504</v>
       </c>
     </row>
     <row r="34" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="1" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>86</v>
+        <v>31</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>87</v>
+        <v>32</v>
       </c>
     </row>
     <row r="35" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="1" t="s">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>89</v>
+        <v>95</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
     </row>
     <row r="36" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="1" t="s">
-        <v>91</v>
+        <v>97</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>93</v>
+        <v>99</v>
       </c>
     </row>
     <row r="37" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" s="1" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>96</v>
+        <v>102</v>
       </c>
     </row>
     <row r="38" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" s="1" t="s">
-        <v>97</v>
+        <v>103</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>98</v>
+        <v>104</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
     </row>
     <row r="39" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A39" s="1" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>101</v>
+        <v>107</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>102</v>
+        <v>108</v>
       </c>
     </row>
     <row r="40" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" s="1" t="s">
-        <v>103</v>
+        <v>109</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>104</v>
+        <v>110</v>
       </c>
       <c r="C40" s="1" t="s">
-        <v>104</v>
+        <v>111</v>
       </c>
     </row>
     <row r="41" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" s="1" t="s">
-        <v>105</v>
+        <v>112</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>106</v>
+        <v>113</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>107</v>
+        <v>113</v>
       </c>
     </row>
     <row r="42" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" s="1" t="s">
-        <v>108</v>
+        <v>114</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>109</v>
+        <v>115</v>
       </c>
       <c r="C42" s="1" t="s">
-        <v>110</v>
+        <v>116</v>
       </c>
     </row>
     <row r="43" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="1" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>112</v>
+        <v>118</v>
       </c>
       <c r="C43" s="1" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
     </row>
     <row r="44" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A44" s="1" t="s">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>115</v>
+        <v>121</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>116</v>
+        <v>122</v>
       </c>
     </row>
     <row r="45" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A45" s="1" t="s">
-        <v>117</v>
+        <v>123</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>118</v>
+        <v>124</v>
       </c>
       <c r="C45" s="1" t="s">
-        <v>119</v>
+        <v>125</v>
       </c>
     </row>
     <row r="46" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A46" s="1" t="s">
-        <v>120</v>
+        <v>126</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>121</v>
+        <v>127</v>
       </c>
       <c r="C46" s="1" t="s">
-        <v>122</v>
+        <v>128</v>
       </c>
     </row>
     <row r="47" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A47" s="1" t="s">
-        <v>123</v>
+        <v>129</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>124</v>
+        <v>130</v>
       </c>
       <c r="C47" s="1" t="s">
-        <v>125</v>
+        <v>131</v>
       </c>
     </row>
     <row r="48" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A48" s="1" t="s">
-        <v>126</v>
+        <v>132</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>127</v>
+        <v>133</v>
       </c>
       <c r="C48" s="1" t="s">
-        <v>128</v>
+        <v>134</v>
       </c>
     </row>
     <row r="49" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A49" s="1" t="s">
-        <v>129</v>
+        <v>135</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>130</v>
+        <v>136</v>
       </c>
       <c r="C49" s="1" t="s">
-        <v>131</v>
+        <v>137</v>
       </c>
     </row>
     <row r="50" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A50" s="1" t="s">
-        <v>132</v>
+        <v>138</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>130</v>
+        <v>139</v>
       </c>
       <c r="C50" s="1" t="s">
-        <v>131</v>
+        <v>140</v>
       </c>
     </row>
     <row r="51" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A51" s="1" t="s">
-        <v>133</v>
+        <v>141</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>134</v>
+        <v>139</v>
       </c>
       <c r="C51" s="1" t="s">
-        <v>135</v>
+        <v>140</v>
       </c>
     </row>
     <row r="52" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A52" s="1" t="s">
-        <v>136</v>
+        <v>142</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>134</v>
+        <v>143</v>
       </c>
       <c r="C52" s="1" t="s">
-        <v>135</v>
+        <v>144</v>
       </c>
     </row>
     <row r="53" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A53" s="1" t="s">
-        <v>137</v>
+        <v>145</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>138</v>
+        <v>143</v>
       </c>
       <c r="C53" s="1" t="s">
-        <v>139</v>
+        <v>144</v>
       </c>
     </row>
     <row r="54" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A54" s="1" t="s">
-        <v>140</v>
+        <v>146</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>138</v>
+        <v>147</v>
       </c>
       <c r="C54" s="1" t="s">
-        <v>139</v>
+        <v>148</v>
       </c>
     </row>
     <row r="55" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A55" s="1" t="s">
-        <v>141</v>
+        <v>149</v>
       </c>
       <c r="B55" s="1" t="s">
-        <v>142</v>
+        <v>147</v>
       </c>
       <c r="C55" s="1" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
     </row>
     <row r="56" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A56" s="1" t="s">
-        <v>144</v>
+        <v>150</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>145</v>
+        <v>151</v>
       </c>
       <c r="C56" s="1" t="s">
-        <v>146</v>
+        <v>152</v>
       </c>
     </row>
     <row r="57" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A57" s="1" t="s">
-        <v>147</v>
+        <v>153</v>
       </c>
       <c r="B57" s="1" t="s">
-        <v>148</v>
+        <v>154</v>
       </c>
       <c r="C57" s="1" t="s">
-        <v>149</v>
+        <v>155</v>
       </c>
     </row>
     <row r="58" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A58" s="1" t="s">
-        <v>150</v>
+        <v>156</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>151</v>
+        <v>157</v>
       </c>
       <c r="C58" s="1" t="s">
-        <v>152</v>
+        <v>158</v>
       </c>
     </row>
     <row r="59" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A59" s="1" t="s">
-        <v>153</v>
+        <v>159</v>
       </c>
       <c r="B59" s="1" t="s">
-        <v>154</v>
+        <v>160</v>
       </c>
       <c r="C59" s="1" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
     </row>
     <row r="60" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A60" s="1" t="s">
-        <v>156</v>
+        <v>162</v>
       </c>
       <c r="B60" s="1" t="s">
-        <v>157</v>
+        <v>163</v>
       </c>
       <c r="C60" s="1" t="s">
-        <v>158</v>
+        <v>164</v>
       </c>
     </row>
     <row r="61" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A61" s="1" t="s">
-        <v>159</v>
+        <v>165</v>
       </c>
       <c r="B61" s="1" t="s">
-        <v>130</v>
+        <v>166</v>
       </c>
       <c r="C61" s="1" t="s">
-        <v>131</v>
+        <v>167</v>
       </c>
     </row>
     <row r="62" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A62" s="1" t="s">
-        <v>160</v>
+        <v>168</v>
       </c>
       <c r="B62" s="1" t="s">
-        <v>161</v>
+        <v>139</v>
       </c>
       <c r="C62" s="1" t="s">
-        <v>162</v>
+        <v>140</v>
       </c>
     </row>
     <row r="63" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A63" s="1" t="s">
-        <v>163</v>
+        <v>169</v>
       </c>
       <c r="B63" s="1" t="s">
-        <v>164</v>
+        <v>170</v>
       </c>
       <c r="C63" s="1" t="s">
-        <v>165</v>
+        <v>171</v>
       </c>
     </row>
     <row r="64" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A64" s="1" t="s">
-        <v>166</v>
+        <v>172</v>
       </c>
       <c r="B64" s="1" t="s">
-        <v>167</v>
+        <v>173</v>
       </c>
       <c r="C64" s="1" t="s">
-        <v>168</v>
+        <v>174</v>
       </c>
     </row>
     <row r="65" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A65" s="1" t="s">
-        <v>169</v>
+        <v>175</v>
       </c>
       <c r="B65" s="1" t="s">
-        <v>170</v>
+        <v>176</v>
       </c>
       <c r="C65" s="1" t="s">
-        <v>171</v>
+        <v>177</v>
       </c>
     </row>
     <row r="66" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A66" s="1" t="s">
-        <v>172</v>
+        <v>178</v>
       </c>
       <c r="B66" s="1" t="s">
-        <v>173</v>
+        <v>179</v>
       </c>
       <c r="C66" s="1" t="s">
-        <v>174</v>
+        <v>180</v>
       </c>
     </row>
     <row r="67" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A67" s="1" t="s">
-        <v>175</v>
+        <v>181</v>
       </c>
       <c r="B67" s="1" t="s">
-        <v>176</v>
+        <v>182</v>
       </c>
       <c r="C67" s="1" t="s">
-        <v>177</v>
+        <v>183</v>
       </c>
     </row>
     <row r="68" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A68" s="1" t="s">
-        <v>178</v>
+        <v>184</v>
       </c>
       <c r="B68" s="1" t="s">
-        <v>176</v>
+        <v>185</v>
       </c>
       <c r="C68" s="1" t="s">
-        <v>177</v>
+        <v>186</v>
       </c>
     </row>
     <row r="69" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A69" s="1" t="s">
-        <v>179</v>
+        <v>187</v>
       </c>
       <c r="B69" s="1" t="s">
-        <v>180</v>
+        <v>185</v>
       </c>
       <c r="C69" s="1" t="s">
-        <v>181</v>
+        <v>186</v>
       </c>
     </row>
     <row r="70" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A70" s="1" t="s">
-        <v>182</v>
+        <v>188</v>
       </c>
       <c r="B70" s="1" t="s">
-        <v>180</v>
+        <v>189</v>
       </c>
       <c r="C70" s="1" t="s">
-        <v>181</v>
+        <v>190</v>
       </c>
     </row>
     <row r="71" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A71" s="1" t="s">
-        <v>183</v>
+        <v>191</v>
       </c>
       <c r="B71" s="1" t="s">
-        <v>184</v>
+        <v>189</v>
       </c>
       <c r="C71" s="1" t="s">
-        <v>185</v>
+        <v>190</v>
       </c>
     </row>
     <row r="72" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A72" s="1" t="s">
-        <v>186</v>
+        <v>192</v>
       </c>
       <c r="B72" s="1" t="s">
-        <v>187</v>
+        <v>193</v>
       </c>
       <c r="C72" s="1" t="s">
-        <v>187</v>
+        <v>194</v>
       </c>
     </row>
     <row r="73" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A73" s="1" t="s">
-        <v>188</v>
+        <v>195</v>
       </c>
       <c r="B73" s="1" t="s">
-        <v>187</v>
+        <v>196</v>
       </c>
       <c r="C73" s="1" t="s">
-        <v>187</v>
+        <v>196</v>
       </c>
     </row>
     <row r="74" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A74" s="1" t="s">
-        <v>189</v>
+        <v>197</v>
       </c>
       <c r="B74" s="1" t="s">
-        <v>190</v>
+        <v>196</v>
       </c>
       <c r="C74" s="1" t="s">
-        <v>191</v>
+        <v>196</v>
       </c>
     </row>
     <row r="75" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A75" s="1" t="s">
-        <v>192</v>
+        <v>198</v>
       </c>
       <c r="B75" s="1" t="s">
-        <v>157</v>
+        <v>199</v>
       </c>
       <c r="C75" s="1" t="s">
-        <v>158</v>
+        <v>200</v>
       </c>
     </row>
     <row r="76" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A76" s="1" t="s">
-        <v>193</v>
+        <v>201</v>
       </c>
       <c r="B76" s="1" t="s">
-        <v>194</v>
+        <v>166</v>
       </c>
       <c r="C76" s="1" t="s">
-        <v>195</v>
+        <v>167</v>
       </c>
     </row>
     <row r="77" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A77" s="1" t="s">
-        <v>196</v>
+        <v>202</v>
       </c>
       <c r="B77" s="1" t="s">
-        <v>157</v>
+        <v>203</v>
       </c>
       <c r="C77" s="1" t="s">
-        <v>158</v>
+        <v>204</v>
       </c>
     </row>
     <row r="78" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A78" s="1" t="s">
-        <v>197</v>
+        <v>205</v>
       </c>
       <c r="B78" s="1" t="s">
-        <v>198</v>
+        <v>166</v>
       </c>
       <c r="C78" s="1" t="s">
-        <v>199</v>
+        <v>167</v>
       </c>
     </row>
     <row r="79" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A79" s="1" t="s">
-        <v>200</v>
+        <v>206</v>
       </c>
       <c r="B79" s="1" t="s">
-        <v>201</v>
+        <v>207</v>
       </c>
       <c r="C79" s="1" t="s">
-        <v>202</v>
+        <v>208</v>
       </c>
     </row>
     <row r="80" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A80" s="1" t="s">
-        <v>203</v>
+        <v>209</v>
       </c>
       <c r="B80" s="1" t="s">
-        <v>204</v>
+        <v>210</v>
       </c>
       <c r="C80" s="1" t="s">
-        <v>205</v>
+        <v>211</v>
       </c>
     </row>
     <row r="81" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A81" s="1" t="s">
-        <v>206</v>
+        <v>212</v>
       </c>
       <c r="B81" s="1" t="s">
-        <v>207</v>
+        <v>213</v>
       </c>
       <c r="C81" s="1" t="s">
-        <v>208</v>
+        <v>214</v>
       </c>
     </row>
     <row r="82" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A82" s="1" t="s">
-        <v>209</v>
+        <v>215</v>
       </c>
       <c r="B82" s="1" t="s">
-        <v>157</v>
+        <v>216</v>
       </c>
       <c r="C82" s="1" t="s">
-        <v>158</v>
+        <v>217</v>
       </c>
     </row>
     <row r="83" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A83" s="1" t="s">
-        <v>210</v>
+        <v>218</v>
       </c>
       <c r="B83" s="1" t="s">
-        <v>211</v>
+        <v>166</v>
       </c>
       <c r="C83" s="1" t="s">
-        <v>212</v>
+        <v>167</v>
       </c>
     </row>
     <row r="84" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A84" s="1" t="s">
-        <v>213</v>
+        <v>219</v>
       </c>
       <c r="B84" s="1" t="s">
-        <v>148</v>
+        <v>220</v>
       </c>
       <c r="C84" s="1" t="s">
-        <v>149</v>
+        <v>221</v>
       </c>
     </row>
     <row r="85" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A85" s="1" t="s">
-        <v>214</v>
+        <v>222</v>
       </c>
       <c r="B85" s="1" t="s">
-        <v>138</v>
+        <v>157</v>
       </c>
       <c r="C85" s="1" t="s">
-        <v>139</v>
+        <v>158</v>
       </c>
     </row>
     <row r="86" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A86" s="1" t="s">
-        <v>215</v>
+        <v>223</v>
       </c>
       <c r="B86" s="1" t="s">
-        <v>138</v>
+        <v>147</v>
       </c>
       <c r="C86" s="1" t="s">
-        <v>139</v>
+        <v>148</v>
       </c>
     </row>
     <row r="87" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A87" s="1" t="s">
-        <v>216</v>
+        <v>224</v>
       </c>
       <c r="B87" s="1" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="C87" s="1" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
     </row>
     <row r="88" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A88" s="1" t="s">
-        <v>217</v>
+        <v>225</v>
       </c>
       <c r="B88" s="1" t="s">
-        <v>218</v>
+        <v>154</v>
       </c>
       <c r="C88" s="1" t="s">
-        <v>219</v>
+        <v>155</v>
       </c>
     </row>
     <row r="89" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A89" s="1" t="s">
-        <v>220</v>
+        <v>226</v>
       </c>
       <c r="B89" s="1" t="s">
-        <v>134</v>
+        <v>227</v>
       </c>
       <c r="C89" s="1" t="s">
-        <v>135</v>
+        <v>228</v>
       </c>
     </row>
     <row r="90" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A90" s="1" t="s">
-        <v>221</v>
+        <v>229</v>
       </c>
       <c r="B90" s="1" t="s">
-        <v>134</v>
+        <v>143</v>
       </c>
       <c r="C90" s="1" t="s">
-        <v>135</v>
+        <v>144</v>
       </c>
     </row>
     <row r="91" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A91" s="1" t="s">
-        <v>222</v>
+        <v>230</v>
       </c>
       <c r="B91" s="1" t="s">
-        <v>223</v>
+        <v>143</v>
       </c>
       <c r="C91" s="1" t="s">
-        <v>155</v>
+        <v>144</v>
       </c>
     </row>
     <row r="92" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A92" s="1" t="s">
-        <v>224</v>
+        <v>231</v>
       </c>
       <c r="B92" s="1" t="s">
-        <v>223</v>
+        <v>232</v>
       </c>
       <c r="C92" s="1" t="s">
-        <v>155</v>
+        <v>164</v>
       </c>
     </row>
     <row r="93" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A93" s="1" t="s">
-        <v>225</v>
+        <v>233</v>
       </c>
       <c r="B93" s="1" t="s">
-        <v>190</v>
+        <v>232</v>
       </c>
       <c r="C93" s="1" t="s">
-        <v>191</v>
+        <v>164</v>
       </c>
     </row>
     <row r="94" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A94" s="1" t="s">
-        <v>226</v>
+        <v>234</v>
       </c>
       <c r="B94" s="1" t="s">
-        <v>154</v>
+        <v>199</v>
       </c>
       <c r="C94" s="1" t="s">
-        <v>155</v>
+        <v>200</v>
       </c>
     </row>
     <row r="95" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A95" s="1" t="s">
-        <v>227</v>
+        <v>235</v>
       </c>
       <c r="B95" s="1" t="s">
-        <v>228</v>
+        <v>163</v>
       </c>
       <c r="C95" s="1" t="s">
-        <v>229</v>
+        <v>164</v>
       </c>
     </row>
     <row r="96" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A96" s="1" t="s">
-        <v>230</v>
+        <v>236</v>
       </c>
       <c r="B96" s="1" t="s">
-        <v>231</v>
+        <v>237</v>
       </c>
       <c r="C96" s="1" t="s">
-        <v>232</v>
+        <v>238</v>
       </c>
     </row>
     <row r="97" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A97" s="1" t="s">
-        <v>233</v>
+        <v>239</v>
       </c>
       <c r="B97" s="1" t="s">
-        <v>234</v>
+        <v>240</v>
       </c>
       <c r="C97" s="1" t="s">
-        <v>235</v>
+        <v>241</v>
       </c>
     </row>
     <row r="98" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A98" s="1" t="s">
-        <v>236</v>
+        <v>242</v>
       </c>
       <c r="B98" s="1" t="s">
-        <v>237</v>
+        <v>243</v>
       </c>
       <c r="C98" s="1" t="s">
-        <v>238</v>
+        <v>244</v>
       </c>
     </row>
     <row r="99" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A99" s="1" t="s">
-        <v>239</v>
+        <v>245</v>
       </c>
       <c r="B99" s="1" t="s">
-        <v>234</v>
+        <v>246</v>
       </c>
       <c r="C99" s="1" t="s">
-        <v>235</v>
+        <v>247</v>
       </c>
     </row>
     <row r="100" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A100" s="1" t="s">
-        <v>240</v>
+        <v>248</v>
       </c>
       <c r="B100" s="1" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="C100" s="1" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
     </row>
     <row r="101" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A101" s="1" t="s">
-        <v>243</v>
+        <v>249</v>
       </c>
       <c r="B101" s="1" t="s">
-        <v>244</v>
+        <v>250</v>
       </c>
       <c r="C101" s="1" t="s">
-        <v>245</v>
+        <v>251</v>
       </c>
     </row>
     <row r="102" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A102" s="1" t="s">
-        <v>246</v>
+        <v>252</v>
       </c>
       <c r="B102" s="1" t="s">
-        <v>247</v>
+        <v>253</v>
       </c>
       <c r="C102" s="1" t="s">
-        <v>248</v>
+        <v>254</v>
       </c>
     </row>
     <row r="103" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A103" s="1" t="s">
-        <v>249</v>
+        <v>255</v>
       </c>
       <c r="B103" s="1" t="s">
-        <v>190</v>
+        <v>256</v>
       </c>
       <c r="C103" s="1" t="s">
-        <v>250</v>
+        <v>257</v>
       </c>
     </row>
     <row r="104" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A104" s="1" t="s">
-        <v>251</v>
+        <v>258</v>
       </c>
       <c r="B104" s="1" t="s">
-        <v>252</v>
+        <v>199</v>
       </c>
       <c r="C104" s="1" t="s">
-        <v>235</v>
+        <v>259</v>
       </c>
     </row>
     <row r="105" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A105" s="1" t="s">
-        <v>253</v>
+        <v>260</v>
       </c>
       <c r="B105" s="1" t="s">
-        <v>254</v>
+        <v>261</v>
       </c>
       <c r="C105" s="1" t="s">
-        <v>255</v>
+        <v>244</v>
       </c>
     </row>
     <row r="106" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A106" s="1" t="s">
-        <v>256</v>
+        <v>262</v>
       </c>
       <c r="B106" s="1" t="s">
-        <v>257</v>
+        <v>263</v>
       </c>
       <c r="C106" s="1" t="s">
-        <v>258</v>
+        <v>264</v>
       </c>
     </row>
     <row r="107" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A107" s="1" t="s">
-        <v>259</v>
+        <v>265</v>
       </c>
       <c r="B107" s="1" t="s">
-        <v>260</v>
+        <v>266</v>
       </c>
       <c r="C107" s="1" t="s">
-        <v>261</v>
+        <v>267</v>
       </c>
     </row>
     <row r="108" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A108" s="1" t="s">
-        <v>262</v>
+        <v>268</v>
       </c>
       <c r="B108" s="1" t="s">
-        <v>263</v>
+        <v>269</v>
       </c>
       <c r="C108" s="1" t="s">
-        <v>264</v>
+        <v>270</v>
       </c>
     </row>
     <row r="109" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A109" s="1" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="B109" s="1" t="s">
-        <v>266</v>
+        <v>272</v>
       </c>
       <c r="C109" s="1" t="s">
-        <v>267</v>
+        <v>273</v>
       </c>
     </row>
     <row r="110" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A110" s="1" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
       <c r="B110" s="1" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
       <c r="C110" s="1" t="s">
-        <v>270</v>
+        <v>276</v>
       </c>
     </row>
     <row r="111" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A111" s="1" t="s">
-        <v>271</v>
+        <v>277</v>
       </c>
       <c r="B111" s="1" t="s">
-        <v>272</v>
+        <v>278</v>
       </c>
       <c r="C111" s="1" t="s">
-        <v>273</v>
+        <v>279</v>
       </c>
     </row>
     <row r="112" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A112" s="1" t="s">
-        <v>274</v>
+        <v>280</v>
       </c>
       <c r="B112" s="1" t="s">
-        <v>275</v>
+        <v>281</v>
       </c>
       <c r="C112" s="1" t="s">
-        <v>276</v>
+        <v>282</v>
       </c>
     </row>
     <row r="113" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A113" s="1" t="s">
-        <v>277</v>
+        <v>283</v>
       </c>
       <c r="B113" s="1" t="s">
-        <v>278</v>
+        <v>284</v>
       </c>
       <c r="C113" s="1" t="s">
-        <v>279</v>
+        <v>285</v>
       </c>
     </row>
     <row r="114" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A114" s="1" t="s">
-        <v>280</v>
+        <v>286</v>
       </c>
       <c r="B114" s="1" t="s">
-        <v>281</v>
+        <v>287</v>
       </c>
       <c r="C114" s="1" t="s">
-        <v>282</v>
+        <v>288</v>
       </c>
     </row>
     <row r="115" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A115" s="1" t="s">
-        <v>283</v>
+        <v>289</v>
       </c>
       <c r="B115" s="1" t="s">
-        <v>284</v>
+        <v>290</v>
       </c>
       <c r="C115" s="1" t="s">
-        <v>285</v>
+        <v>291</v>
       </c>
     </row>
     <row r="116" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A116" s="1" t="s">
-        <v>286</v>
+        <v>292</v>
       </c>
       <c r="B116" s="1" t="s">
-        <v>287</v>
+        <v>293</v>
       </c>
       <c r="C116" s="1" t="s">
-        <v>288</v>
+        <v>294</v>
       </c>
     </row>
     <row r="117" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A117" s="1" t="s">
-        <v>289</v>
+        <v>295</v>
       </c>
       <c r="B117" s="1" t="s">
-        <v>290</v>
+        <v>296</v>
       </c>
       <c r="C117" s="1" t="s">
-        <v>291</v>
+        <v>297</v>
       </c>
     </row>
     <row r="118" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A118" s="1" t="s">
-        <v>292</v>
+        <v>298</v>
       </c>
       <c r="B118" s="1" t="s">
-        <v>293</v>
+        <v>299</v>
       </c>
       <c r="C118" s="1" t="s">
-        <v>294</v>
+        <v>300</v>
       </c>
     </row>
     <row r="119" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A119" s="1" t="s">
-        <v>295</v>
+        <v>301</v>
       </c>
       <c r="B119" s="1" t="s">
-        <v>296</v>
+        <v>302</v>
       </c>
       <c r="C119" s="1" t="s">
-        <v>297</v>
+        <v>303</v>
       </c>
     </row>
     <row r="120" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A120" s="1" t="s">
-        <v>298</v>
+        <v>304</v>
       </c>
       <c r="B120" s="1" t="s">
-        <v>299</v>
+        <v>305</v>
       </c>
       <c r="C120" s="1" t="s">
-        <v>300</v>
+        <v>306</v>
       </c>
     </row>
     <row r="121" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A121" s="1" t="s">
-        <v>301</v>
+        <v>307</v>
       </c>
       <c r="B121" s="1" t="s">
-        <v>302</v>
+        <v>308</v>
       </c>
       <c r="C121" s="1" t="s">
-        <v>303</v>
+        <v>309</v>
       </c>
     </row>
     <row r="122" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A122" s="1" t="s">
-        <v>304</v>
+        <v>310</v>
       </c>
       <c r="B122" s="1" t="s">
-        <v>305</v>
+        <v>311</v>
       </c>
       <c r="C122" s="1" t="s">
-        <v>306</v>
+        <v>312</v>
       </c>
     </row>
     <row r="123" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A123" s="1" t="s">
-        <v>307</v>
+        <v>313</v>
       </c>
       <c r="B123" s="1" t="s">
-        <v>293</v>
+        <v>314</v>
       </c>
       <c r="C123" s="1" t="s">
-        <v>294</v>
+        <v>315</v>
       </c>
     </row>
     <row r="124" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A124" s="1" t="s">
-        <v>308</v>
+        <v>316</v>
       </c>
       <c r="B124" s="1" t="s">
-        <v>184</v>
+        <v>302</v>
       </c>
       <c r="C124" s="1" t="s">
-        <v>185</v>
+        <v>303</v>
       </c>
     </row>
     <row r="125" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A125" s="1" t="s">
-        <v>309</v>
+        <v>317</v>
       </c>
       <c r="B125" s="1" t="s">
-        <v>310</v>
+        <v>193</v>
       </c>
       <c r="C125" s="1" t="s">
-        <v>311</v>
+        <v>194</v>
       </c>
     </row>
     <row r="126" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A126" s="1" t="s">
-        <v>312</v>
+        <v>318</v>
       </c>
       <c r="B126" s="1" t="s">
-        <v>313</v>
+        <v>319</v>
       </c>
       <c r="C126" s="1" t="s">
-        <v>314</v>
+        <v>320</v>
       </c>
     </row>
     <row r="127" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A127" s="1" t="s">
-        <v>315</v>
+        <v>321</v>
       </c>
       <c r="B127" s="1" t="s">
-        <v>293</v>
+        <v>322</v>
       </c>
       <c r="C127" s="1" t="s">
-        <v>294</v>
+        <v>323</v>
       </c>
     </row>
     <row r="128" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A128" s="1" t="s">
-        <v>316</v>
+        <v>324</v>
       </c>
       <c r="B128" s="1" t="s">
-        <v>317</v>
+        <v>302</v>
       </c>
       <c r="C128" s="1" t="s">
-        <v>318</v>
+        <v>303</v>
       </c>
     </row>
     <row r="129" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A129" s="1" t="s">
-        <v>319</v>
+        <v>325</v>
       </c>
       <c r="B129" s="1" t="s">
-        <v>320</v>
+        <v>326</v>
       </c>
       <c r="C129" s="1" t="s">
-        <v>321</v>
+        <v>327</v>
       </c>
     </row>
     <row r="130" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A130" s="1" t="s">
-        <v>322</v>
+        <v>328</v>
       </c>
       <c r="B130" s="1" t="s">
-        <v>323</v>
+        <v>329</v>
       </c>
       <c r="C130" s="1" t="s">
-        <v>324</v>
+        <v>330</v>
       </c>
     </row>
     <row r="131" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A131" s="1" t="s">
-        <v>325</v>
+        <v>331</v>
       </c>
       <c r="B131" s="1" t="s">
-        <v>293</v>
+        <v>332</v>
       </c>
       <c r="C131" s="1" t="s">
-        <v>294</v>
+        <v>333</v>
       </c>
     </row>
     <row r="132" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A132" s="1" t="s">
-        <v>326</v>
+        <v>334</v>
       </c>
       <c r="B132" s="1" t="s">
-        <v>317</v>
+        <v>302</v>
       </c>
       <c r="C132" s="1" t="s">
-        <v>318</v>
+        <v>303</v>
       </c>
     </row>
     <row r="133" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A133" s="1" t="s">
+        <v>335</v>
+      </c>
+      <c r="B133" s="1" t="s">
+        <v>326</v>
+      </c>
+      <c r="C133" s="1" t="s">
         <v>327</v>
-      </c>
-      <c r="B133" s="1" t="s">
-        <v>328</v>
-      </c>
-      <c r="C133" s="1" t="s">
-        <v>329</v>
       </c>
     </row>
     <row r="134" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A134" s="1" t="s">
-        <v>330</v>
+        <v>336</v>
       </c>
       <c r="B134" s="1" t="s">
-        <v>331</v>
+        <v>337</v>
       </c>
       <c r="C134" s="1" t="s">
-        <v>332</v>
+        <v>338</v>
       </c>
     </row>
     <row r="135" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A135" s="1" t="s">
-        <v>333</v>
+        <v>339</v>
       </c>
       <c r="B135" s="1" t="s">
-        <v>293</v>
+        <v>340</v>
       </c>
       <c r="C135" s="1" t="s">
-        <v>294</v>
+        <v>341</v>
       </c>
     </row>
     <row r="136" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A136" s="1" t="s">
-        <v>334</v>
+        <v>342</v>
       </c>
       <c r="B136" s="1" t="s">
-        <v>335</v>
+        <v>302</v>
       </c>
       <c r="C136" s="1" t="s">
-        <v>336</v>
+        <v>303</v>
       </c>
     </row>
     <row r="137" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A137" s="1" t="s">
-        <v>337</v>
+        <v>343</v>
       </c>
       <c r="B137" s="1" t="s">
-        <v>320</v>
+        <v>344</v>
       </c>
       <c r="C137" s="1" t="s">
-        <v>321</v>
+        <v>345</v>
       </c>
     </row>
     <row r="138" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A138" s="1" t="s">
-        <v>338</v>
+        <v>346</v>
       </c>
       <c r="B138" s="1" t="s">
-        <v>339</v>
+        <v>329</v>
       </c>
       <c r="C138" s="1" t="s">
-        <v>340</v>
+        <v>330</v>
       </c>
     </row>
     <row r="139" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A139" s="1" t="s">
-        <v>341</v>
+        <v>347</v>
       </c>
       <c r="B139" s="1" t="s">
-        <v>342</v>
+        <v>348</v>
       </c>
       <c r="C139" s="1" t="s">
-        <v>343</v>
+        <v>349</v>
       </c>
     </row>
     <row r="140" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A140" s="1" t="s">
-        <v>344</v>
+        <v>350</v>
       </c>
       <c r="B140" s="1" t="s">
-        <v>293</v>
+        <v>351</v>
       </c>
       <c r="C140" s="1" t="s">
-        <v>294</v>
+        <v>352</v>
       </c>
     </row>
     <row r="141" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A141" s="1" t="s">
-        <v>345</v>
+        <v>353</v>
       </c>
       <c r="B141" s="1" t="s">
-        <v>346</v>
+        <v>302</v>
       </c>
       <c r="C141" s="1" t="s">
-        <v>347</v>
+        <v>303</v>
       </c>
     </row>
     <row r="142" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A142" s="1" t="s">
-        <v>348</v>
+        <v>354</v>
       </c>
       <c r="B142" s="1" t="s">
-        <v>349</v>
+        <v>355</v>
       </c>
       <c r="C142" s="1" t="s">
-        <v>350</v>
+        <v>356</v>
       </c>
     </row>
     <row r="143" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A143" s="1" t="s">
-        <v>351</v>
+        <v>357</v>
       </c>
       <c r="B143" s="1" t="s">
-        <v>352</v>
+        <v>358</v>
       </c>
       <c r="C143" s="1" t="s">
-        <v>353</v>
+        <v>359</v>
       </c>
     </row>
     <row r="144" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A144" s="1" t="s">
-        <v>354</v>
+        <v>360</v>
       </c>
       <c r="B144" s="1" t="s">
-        <v>293</v>
+        <v>361</v>
       </c>
       <c r="C144" s="1" t="s">
-        <v>294</v>
+        <v>362</v>
       </c>
     </row>
     <row r="145" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A145" s="1" t="s">
-        <v>355</v>
+        <v>363</v>
       </c>
       <c r="B145" s="1" t="s">
-        <v>356</v>
+        <v>302</v>
       </c>
       <c r="C145" s="1" t="s">
-        <v>357</v>
+        <v>303</v>
       </c>
     </row>
     <row r="146" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A146" s="1" t="s">
-        <v>358</v>
+        <v>364</v>
       </c>
       <c r="B146" s="1" t="s">
-        <v>359</v>
+        <v>365</v>
       </c>
       <c r="C146" s="1" t="s">
-        <v>360</v>
+        <v>366</v>
       </c>
     </row>
     <row r="147" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A147" s="1" t="s">
-        <v>361</v>
+        <v>367</v>
       </c>
       <c r="B147" s="1" t="s">
-        <v>362</v>
+        <v>368</v>
       </c>
       <c r="C147" s="1" t="s">
-        <v>363</v>
+        <v>369</v>
       </c>
     </row>
     <row r="148" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A148" s="1" t="s">
-        <v>364</v>
+        <v>370</v>
       </c>
       <c r="B148" s="1" t="s">
-        <v>365</v>
+        <v>371</v>
       </c>
       <c r="C148" s="1" t="s">
-        <v>366</v>
+        <v>372</v>
       </c>
     </row>
     <row r="149" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A149" s="1" t="s">
-        <v>367</v>
+        <v>373</v>
       </c>
       <c r="B149" s="1" t="s">
-        <v>368</v>
+        <v>374</v>
       </c>
       <c r="C149" s="1" t="s">
-        <v>369</v>
+        <v>375</v>
       </c>
     </row>
     <row r="150" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A150" s="1" t="s">
-        <v>370</v>
+        <v>376</v>
       </c>
       <c r="B150" s="1" t="s">
-        <v>293</v>
+        <v>377</v>
       </c>
       <c r="C150" s="1" t="s">
-        <v>294</v>
+        <v>378</v>
       </c>
     </row>
     <row r="151" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A151" s="1" t="s">
-        <v>371</v>
+        <v>379</v>
       </c>
       <c r="B151" s="1" t="s">
-        <v>372</v>
+        <v>302</v>
       </c>
       <c r="C151" s="1" t="s">
-        <v>373</v>
+        <v>303</v>
       </c>
     </row>
     <row r="152" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A152" s="1" t="s">
-        <v>374</v>
+        <v>380</v>
       </c>
       <c r="B152" s="1" t="s">
-        <v>375</v>
+        <v>381</v>
       </c>
       <c r="C152" s="1" t="s">
-        <v>376</v>
+        <v>382</v>
       </c>
     </row>
     <row r="153" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A153" s="1" t="s">
-        <v>377</v>
+        <v>383</v>
       </c>
       <c r="B153" s="1" t="s">
-        <v>378</v>
+        <v>384</v>
       </c>
       <c r="C153" s="1" t="s">
-        <v>379</v>
+        <v>385</v>
       </c>
     </row>
     <row r="154" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A154" s="1" t="s">
-        <v>380</v>
+        <v>386</v>
       </c>
       <c r="B154" s="1" t="s">
-        <v>293</v>
+        <v>387</v>
       </c>
       <c r="C154" s="1" t="s">
-        <v>294</v>
+        <v>388</v>
       </c>
     </row>
     <row r="155" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A155" s="1" t="s">
-        <v>381</v>
+        <v>389</v>
       </c>
       <c r="B155" s="1" t="s">
-        <v>244</v>
+        <v>302</v>
       </c>
       <c r="C155" s="1" t="s">
-        <v>245</v>
+        <v>303</v>
       </c>
     </row>
     <row r="156" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A156" s="1" t="s">
-        <v>382</v>
+        <v>390</v>
       </c>
       <c r="B156" s="1" t="s">
-        <v>383</v>
+        <v>253</v>
       </c>
       <c r="C156" s="1" t="s">
-        <v>384</v>
+        <v>254</v>
       </c>
     </row>
     <row r="157" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A157" s="1" t="s">
-        <v>385</v>
+        <v>391</v>
       </c>
       <c r="B157" s="1" t="s">
-        <v>386</v>
+        <v>392</v>
       </c>
       <c r="C157" s="1" t="s">
-        <v>387</v>
+        <v>393</v>
       </c>
     </row>
     <row r="158" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A158" s="1" t="s">
-        <v>388</v>
+        <v>394</v>
       </c>
       <c r="B158" s="1" t="s">
-        <v>389</v>
+        <v>395</v>
       </c>
       <c r="C158" s="1" t="s">
-        <v>390</v>
+        <v>396</v>
       </c>
     </row>
     <row r="159" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A159" s="1" t="s">
-        <v>391</v>
+        <v>397</v>
       </c>
       <c r="B159" s="1" t="s">
-        <v>392</v>
+        <v>398</v>
       </c>
       <c r="C159" s="1" t="s">
-        <v>393</v>
+        <v>399</v>
       </c>
     </row>
     <row r="160" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A160" s="1" t="s">
-        <v>394</v>
+        <v>400</v>
       </c>
       <c r="B160" s="1" t="s">
-        <v>395</v>
+        <v>401</v>
       </c>
       <c r="C160" s="1" t="s">
-        <v>396</v>
+        <v>402</v>
       </c>
     </row>
     <row r="161" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A161" s="1" t="s">
-        <v>397</v>
+        <v>403</v>
       </c>
       <c r="B161" s="1" t="s">
-        <v>293</v>
+        <v>404</v>
       </c>
       <c r="C161" s="1" t="s">
-        <v>294</v>
+        <v>405</v>
       </c>
     </row>
     <row r="162" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A162" s="1" t="s">
-        <v>398</v>
+        <v>406</v>
       </c>
       <c r="B162" s="1" t="s">
-        <v>317</v>
+        <v>302</v>
       </c>
       <c r="C162" s="1" t="s">
-        <v>318</v>
+        <v>303</v>
       </c>
     </row>
     <row r="163" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A163" s="1" t="s">
-        <v>399</v>
+        <v>407</v>
       </c>
       <c r="B163" s="1" t="s">
-        <v>400</v>
+        <v>326</v>
       </c>
       <c r="C163" s="1" t="s">
-        <v>401</v>
+        <v>327</v>
       </c>
     </row>
     <row r="164" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A164" s="1" t="s">
-        <v>402</v>
+        <v>408</v>
       </c>
       <c r="B164" s="1" t="s">
-        <v>320</v>
+        <v>409</v>
       </c>
       <c r="C164" s="1" t="s">
-        <v>321</v>
+        <v>410</v>
       </c>
     </row>
     <row r="165" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A165" s="1" t="s">
-        <v>403</v>
+        <v>411</v>
       </c>
       <c r="B165" s="1" t="s">
-        <v>404</v>
+        <v>329</v>
       </c>
       <c r="C165" s="1" t="s">
-        <v>405</v>
+        <v>330</v>
       </c>
     </row>
     <row r="166" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A166" s="1" t="s">
-        <v>406</v>
+        <v>412</v>
       </c>
       <c r="B166" s="1" t="s">
-        <v>407</v>
+        <v>413</v>
       </c>
       <c r="C166" s="1" t="s">
-        <v>408</v>
+        <v>414</v>
       </c>
     </row>
     <row r="167" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A167" s="1" t="s">
-        <v>409</v>
+        <v>415</v>
       </c>
       <c r="B167" s="1" t="s">
-        <v>410</v>
+        <v>416</v>
       </c>
       <c r="C167" s="1" t="s">
-        <v>411</v>
+        <v>417</v>
       </c>
     </row>
     <row r="168" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A168" s="1" t="s">
-        <v>412</v>
+        <v>418</v>
       </c>
       <c r="B168" s="1" t="s">
-        <v>413</v>
+        <v>419</v>
       </c>
       <c r="C168" s="1" t="s">
-        <v>414</v>
+        <v>420</v>
       </c>
     </row>
     <row r="169" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A169" s="1" t="s">
-        <v>415</v>
+        <v>421</v>
       </c>
       <c r="B169" s="1" t="s">
-        <v>416</v>
+        <v>422</v>
       </c>
       <c r="C169" s="1" t="s">
-        <v>417</v>
+        <v>423</v>
       </c>
     </row>
     <row r="170" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A170" s="1" t="s">
-        <v>418</v>
+        <v>424</v>
       </c>
       <c r="B170" s="1" t="s">
-        <v>419</v>
+        <v>425</v>
       </c>
       <c r="C170" s="1" t="s">
-        <v>420</v>
+        <v>426</v>
       </c>
     </row>
     <row r="171" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A171" s="1" t="s">
-        <v>421</v>
+        <v>427</v>
       </c>
       <c r="B171" s="1" t="s">
-        <v>422</v>
+        <v>428</v>
       </c>
       <c r="C171" s="1" t="s">
-        <v>423</v>
+        <v>429</v>
       </c>
     </row>
     <row r="172" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A172" s="1" t="s">
-        <v>424</v>
+        <v>430</v>
       </c>
       <c r="B172" s="1" t="s">
-        <v>425</v>
+        <v>431</v>
       </c>
       <c r="C172" s="1" t="s">
-        <v>426</v>
+        <v>432</v>
       </c>
     </row>
     <row r="173" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A173" s="1" t="s">
-        <v>427</v>
+        <v>433</v>
       </c>
       <c r="B173" s="1" t="s">
-        <v>428</v>
+        <v>434</v>
       </c>
       <c r="C173" s="1" t="s">
-        <v>429</v>
+        <v>435</v>
       </c>
     </row>
     <row r="174" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A174" s="1" t="s">
-        <v>430</v>
+        <v>436</v>
       </c>
       <c r="B174" s="1" t="s">
-        <v>431</v>
+        <v>437</v>
       </c>
       <c r="C174" s="1" t="s">
-        <v>432</v>
+        <v>438</v>
       </c>
     </row>
     <row r="175" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A175" s="1" t="s">
-        <v>433</v>
+        <v>439</v>
       </c>
       <c r="B175" s="1" t="s">
-        <v>434</v>
+        <v>440</v>
       </c>
       <c r="C175" s="1" t="s">
-        <v>435</v>
+        <v>441</v>
       </c>
     </row>
     <row r="176" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A176" s="1" t="s">
-        <v>436</v>
+        <v>442</v>
       </c>
       <c r="B176" s="1" t="s">
-        <v>437</v>
+        <v>443</v>
       </c>
       <c r="C176" s="1" t="s">
-        <v>438</v>
+        <v>444</v>
       </c>
     </row>
     <row r="177" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A177" s="1" t="s">
-        <v>439</v>
+        <v>445</v>
       </c>
       <c r="B177" s="1" t="s">
-        <v>440</v>
+        <v>446</v>
       </c>
       <c r="C177" s="1" t="s">
-        <v>441</v>
+        <v>444</v>
       </c>
     </row>
     <row r="178" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A178" s="1" t="s">
-        <v>442</v>
+        <v>447</v>
       </c>
       <c r="B178" s="1" t="s">
-        <v>443</v>
+        <v>448</v>
       </c>
       <c r="C178" s="1" t="s">
-        <v>444</v>
+        <v>449</v>
       </c>
     </row>
     <row r="179" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A179" s="1" t="s">
-        <v>445</v>
+        <v>450</v>
       </c>
       <c r="B179" s="1" t="s">
-        <v>446</v>
+        <v>451</v>
       </c>
       <c r="C179" s="1" t="s">
-        <v>447</v>
+        <v>452</v>
       </c>
     </row>
     <row r="180" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A180" s="1" t="s">
-        <v>448</v>
+        <v>453</v>
       </c>
       <c r="B180" s="1" t="s">
-        <v>449</v>
+        <v>454</v>
       </c>
       <c r="C180" s="1" t="s">
-        <v>432</v>
+        <v>455</v>
       </c>
     </row>
     <row r="181" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A181" s="1" t="s">
-        <v>450</v>
+        <v>456</v>
       </c>
       <c r="B181" s="1" t="s">
-        <v>293</v>
+        <v>302</v>
       </c>
       <c r="C181" s="1" t="s">
-        <v>294</v>
+        <v>303</v>
       </c>
     </row>
     <row r="182" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A182" s="1" t="s">
-        <v>451</v>
+        <v>457</v>
       </c>
       <c r="B182" s="1" t="s">
-        <v>446</v>
+        <v>458</v>
       </c>
       <c r="C182" s="1" t="s">
-        <v>447</v>
+        <v>459</v>
       </c>
     </row>
     <row r="183" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A183" s="1" t="s">
-        <v>452</v>
+        <v>460</v>
       </c>
       <c r="B183" s="1" t="s">
-        <v>443</v>
+        <v>461</v>
       </c>
       <c r="C183" s="1" t="s">
-        <v>444</v>
+        <v>462</v>
       </c>
     </row>
     <row r="184" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A184" s="1" t="s">
-        <v>453</v>
+        <v>463</v>
       </c>
       <c r="B184" s="1" t="s">
-        <v>437</v>
+        <v>329</v>
       </c>
       <c r="C184" s="1" t="s">
-        <v>438</v>
-      </c>
-    </row>
-    <row r="185" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A185" t="s">
-        <v>454</v>
-      </c>
-      <c r="B185" t="s">
-        <v>293</v>
-      </c>
-      <c r="C185" t="s">
-        <v>294</v>
-      </c>
-    </row>
-    <row r="186" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A186" t="s">
-        <v>455</v>
-      </c>
-      <c r="B186" t="s">
-        <v>434</v>
-      </c>
-      <c r="C186" t="s">
-        <v>435</v>
+        <v>330</v>
+      </c>
+    </row>
+    <row r="185" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A185" s="1" t="s">
+        <v>464</v>
+      </c>
+      <c r="B185" s="1" t="s">
+        <v>465</v>
+      </c>
+      <c r="C185" s="1" t="s">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="186" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A186" s="1" t="s">
+        <v>467</v>
+      </c>
+      <c r="B186" s="1" t="s">
+        <v>468</v>
+      </c>
+      <c r="C186" s="1" t="s">
+        <v>469</v>
       </c>
     </row>
     <row r="187" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A187" t="s">
-        <v>456</v>
+        <v>470</v>
       </c>
       <c r="B187" t="s">
-        <v>457</v>
+        <v>471</v>
       </c>
       <c r="C187" t="s">
-        <v>458</v>
+        <v>472</v>
       </c>
     </row>
     <row r="188" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A188" t="s">
-        <v>459</v>
+        <v>473</v>
       </c>
       <c r="B188" t="s">
-        <v>460</v>
+        <v>474</v>
       </c>
       <c r="C188" t="s">
-        <v>461</v>
+        <v>475</v>
       </c>
     </row>
     <row r="189" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A189" t="s">
-        <v>462</v>
+        <v>476</v>
       </c>
       <c r="B189" t="s">
-        <v>463</v>
+        <v>477</v>
       </c>
       <c r="C189" t="s">
-        <v>464</v>
+        <v>478</v>
       </c>
     </row>
     <row r="190" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A190" t="s">
-        <v>465</v>
+        <v>479</v>
       </c>
       <c r="B190" t="s">
-        <v>466</v>
+        <v>480</v>
       </c>
       <c r="C190" t="s">
-        <v>467</v>
+        <v>481</v>
+      </c>
+    </row>
+    <row r="191" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A191" t="s">
+        <v>482</v>
+      </c>
+      <c r="B191" t="s">
+        <v>483</v>
+      </c>
+      <c r="C191" t="s">
+        <v>441</v>
+      </c>
+    </row>
+    <row r="192" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A192" t="s">
+        <v>484</v>
+      </c>
+      <c r="B192" t="s">
+        <v>302</v>
+      </c>
+      <c r="C192" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="193" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A193" t="s">
+        <v>485</v>
+      </c>
+      <c r="B193" t="s">
+        <v>480</v>
+      </c>
+      <c r="C193" t="s">
+        <v>481</v>
+      </c>
+    </row>
+    <row r="194" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A194" t="s">
+        <v>486</v>
+      </c>
+      <c r="B194" t="s">
+        <v>477</v>
+      </c>
+      <c r="C194" t="s">
+        <v>478</v>
+      </c>
+    </row>
+    <row r="195" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A195" t="s">
+        <v>487</v>
+      </c>
+      <c r="B195" t="s">
+        <v>471</v>
+      </c>
+      <c r="C195" t="s">
+        <v>472</v>
+      </c>
+    </row>
+    <row r="196" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A196" t="s">
+        <v>488</v>
+      </c>
+      <c r="B196" t="s">
+        <v>302</v>
+      </c>
+      <c r="C196" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="197" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A197" t="s">
+        <v>489</v>
+      </c>
+      <c r="B197" t="s">
+        <v>468</v>
+      </c>
+      <c r="C197" t="s">
+        <v>469</v>
+      </c>
+    </row>
+    <row r="198" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A198" t="s">
+        <v>490</v>
+      </c>
+      <c r="B198" t="s">
+        <v>491</v>
+      </c>
+      <c r="C198" t="s">
+        <v>492</v>
+      </c>
+    </row>
+    <row r="199" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A199" t="s">
+        <v>493</v>
+      </c>
+      <c r="B199" t="s">
+        <v>494</v>
+      </c>
+      <c r="C199" t="s">
+        <v>495</v>
+      </c>
+    </row>
+    <row r="200" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A200" t="s">
+        <v>496</v>
+      </c>
+      <c r="B200" t="s">
+        <v>497</v>
+      </c>
+      <c r="C200" t="s">
+        <v>498</v>
+      </c>
+    </row>
+    <row r="201" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A201" t="s">
+        <v>499</v>
+      </c>
+      <c r="B201" t="s">
+        <v>500</v>
+      </c>
+      <c r="C201" t="s">
+        <v>501</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
- add user daily tasks to retrieve bonus coin: lucky wheel, bonus coin and daily task - update recalculate amounts api and job - more responsive for mobile and desktop mode - fix incorrect unread bug - edit profile feature - flip board feature, snackbar notification feature
</commit_message>
<xml_diff>
--- a/tools/languages.xlsx
+++ b/tools/languages.xlsx
@@ -325,7 +325,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C351"/>
+  <dimension ref="A1:C378"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -350,7 +350,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="17" customHeight="1">
+    <row r="2" ht="18" customHeight="1">
       <c r="A2" s="1" t="inlineStr">
         <is>
           <t>common.input.is-required</t>
@@ -367,7 +367,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="17" customHeight="1">
+    <row r="3" ht="18" customHeight="1">
       <c r="A3" s="1" t="inlineStr">
         <is>
           <t>common.loading</t>
@@ -384,7 +384,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="17" customHeight="1">
+    <row r="4" ht="18" customHeight="1">
       <c r="A4" s="1" t="inlineStr">
         <is>
           <t>common.password.policy-1</t>
@@ -401,7 +401,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="17" customHeight="1">
+    <row r="5" ht="18" customHeight="1">
       <c r="A5" s="1" t="inlineStr">
         <is>
           <t>common.password.policy-2</t>
@@ -418,7 +418,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="17" customHeight="1">
+    <row r="6" ht="18" customHeight="1">
       <c r="A6" s="1" t="inlineStr">
         <is>
           <t>common.password.policy-3</t>
@@ -639,7 +639,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="17" customHeight="1">
+    <row r="19" ht="18" customHeight="1">
       <c r="A19" s="1" t="inlineStr">
         <is>
           <t>page.history.no-games</t>
@@ -656,7 +656,7 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="17" customHeight="1">
+    <row r="20" ht="18" customHeight="1">
       <c r="A20" s="1" t="inlineStr">
         <is>
           <t>page.history.point-label</t>
@@ -673,7 +673,7 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="17" customHeight="1">
+    <row r="21" ht="18" customHeight="1">
       <c r="A21" s="1" t="inlineStr">
         <is>
           <t>page.about.title</t>
@@ -690,7 +690,7 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="17" customHeight="1">
+    <row r="22" ht="18" customHeight="1">
       <c r="A22" s="1" t="inlineStr">
         <is>
           <t>menu.app-name</t>
@@ -707,7 +707,7 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="17" customHeight="1">
+    <row r="23" ht="18" customHeight="1">
       <c r="A23" s="1" t="inlineStr">
         <is>
           <t>menu.profile</t>
@@ -724,7 +724,7 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="17" customHeight="1">
+    <row r="24" ht="18" customHeight="1">
       <c r="A24" s="1" t="inlineStr">
         <is>
           <t>menu.messages</t>
@@ -741,7 +741,7 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="17" customHeight="1">
+    <row r="25" ht="18" customHeight="1">
       <c r="A25" s="1" t="inlineStr">
         <is>
           <t>menu.guide</t>
@@ -758,7 +758,7 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="17" customHeight="1">
+    <row r="26" ht="18" customHeight="1">
       <c r="A26" s="1" t="inlineStr">
         <is>
           <t>menu.announce</t>
@@ -775,75 +775,75 @@
         </is>
       </c>
     </row>
-    <row r="27" ht="17" customHeight="1">
+    <row r="27" ht="18" customHeight="1">
       <c r="A27" s="1" t="inlineStr">
         <is>
+          <t>menu.extra</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>Daily tasks</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>Tác vụ thường nhật</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="18" customHeight="1">
+      <c r="A28" s="1" t="inlineStr">
+        <is>
           <t>menu.setting.button</t>
         </is>
       </c>
-      <c r="B27" s="2" t="inlineStr">
+      <c r="B28" s="2" t="inlineStr">
         <is>
           <t>Settings</t>
         </is>
       </c>
-      <c r="C27" s="2" t="inlineStr">
+      <c r="C28" s="2" t="inlineStr">
         <is>
           <t>Cài đặt</t>
         </is>
       </c>
     </row>
-    <row r="28" ht="17" customHeight="1">
-      <c r="A28" s="1" t="inlineStr">
+    <row r="29" ht="18" customHeight="1">
+      <c r="A29" s="1" t="inlineStr">
         <is>
           <t>menu.app-name</t>
         </is>
       </c>
-      <c r="B28" s="2" t="inlineStr">
+      <c r="B29" s="2" t="inlineStr">
         <is>
           <t>Xiangqi</t>
         </is>
       </c>
-      <c r="C28" s="2" t="inlineStr">
+      <c r="C29" s="2" t="inlineStr">
         <is>
           <t>Cờ tướng</t>
         </is>
       </c>
     </row>
-    <row r="29" ht="17" customHeight="1">
-      <c r="A29" s="1" t="inlineStr">
+    <row r="30" ht="18" customHeight="1">
+      <c r="A30" s="1" t="inlineStr">
         <is>
           <t>menu.home</t>
         </is>
       </c>
-      <c r="B29" s="2" t="inlineStr">
+      <c r="B30" s="2" t="inlineStr">
         <is>
           <t>Home</t>
         </is>
       </c>
-      <c r="C29" s="2" t="inlineStr">
+      <c r="C30" s="2" t="inlineStr">
         <is>
           <t>Trang chủ</t>
         </is>
       </c>
     </row>
-    <row r="30" ht="17" customHeight="1">
-      <c r="A30" s="1" t="inlineStr">
-        <is>
-          <t>menu.profile</t>
-        </is>
-      </c>
-      <c r="B30" s="2" t="inlineStr">
-        <is>
-          <t>Profile</t>
-        </is>
-      </c>
-      <c r="C30" s="2" t="inlineStr">
-        <is>
-          <t>Trang cá nhân</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="17" customHeight="1">
+    <row r="31" ht="18" customHeight="1">
       <c r="A31" s="1" t="inlineStr">
         <is>
           <t>menu.expired</t>
@@ -860,7 +860,7 @@
         </is>
       </c>
     </row>
-    <row r="32" ht="17" customHeight="1">
+    <row r="32" ht="18" customHeight="1">
       <c r="A32" s="1" t="inlineStr">
         <is>
           <t>menu.logout</t>
@@ -877,7 +877,7 @@
         </is>
       </c>
     </row>
-    <row r="33" ht="17" customHeight="1">
+    <row r="33" ht="18" customHeight="1">
       <c r="A33" s="1" t="inlineStr">
         <is>
           <t>menu.rooms</t>
@@ -894,7 +894,7 @@
         </is>
       </c>
     </row>
-    <row r="34" ht="17" customHeight="1">
+    <row r="34" ht="18" customHeight="1">
       <c r="A34" s="1" t="inlineStr">
         <is>
           <t>announce.title</t>
@@ -911,7 +911,7 @@
         </is>
       </c>
     </row>
-    <row r="35" ht="17" customHeight="1">
+    <row r="35" ht="18" customHeight="1">
       <c r="A35" s="1" t="inlineStr">
         <is>
           <t>announce.placeholder</t>
@@ -928,7 +928,7 @@
         </is>
       </c>
     </row>
-    <row r="36" ht="17" customHeight="1">
+    <row r="36" ht="18" customHeight="1">
       <c r="A36" s="1" t="inlineStr">
         <is>
           <t>announce.empty</t>
@@ -945,7 +945,7 @@
         </is>
       </c>
     </row>
-    <row r="37" ht="17" customHeight="1">
+    <row r="37" ht="18" customHeight="1">
       <c r="A37" s="1" t="inlineStr">
         <is>
           <t>announce.loading-older</t>
@@ -962,7 +962,7 @@
         </is>
       </c>
     </row>
-    <row r="38" ht="17" customHeight="1">
+    <row r="38" ht="36" customHeight="1">
       <c r="A38" s="1" t="inlineStr">
         <is>
           <t>archivement.title-01</t>
@@ -979,7 +979,7 @@
         </is>
       </c>
     </row>
-    <row r="39" ht="17" customHeight="1">
+    <row r="39" ht="18" customHeight="1">
       <c r="A39" s="1" t="inlineStr">
         <is>
           <t>archivement.title-02</t>
@@ -996,7 +996,7 @@
         </is>
       </c>
     </row>
-    <row r="40" ht="17" customHeight="1">
+    <row r="40" ht="18" customHeight="1">
       <c r="A40" s="1" t="inlineStr">
         <is>
           <t>archivement.title-03</t>
@@ -1013,7 +1013,7 @@
         </is>
       </c>
     </row>
-    <row r="41" ht="17" customHeight="1">
+    <row r="41" ht="18" customHeight="1">
       <c r="A41" s="1" t="inlineStr">
         <is>
           <t>archivement.title-04</t>
@@ -1030,7 +1030,7 @@
         </is>
       </c>
     </row>
-    <row r="42" ht="17" customHeight="1">
+    <row r="42" ht="18" customHeight="1">
       <c r="A42" s="1" t="inlineStr">
         <is>
           <t>archivement.title-05</t>
@@ -1047,7 +1047,7 @@
         </is>
       </c>
     </row>
-    <row r="43" ht="17" customHeight="1">
+    <row r="43" ht="18" customHeight="1">
       <c r="A43" s="1" t="inlineStr">
         <is>
           <t>archivement.title-06</t>
@@ -1064,7 +1064,7 @@
         </is>
       </c>
     </row>
-    <row r="44" ht="17" customHeight="1">
+    <row r="44" ht="18" customHeight="1">
       <c r="A44" s="1" t="inlineStr">
         <is>
           <t>archivement.title-07</t>
@@ -1081,7 +1081,7 @@
         </is>
       </c>
     </row>
-    <row r="45" ht="17" customHeight="1">
+    <row r="45" ht="36" customHeight="1">
       <c r="A45" s="1" t="inlineStr">
         <is>
           <t>archivement.title-08</t>
@@ -1098,7 +1098,7 @@
         </is>
       </c>
     </row>
-    <row r="46" ht="17" customHeight="1">
+    <row r="46" ht="36" customHeight="1">
       <c r="A46" s="1" t="inlineStr">
         <is>
           <t>archivement.title-09</t>
@@ -1115,7 +1115,7 @@
         </is>
       </c>
     </row>
-    <row r="47" ht="17" customHeight="1">
+    <row r="47" ht="18" customHeight="1">
       <c r="A47" s="1" t="inlineStr">
         <is>
           <t>archivement.title-10</t>
@@ -1132,7 +1132,7 @@
         </is>
       </c>
     </row>
-    <row r="48" ht="17" customHeight="1">
+    <row r="48" ht="36" customHeight="1">
       <c r="A48" s="1" t="inlineStr">
         <is>
           <t>archivement.title-11</t>
@@ -1149,7 +1149,7 @@
         </is>
       </c>
     </row>
-    <row r="49" ht="17" customHeight="1">
+    <row r="49" ht="18" customHeight="1">
       <c r="A49" s="1" t="inlineStr">
         <is>
           <t>archivement.title-12</t>
@@ -1166,7 +1166,7 @@
         </is>
       </c>
     </row>
-    <row r="50" ht="17" customHeight="1">
+    <row r="50" ht="18" customHeight="1">
       <c r="A50" s="1" t="inlineStr">
         <is>
           <t>chat.conversation.you</t>
@@ -1183,7 +1183,7 @@
         </is>
       </c>
     </row>
-    <row r="51" ht="17" customHeight="1">
+    <row r="51" ht="18" customHeight="1">
       <c r="A51" s="1" t="inlineStr">
         <is>
           <t>chat.conversation.new</t>
@@ -1200,7 +1200,7 @@
         </is>
       </c>
     </row>
-    <row r="52" ht="17" customHeight="1">
+    <row r="52" ht="18" customHeight="1">
       <c r="A52" s="1" t="inlineStr">
         <is>
           <t>chat.messages.unread</t>
@@ -1217,7 +1217,7 @@
         </is>
       </c>
     </row>
-    <row r="53" ht="17" customHeight="1">
+    <row r="53" ht="18" customHeight="1">
       <c r="A53" s="1" t="inlineStr">
         <is>
           <t>search.user.title</t>
@@ -1234,7 +1234,7 @@
         </is>
       </c>
     </row>
-    <row r="54" ht="17" customHeight="1">
+    <row r="54" ht="18" customHeight="1">
       <c r="A54" s="1" t="inlineStr">
         <is>
           <t>search.user.placeholder</t>
@@ -1251,7 +1251,7 @@
         </is>
       </c>
     </row>
-    <row r="55" ht="17" customHeight="1">
+    <row r="55" ht="18" customHeight="1">
       <c r="A55" s="1" t="inlineStr">
         <is>
           <t>search.user.no-results</t>
@@ -1268,7 +1268,7 @@
         </is>
       </c>
     </row>
-    <row r="56" ht="17" customHeight="1">
+    <row r="56" ht="18" customHeight="1">
       <c r="A56" s="1" t="inlineStr">
         <is>
           <t>search.button.search</t>
@@ -1285,7 +1285,7 @@
         </is>
       </c>
     </row>
-    <row r="57" ht="17" customHeight="1">
+    <row r="57" ht="18" customHeight="1">
       <c r="A57" s="1" t="inlineStr">
         <is>
           <t>dashboard.page.title</t>
@@ -1302,7 +1302,7 @@
         </is>
       </c>
     </row>
-    <row r="58" ht="17" customHeight="1">
+    <row r="58" ht="18" customHeight="1">
       <c r="A58" s="1" t="inlineStr">
         <is>
           <t>dashboard.filters.all</t>
@@ -1319,7 +1319,7 @@
         </is>
       </c>
     </row>
-    <row r="59" ht="17" customHeight="1">
+    <row r="59" ht="18" customHeight="1">
       <c r="A59" s="1" t="inlineStr">
         <is>
           <t>dashboard.filters.available</t>
@@ -1336,7 +1336,7 @@
         </is>
       </c>
     </row>
-    <row r="60" ht="17" customHeight="1">
+    <row r="60" ht="18" customHeight="1">
       <c r="A60" s="1" t="inlineStr">
         <is>
           <t>dashboard.filters.playing</t>
@@ -1353,7 +1353,7 @@
         </is>
       </c>
     </row>
-    <row r="61" ht="17" customHeight="1">
+    <row r="61" ht="18" customHeight="1">
       <c r="A61" s="1" t="inlineStr">
         <is>
           <t>dashboard.feedback.empty</t>
@@ -1370,7 +1370,7 @@
         </is>
       </c>
     </row>
-    <row r="62" ht="17" customHeight="1">
+    <row r="62" ht="18" customHeight="1">
       <c r="A62" s="1" t="inlineStr">
         <is>
           <t>dashboard.feedback.error</t>
@@ -1387,7 +1387,7 @@
         </is>
       </c>
     </row>
-    <row r="63" ht="17" customHeight="1">
+    <row r="63" ht="18" customHeight="1">
       <c r="A63" s="1" t="inlineStr">
         <is>
           <t>dashboard.status.unknown</t>
@@ -1404,7 +1404,7 @@
         </is>
       </c>
     </row>
-    <row r="64" ht="17" customHeight="1">
+    <row r="64" ht="18" customHeight="1">
       <c r="A64" s="1" t="inlineStr">
         <is>
           <t>dashboard.feedback.result-count</t>
@@ -1421,7 +1421,7 @@
         </is>
       </c>
     </row>
-    <row r="65" ht="17" customHeight="1">
+    <row r="65" ht="18" customHeight="1">
       <c r="A65" s="1" t="inlineStr">
         <is>
           <t>dashboard.room.create</t>
@@ -1438,7 +1438,7 @@
         </is>
       </c>
     </row>
-    <row r="66" ht="17" customHeight="1">
+    <row r="66" ht="18" customHeight="1">
       <c r="A66" s="1" t="inlineStr">
         <is>
           <t>dashboard.popup.piece-selection</t>
@@ -1455,7 +1455,7 @@
         </is>
       </c>
     </row>
-    <row r="67" ht="17" customHeight="1">
+    <row r="67" ht="18" customHeight="1">
       <c r="A67" s="1" t="inlineStr">
         <is>
           <t>dashboard.popup.red-first</t>
@@ -1472,7 +1472,7 @@
         </is>
       </c>
     </row>
-    <row r="68" ht="17" customHeight="1">
+    <row r="68" ht="18" customHeight="1">
       <c r="A68" s="1" t="inlineStr">
         <is>
           <t>dashboard.popup.pve-mode</t>
@@ -1489,7 +1489,7 @@
         </is>
       </c>
     </row>
-    <row r="69" ht="17" customHeight="1">
+    <row r="69" ht="18" customHeight="1">
       <c r="A69" s="1" t="inlineStr">
         <is>
           <t>dashboard.popup.bet-amount</t>
@@ -1506,7 +1506,7 @@
         </is>
       </c>
     </row>
-    <row r="70" ht="17" customHeight="1">
+    <row r="70" ht="18" customHeight="1">
       <c r="A70" s="1" t="inlineStr">
         <is>
           <t>dashboard.popup.room-name-label</t>
@@ -1523,7 +1523,7 @@
         </is>
       </c>
     </row>
-    <row r="71" ht="17" customHeight="1">
+    <row r="71" ht="18" customHeight="1">
       <c r="A71" s="1" t="inlineStr">
         <is>
           <t>dashboard.popup.room-name-helptext</t>
@@ -1540,7 +1540,7 @@
         </is>
       </c>
     </row>
-    <row r="72" ht="17" customHeight="1">
+    <row r="72" ht="18" customHeight="1">
       <c r="A72" s="1" t="inlineStr">
         <is>
           <t>dashboard.popup.play</t>
@@ -1557,7 +1557,7 @@
         </is>
       </c>
     </row>
-    <row r="73" ht="17" customHeight="1">
+    <row r="73" ht="18" customHeight="1">
       <c r="A73" s="1" t="inlineStr">
         <is>
           <t>dashboard.popup.view</t>
@@ -1574,7 +1574,7 @@
         </is>
       </c>
     </row>
-    <row r="74" ht="17" customHeight="1">
+    <row r="74" ht="18" customHeight="1">
       <c r="A74" s="1" t="inlineStr">
         <is>
           <t>settings.header</t>
@@ -1591,7 +1591,7 @@
         </is>
       </c>
     </row>
-    <row r="75" ht="17" customHeight="1">
+    <row r="75" ht="18" customHeight="1">
       <c r="A75" s="1" t="inlineStr">
         <is>
           <t>settings.language</t>
@@ -1608,7 +1608,7 @@
         </is>
       </c>
     </row>
-    <row r="76" ht="17" customHeight="1">
+    <row r="76" ht="18" customHeight="1">
       <c r="A76" s="1" t="inlineStr">
         <is>
           <t>settings.dark-mode</t>
@@ -1625,7 +1625,7 @@
         </is>
       </c>
     </row>
-    <row r="77" ht="17" customHeight="1">
+    <row r="77" ht="18" customHeight="1">
       <c r="A77" s="1" t="inlineStr">
         <is>
           <t>settings.debug-mode</t>
@@ -1642,7 +1642,7 @@
         </is>
       </c>
     </row>
-    <row r="78" ht="17" customHeight="1">
+    <row r="78" ht="18" customHeight="1">
       <c r="A78" s="1" t="inlineStr">
         <is>
           <t>settings.close</t>
@@ -1659,7 +1659,7 @@
         </is>
       </c>
     </row>
-    <row r="79" ht="17" customHeight="1">
+    <row r="79" ht="18" customHeight="1">
       <c r="A79" s="1" t="inlineStr">
         <is>
           <t>settings.change-password</t>
@@ -1676,7 +1676,7 @@
         </is>
       </c>
     </row>
-    <row r="80" ht="17" customHeight="1">
+    <row r="80" ht="18" customHeight="1">
       <c r="A80" s="1" t="inlineStr">
         <is>
           <t>popup.alert.title</t>
@@ -1693,7 +1693,7 @@
         </is>
       </c>
     </row>
-    <row r="81" ht="17" customHeight="1">
+    <row r="81" ht="18" customHeight="1">
       <c r="A81" s="1" t="inlineStr">
         <is>
           <t>popup.confirm.title</t>
@@ -1710,7 +1710,7 @@
         </is>
       </c>
     </row>
-    <row r="82" ht="17" customHeight="1">
+    <row r="82" ht="18" customHeight="1">
       <c r="A82" s="1" t="inlineStr">
         <is>
           <t>popup.confirm.ok</t>
@@ -1727,7 +1727,7 @@
         </is>
       </c>
     </row>
-    <row r="83" ht="17" customHeight="1">
+    <row r="83" ht="18" customHeight="1">
       <c r="A83" s="1" t="inlineStr">
         <is>
           <t>popup.confirm.cancel</t>
@@ -1744,7 +1744,7 @@
         </is>
       </c>
     </row>
-    <row r="84" ht="17" customHeight="1">
+    <row r="84" ht="18" customHeight="1">
       <c r="A84" s="1" t="inlineStr">
         <is>
           <t>home.turn.title</t>
@@ -1761,7 +1761,7 @@
         </is>
       </c>
     </row>
-    <row r="85" ht="17" customHeight="1">
+    <row r="85" ht="18" customHeight="1">
       <c r="A85" s="1" t="inlineStr">
         <is>
           <t>game.general.captured</t>
@@ -1778,7 +1778,7 @@
         </is>
       </c>
     </row>
-    <row r="86" ht="17" customHeight="1">
+    <row r="86" ht="18" customHeight="1">
       <c r="A86" s="1" t="inlineStr">
         <is>
           <t>game.general.in-check</t>
@@ -1795,7 +1795,7 @@
         </is>
       </c>
     </row>
-    <row r="87" ht="17" customHeight="1">
+    <row r="87" ht="18" customHeight="1">
       <c r="A87" s="1" t="inlineStr">
         <is>
           <t>room.bot-difficulty.title</t>
@@ -1812,7 +1812,7 @@
         </is>
       </c>
     </row>
-    <row r="88" ht="17" customHeight="1">
+    <row r="88" ht="18" customHeight="1">
       <c r="A88" s="1" t="inlineStr">
         <is>
           <t>room.bot-difficulty.beginner</t>
@@ -1829,7 +1829,7 @@
         </is>
       </c>
     </row>
-    <row r="89" ht="17" customHeight="1">
+    <row r="89" ht="18" customHeight="1">
       <c r="A89" s="1" t="inlineStr">
         <is>
           <t>room.bot-difficulty.amateur</t>
@@ -1846,7 +1846,7 @@
         </is>
       </c>
     </row>
-    <row r="90" ht="17" customHeight="1">
+    <row r="90" ht="18" customHeight="1">
       <c r="A90" s="1" t="inlineStr">
         <is>
           <t>room.bot-difficulty.intermediate</t>
@@ -1863,7 +1863,7 @@
         </is>
       </c>
     </row>
-    <row r="91" ht="17" customHeight="1">
+    <row r="91" ht="18" customHeight="1">
       <c r="A91" s="1" t="inlineStr">
         <is>
           <t>room.bot-difficulty.advanced</t>
@@ -1880,7 +1880,7 @@
         </is>
       </c>
     </row>
-    <row r="92" ht="17" customHeight="1">
+    <row r="92" ht="18" customHeight="1">
       <c r="A92" s="1" t="inlineStr">
         <is>
           <t>room.bot-difficulty.master</t>
@@ -1897,7 +1897,7 @@
         </is>
       </c>
     </row>
-    <row r="93" ht="17" customHeight="1">
+    <row r="93" ht="18" customHeight="1">
       <c r="A93" s="1" t="inlineStr">
         <is>
           <t>login.page.title</t>
@@ -1914,7 +1914,7 @@
         </is>
       </c>
     </row>
-    <row r="94" ht="17" customHeight="1">
+    <row r="94" ht="18" customHeight="1">
       <c r="A94" s="1" t="inlineStr">
         <is>
           <t>login.form.title</t>
@@ -1931,7 +1931,7 @@
         </is>
       </c>
     </row>
-    <row r="95" ht="17" customHeight="1">
+    <row r="95" ht="18" customHeight="1">
       <c r="A95" s="1" t="inlineStr">
         <is>
           <t>login.username.label</t>
@@ -1948,7 +1948,7 @@
         </is>
       </c>
     </row>
-    <row r="96" ht="17" customHeight="1">
+    <row r="96" ht="18" customHeight="1">
       <c r="A96" s="1" t="inlineStr">
         <is>
           <t>login.username.placeholder</t>
@@ -1965,7 +1965,7 @@
         </is>
       </c>
     </row>
-    <row r="97" ht="17" customHeight="1">
+    <row r="97" ht="18" customHeight="1">
       <c r="A97" s="1" t="inlineStr">
         <is>
           <t>login.password.label</t>
@@ -1982,7 +1982,7 @@
         </is>
       </c>
     </row>
-    <row r="98" ht="17" customHeight="1">
+    <row r="98" ht="18" customHeight="1">
       <c r="A98" s="1" t="inlineStr">
         <is>
           <t>login.password.placeholder</t>
@@ -1999,7 +1999,7 @@
         </is>
       </c>
     </row>
-    <row r="99" ht="17" customHeight="1">
+    <row r="99" ht="18" customHeight="1">
       <c r="A99" s="1" t="inlineStr">
         <is>
           <t>login.password.error1</t>
@@ -2016,7 +2016,7 @@
         </is>
       </c>
     </row>
-    <row r="100" ht="17" customHeight="1">
+    <row r="100" ht="18" customHeight="1">
       <c r="A100" s="1" t="inlineStr">
         <is>
           <t>login.password.show</t>
@@ -2033,7 +2033,7 @@
         </is>
       </c>
     </row>
-    <row r="101" ht="17" customHeight="1">
+    <row r="101" ht="18" customHeight="1">
       <c r="A101" s="1" t="inlineStr">
         <is>
           <t>login.password.hide</t>
@@ -2050,7 +2050,7 @@
         </is>
       </c>
     </row>
-    <row r="102" ht="17" customHeight="1">
+    <row r="102" ht="18" customHeight="1">
       <c r="A102" s="1" t="inlineStr">
         <is>
           <t>login.form.error1</t>
@@ -2067,7 +2067,7 @@
         </is>
       </c>
     </row>
-    <row r="103" ht="17" customHeight="1">
+    <row r="103" ht="18" customHeight="1">
       <c r="A103" s="1" t="inlineStr">
         <is>
           <t>login.form.forgot-password</t>
@@ -2084,7 +2084,7 @@
         </is>
       </c>
     </row>
-    <row r="104" ht="17" customHeight="1">
+    <row r="104" ht="18" customHeight="1">
       <c r="A104" s="1" t="inlineStr">
         <is>
           <t>login.form.register</t>
@@ -2101,7 +2101,7 @@
         </is>
       </c>
     </row>
-    <row r="105" ht="17" customHeight="1">
+    <row r="105" ht="18" customHeight="1">
       <c r="A105" s="1" t="inlineStr">
         <is>
           <t>login.form.submit</t>
@@ -2118,7 +2118,7 @@
         </is>
       </c>
     </row>
-    <row r="106" ht="17" customHeight="1">
+    <row r="106" ht="18" customHeight="1">
       <c r="A106" s="1" t="inlineStr">
         <is>
           <t>notfound.title</t>
@@ -2135,7 +2135,7 @@
         </is>
       </c>
     </row>
-    <row r="107" ht="17" customHeight="1">
+    <row r="107" ht="36" customHeight="1">
       <c r="A107" s="1" t="inlineStr">
         <is>
           <t>notfound.description</t>
@@ -2152,7 +2152,7 @@
         </is>
       </c>
     </row>
-    <row r="108" ht="17" customHeight="1">
+    <row r="108" ht="18" customHeight="1">
       <c r="A108" s="1" t="inlineStr">
         <is>
           <t>notfound.home</t>
@@ -2169,7 +2169,7 @@
         </is>
       </c>
     </row>
-    <row r="109" ht="17" customHeight="1">
+    <row r="109" ht="18" customHeight="1">
       <c r="A109" s="1" t="inlineStr">
         <is>
           <t>notfound.back</t>
@@ -2186,7 +2186,7 @@
         </is>
       </c>
     </row>
-    <row r="110" ht="17" customHeight="1">
+    <row r="110" ht="18" customHeight="1">
       <c r="A110" s="1" t="inlineStr">
         <is>
           <t>register.confirm-password.error1</t>
@@ -2203,7 +2203,7 @@
         </is>
       </c>
     </row>
-    <row r="111" ht="17" customHeight="1">
+    <row r="111" ht="18" customHeight="1">
       <c r="A111" s="1" t="inlineStr">
         <is>
           <t>register.confirm-password.label</t>
@@ -2220,7 +2220,7 @@
         </is>
       </c>
     </row>
-    <row r="112" ht="17" customHeight="1">
+    <row r="112" ht="18" customHeight="1">
       <c r="A112" s="1" t="inlineStr">
         <is>
           <t>register.confirm-password.placeholder</t>
@@ -2237,7 +2237,7 @@
         </is>
       </c>
     </row>
-    <row r="113" ht="17" customHeight="1">
+    <row r="113" ht="18" customHeight="1">
       <c r="A113" s="1" t="inlineStr">
         <is>
           <t>register.display-name.label</t>
@@ -2254,7 +2254,7 @@
         </is>
       </c>
     </row>
-    <row r="114" ht="17" customHeight="1">
+    <row r="114" ht="18" customHeight="1">
       <c r="A114" s="1" t="inlineStr">
         <is>
           <t>register.display-name.placeholder</t>
@@ -2271,7 +2271,7 @@
         </is>
       </c>
     </row>
-    <row r="115" ht="17" customHeight="1">
+    <row r="115" ht="18" customHeight="1">
       <c r="A115" s="1" t="inlineStr">
         <is>
           <t>register.email.error1</t>
@@ -2288,7 +2288,7 @@
         </is>
       </c>
     </row>
-    <row r="116" ht="17" customHeight="1">
+    <row r="116" ht="18" customHeight="1">
       <c r="A116" s="1" t="inlineStr">
         <is>
           <t>register.email.label</t>
@@ -2305,7 +2305,7 @@
         </is>
       </c>
     </row>
-    <row r="117" ht="17" customHeight="1">
+    <row r="117" ht="18" customHeight="1">
       <c r="A117" s="1" t="inlineStr">
         <is>
           <t>register.email.placeholder</t>
@@ -2322,7 +2322,7 @@
         </is>
       </c>
     </row>
-    <row r="118" ht="17" customHeight="1">
+    <row r="118" ht="18" customHeight="1">
       <c r="A118" s="1" t="inlineStr">
         <is>
           <t>register.form.login</t>
@@ -2339,7 +2339,7 @@
         </is>
       </c>
     </row>
-    <row r="119" ht="17" customHeight="1">
+    <row r="119" ht="18" customHeight="1">
       <c r="A119" s="1" t="inlineStr">
         <is>
           <t>register.form.submit</t>
@@ -2356,7 +2356,7 @@
         </is>
       </c>
     </row>
-    <row r="120" ht="17" customHeight="1">
+    <row r="120" ht="18" customHeight="1">
       <c r="A120" s="1" t="inlineStr">
         <is>
           <t>register.form.success</t>
@@ -2373,7 +2373,7 @@
         </is>
       </c>
     </row>
-    <row r="121" ht="17" customHeight="1">
+    <row r="121" ht="18" customHeight="1">
       <c r="A121" s="1" t="inlineStr">
         <is>
           <t>register.form.title</t>
@@ -2390,7 +2390,7 @@
         </is>
       </c>
     </row>
-    <row r="122" ht="17" customHeight="1">
+    <row r="122" ht="18" customHeight="1">
       <c r="A122" s="1" t="inlineStr">
         <is>
           <t>register.gender.female</t>
@@ -2407,7 +2407,7 @@
         </is>
       </c>
     </row>
-    <row r="123" ht="17" customHeight="1">
+    <row r="123" ht="18" customHeight="1">
       <c r="A123" s="1" t="inlineStr">
         <is>
           <t>register.gender.label</t>
@@ -2424,7 +2424,7 @@
         </is>
       </c>
     </row>
-    <row r="124" ht="17" customHeight="1">
+    <row r="124" ht="18" customHeight="1">
       <c r="A124" s="1" t="inlineStr">
         <is>
           <t>register.gender.male</t>
@@ -2441,7 +2441,7 @@
         </is>
       </c>
     </row>
-    <row r="125" ht="17" customHeight="1">
+    <row r="125" ht="18" customHeight="1">
       <c r="A125" s="1" t="inlineStr">
         <is>
           <t>register.gender.select</t>
@@ -2458,7 +2458,7 @@
         </is>
       </c>
     </row>
-    <row r="126" ht="17" customHeight="1">
+    <row r="126" ht="18" customHeight="1">
       <c r="A126" s="1" t="inlineStr">
         <is>
           <t>register.page.title</t>
@@ -2475,7 +2475,7 @@
         </is>
       </c>
     </row>
-    <row r="127" ht="17" customHeight="1">
+    <row r="127" ht="36" customHeight="1">
       <c r="A127" s="1" t="inlineStr">
         <is>
           <t>register.password.error1</t>
@@ -2492,7 +2492,7 @@
         </is>
       </c>
     </row>
-    <row r="128" ht="17" customHeight="1">
+    <row r="128" ht="18" customHeight="1">
       <c r="A128" s="1" t="inlineStr">
         <is>
           <t>register.password.hide</t>
@@ -2509,7 +2509,7 @@
         </is>
       </c>
     </row>
-    <row r="129" ht="17" customHeight="1">
+    <row r="129" ht="18" customHeight="1">
       <c r="A129" s="1" t="inlineStr">
         <is>
           <t>register.password.label</t>
@@ -2526,7 +2526,7 @@
         </is>
       </c>
     </row>
-    <row r="130" ht="17" customHeight="1">
+    <row r="130" ht="18" customHeight="1">
       <c r="A130" s="1" t="inlineStr">
         <is>
           <t>register.password.placeholder</t>
@@ -2543,7 +2543,7 @@
         </is>
       </c>
     </row>
-    <row r="131" ht="17" customHeight="1">
+    <row r="131" ht="18" customHeight="1">
       <c r="A131" s="1" t="inlineStr">
         <is>
           <t>register.password.show</t>
@@ -2560,7 +2560,7 @@
         </is>
       </c>
     </row>
-    <row r="132" ht="17" customHeight="1">
+    <row r="132" ht="36" customHeight="1">
       <c r="A132" s="1" t="inlineStr">
         <is>
           <t>register.username.error1</t>
@@ -2577,7 +2577,7 @@
         </is>
       </c>
     </row>
-    <row r="133" ht="17" customHeight="1">
+    <row r="133" ht="18" customHeight="1">
       <c r="A133" s="1" t="inlineStr">
         <is>
           <t>register.username.label</t>
@@ -2594,7 +2594,7 @@
         </is>
       </c>
     </row>
-    <row r="134" ht="17" customHeight="1">
+    <row r="134" ht="18" customHeight="1">
       <c r="A134" s="1" t="inlineStr">
         <is>
           <t>register.username.placeholder</t>
@@ -2611,7 +2611,7 @@
         </is>
       </c>
     </row>
-    <row r="135" ht="17" customHeight="1">
+    <row r="135" ht="18" customHeight="1">
       <c r="A135" s="1" t="inlineStr">
         <is>
           <t>forgot-password.page.title</t>
@@ -2628,7 +2628,7 @@
         </is>
       </c>
     </row>
-    <row r="136" ht="17" customHeight="1">
+    <row r="136" ht="18" customHeight="1">
       <c r="A136" s="1" t="inlineStr">
         <is>
           <t>forgot-password.form.title</t>
@@ -2645,7 +2645,7 @@
         </is>
       </c>
     </row>
-    <row r="137" ht="17" customHeight="1">
+    <row r="137" ht="18" customHeight="1">
       <c r="A137" s="1" t="inlineStr">
         <is>
           <t>forgot-password.form.login</t>
@@ -2662,7 +2662,7 @@
         </is>
       </c>
     </row>
-    <row r="138" ht="17" customHeight="1">
+    <row r="138" ht="18" customHeight="1">
       <c r="A138" s="1" t="inlineStr">
         <is>
           <t>forgot-password.form.submit</t>
@@ -2679,7 +2679,7 @@
         </is>
       </c>
     </row>
-    <row r="139" ht="17" customHeight="1">
+    <row r="139" ht="36" customHeight="1">
       <c r="A139" s="1" t="inlineStr">
         <is>
           <t>forgot-password.form.success</t>
@@ -2696,7 +2696,7 @@
         </is>
       </c>
     </row>
-    <row r="140" ht="17" customHeight="1">
+    <row r="140" ht="18" customHeight="1">
       <c r="A140" s="1" t="inlineStr">
         <is>
           <t>forgot-password.form.error1</t>
@@ -2713,7 +2713,7 @@
         </is>
       </c>
     </row>
-    <row r="141" ht="17" customHeight="1">
+    <row r="141" ht="18" customHeight="1">
       <c r="A141" s="1" t="inlineStr">
         <is>
           <t>reset-password.page.title</t>
@@ -2730,7 +2730,7 @@
         </is>
       </c>
     </row>
-    <row r="142" ht="17" customHeight="1">
+    <row r="142" ht="18" customHeight="1">
       <c r="A142" s="1" t="inlineStr">
         <is>
           <t>reset-password.form.title</t>
@@ -2747,7 +2747,7 @@
         </is>
       </c>
     </row>
-    <row r="143" ht="17" customHeight="1">
+    <row r="143" ht="18" customHeight="1">
       <c r="A143" s="1" t="inlineStr">
         <is>
           <t>reset-password.form.submit</t>
@@ -2764,7 +2764,7 @@
         </is>
       </c>
     </row>
-    <row r="144" ht="17" customHeight="1">
+    <row r="144" ht="36" customHeight="1">
       <c r="A144" s="1" t="inlineStr">
         <is>
           <t>reset-password.form.error1</t>
@@ -2781,7 +2781,7 @@
         </is>
       </c>
     </row>
-    <row r="145" ht="17" customHeight="1">
+    <row r="145" ht="18" customHeight="1">
       <c r="A145" s="1" t="inlineStr">
         <is>
           <t>reset-password.form.invalid-token</t>
@@ -2798,7 +2798,7 @@
         </is>
       </c>
     </row>
-    <row r="146" ht="17" customHeight="1">
+    <row r="146" ht="36" customHeight="1">
       <c r="A146" s="1" t="inlineStr">
         <is>
           <t>reset-password.form.success</t>
@@ -2815,7 +2815,7 @@
         </is>
       </c>
     </row>
-    <row r="147" ht="17" customHeight="1">
+    <row r="147" ht="18" customHeight="1">
       <c r="A147" s="1" t="inlineStr">
         <is>
           <t>reset-password.action.back-to-login</t>
@@ -2832,7 +2832,7 @@
         </is>
       </c>
     </row>
-    <row r="148" ht="17" customHeight="1">
+    <row r="148" ht="18" customHeight="1">
       <c r="A148" s="1" t="inlineStr">
         <is>
           <t>reset-password.action.submit</t>
@@ -2849,7 +2849,7 @@
         </is>
       </c>
     </row>
-    <row r="149" ht="17" customHeight="1">
+    <row r="149" ht="18" customHeight="1">
       <c r="A149" s="1" t="inlineStr">
         <is>
           <t>auth-middleware.messages.invalid-token-payload</t>
@@ -2866,7 +2866,7 @@
         </is>
       </c>
     </row>
-    <row r="150" ht="17" customHeight="1">
+    <row r="150" ht="18" customHeight="1">
       <c r="A150" s="1" t="inlineStr">
         <is>
           <t>auth-middleware.messages.session-not-found</t>
@@ -2883,7 +2883,7 @@
         </is>
       </c>
     </row>
-    <row r="151" ht="17" customHeight="1">
+    <row r="151" ht="18" customHeight="1">
       <c r="A151" s="1" t="inlineStr">
         <is>
           <t>auth-middleware.messages.token-expired</t>
@@ -2900,7 +2900,7 @@
         </is>
       </c>
     </row>
-    <row r="152" ht="17" customHeight="1">
+    <row r="152" ht="18" customHeight="1">
       <c r="A152" s="1" t="inlineStr">
         <is>
           <t>auth-middleware.messages.token-invalid</t>
@@ -2917,7 +2917,7 @@
         </is>
       </c>
     </row>
-    <row r="153" ht="17" customHeight="1">
+    <row r="153" ht="18" customHeight="1">
       <c r="A153" s="1" t="inlineStr">
         <is>
           <t>auth-middleware.messages.token-required</t>
@@ -2934,7 +2934,7 @@
         </is>
       </c>
     </row>
-    <row r="154" ht="17" customHeight="1">
+    <row r="154" ht="18" customHeight="1">
       <c r="A154" s="1" t="inlineStr">
         <is>
           <t>auth-middleware.messages.token-subject-mismatch</t>
@@ -2951,7 +2951,7 @@
         </is>
       </c>
     </row>
-    <row r="155" ht="17" customHeight="1">
+    <row r="155" ht="18" customHeight="1">
       <c r="A155" s="1" t="inlineStr">
         <is>
           <t>auth-middleware.messages.token-validation-failed</t>
@@ -2968,7 +2968,7 @@
         </is>
       </c>
     </row>
-    <row r="156" ht="17" customHeight="1">
+    <row r="156" ht="36" customHeight="1">
       <c r="A156" s="1" t="inlineStr">
         <is>
           <t>create-room.messages.insufficient-amount</t>
@@ -2985,7 +2985,7 @@
         </is>
       </c>
     </row>
-    <row r="157" ht="17" customHeight="1">
+    <row r="157" ht="18" customHeight="1">
       <c r="A157" s="1" t="inlineStr">
         <is>
           <t>create-room.messages.internal-server-error</t>
@@ -3002,7 +3002,7 @@
         </is>
       </c>
     </row>
-    <row r="158" ht="17" customHeight="1">
+    <row r="158" ht="36" customHeight="1">
       <c r="A158" s="1" t="inlineStr">
         <is>
           <t>create-room.messages.invalid-bet-amount</t>
@@ -3019,7 +3019,7 @@
         </is>
       </c>
     </row>
-    <row r="159" ht="17" customHeight="1">
+    <row r="159" ht="18" customHeight="1">
       <c r="A159" s="1" t="inlineStr">
         <is>
           <t>create-room.messages.invalid-redFirst</t>
@@ -3036,7 +3036,7 @@
         </is>
       </c>
     </row>
-    <row r="160" ht="17" customHeight="1">
+    <row r="160" ht="18" customHeight="1">
       <c r="A160" s="1" t="inlineStr">
         <is>
           <t>create-room.messages.invalid-team-name</t>
@@ -3053,7 +3053,7 @@
         </is>
       </c>
     </row>
-    <row r="161" ht="17" customHeight="1">
+    <row r="161" ht="36" customHeight="1">
       <c r="A161" s="1" t="inlineStr">
         <is>
           <t>create-room.messages.name-required</t>
@@ -3070,7 +3070,7 @@
         </is>
       </c>
     </row>
-    <row r="162" ht="17" customHeight="1">
+    <row r="162" ht="18" customHeight="1">
       <c r="A162" s="1" t="inlineStr">
         <is>
           <t>create-room.messages.room-created</t>
@@ -3087,7 +3087,7 @@
         </is>
       </c>
     </row>
-    <row r="163" ht="17" customHeight="1">
+    <row r="163" ht="18" customHeight="1">
       <c r="A163" s="1" t="inlineStr">
         <is>
           <t>fetch-rooms.messages.internal-server-error</t>
@@ -3104,7 +3104,7 @@
         </is>
       </c>
     </row>
-    <row r="164" ht="17" customHeight="1">
+    <row r="164" ht="18" customHeight="1">
       <c r="A164" s="1" t="inlineStr">
         <is>
           <t>fetch-rooms.messages.invalid-status</t>
@@ -3121,7 +3121,7 @@
         </is>
       </c>
     </row>
-    <row r="165" ht="17" customHeight="1">
+    <row r="165" ht="18" customHeight="1">
       <c r="A165" s="1" t="inlineStr">
         <is>
           <t>fetch-rooms.messages.success</t>
@@ -3138,7 +3138,7 @@
         </is>
       </c>
     </row>
-    <row r="166" ht="17" customHeight="1">
+    <row r="166" ht="18" customHeight="1">
       <c r="A166" s="1" t="inlineStr">
         <is>
           <t>forgot-password.messages.email-not-found</t>
@@ -3155,7 +3155,7 @@
         </is>
       </c>
     </row>
-    <row r="167" ht="17" customHeight="1">
+    <row r="167" ht="18" customHeight="1">
       <c r="A167" s="1" t="inlineStr">
         <is>
           <t>forgot-password.messages.email-service-not-configured</t>
@@ -3172,7 +3172,7 @@
         </is>
       </c>
     </row>
-    <row r="168" ht="17" customHeight="1">
+    <row r="168" ht="18" customHeight="1">
       <c r="A168" s="1" t="inlineStr">
         <is>
           <t>forgot-password.messages.internal-server-error</t>
@@ -3189,7 +3189,7 @@
         </is>
       </c>
     </row>
-    <row r="169" ht="17" customHeight="1">
+    <row r="169" ht="18" customHeight="1">
       <c r="A169" s="1" t="inlineStr">
         <is>
           <t>forgot-password.messages.invalid-email-format</t>
@@ -3206,7 +3206,7 @@
         </is>
       </c>
     </row>
-    <row r="170" ht="17" customHeight="1">
+    <row r="170" ht="18" customHeight="1">
       <c r="A170" s="1" t="inlineStr">
         <is>
           <t>forgot-password.messages.missing-email</t>
@@ -3223,7 +3223,7 @@
         </is>
       </c>
     </row>
-    <row r="171" ht="17" customHeight="1">
+    <row r="171" ht="18" customHeight="1">
       <c r="A171" s="1" t="inlineStr">
         <is>
           <t>forgot-password.messages.success</t>
@@ -3240,7 +3240,7 @@
         </is>
       </c>
     </row>
-    <row r="172" ht="17" customHeight="1">
+    <row r="172" ht="18" customHeight="1">
       <c r="A172" s="1" t="inlineStr">
         <is>
           <t>join-room.messages.internal-server-error</t>
@@ -3257,7 +3257,7 @@
         </is>
       </c>
     </row>
-    <row r="173" ht="17" customHeight="1">
+    <row r="173" ht="36" customHeight="1">
       <c r="A173" s="1" t="inlineStr">
         <is>
           <t>join-room.messages.invalid-team</t>
@@ -3274,7 +3274,7 @@
         </is>
       </c>
     </row>
-    <row r="174" ht="17" customHeight="1">
+    <row r="174" ht="18" customHeight="1">
       <c r="A174" s="1" t="inlineStr">
         <is>
           <t>join-room.messages.invalid-room-id</t>
@@ -3291,7 +3291,7 @@
         </is>
       </c>
     </row>
-    <row r="175" ht="17" customHeight="1">
+    <row r="175" ht="18" customHeight="1">
       <c r="A175" s="1" t="inlineStr">
         <is>
           <t>join-room.messages.room-not-found</t>
@@ -3308,7 +3308,7 @@
         </is>
       </c>
     </row>
-    <row r="176" ht="17" customHeight="1">
+    <row r="176" ht="18" customHeight="1">
       <c r="A176" s="1" t="inlineStr">
         <is>
           <t>join-room.messages.success</t>
@@ -3325,7 +3325,7 @@
         </is>
       </c>
     </row>
-    <row r="177" ht="17" customHeight="1">
+    <row r="177" ht="18" customHeight="1">
       <c r="A177" s="1" t="inlineStr">
         <is>
           <t>join-room.messages.team-seat-occupied</t>
@@ -3342,7 +3342,7 @@
         </is>
       </c>
     </row>
-    <row r="178" ht="17" customHeight="1">
+    <row r="178" ht="18" customHeight="1">
       <c r="A178" s="1" t="inlineStr">
         <is>
           <t>kick-user.messages.cannot-kick-self</t>
@@ -3359,7 +3359,7 @@
         </is>
       </c>
     </row>
-    <row r="179" ht="17" customHeight="1">
+    <row r="179" ht="18" customHeight="1">
       <c r="A179" s="1" t="inlineStr">
         <is>
           <t>kick-user.messages.forbidden</t>
@@ -3376,7 +3376,7 @@
         </is>
       </c>
     </row>
-    <row r="180" ht="17" customHeight="1">
+    <row r="180" ht="18" customHeight="1">
       <c r="A180" s="1" t="inlineStr">
         <is>
           <t>kick-user.messages.internal-server-error</t>
@@ -3393,7 +3393,7 @@
         </is>
       </c>
     </row>
-    <row r="181" ht="17" customHeight="1">
+    <row r="181" ht="18" customHeight="1">
       <c r="A181" s="1" t="inlineStr">
         <is>
           <t>kick-user.messages.invalid-room-id</t>
@@ -3410,7 +3410,7 @@
         </is>
       </c>
     </row>
-    <row r="182" ht="17" customHeight="1">
+    <row r="182" ht="36" customHeight="1">
       <c r="A182" s="1" t="inlineStr">
         <is>
           <t>kick-user.messages.invalid-user-id</t>
@@ -3427,7 +3427,7 @@
         </is>
       </c>
     </row>
-    <row r="183" ht="17" customHeight="1">
+    <row r="183" ht="18" customHeight="1">
       <c r="A183" s="1" t="inlineStr">
         <is>
           <t>kick-user.messages.room-not-found</t>
@@ -3444,7 +3444,7 @@
         </is>
       </c>
     </row>
-    <row r="184" ht="17" customHeight="1">
+    <row r="184" ht="36" customHeight="1">
       <c r="A184" s="1" t="inlineStr">
         <is>
           <t>kick-user.messages.room-not-waiting</t>
@@ -3461,7 +3461,7 @@
         </is>
       </c>
     </row>
-    <row r="185" ht="17" customHeight="1">
+    <row r="185" ht="18" customHeight="1">
       <c r="A185" s="1" t="inlineStr">
         <is>
           <t>kick-user.messages.success</t>
@@ -3478,7 +3478,7 @@
         </is>
       </c>
     </row>
-    <row r="186" ht="17" customHeight="1">
+    <row r="186" ht="18" customHeight="1">
       <c r="A186" s="1" t="inlineStr">
         <is>
           <t>kick-user.messages.user-not-in-room</t>
@@ -3495,7 +3495,7 @@
         </is>
       </c>
     </row>
-    <row r="187" ht="17" customHeight="1">
+    <row r="187" ht="18" customHeight="1">
       <c r="A187" s="1" t="inlineStr">
         <is>
           <t>kick-user.messages.you-were-kicked</t>
@@ -3512,7 +3512,7 @@
         </is>
       </c>
     </row>
-    <row r="188" ht="36" customHeight="1">
+    <row r="188" ht="18" customHeight="1">
       <c r="A188" s="1" t="inlineStr">
         <is>
           <t>leave-room.messages.internal-server-error</t>
@@ -3529,7 +3529,7 @@
         </is>
       </c>
     </row>
-    <row r="189" ht="17" customHeight="1">
+    <row r="189" ht="18" customHeight="1">
       <c r="A189" s="1" t="inlineStr">
         <is>
           <t>leave-room.messages.invalid-room-id</t>
@@ -3546,7 +3546,7 @@
         </is>
       </c>
     </row>
-    <row r="190" ht="17" customHeight="1">
+    <row r="190" ht="18" customHeight="1">
       <c r="A190" s="1" t="inlineStr">
         <is>
           <t>leave-room.messages.player-not-in-room</t>
@@ -3563,7 +3563,7 @@
         </is>
       </c>
     </row>
-    <row r="191" ht="17" customHeight="1">
+    <row r="191" ht="18" customHeight="1">
       <c r="A191" s="1" t="inlineStr">
         <is>
           <t>leave-room.messages.success</t>
@@ -3580,7 +3580,7 @@
         </is>
       </c>
     </row>
-    <row r="192" ht="17" customHeight="1">
+    <row r="192" ht="18" customHeight="1">
       <c r="A192" s="1" t="inlineStr">
         <is>
           <t>load-room.messages.internal-server-error</t>
@@ -3597,7 +3597,7 @@
         </is>
       </c>
     </row>
-    <row r="193" ht="17" customHeight="1">
+    <row r="193" ht="18" customHeight="1">
       <c r="A193" s="1" t="inlineStr">
         <is>
           <t>load-room.messages.invalid-room-id</t>
@@ -3614,7 +3614,7 @@
         </is>
       </c>
     </row>
-    <row r="194" ht="17" customHeight="1">
+    <row r="194" ht="18" customHeight="1">
       <c r="A194" s="1" t="inlineStr">
         <is>
           <t>load-room.messages.room-not-found</t>
@@ -3631,7 +3631,7 @@
         </is>
       </c>
     </row>
-    <row r="195" ht="17" customHeight="1">
+    <row r="195" ht="18" customHeight="1">
       <c r="A195" s="1" t="inlineStr">
         <is>
           <t>load-room.messages.success</t>
@@ -3648,7 +3648,7 @@
         </is>
       </c>
     </row>
-    <row r="196" ht="17" customHeight="1">
+    <row r="196" ht="18" customHeight="1">
       <c r="A196" s="1" t="inlineStr">
         <is>
           <t>login.messages.incorrect-login</t>
@@ -3665,7 +3665,7 @@
         </is>
       </c>
     </row>
-    <row r="197" ht="17" customHeight="1">
+    <row r="197" ht="18" customHeight="1">
       <c r="A197" s="1" t="inlineStr">
         <is>
           <t>login.messages.internal-server-error</t>
@@ -3682,7 +3682,7 @@
         </is>
       </c>
     </row>
-    <row r="198" ht="17" customHeight="1">
+    <row r="198" ht="18" customHeight="1">
       <c r="A198" s="1" t="inlineStr">
         <is>
           <t>login.messages.missing-credentials</t>
@@ -3699,7 +3699,7 @@
         </is>
       </c>
     </row>
-    <row r="199" ht="17" customHeight="1">
+    <row r="199" ht="18" customHeight="1">
       <c r="A199" s="1" t="inlineStr">
         <is>
           <t>login.messages.success</t>
@@ -3716,7 +3716,7 @@
         </is>
       </c>
     </row>
-    <row r="200" ht="17" customHeight="1">
+    <row r="200" ht="18" customHeight="1">
       <c r="A200" s="1" t="inlineStr">
         <is>
           <t>logout.messages.already-inactive</t>
@@ -3733,7 +3733,7 @@
         </is>
       </c>
     </row>
-    <row r="201" ht="17" customHeight="1">
+    <row r="201" ht="18" customHeight="1">
       <c r="A201" s="1" t="inlineStr">
         <is>
           <t>logout.messages.internal-server-error</t>
@@ -3750,7 +3750,7 @@
         </is>
       </c>
     </row>
-    <row r="202" ht="17" customHeight="1">
+    <row r="202" ht="18" customHeight="1">
       <c r="A202" s="1" t="inlineStr">
         <is>
           <t>logout.messages.success</t>
@@ -3767,7 +3767,7 @@
         </is>
       </c>
     </row>
-    <row r="203" ht="17" customHeight="1">
+    <row r="203" ht="18" customHeight="1">
       <c r="A203" s="1" t="inlineStr">
         <is>
           <t>refresh-token.messages.missing-refresh-token</t>
@@ -3784,7 +3784,7 @@
         </is>
       </c>
     </row>
-    <row r="204" ht="17" customHeight="1">
+    <row r="204" ht="18" customHeight="1">
       <c r="A204" s="1" t="inlineStr">
         <is>
           <t>refresh-token.messages.mismatch-or-expired</t>
@@ -3801,7 +3801,7 @@
         </is>
       </c>
     </row>
-    <row r="205" ht="17" customHeight="1">
+    <row r="205" ht="18" customHeight="1">
       <c r="A205" s="1" t="inlineStr">
         <is>
           <t>refresh-token.messages.success</t>
@@ -3818,7 +3818,7 @@
         </is>
       </c>
     </row>
-    <row r="206" ht="17" customHeight="1">
+    <row r="206" ht="18" customHeight="1">
       <c r="A206" s="1" t="inlineStr">
         <is>
           <t>register.messages.email-exists</t>
@@ -3835,7 +3835,7 @@
         </is>
       </c>
     </row>
-    <row r="207" ht="17" customHeight="1">
+    <row r="207" ht="18" customHeight="1">
       <c r="A207" s="1" t="inlineStr">
         <is>
           <t>register.messages.internal-server-error</t>
@@ -3852,7 +3852,7 @@
         </is>
       </c>
     </row>
-    <row r="208" ht="17" customHeight="1">
+    <row r="208" ht="36" customHeight="1">
       <c r="A208" s="1" t="inlineStr">
         <is>
           <t>register.messages.missing-fields</t>
@@ -3869,7 +3869,7 @@
         </is>
       </c>
     </row>
-    <row r="209" ht="17" customHeight="1">
+    <row r="209" ht="18" customHeight="1">
       <c r="A209" s="1" t="inlineStr">
         <is>
           <t>register.messages.success</t>
@@ -3886,7 +3886,7 @@
         </is>
       </c>
     </row>
-    <row r="210" ht="17" customHeight="1">
+    <row r="210" ht="18" customHeight="1">
       <c r="A210" s="1" t="inlineStr">
         <is>
           <t>register.messages.username-exists</t>
@@ -3903,7 +3903,7 @@
         </is>
       </c>
     </row>
-    <row r="211" ht="17" customHeight="1">
+    <row r="211" ht="18" customHeight="1">
       <c r="A211" s="1" t="inlineStr">
         <is>
           <t>reset-password.messages.internal-server-error</t>
@@ -3920,7 +3920,7 @@
         </is>
       </c>
     </row>
-    <row r="212" ht="17" customHeight="1">
+    <row r="212" ht="18" customHeight="1">
       <c r="A212" s="1" t="inlineStr">
         <is>
           <t>reset-password.messages.invalid-or-expired-token</t>
@@ -3937,7 +3937,7 @@
         </is>
       </c>
     </row>
-    <row r="213" ht="17" customHeight="1">
+    <row r="213" ht="18" customHeight="1">
       <c r="A213" s="1" t="inlineStr">
         <is>
           <t>reset-password.messages.invalid-user-id</t>
@@ -3954,7 +3954,7 @@
         </is>
       </c>
     </row>
-    <row r="214" ht="17" customHeight="1">
+    <row r="214" ht="18" customHeight="1">
       <c r="A214" s="1" t="inlineStr">
         <is>
           <t>reset-password.messages.missing-id-or-token</t>
@@ -3971,7 +3971,7 @@
         </is>
       </c>
     </row>
-    <row r="215" ht="17" customHeight="1">
+    <row r="215" ht="18" customHeight="1">
       <c r="A215" s="1" t="inlineStr">
         <is>
           <t>reset-password.messages.missing-userId-or-password</t>
@@ -3988,7 +3988,7 @@
         </is>
       </c>
     </row>
-    <row r="216" ht="17" customHeight="1">
+    <row r="216" ht="18" customHeight="1">
       <c r="A216" s="1" t="inlineStr">
         <is>
           <t>reset-password.messages.token-valid</t>
@@ -4005,7 +4005,7 @@
         </is>
       </c>
     </row>
-    <row r="217" ht="17" customHeight="1">
+    <row r="217" ht="18" customHeight="1">
       <c r="A217" s="1" t="inlineStr">
         <is>
           <t>reset-password.messages.user-not-found</t>
@@ -4022,7 +4022,7 @@
         </is>
       </c>
     </row>
-    <row r="218" ht="17" customHeight="1">
+    <row r="218" ht="18" customHeight="1">
       <c r="A218" s="1" t="inlineStr">
         <is>
           <t>set-room-status.messages.internal-server-error</t>
@@ -4039,7 +4039,7 @@
         </is>
       </c>
     </row>
-    <row r="219" ht="17" customHeight="1">
+    <row r="219" ht="18" customHeight="1">
       <c r="A219" s="1" t="inlineStr">
         <is>
           <t>set-room-status.messages.invalid-room-id</t>
@@ -4229,721 +4229,721 @@
     <row r="230" ht="18" customHeight="1">
       <c r="A230" s="1" t="inlineStr">
         <is>
-          <t>room.actions.accept-draw</t>
+          <t>room.actions.flip-board</t>
         </is>
       </c>
       <c r="B230" s="2" t="inlineStr">
         <is>
-          <t>Accept</t>
+          <t>Flip board</t>
         </is>
       </c>
       <c r="C230" s="2" t="inlineStr">
         <is>
-          <t>Chấp nhận</t>
+          <t>Đảo chiều bàn cờ</t>
         </is>
       </c>
     </row>
     <row r="231" ht="18" customHeight="1">
       <c r="A231" s="1" t="inlineStr">
         <is>
-          <t>room.actions.reject-draw</t>
+          <t>room.actions.accept-draw</t>
         </is>
       </c>
       <c r="B231" s="2" t="inlineStr">
         <is>
-          <t>Reject</t>
+          <t>Accept</t>
         </is>
       </c>
       <c r="C231" s="2" t="inlineStr">
         <is>
-          <t>Từ chối</t>
+          <t>Chấp nhận</t>
         </is>
       </c>
     </row>
     <row r="232" ht="18" customHeight="1">
       <c r="A232" s="1" t="inlineStr">
         <is>
-          <t>room.actions.send-pm</t>
+          <t>room.actions.reject-draw</t>
         </is>
       </c>
       <c r="B232" s="2" t="inlineStr">
         <is>
-          <t>Send PM</t>
+          <t>Reject</t>
         </is>
       </c>
       <c r="C232" s="2" t="inlineStr">
         <is>
-          <t>Chat</t>
+          <t>Từ chối</t>
         </is>
       </c>
     </row>
     <row r="233" ht="18" customHeight="1">
       <c r="A233" s="1" t="inlineStr">
         <is>
-          <t>room.actions.view-history</t>
+          <t>room.actions.send-pm</t>
         </is>
       </c>
       <c r="B233" s="2" t="inlineStr">
         <is>
-          <t>History</t>
+          <t>Send PM</t>
         </is>
       </c>
       <c r="C233" s="2" t="inlineStr">
         <is>
-          <t>Lịch sử</t>
+          <t>Chat</t>
         </is>
       </c>
     </row>
     <row r="234" ht="18" customHeight="1">
       <c r="A234" s="1" t="inlineStr">
         <is>
-          <t>room.actions.kick</t>
+          <t>room.actions.view-history</t>
         </is>
       </c>
       <c r="B234" s="2" t="inlineStr">
         <is>
-          <t>Kick</t>
+          <t>History</t>
         </is>
       </c>
       <c r="C234" s="2" t="inlineStr">
         <is>
-          <t>Kick</t>
+          <t>Lịch sử</t>
         </is>
       </c>
     </row>
     <row r="235" ht="18" customHeight="1">
       <c r="A235" s="1" t="inlineStr">
         <is>
-          <t>room.actions.settings</t>
+          <t>room.actions.kick</t>
         </is>
       </c>
       <c r="B235" s="2" t="inlineStr">
         <is>
-          <t>Room settings</t>
+          <t>Kick</t>
         </is>
       </c>
       <c r="C235" s="2" t="inlineStr">
         <is>
-          <t>Cài đặt phòng</t>
+          <t>Kick</t>
         </is>
       </c>
     </row>
     <row r="236" ht="18" customHeight="1">
       <c r="A236" s="1" t="inlineStr">
         <is>
-          <t>room.messages.draw-accepted</t>
+          <t>room.actions.settings</t>
         </is>
       </c>
       <c r="B236" s="2" t="inlineStr">
         <is>
-          <t>Opponent accepted the draw</t>
+          <t>Room settings</t>
         </is>
       </c>
       <c r="C236" s="2" t="inlineStr">
         <is>
-          <t>Đối phương đã đồng ý hòa</t>
+          <t>Cài đặt phòng</t>
         </is>
       </c>
     </row>
     <row r="237" ht="18" customHeight="1">
       <c r="A237" s="1" t="inlineStr">
         <is>
-          <t>room.messages.draw-rejected</t>
+          <t>room.messages.draw-accepted</t>
         </is>
       </c>
       <c r="B237" s="2" t="inlineStr">
         <is>
-          <t>Opponent rejected the draw</t>
+          <t>Opponent accepted the draw</t>
         </is>
       </c>
       <c r="C237" s="2" t="inlineStr">
         <is>
-          <t>Đối phương từ chối hòa</t>
+          <t>Đối phương đã đồng ý hòa</t>
         </is>
       </c>
     </row>
     <row r="238" ht="18" customHeight="1">
       <c r="A238" s="1" t="inlineStr">
         <is>
-          <t>room.messages.draw-completed</t>
+          <t>room.messages.draw-rejected</t>
         </is>
       </c>
       <c r="B238" s="2" t="inlineStr">
         <is>
-          <t>Draw completed</t>
+          <t>Opponent rejected the draw</t>
         </is>
       </c>
       <c r="C238" s="2" t="inlineStr">
         <is>
-          <t>Hòa cờ thành công</t>
+          <t>Đối phương từ chối hòa</t>
         </is>
       </c>
     </row>
     <row r="239" ht="18" customHeight="1">
       <c r="A239" s="1" t="inlineStr">
         <is>
-          <t>room.messages.opponent-surrendered</t>
+          <t>room.messages.draw-completed</t>
         </is>
       </c>
       <c r="B239" s="2" t="inlineStr">
         <is>
-          <t>Opponent surrendered! You won!</t>
+          <t>Draw completed</t>
         </is>
       </c>
       <c r="C239" s="2" t="inlineStr">
         <is>
-          <t>Đối phương đã đầu hàng! Bạn thắng!</t>
+          <t>Hòa cờ thành công</t>
         </is>
       </c>
     </row>
     <row r="240" ht="18" customHeight="1">
       <c r="A240" s="1" t="inlineStr">
         <is>
-          <t>room.messages.confirm-leave</t>
+          <t>room.messages.opponent-surrendered</t>
         </is>
       </c>
       <c r="B240" s="2" t="inlineStr">
         <is>
-          <t>Are you sure you want to leave room?</t>
+          <t>Opponent surrendered! You won!</t>
         </is>
       </c>
       <c r="C240" s="2" t="inlineStr">
         <is>
-          <t>Bạn có chắc muốn rời bàn chơi?</t>
+          <t>Đối phương đã đầu hàng! Bạn thắng!</t>
         </is>
       </c>
     </row>
     <row r="241" ht="18" customHeight="1">
       <c r="A241" s="1" t="inlineStr">
         <is>
-          <t>room.messages.confirm-surrender</t>
+          <t>room.messages.confirm-leave</t>
         </is>
       </c>
       <c r="B241" s="2" t="inlineStr">
         <is>
-          <t>Are you sure you want to surrender?</t>
+          <t>Are you sure you want to leave room?</t>
         </is>
       </c>
       <c r="C241" s="2" t="inlineStr">
         <is>
-          <t>Bạn có chắc chắn muốn đầu hàng không?</t>
+          <t>Bạn có chắc muốn rời bàn chơi?</t>
         </is>
       </c>
     </row>
     <row r="242" ht="18" customHeight="1">
       <c r="A242" s="1" t="inlineStr">
         <is>
-          <t>room.messages.confirm-draw</t>
+          <t>room.messages.confirm-surrender</t>
         </is>
       </c>
       <c r="B242" s="2" t="inlineStr">
         <is>
-          <t>Are you sure you want to draw?</t>
+          <t>Are you sure you want to surrender?</t>
         </is>
       </c>
       <c r="C242" s="2" t="inlineStr">
         <is>
-          <t>Bạn có chắc chắn muốn hòa không?</t>
+          <t>Bạn có chắc chắn muốn đầu hàng không?</t>
         </is>
       </c>
     </row>
     <row r="243" ht="18" customHeight="1">
       <c r="A243" s="1" t="inlineStr">
         <is>
-          <t>room.messages.confirm-accept-draw</t>
+          <t>room.messages.confirm-draw</t>
         </is>
       </c>
       <c r="B243" s="2" t="inlineStr">
         <is>
-          <t>Opponent has proposed a draw. Do you accept?</t>
+          <t>Are you sure you want to draw?</t>
         </is>
       </c>
       <c r="C243" s="2" t="inlineStr">
         <is>
-          <t>Đối phương đã chủ hòa, bạn có đồng ý không?</t>
+          <t>Bạn có chắc chắn muốn hòa không?</t>
         </is>
       </c>
     </row>
     <row r="244" ht="18" customHeight="1">
       <c r="A244" s="1" t="inlineStr">
         <is>
-          <t>room.messages.insufficient-amount</t>
+          <t>room.messages.confirm-accept-draw</t>
         </is>
       </c>
       <c r="B244" s="2" t="inlineStr">
         <is>
-          <t>You do not have enough balance to join this room</t>
+          <t>Opponent has proposed a draw. Do you accept?</t>
         </is>
       </c>
       <c r="C244" s="2" t="inlineStr">
         <is>
-          <t>Bạn không đủ tiền để tham gia bàn chơi này</t>
+          <t>Đối phương đã chủ hòa, bạn có đồng ý không?</t>
         </is>
       </c>
     </row>
     <row r="245" ht="18" customHeight="1">
       <c r="A245" s="1" t="inlineStr">
         <is>
-          <t>room.messages.all-seats-occupied</t>
+          <t>room.messages.insufficient-amount</t>
         </is>
       </c>
       <c r="B245" s="2" t="inlineStr">
         <is>
-          <t>All player seats are occupied</t>
+          <t>You do not have enough balance to join this room</t>
         </is>
       </c>
       <c r="C245" s="2" t="inlineStr">
         <is>
-          <t>Tất cả ghế chơi đã được chiếm</t>
+          <t>Bạn không đủ tiền để tham gia bàn chơi này</t>
         </is>
       </c>
     </row>
     <row r="246" ht="18" customHeight="1">
       <c r="A246" s="1" t="inlineStr">
         <is>
-          <t>room.settings.title</t>
+          <t>room.messages.all-seats-occupied</t>
         </is>
       </c>
       <c r="B246" s="2" t="inlineStr">
         <is>
-          <t>Room Settings</t>
+          <t>All player seats are occupied</t>
         </is>
       </c>
       <c r="C246" s="2" t="inlineStr">
         <is>
-          <t>Cài đặt phòng</t>
+          <t>Tất cả ghế chơi đã được chiếm</t>
         </is>
       </c>
     </row>
     <row r="247" ht="18" customHeight="1">
       <c r="A247" s="1" t="inlineStr">
         <is>
+          <t>room.notifications.joined</t>
+        </is>
+      </c>
+      <c r="B247" s="2" t="inlineStr">
+        <is>
+          <t>{0} joined the room</t>
+        </is>
+      </c>
+      <c r="C247" s="2" t="inlineStr">
+        <is>
+          <t>{0} đã vào phòng</t>
+        </is>
+      </c>
+    </row>
+    <row r="248" ht="18" customHeight="1">
+      <c r="A248" s="1" t="inlineStr">
+        <is>
+          <t>room.notifications.left</t>
+        </is>
+      </c>
+      <c r="B248" s="2" t="inlineStr">
+        <is>
+          <t>{0} left the room</t>
+        </is>
+      </c>
+      <c r="C248" s="2" t="inlineStr">
+        <is>
+          <t>{0} đã rời phòng</t>
+        </is>
+      </c>
+    </row>
+    <row r="249" ht="18" customHeight="1">
+      <c r="A249" s="1" t="inlineStr">
+        <is>
+          <t>room.settings.title</t>
+        </is>
+      </c>
+      <c r="B249" s="2" t="inlineStr">
+        <is>
+          <t>Room Settings</t>
+        </is>
+      </c>
+      <c r="C249" s="2" t="inlineStr">
+        <is>
+          <t>Cài đặt phòng</t>
+        </is>
+      </c>
+    </row>
+    <row r="250" ht="18" customHeight="1">
+      <c r="A250" s="1" t="inlineStr">
+        <is>
           <t>room.settings.room-name</t>
         </is>
       </c>
-      <c r="B247" s="2" t="inlineStr">
+      <c r="B250" s="2" t="inlineStr">
         <is>
           <t>Room name</t>
         </is>
       </c>
-      <c r="C247" s="2" t="inlineStr">
+      <c r="C250" s="2" t="inlineStr">
         <is>
           <t>Tên phòng</t>
         </is>
       </c>
     </row>
-    <row r="248" ht="17" customHeight="1">
-      <c r="A248" s="1" t="inlineStr">
+    <row r="251" ht="18" customHeight="1">
+      <c r="A251" s="1" t="inlineStr">
         <is>
           <t>room.settings.players</t>
         </is>
       </c>
-      <c r="B248" s="2" t="inlineStr">
+      <c r="B251" s="2" t="inlineStr">
         <is>
           <t>Spectators</t>
         </is>
       </c>
-      <c r="C248" s="2" t="inlineStr">
+      <c r="C251" s="2" t="inlineStr">
         <is>
           <t>Người xem</t>
         </is>
       </c>
     </row>
-    <row r="249" ht="17" customHeight="1">
-      <c r="A249" s="1" t="inlineStr">
+    <row r="252" ht="18" customHeight="1">
+      <c r="A252" s="1" t="inlineStr">
         <is>
           <t>room.settings.save</t>
         </is>
       </c>
-      <c r="B249" s="2" t="inlineStr">
+      <c r="B252" s="2" t="inlineStr">
         <is>
           <t>Save</t>
         </is>
       </c>
-      <c r="C249" s="2" t="inlineStr">
+      <c r="C252" s="2" t="inlineStr">
         <is>
           <t>Lưu</t>
         </is>
       </c>
     </row>
-    <row r="250" ht="17" customHeight="1">
-      <c r="A250" s="1" t="inlineStr">
+    <row r="253" ht="18" customHeight="1">
+      <c r="A253" s="1" t="inlineStr">
         <is>
           <t>room-invite.messages.title</t>
         </is>
       </c>
-      <c r="B250" s="2" t="inlineStr">
+      <c r="B253" s="2" t="inlineStr">
         <is>
           <t>Room Invitation</t>
         </is>
       </c>
-      <c r="C250" s="2" t="inlineStr">
+      <c r="C253" s="2" t="inlineStr">
         <is>
           <t>Lời mời vào phòng</t>
         </is>
       </c>
     </row>
-    <row r="251" ht="17" customHeight="1">
-      <c r="A251" s="1" t="inlineStr">
+    <row r="254" ht="18" customHeight="1">
+      <c r="A254" s="1" t="inlineStr">
         <is>
           <t>start-game.messages.success</t>
         </is>
       </c>
-      <c r="B251" s="2" t="inlineStr">
+      <c r="B254" s="2" t="inlineStr">
         <is>
           <t>Game started successfully</t>
         </is>
       </c>
-      <c r="C251" s="2" t="inlineStr">
+      <c r="C254" s="2" t="inlineStr">
         <is>
           <t>Bắt đầu trò chơi thành công</t>
         </is>
       </c>
     </row>
-    <row r="252" ht="17" customHeight="1">
-      <c r="A252" s="1" t="inlineStr">
+    <row r="255" ht="18" customHeight="1">
+      <c r="A255" s="1" t="inlineStr">
         <is>
           <t>start-game.messages.internal-server-error</t>
         </is>
       </c>
-      <c r="B252" s="2" t="inlineStr">
+      <c r="B255" s="2" t="inlineStr">
         <is>
           <t>Internal server error while starting game</t>
         </is>
       </c>
-      <c r="C252" s="2" t="inlineStr">
+      <c r="C255" s="2" t="inlineStr">
         <is>
           <t>Lỗi máy chủ nội bộ khi bắt đầu trò chơi</t>
         </is>
       </c>
     </row>
-    <row r="253" ht="17" customHeight="1">
-      <c r="A253" s="1" t="inlineStr">
+    <row r="256" ht="18" customHeight="1">
+      <c r="A256" s="1" t="inlineStr">
         <is>
           <t>start-game.messages.invalid-room-id</t>
         </is>
       </c>
-      <c r="B253" s="2" t="inlineStr">
+      <c r="B256" s="2" t="inlineStr">
         <is>
           <t>Field 'id' is required and must be a positive integer</t>
         </is>
       </c>
-      <c r="C253" s="2" t="inlineStr">
+      <c r="C256" s="2" t="inlineStr">
         <is>
           <t>Trường 'id' là bắt buộc và phải là số nguyên dương</t>
         </is>
       </c>
     </row>
-    <row r="254" ht="17" customHeight="1">
-      <c r="A254" s="1" t="inlineStr">
+    <row r="257" ht="36" customHeight="1">
+      <c r="A257" s="1" t="inlineStr">
         <is>
           <t>start-game.messages.invalid-difficulty</t>
         </is>
       </c>
-      <c r="B254" s="2" t="inlineStr">
+      <c r="B257" s="2" t="inlineStr">
         <is>
           <t>Bot difficulty must be between 1 and 5</t>
         </is>
       </c>
-      <c r="C254" s="2" t="inlineStr">
+      <c r="C257" s="2" t="inlineStr">
         <is>
           <t>Độ khó của bot phải từ 1 đến 5</t>
         </is>
       </c>
     </row>
-    <row r="255" ht="17" customHeight="1">
-      <c r="A255" s="1" t="inlineStr">
+    <row r="258" ht="36" customHeight="1">
+      <c r="A258" s="1" t="inlineStr">
         <is>
           <t>start-game.messages.room-not-found</t>
         </is>
       </c>
-      <c r="B255" s="2" t="inlineStr">
+      <c r="B258" s="2" t="inlineStr">
         <is>
           <t>Room not found</t>
         </is>
       </c>
-      <c r="C255" s="2" t="inlineStr">
+      <c r="C258" s="2" t="inlineStr">
         <is>
           <t>Không tìm thấy phòng</t>
         </is>
       </c>
     </row>
-    <row r="256" ht="17" customHeight="1">
-      <c r="A256" s="1" t="inlineStr">
+    <row r="259" ht="18" customHeight="1">
+      <c r="A259" s="1" t="inlineStr">
         <is>
           <t>start-game.messages.forbidden</t>
         </is>
       </c>
-      <c r="B256" s="2" t="inlineStr">
+      <c r="B259" s="2" t="inlineStr">
         <is>
           <t>Only the room host can start the game</t>
         </is>
       </c>
-      <c r="C256" s="2" t="inlineStr">
+      <c r="C259" s="2" t="inlineStr">
         <is>
           <t>Chỉ chủ phòng mới có thể bắt đầu trò chơi</t>
         </is>
       </c>
     </row>
-    <row r="257" ht="17" customHeight="1">
-      <c r="A257" s="1" t="inlineStr">
+    <row r="260" ht="18" customHeight="1">
+      <c r="A260" s="1" t="inlineStr">
         <is>
           <t>start-game.messages.insufficient-amount</t>
         </is>
       </c>
-      <c r="B257" s="2" t="inlineStr">
+      <c r="B260" s="2" t="inlineStr">
         <is>
           <t>You do not have enough balance to start a game with this bet</t>
         </is>
       </c>
-      <c r="C257" s="2" t="inlineStr">
+      <c r="C260" s="2" t="inlineStr">
         <is>
           <t>Bạn không còn đủ amount để start room</t>
         </is>
       </c>
     </row>
-    <row r="258" ht="17" customHeight="1">
-      <c r="A258" s="1" t="inlineStr">
+    <row r="261" ht="18" customHeight="1">
+      <c r="A261" s="1" t="inlineStr">
         <is>
           <t>start-game.messages.requester-must-pick-team</t>
         </is>
       </c>
-      <c r="B258" s="2" t="inlineStr">
+      <c r="B261" s="2" t="inlineStr">
         <is>
           <t>You must select a team before starting a game with bot</t>
         </is>
       </c>
-      <c r="C258" s="2" t="inlineStr">
+      <c r="C261" s="2" t="inlineStr">
         <is>
           <t>Bạn phải chọn team trước khi bắt đầu trò chơi với bot</t>
-        </is>
-      </c>
-    </row>
-    <row r="259" ht="17" customHeight="1">
-      <c r="A259" s="1" t="inlineStr">
-        <is>
-          <t>update-room.messages.success</t>
-        </is>
-      </c>
-      <c r="B259" s="2" t="inlineStr">
-        <is>
-          <t>Room updated successfully</t>
-        </is>
-      </c>
-      <c r="C259" s="2" t="inlineStr">
-        <is>
-          <t>Cập nhật phòng thành công</t>
-        </is>
-      </c>
-    </row>
-    <row r="260" ht="17" customHeight="1">
-      <c r="A260" s="1" t="inlineStr">
-        <is>
-          <t>update-room.messages.internal-server-error</t>
-        </is>
-      </c>
-      <c r="B260" s="2" t="inlineStr">
-        <is>
-          <t>Internal server error</t>
-        </is>
-      </c>
-      <c r="C260" s="2" t="inlineStr">
-        <is>
-          <t>Lỗi máy chủ nội bộ</t>
-        </is>
-      </c>
-    </row>
-    <row r="261" ht="17" customHeight="1">
-      <c r="A261" s="1" t="inlineStr">
-        <is>
-          <t>update-room.messages.invalid-room-id</t>
-        </is>
-      </c>
-      <c r="B261" s="2" t="inlineStr">
-        <is>
-          <t>Invalid room ID</t>
-        </is>
-      </c>
-      <c r="C261" s="2" t="inlineStr">
-        <is>
-          <t>ID phòng không hợp lệ</t>
         </is>
       </c>
     </row>
     <row r="262" ht="17" customHeight="1">
       <c r="A262" s="1" t="inlineStr">
         <is>
-          <t>update-room.messages.name-required</t>
+          <t>update-room.messages.success</t>
         </is>
       </c>
       <c r="B262" s="1" t="inlineStr">
         <is>
-          <t>Room name is required</t>
+          <t>Room updated successfully</t>
         </is>
       </c>
       <c r="C262" s="1" t="inlineStr">
         <is>
-          <t>Tên phòng không được để trống</t>
-        </is>
-      </c>
-    </row>
-    <row r="263" ht="17" customHeight="1">
+          <t>Cập nhật phòng thành công</t>
+        </is>
+      </c>
+    </row>
+    <row r="263" ht="18" customHeight="1">
       <c r="A263" s="2" t="inlineStr">
         <is>
-          <t>update-room.messages.room-not-found</t>
+          <t>update-room.messages.internal-server-error</t>
         </is>
       </c>
       <c r="B263" s="2" t="inlineStr">
         <is>
-          <t>Room not found</t>
+          <t>Internal server error</t>
         </is>
       </c>
       <c r="C263" s="2" t="inlineStr">
         <is>
-          <t>Không tìm thấy phòng</t>
-        </is>
-      </c>
-    </row>
-    <row r="264" ht="36" customHeight="1">
+          <t>Lỗi máy chủ nội bộ</t>
+        </is>
+      </c>
+    </row>
+    <row r="264" ht="18" customHeight="1">
       <c r="A264" s="2" t="inlineStr">
         <is>
-          <t>update-room.messages.forbidden</t>
+          <t>update-room.messages.invalid-room-id</t>
         </is>
       </c>
       <c r="B264" s="2" t="inlineStr">
         <is>
-          <t>You are not the host of this room</t>
+          <t>Invalid room ID</t>
         </is>
       </c>
       <c r="C264" s="2" t="inlineStr">
         <is>
-          <t>Bạn không phải chủ phòng</t>
+          <t>ID phòng không hợp lệ</t>
         </is>
       </c>
     </row>
     <row r="265" ht="18" customHeight="1">
       <c r="A265" s="2" t="inlineStr">
         <is>
-          <t>draw-game.messages.invalid-game-id</t>
+          <t>update-room.messages.name-required</t>
         </is>
       </c>
       <c r="B265" s="2" t="inlineStr">
         <is>
-          <t>Invalid game ID</t>
+          <t>Room name is required</t>
         </is>
       </c>
       <c r="C265" s="2" t="inlineStr">
         <is>
-          <t>ID trò chơi không hợp lệ</t>
+          <t>Tên phòng không được để trống</t>
         </is>
       </c>
     </row>
     <row r="266" ht="18" customHeight="1">
       <c r="A266" s="2" t="inlineStr">
         <is>
-          <t>draw-game.messages.game-not-found</t>
+          <t>update-room.messages.room-not-found</t>
         </is>
       </c>
       <c r="B266" s="2" t="inlineStr">
         <is>
-          <t>Game not found</t>
+          <t>Room not found</t>
         </is>
       </c>
       <c r="C266" s="2" t="inlineStr">
         <is>
-          <t>Không tìm thấy trò chơi</t>
+          <t>Không tìm thấy phòng</t>
         </is>
       </c>
     </row>
     <row r="267" ht="18" customHeight="1">
       <c r="A267" s="2" t="inlineStr">
         <is>
-          <t>draw-game.messages.forbidden</t>
+          <t>update-room.messages.forbidden</t>
         </is>
       </c>
       <c r="B267" s="2" t="inlineStr">
         <is>
-          <t>You are not in this room</t>
+          <t>You are not the host of this room</t>
         </is>
       </c>
       <c r="C267" s="2" t="inlineStr">
         <is>
-          <t>Bạn không có trong phòng này</t>
-        </is>
-      </c>
-    </row>
-    <row r="268" ht="18" customHeight="1">
+          <t>Bạn không phải chủ phòng</t>
+        </is>
+      </c>
+    </row>
+    <row r="268" ht="36" customHeight="1">
       <c r="A268" s="2" t="inlineStr">
         <is>
-          <t>draw-game.messages.game-history-not-found</t>
+          <t>draw-game.messages.invalid-game-id</t>
         </is>
       </c>
       <c r="B268" s="2" t="inlineStr">
         <is>
-          <t>Game history not found</t>
+          <t>Invalid game ID</t>
         </is>
       </c>
       <c r="C268" s="2" t="inlineStr">
         <is>
-          <t>Không tìm thấy lịch sử trò chơi</t>
+          <t>ID trò chơi không hợp lệ</t>
         </is>
       </c>
     </row>
     <row r="269" ht="36" customHeight="1">
       <c r="A269" s="2" t="inlineStr">
         <is>
-          <t>draw-game.messages.game-already-finished</t>
+          <t>draw-game.messages.game-not-found</t>
         </is>
       </c>
       <c r="B269" s="2" t="inlineStr">
         <is>
-          <t>Game is already finished</t>
+          <t>Game not found</t>
         </is>
       </c>
       <c r="C269" s="2" t="inlineStr">
         <is>
-          <t>Trò chơi đã kết thúc</t>
+          <t>Không tìm thấy trò chơi</t>
         </is>
       </c>
     </row>
     <row r="270" ht="18" customHeight="1">
       <c r="A270" s="2" t="inlineStr">
         <is>
-          <t>draw-game.messages.success</t>
+          <t>draw-game.messages.forbidden</t>
         </is>
       </c>
       <c r="B270" s="2" t="inlineStr">
         <is>
-          <t>Draw game successfully</t>
+          <t>You are not in this room</t>
         </is>
       </c>
       <c r="C270" s="2" t="inlineStr">
         <is>
-          <t>Hòa cờ thành công</t>
+          <t>Bạn không có trong phòng này</t>
         </is>
       </c>
     </row>
     <row r="271" ht="18" customHeight="1">
       <c r="A271" s="1" t="inlineStr">
         <is>
-          <t>draw-game.messages.internal-server-error</t>
+          <t>draw-game.messages.game-history-not-found</t>
         </is>
       </c>
       <c r="B271" s="2" t="inlineStr">
         <is>
-          <t>Internal server error</t>
+          <t>Game history not found</t>
         </is>
       </c>
       <c r="C271" s="2" t="inlineStr">
         <is>
-          <t>Lỗi máy chủ nội bộ</t>
+          <t>Không tìm thấy lịch sử trò chơi</t>
         </is>
       </c>
     </row>
     <row r="272" ht="18" customHeight="1">
       <c r="A272" s="1" t="inlineStr">
         <is>
-          <t>surrender.messages.game-already-finished</t>
+          <t>draw-game.messages.game-already-finished</t>
         </is>
       </c>
       <c r="B272" s="2" t="inlineStr">
@@ -4960,1213 +4960,1576 @@
     <row r="273" ht="18" customHeight="1">
       <c r="A273" s="1" t="inlineStr">
         <is>
-          <t>surrender.messages.game-history-not-found</t>
+          <t>draw-game.messages.success</t>
         </is>
       </c>
       <c r="B273" s="2" t="inlineStr">
         <is>
-          <t>Game history not found</t>
+          <t>Draw game successfully</t>
         </is>
       </c>
       <c r="C273" s="2" t="inlineStr">
         <is>
-          <t>Không tìm thấy lịch sử trò chơi</t>
+          <t>Hòa cờ thành công</t>
         </is>
       </c>
     </row>
     <row r="274" ht="18" customHeight="1">
       <c r="A274" s="1" t="inlineStr">
         <is>
-          <t>surrender.messages.game-not-found</t>
+          <t>draw-game.messages.internal-server-error</t>
         </is>
       </c>
       <c r="B274" s="2" t="inlineStr">
         <is>
-          <t>Game not found</t>
+          <t>Internal server error</t>
         </is>
       </c>
       <c r="C274" s="2" t="inlineStr">
         <is>
-          <t>Không tìm thấy trò chơi</t>
+          <t>Lỗi máy chủ nội bộ</t>
         </is>
       </c>
     </row>
     <row r="275" ht="18" customHeight="1">
       <c r="A275" s="1" t="inlineStr">
         <is>
-          <t>surrender.messages.internal-server-error</t>
+          <t>surrender.messages.game-already-finished</t>
         </is>
       </c>
       <c r="B275" s="2" t="inlineStr">
         <is>
-          <t>Internal server error</t>
+          <t>Game is already finished</t>
         </is>
       </c>
       <c r="C275" s="2" t="inlineStr">
         <is>
-          <t>Lỗi máy chủ nội bộ</t>
+          <t>Trò chơi đã kết thúc</t>
         </is>
       </c>
     </row>
     <row r="276" ht="18" customHeight="1">
       <c r="A276" s="1" t="inlineStr">
         <is>
-          <t>surrender.messages.invalid-game-id</t>
+          <t>surrender.messages.game-history-not-found</t>
         </is>
       </c>
       <c r="B276" s="2" t="inlineStr">
         <is>
-          <t>Invalid game ID</t>
+          <t>Game history not found</t>
         </is>
       </c>
       <c r="C276" s="2" t="inlineStr">
         <is>
-          <t>ID trò chơi không hợp lệ</t>
+          <t>Không tìm thấy lịch sử trò chơi</t>
         </is>
       </c>
     </row>
     <row r="277" ht="18" customHeight="1">
       <c r="A277" s="1" t="inlineStr">
         <is>
-          <t>surrender.messages.invalid-surrender-player</t>
+          <t>surrender.messages.game-not-found</t>
         </is>
       </c>
       <c r="B277" s="2" t="inlineStr">
         <is>
-          <t>You are not a player in this game</t>
+          <t>Game not found</t>
         </is>
       </c>
       <c r="C277" s="2" t="inlineStr">
         <is>
-          <t>Bạn không phải là người chơi trong trò chơi này</t>
+          <t>Không tìm thấy trò chơi</t>
         </is>
       </c>
     </row>
     <row r="278" ht="18" customHeight="1">
       <c r="A278" s="1" t="inlineStr">
         <is>
-          <t>surrender.messages.opponent-not-found</t>
+          <t>surrender.messages.internal-server-error</t>
         </is>
       </c>
       <c r="B278" s="2" t="inlineStr">
         <is>
-          <t>Opponent not found</t>
+          <t>Internal server error</t>
         </is>
       </c>
       <c r="C278" s="2" t="inlineStr">
         <is>
-          <t>Không tìm thấy đối thủ</t>
+          <t>Lỗi máy chủ nội bộ</t>
         </is>
       </c>
     </row>
     <row r="279" ht="18" customHeight="1">
       <c r="A279" s="1" t="inlineStr">
         <is>
-          <t>surrender.messages.success</t>
+          <t>surrender.messages.invalid-game-id</t>
         </is>
       </c>
       <c r="B279" s="2" t="inlineStr">
         <is>
-          <t>Surrendered</t>
+          <t>Invalid game ID</t>
         </is>
       </c>
       <c r="C279" s="2" t="inlineStr">
         <is>
-          <t>Đã đầu hàng</t>
+          <t>ID trò chơi không hợp lệ</t>
         </is>
       </c>
     </row>
     <row r="280" ht="18" customHeight="1">
       <c r="A280" s="1" t="inlineStr">
         <is>
-          <t>undo.messages.invalid-game-id</t>
+          <t>surrender.messages.invalid-surrender-player</t>
         </is>
       </c>
       <c r="B280" s="2" t="inlineStr">
         <is>
-          <t>Invalid game ID</t>
+          <t>You are not a player in this game</t>
         </is>
       </c>
       <c r="C280" s="2" t="inlineStr">
         <is>
-          <t>ID trò chơi không hợp lệ</t>
+          <t>Bạn không phải là người chơi trong trò chơi này</t>
         </is>
       </c>
     </row>
     <row r="281" ht="18" customHeight="1">
       <c r="A281" s="1" t="inlineStr">
         <is>
-          <t>undo.messages.unauthorized</t>
+          <t>surrender.messages.opponent-not-found</t>
         </is>
       </c>
       <c r="B281" s="2" t="inlineStr">
         <is>
-          <t>Unauthorized</t>
+          <t>Opponent not found</t>
         </is>
       </c>
       <c r="C281" s="2" t="inlineStr">
         <is>
-          <t>Không được phép truy cập</t>
+          <t>Không tìm thấy đối thủ</t>
         </is>
       </c>
     </row>
     <row r="282" ht="18" customHeight="1">
       <c r="A282" s="1" t="inlineStr">
         <is>
-          <t>undo.messages.game-not-found</t>
+          <t>surrender.messages.success</t>
         </is>
       </c>
       <c r="B282" s="2" t="inlineStr">
         <is>
-          <t>Game not found</t>
+          <t>Surrendered</t>
         </is>
       </c>
       <c r="C282" s="2" t="inlineStr">
         <is>
-          <t>Không tìm thấy trò chơi</t>
+          <t>Đã đầu hàng</t>
         </is>
       </c>
     </row>
     <row r="283" ht="18" customHeight="1">
       <c r="A283" s="1" t="inlineStr">
         <is>
-          <t>undo.messages.not-in-game</t>
+          <t>undo.messages.invalid-game-id</t>
         </is>
       </c>
       <c r="B283" s="2" t="inlineStr">
         <is>
-          <t>You are not part of this game</t>
+          <t>Invalid game ID</t>
         </is>
       </c>
       <c r="C283" s="2" t="inlineStr">
         <is>
-          <t>Bạn không phải là người chơi trong trò chơi này</t>
+          <t>ID trò chơi không hợp lệ</t>
         </is>
       </c>
     </row>
     <row r="284" ht="18" customHeight="1">
       <c r="A284" s="1" t="inlineStr">
         <is>
-          <t>undo.messages.not-in-room</t>
+          <t>undo.messages.unauthorized</t>
         </is>
       </c>
       <c r="B284" s="2" t="inlineStr">
         <is>
-          <t>You are not in this room</t>
+          <t>Unauthorized</t>
         </is>
       </c>
       <c r="C284" s="2" t="inlineStr">
         <is>
-          <t>Bạn không trong phòng này</t>
+          <t>Không được phép truy cập</t>
         </is>
       </c>
     </row>
     <row r="285" ht="18" customHeight="1">
       <c r="A285" s="1" t="inlineStr">
         <is>
-          <t>undo.messages.spectator-cannot-undo</t>
+          <t>undo.messages.game-not-found</t>
         </is>
       </c>
       <c r="B285" s="2" t="inlineStr">
         <is>
-          <t>Spectators cannot undo moves</t>
+          <t>Game not found</t>
         </is>
       </c>
       <c r="C285" s="2" t="inlineStr">
         <is>
-          <t>Người xem không thể hoàn tác nước đi</t>
+          <t>Không tìm thấy trò chơi</t>
         </is>
       </c>
     </row>
     <row r="286" ht="18" customHeight="1">
       <c r="A286" s="1" t="inlineStr">
         <is>
-          <t>undo.messages.no-moves</t>
+          <t>undo.messages.not-in-game</t>
         </is>
       </c>
       <c r="B286" s="2" t="inlineStr">
         <is>
-          <t>No moves to undo</t>
+          <t>You are not part of this game</t>
         </is>
       </c>
       <c r="C286" s="2" t="inlineStr">
         <is>
-          <t>Không có nước đi để hoàn tác</t>
+          <t>Bạn không phải là người chơi trong trò chơi này</t>
         </is>
       </c>
     </row>
     <row r="287" ht="18" customHeight="1">
       <c r="A287" s="1" t="inlineStr">
         <is>
-          <t>undo.messages.delete-failed</t>
+          <t>undo.messages.not-in-room</t>
         </is>
       </c>
       <c r="B287" s="2" t="inlineStr">
         <is>
-          <t>Failed to undo move</t>
+          <t>You are not in this room</t>
         </is>
       </c>
       <c r="C287" s="2" t="inlineStr">
         <is>
-          <t>Không thể hoàn tác nước đi</t>
+          <t>Bạn không trong phòng này</t>
         </is>
       </c>
     </row>
     <row r="288" ht="18" customHeight="1">
       <c r="A288" s="1" t="inlineStr">
         <is>
-          <t>undo.messages.undo-limit-exceeded</t>
+          <t>undo.messages.spectator-cannot-undo</t>
         </is>
       </c>
       <c r="B288" s="2" t="inlineStr">
         <is>
-          <t>Maximum 3 undo per game exceeded</t>
+          <t>Spectators cannot undo moves</t>
         </is>
       </c>
       <c r="C288" s="2" t="inlineStr">
         <is>
-          <t>Đã đạt tối đa 3 lần hoàn tác trong trò chơi</t>
+          <t>Người xem không thể hoàn tác nước đi</t>
         </is>
       </c>
     </row>
     <row r="289" ht="18" customHeight="1">
       <c r="A289" s="1" t="inlineStr">
         <is>
-          <t>undo.messages.success</t>
+          <t>undo.messages.no-moves</t>
         </is>
       </c>
       <c r="B289" s="2" t="inlineStr">
         <is>
-          <t>Move undone successfully</t>
+          <t>No moves to undo</t>
         </is>
       </c>
       <c r="C289" s="2" t="inlineStr">
         <is>
-          <t>Hoàn tác nước đi thành công</t>
+          <t>Không có nước đi để hoàn tác</t>
         </is>
       </c>
     </row>
     <row r="290" ht="18" customHeight="1">
       <c r="A290" s="1" t="inlineStr">
         <is>
-          <t>undo.messages.internal-server-error</t>
+          <t>undo.messages.delete-failed</t>
         </is>
       </c>
       <c r="B290" s="2" t="inlineStr">
         <is>
-          <t>Internal server error</t>
+          <t>Failed to undo move</t>
         </is>
       </c>
       <c r="C290" s="2" t="inlineStr">
         <is>
-          <t>Lỗi máy chủ nội bộ</t>
+          <t>Không thể hoàn tác nước đi</t>
         </is>
       </c>
     </row>
     <row r="291" ht="18" customHeight="1">
       <c r="A291" s="1" t="inlineStr">
         <is>
-          <t>player-history.messages.invalid-user-id</t>
+          <t>undo.messages.undo-limit-exceeded</t>
         </is>
       </c>
       <c r="B291" s="2" t="inlineStr">
         <is>
-          <t>Invalid user ID</t>
+          <t>Maximum 3 undo per game exceeded</t>
         </is>
       </c>
       <c r="C291" s="2" t="inlineStr">
         <is>
-          <t>ID người dùng không hợp lệ</t>
+          <t>Đã đạt tối đa 3 lần hoàn tác trong trò chơi</t>
         </is>
       </c>
     </row>
     <row r="292" ht="18" customHeight="1">
       <c r="A292" s="1" t="inlineStr">
         <is>
-          <t>player-history.messages.success</t>
+          <t>undo.messages.success</t>
         </is>
       </c>
       <c r="B292" s="2" t="inlineStr">
         <is>
-          <t>Fetch game history successfully</t>
+          <t>Move undone successfully</t>
         </is>
       </c>
       <c r="C292" s="2" t="inlineStr">
         <is>
-          <t>Lấy lịch sử trò chơi thành công</t>
+          <t>Hoàn tác nước đi thành công</t>
         </is>
       </c>
     </row>
     <row r="293" ht="18" customHeight="1">
       <c r="A293" s="1" t="inlineStr">
         <is>
-          <t>validate-token.messages.success</t>
+          <t>undo.messages.internal-server-error</t>
         </is>
       </c>
       <c r="B293" s="2" t="inlineStr">
         <is>
-          <t>Token is valid</t>
+          <t>Internal server error</t>
         </is>
       </c>
       <c r="C293" s="2" t="inlineStr">
         <is>
-          <t>Token hợp lệ</t>
+          <t>Lỗi máy chủ nội bộ</t>
         </is>
       </c>
     </row>
     <row r="294" ht="18" customHeight="1">
       <c r="A294" s="1" t="inlineStr">
         <is>
-          <t>guide.section.objective</t>
+          <t>player-history.messages.invalid-user-id</t>
         </is>
       </c>
       <c r="B294" s="2" t="inlineStr">
         <is>
-          <t>Objective of the game</t>
+          <t>Invalid user ID</t>
         </is>
       </c>
       <c r="C294" s="2" t="inlineStr">
         <is>
-          <t>Mục tiêu của trò chơi</t>
+          <t>ID người dùng không hợp lệ</t>
         </is>
       </c>
     </row>
     <row r="295" ht="18" customHeight="1">
       <c r="A295" s="1" t="inlineStr">
         <is>
-          <t>guide.section.pieces</t>
+          <t>player-history.messages.success</t>
         </is>
       </c>
       <c r="B295" s="2" t="inlineStr">
         <is>
-          <t>Pieces</t>
+          <t>Fetch game history successfully</t>
         </is>
       </c>
       <c r="C295" s="2" t="inlineStr">
         <is>
-          <t>Quân cờ</t>
+          <t>Lấy lịch sử trò chơi thành công</t>
         </is>
       </c>
     </row>
     <row r="296" ht="18" customHeight="1">
       <c r="A296" s="1" t="inlineStr">
         <is>
-          <t>guide.section.moving-pieces</t>
+          <t>validate-token.messages.success</t>
         </is>
       </c>
       <c r="B296" s="2" t="inlineStr">
         <is>
-          <t>Moving pieces</t>
+          <t>Token is valid</t>
         </is>
       </c>
       <c r="C296" s="2" t="inlineStr">
         <is>
-          <t>Đi quân</t>
+          <t>Token hợp lệ</t>
         </is>
       </c>
     </row>
     <row r="297" ht="18" customHeight="1">
       <c r="A297" s="1" t="inlineStr">
         <is>
-          <t>guide.section.capturing</t>
+          <t>guide.section.objective</t>
         </is>
       </c>
       <c r="B297" s="2" t="inlineStr">
         <is>
-          <t>Capturing</t>
+          <t>Objective of the game</t>
         </is>
       </c>
       <c r="C297" s="2" t="inlineStr">
         <is>
-          <t>Bắt quân</t>
+          <t>Mục tiêu của trò chơi</t>
         </is>
       </c>
     </row>
     <row r="298" ht="18" customHeight="1">
       <c r="A298" s="1" t="inlineStr">
         <is>
-          <t>guide.section.check</t>
+          <t>guide.section.pieces</t>
         </is>
       </c>
       <c r="B298" s="2" t="inlineStr">
         <is>
-          <t>Check</t>
+          <t>Pieces</t>
         </is>
       </c>
       <c r="C298" s="2" t="inlineStr">
         <is>
-          <t>Chiếu tướng</t>
-        </is>
-      </c>
-    </row>
-    <row r="299" ht="90" customHeight="1">
+          <t>Quân cờ</t>
+        </is>
+      </c>
+    </row>
+    <row r="299" ht="18" customHeight="1">
       <c r="A299" s="1" t="inlineStr">
         <is>
-          <t>guide.section.result</t>
+          <t>guide.section.moving-pieces</t>
         </is>
       </c>
       <c r="B299" s="2" t="inlineStr">
         <is>
-          <t>Result</t>
+          <t>Moving pieces</t>
         </is>
       </c>
       <c r="C299" s="2" t="inlineStr">
         <is>
-          <t>Kết quả</t>
-        </is>
-      </c>
-    </row>
-    <row r="300" ht="90" customHeight="1">
+          <t>Đi quân</t>
+        </is>
+      </c>
+    </row>
+    <row r="300" ht="18" customHeight="1">
       <c r="A300" s="1" t="inlineStr">
         <is>
-          <t>guide.table.piece</t>
+          <t>guide.section.capturing</t>
         </is>
       </c>
       <c r="B300" s="2" t="inlineStr">
         <is>
-          <t>Piece</t>
+          <t>Capturing</t>
         </is>
       </c>
       <c r="C300" s="2" t="inlineStr">
         <is>
-          <t>Quân</t>
+          <t>Bắt quân</t>
         </is>
       </c>
     </row>
     <row r="301" ht="18" customHeight="1">
       <c r="A301" s="1" t="inlineStr">
         <is>
-          <t>guide.table.symbol</t>
+          <t>guide.section.check</t>
         </is>
       </c>
       <c r="B301" s="2" t="inlineStr">
         <is>
-          <t>Symbol</t>
+          <t>Check</t>
         </is>
       </c>
       <c r="C301" s="2" t="inlineStr">
         <is>
-          <t>Ký hiệu</t>
+          <t>Chiếu tướng</t>
         </is>
       </c>
     </row>
     <row r="302" ht="18" customHeight="1">
       <c r="A302" s="1" t="inlineStr">
         <is>
-          <t>guide.table.quantity</t>
+          <t>guide.section.result</t>
         </is>
       </c>
       <c r="B302" s="2" t="inlineStr">
         <is>
-          <t>Quantity</t>
+          <t>Result</t>
         </is>
       </c>
       <c r="C302" s="2" t="inlineStr">
         <is>
-          <t>Số lượng</t>
-        </is>
-      </c>
-    </row>
-    <row r="303" ht="18" customHeight="1">
+          <t>Kết quả</t>
+        </is>
+      </c>
+    </row>
+    <row r="303" ht="90" customHeight="1">
       <c r="A303" s="1" t="inlineStr">
         <is>
-          <t>guide.objective.paragraph1</t>
+          <t>guide.table.piece</t>
         </is>
       </c>
       <c r="B303" s="2" t="inlineStr">
         <is>
-          <t>A match is played between two players: one controls the Red pieces, and the other controls the Black pieces. The objective of each player is to use their pieces on the board to &lt;b&gt;checkmate&lt;/b&gt; the opponent's General, and win the game.</t>
+          <t>Piece</t>
         </is>
       </c>
       <c r="C303" s="2" t="inlineStr">
         <is>
-          <t>Ván cờ được tiến hành giữa 2 đấu thủ, một người cầm Quân Đỏ, một người cầm Quân Đen. Mục đích của mỗi đấu thủ là tìm mọi cách sử dụng các quân trên bàn cờ để &lt;b&gt;chiếu bí Tướng&lt;/b&gt; của đối phương, giành thắng lợi.</t>
-        </is>
-      </c>
-    </row>
-    <row r="304" ht="18" customHeight="1">
+          <t>Quân</t>
+        </is>
+      </c>
+    </row>
+    <row r="304" ht="90" customHeight="1">
       <c r="A304" s="1" t="inlineStr">
         <is>
-          <t>guide.pieces.paragraph1</t>
+          <t>guide.table.symbol</t>
         </is>
       </c>
       <c r="B304" s="2" t="inlineStr">
         <is>
-          <t>At the start of each game, there must be 32 pieces in total, consisting of &lt;b&gt;7 piece types&lt;/b&gt; split evenly between both sides: 16 Red pieces and 16 Black pieces. The 7 piece types with their symbols and quantities are as follows:</t>
+          <t>Symbol</t>
         </is>
       </c>
       <c r="C304" s="2" t="inlineStr">
         <is>
-          <t>Mỗi ván cờ lúc bắt đầu phải có đủ 32 quân, gồm 7 loại chia đều cho mỗi bên gồm 16 quân Đỏ và 16 quân Đen. &lt;b&gt;7 loại quân&lt;/b&gt; có ký hiệu và số lượng như sau:</t>
+          <t>Ký hiệu</t>
         </is>
       </c>
     </row>
     <row r="305" ht="18" customHeight="1">
       <c r="A305" s="1" t="inlineStr">
         <is>
-          <t>guide.piece.general</t>
+          <t>guide.table.quantity</t>
         </is>
       </c>
       <c r="B305" s="2" t="inlineStr">
         <is>
-          <t>General</t>
+          <t>Quantity</t>
         </is>
       </c>
       <c r="C305" s="2" t="inlineStr">
         <is>
-          <t>Tướng</t>
+          <t>Số lượng</t>
         </is>
       </c>
     </row>
     <row r="306" ht="18" customHeight="1">
       <c r="A306" s="1" t="inlineStr">
         <is>
-          <t>guide.piece.advisor</t>
+          <t>guide.objective.paragraph1</t>
         </is>
       </c>
       <c r="B306" s="2" t="inlineStr">
         <is>
-          <t>Advisor</t>
+          <t>A match is played between two players: one controls the Red pieces, and the other controls the Black pieces. The objective of each player is to use their pieces on the board to &lt;b&gt;checkmate&lt;/b&gt; the opponent's General, and win the game.</t>
         </is>
       </c>
       <c r="C306" s="2" t="inlineStr">
         <is>
-          <t>Sĩ</t>
+          <t>Ván cờ được tiến hành giữa 2 đấu thủ, một người cầm Quân Đỏ, một người cầm Quân Đen. Mục đích của mỗi đấu thủ là tìm mọi cách sử dụng các quân trên bàn cờ để &lt;b&gt;chiếu bí Tướng&lt;/b&gt; của đối phương, giành thắng lợi.</t>
         </is>
       </c>
     </row>
     <row r="307" ht="18" customHeight="1">
       <c r="A307" s="1" t="inlineStr">
         <is>
-          <t>guide.piece.elephant</t>
+          <t>guide.pieces.paragraph1</t>
         </is>
       </c>
       <c r="B307" s="2" t="inlineStr">
         <is>
-          <t>Elephant</t>
+          <t>At the start of each game, there must be 32 pieces in total, consisting of &lt;b&gt;7 piece types&lt;/b&gt; split evenly between both sides: 16 Red pieces and 16 Black pieces. The 7 piece types with their symbols and quantities are as follows:</t>
         </is>
       </c>
       <c r="C307" s="2" t="inlineStr">
         <is>
-          <t>Tượng</t>
-        </is>
-      </c>
-    </row>
-    <row r="308" ht="54" customHeight="1">
+          <t>Mỗi ván cờ lúc bắt đầu phải có đủ 32 quân, gồm 7 loại chia đều cho mỗi bên gồm 16 quân Đỏ và 16 quân Đen. &lt;b&gt;7 loại quân&lt;/b&gt; có ký hiệu và số lượng như sau:</t>
+        </is>
+      </c>
+    </row>
+    <row r="308" ht="18" customHeight="1">
       <c r="A308" s="2" t="inlineStr">
         <is>
-          <t>guide.piece.chariot</t>
+          <t>guide.piece.general</t>
         </is>
       </c>
       <c r="B308" s="2" t="inlineStr">
         <is>
-          <t>Chariot</t>
+          <t>General</t>
         </is>
       </c>
       <c r="C308" s="2" t="inlineStr">
         <is>
-          <t>Xe</t>
+          <t>Tướng</t>
         </is>
       </c>
     </row>
     <row r="309" ht="18" customHeight="1">
       <c r="A309" s="2" t="inlineStr">
         <is>
-          <t>guide.piece.horse</t>
+          <t>guide.piece.advisor</t>
         </is>
       </c>
       <c r="B309" s="2" t="inlineStr">
         <is>
-          <t>Horse</t>
+          <t>Advisor</t>
         </is>
       </c>
       <c r="C309" s="2" t="inlineStr">
         <is>
-          <t>Mã</t>
-        </is>
-      </c>
-    </row>
-    <row r="310" ht="90" customHeight="1">
+          <t>Sĩ</t>
+        </is>
+      </c>
+    </row>
+    <row r="310" ht="18" customHeight="1">
       <c r="A310" s="2" t="inlineStr">
         <is>
-          <t>guide.piece.cannon</t>
+          <t>guide.piece.elephant</t>
         </is>
       </c>
       <c r="B310" s="2" t="inlineStr">
         <is>
-          <t>Cannon</t>
+          <t>Elephant</t>
         </is>
       </c>
       <c r="C310" s="2" t="inlineStr">
         <is>
-          <t>Pháo</t>
+          <t>Tượng</t>
         </is>
       </c>
     </row>
     <row r="311" ht="18" customHeight="1">
       <c r="A311" s="2" t="inlineStr">
         <is>
-          <t>guide.piece.soldier</t>
+          <t>guide.piece.chariot</t>
         </is>
       </c>
       <c r="B311" s="2" t="inlineStr">
         <is>
-          <t>Soldier</t>
+          <t>Chariot</t>
         </is>
       </c>
       <c r="C311" s="2" t="inlineStr">
         <is>
-          <t>Tốt</t>
-        </is>
-      </c>
-    </row>
-    <row r="312" ht="36" customHeight="1">
+          <t>Xe</t>
+        </is>
+      </c>
+    </row>
+    <row r="312" ht="54" customHeight="1">
       <c r="A312" s="2" t="inlineStr">
         <is>
-          <t>guide.moving-pieces.paragraph1</t>
+          <t>guide.piece.horse</t>
         </is>
       </c>
       <c r="B312" s="2" t="inlineStr">
         <is>
-          <t>On each turn, each side may move only one of its own pieces according to the rules. The movement rules are as follows:</t>
+          <t>Horse</t>
         </is>
       </c>
       <c r="C312" s="2" t="inlineStr">
         <is>
-          <t>Mỗi nước đi, mỗi bên chỉ được di chuyển quân của mình theo đúng quy định. Quy định di chuyển của các quân như sau:</t>
+          <t>Mã</t>
         </is>
       </c>
     </row>
     <row r="313" ht="18" customHeight="1">
       <c r="A313" s="2" t="inlineStr">
         <is>
-          <t>guide.general.paragraph1</t>
+          <t>guide.piece.cannon</t>
         </is>
       </c>
       <c r="B313" s="2" t="inlineStr">
         <is>
-          <t>General</t>
+          <t>Cannon</t>
         </is>
       </c>
       <c r="C313" s="2" t="inlineStr">
         <is>
-          <t>Tướng</t>
-        </is>
-      </c>
-    </row>
-    <row r="314" ht="72" customHeight="1">
+          <t>Pháo</t>
+        </is>
+      </c>
+    </row>
+    <row r="314" ht="90" customHeight="1">
       <c r="A314" s="2" t="inlineStr">
         <is>
-          <t>guide.general.paragraph2</t>
+          <t>guide.piece.soldier</t>
         </is>
       </c>
       <c r="B314" s="2" t="inlineStr">
         <is>
-          <t>Moves one step &lt;b&gt;horizontally or vertically&lt;/b&gt; within the palace. The two Generals may not face each other directly on the same file. If they are facing each other, there must be at least one piece of either side placed between them.</t>
+          <t>Soldier</t>
         </is>
       </c>
       <c r="C314" s="2" t="inlineStr">
         <is>
-          <t>Mỗi nước được đi một bước &lt;b&gt;ngang hoặc dọc&lt;/b&gt; tùy ý trong cung Tướng. Hai tướng của 2 bên không được đối mặt nhau trực tiếp trên cùng một đường thẳng. Nếu đối mặt, bắt buộc phải có quân của bất kỳ bên nào đứng che mặt.</t>
+          <t>Tốt</t>
         </is>
       </c>
     </row>
     <row r="315" ht="18" customHeight="1">
       <c r="A315" s="2" t="inlineStr">
         <is>
-          <t>guide.advisor.paragraph1</t>
+          <t>guide.moving-pieces.paragraph1</t>
         </is>
       </c>
       <c r="B315" s="2" t="inlineStr">
         <is>
-          <t>Advisor</t>
+          <t>On each turn, each side may move only one of its own pieces according to the rules. The movement rules are as follows:</t>
         </is>
       </c>
       <c r="C315" s="2" t="inlineStr">
         <is>
-          <t>Sĩ</t>
-        </is>
-      </c>
-    </row>
-    <row r="316" ht="54" customHeight="1">
+          <t>Mỗi nước đi, mỗi bên chỉ được di chuyển quân của mình theo đúng quy định. Quy định di chuyển của các quân như sau:</t>
+        </is>
+      </c>
+    </row>
+    <row r="316" ht="36" customHeight="1">
       <c r="A316" s="2" t="inlineStr">
         <is>
-          <t>guide.advisor.paragraph2</t>
+          <t>guide.general.paragraph1</t>
         </is>
       </c>
       <c r="B316" s="2" t="inlineStr">
         <is>
-          <t>Moves one step &lt;b&gt;diagonally&lt;/b&gt; within the palace.</t>
+          <t>General</t>
         </is>
       </c>
       <c r="C316" s="2" t="inlineStr">
         <is>
-          <t>Mỗi nước &lt;b&gt;đi chéo một bước&lt;/b&gt; trong cung Tướng.</t>
+          <t>Tướng</t>
         </is>
       </c>
     </row>
     <row r="317" ht="18" customHeight="1">
       <c r="A317" s="2" t="inlineStr">
         <is>
-          <t>guide.elephant.paragraph1</t>
+          <t>guide.general.paragraph2</t>
         </is>
       </c>
       <c r="B317" s="2" t="inlineStr">
         <is>
-          <t>Elephant</t>
+          <t>Moves one step &lt;b&gt;horizontally or vertically&lt;/b&gt; within the palace. The two Generals may not face each other directly on the same file. If they are facing each other, there must be at least one piece of either side placed between them.</t>
         </is>
       </c>
       <c r="C317" s="2" t="inlineStr">
         <is>
-          <t>Tượng</t>
+          <t>Mỗi nước được đi một bước &lt;b&gt;ngang hoặc dọc&lt;/b&gt; tùy ý trong cung Tướng. Hai tướng của 2 bên không được đối mặt nhau trực tiếp trên cùng một đường thẳng. Nếu đối mặt, bắt buộc phải có quân của bất kỳ bên nào đứng che mặt.</t>
         </is>
       </c>
     </row>
     <row r="318" ht="72" customHeight="1">
       <c r="A318" s="2" t="inlineStr">
         <is>
-          <t>guide.elephant.paragraph2</t>
+          <t>guide.advisor.paragraph1</t>
         </is>
       </c>
       <c r="B318" s="2" t="inlineStr">
         <is>
-          <t>Moves &lt;b&gt;two steps diagonally&lt;/b&gt; on its own side of the board and may not cross the river. If there is another piece on the midpoint of that diagonal path, the Elephant is blocked and cannot move.</t>
+          <t>Advisor</t>
         </is>
       </c>
       <c r="C318" s="2" t="inlineStr">
         <is>
-          <t>Mỗi nước &lt;b&gt;đi chéo hai bước&lt;/b&gt; tại trận địa bên mình, không được qua sông. Nếu ở giữa đường chéo đó có quân khác đứng thì quân Tượng bị cản, không đi được.</t>
+          <t>Sĩ</t>
         </is>
       </c>
     </row>
     <row r="319" ht="18" customHeight="1">
       <c r="A319" s="2" t="inlineStr">
         <is>
-          <t>guide.chariot.paragraph1</t>
+          <t>guide.advisor.paragraph2</t>
         </is>
       </c>
       <c r="B319" s="2" t="inlineStr">
         <is>
-          <t>Chariot</t>
+          <t>Moves one step &lt;b&gt;diagonally&lt;/b&gt; within the palace.</t>
         </is>
       </c>
       <c r="C319" s="2" t="inlineStr">
         <is>
-          <t>Xe</t>
-        </is>
-      </c>
-    </row>
-    <row r="320" ht="90" customHeight="1">
+          <t>Mỗi nước &lt;b&gt;đi chéo một bước&lt;/b&gt; trong cung Tướng.</t>
+        </is>
+      </c>
+    </row>
+    <row r="320" ht="54" customHeight="1">
       <c r="A320" s="2" t="inlineStr">
         <is>
-          <t>guide.chariot.paragraph2</t>
+          <t>guide.elephant.paragraph1</t>
         </is>
       </c>
       <c r="B320" s="2" t="inlineStr">
         <is>
-          <t>Moves &lt;b&gt;horizontally or vertically&lt;/b&gt; with no limit on distance, as long as no piece blocks the path.</t>
+          <t>Elephant</t>
         </is>
       </c>
       <c r="C320" s="2" t="inlineStr">
         <is>
-          <t>Mỗi nước được &lt;b&gt;đi dọc hoặc đi ngang&lt;/b&gt;, không hạn chế số bước đi nếu không có quân khác cản đường.</t>
+          <t>Tượng</t>
         </is>
       </c>
     </row>
     <row r="321" ht="18" customHeight="1">
       <c r="A321" s="2" t="inlineStr">
         <is>
-          <t>guide.horse.paragraph1</t>
+          <t>guide.elephant.paragraph2</t>
         </is>
       </c>
       <c r="B321" s="2" t="inlineStr">
         <is>
-          <t>Horse</t>
+          <t>Moves &lt;b&gt;two steps diagonally&lt;/b&gt; on its own side of the board and may not cross the river. If there is another piece on the midpoint of that diagonal path, the Elephant is blocked and cannot move.</t>
         </is>
       </c>
       <c r="C321" s="2" t="inlineStr">
         <is>
-          <t>Mã</t>
+          <t>Mỗi nước &lt;b&gt;đi chéo hai bước&lt;/b&gt; tại trận địa bên mình, không được qua sông. Nếu ở giữa đường chéo đó có quân khác đứng thì quân Tượng bị cản, không đi được.</t>
         </is>
       </c>
     </row>
     <row r="322" ht="72" customHeight="1">
       <c r="A322" s="2" t="inlineStr">
         <is>
+          <t>guide.chariot.paragraph1</t>
+        </is>
+      </c>
+      <c r="B322" s="2" t="inlineStr">
+        <is>
+          <t>Chariot</t>
+        </is>
+      </c>
+      <c r="C322" s="2" t="inlineStr">
+        <is>
+          <t>Xe</t>
+        </is>
+      </c>
+    </row>
+    <row r="323" ht="18" customHeight="1">
+      <c r="A323" s="2" t="inlineStr">
+        <is>
+          <t>guide.chariot.paragraph2</t>
+        </is>
+      </c>
+      <c r="B323" s="2" t="inlineStr">
+        <is>
+          <t>Moves &lt;b&gt;horizontally or vertically&lt;/b&gt; with no limit on distance, as long as no piece blocks the path.</t>
+        </is>
+      </c>
+      <c r="C323" s="2" t="inlineStr">
+        <is>
+          <t>Mỗi nước được &lt;b&gt;đi dọc hoặc đi ngang&lt;/b&gt;, không hạn chế số bước đi nếu không có quân khác cản đường.</t>
+        </is>
+      </c>
+    </row>
+    <row r="324" ht="90" customHeight="1">
+      <c r="A324" s="2" t="inlineStr">
+        <is>
+          <t>guide.horse.paragraph1</t>
+        </is>
+      </c>
+      <c r="B324" s="2" t="inlineStr">
+        <is>
+          <t>Horse</t>
+        </is>
+      </c>
+      <c r="C324" s="2" t="inlineStr">
+        <is>
+          <t>Mã</t>
+        </is>
+      </c>
+    </row>
+    <row r="325" ht="18" customHeight="1">
+      <c r="A325" s="2" t="inlineStr">
+        <is>
           <t>guide.horse.paragraph2</t>
         </is>
       </c>
-      <c r="B322" s="2" t="inlineStr">
+      <c r="B325" s="2" t="inlineStr">
         <is>
           <t>Moves in an &lt;b&gt;L-shape&lt;/b&gt; (one step orthogonally then one step diagonally outward). If the adjacent orthogonal point is occupied by any piece, the Horse is blocked and cannot move.</t>
         </is>
       </c>
-      <c r="C322" s="2" t="inlineStr">
+      <c r="C325" s="2" t="inlineStr">
         <is>
           <t>Đi theo &lt;b&gt;đường chéo hình chữ nhật&lt;/b&gt; của hai ô vuông liền nhau. Nếu giao điểm liền kề bước thẳng dọc ngang có một quân khác đứng thì Mã bị cản, không đi được.</t>
         </is>
       </c>
     </row>
-    <row r="323" ht="54" customHeight="1">
-      <c r="A323" s="2" t="inlineStr">
+    <row r="326" ht="72" customHeight="1">
+      <c r="A326" s="2" t="inlineStr">
         <is>
           <t>guide.cannon.paragraph1</t>
         </is>
       </c>
-      <c r="B323" s="2" t="inlineStr">
+      <c r="B326" s="2" t="inlineStr">
         <is>
           <t>Cannon</t>
         </is>
       </c>
-      <c r="C323" s="2" t="inlineStr">
+      <c r="C326" s="2" t="inlineStr">
         <is>
           <t>Pháo</t>
-        </is>
-      </c>
-    </row>
-    <row r="324" ht="54" customHeight="1">
-      <c r="A324" s="2" t="inlineStr">
-        <is>
-          <t>guide.cannon.paragraph2</t>
-        </is>
-      </c>
-      <c r="B324" s="2" t="inlineStr">
-        <is>
-          <t>Moves &lt;b&gt;horizontally or vertically&lt;/b&gt; like a Chariot when not capturing. To capture, it must &lt;b&gt;jump over exactly one piece&lt;/b&gt; to reach its target. If there are zero or more than one pieces between the Cannon and the target, it cannot capture.</t>
-        </is>
-      </c>
-      <c r="C324" s="2" t="inlineStr">
-        <is>
-          <t>Đi ngang hoặc dọc giống Xe khi không bắt quân. Để bắt quân, nó phải &lt;b&gt;nhảy qua đúng một quân khác&lt;/b&gt; để đến mục tiêu. Nếu không có hoặc có nhiều hơn một quân giữa Pháo và mục tiêu, nó không thể bắt quân.</t>
-        </is>
-      </c>
-    </row>
-    <row r="325" ht="54" customHeight="1">
-      <c r="A325" s="2" t="inlineStr">
-        <is>
-          <t>guide.soldier.paragraph1</t>
-        </is>
-      </c>
-      <c r="B325" s="2" t="inlineStr">
-        <is>
-          <t>Soldier</t>
-        </is>
-      </c>
-      <c r="C325" s="2" t="inlineStr">
-        <is>
-          <t>Tốt</t>
-        </is>
-      </c>
-    </row>
-    <row r="326" ht="90" customHeight="1">
-      <c r="A326" s="2" t="inlineStr">
-        <is>
-          <t>guide.soldier.paragraph2</t>
-        </is>
-      </c>
-      <c r="B326" s="2" t="inlineStr">
-        <is>
-          <t>Moves &lt;b&gt;one step&lt;/b&gt; each turn. Before crossing the river, it can only move forward. After crossing the river, it may move &lt;b&gt;forward or sideways&lt;/b&gt;, but never backward.</t>
-        </is>
-      </c>
-      <c r="C326" s="2" t="inlineStr">
-        <is>
-          <t>Mỗi nước đi &lt;b&gt;một bước&lt;/b&gt;. Khi chưa qua sông, Tốt chỉ được tiến. Khi Tốt đã qua sông được quyền &lt;b&gt;đi tiến và đi ngang&lt;/b&gt;, không được phép lùi.</t>
         </is>
       </c>
     </row>
     <row r="327" ht="54" customHeight="1">
       <c r="A327" s="2" t="inlineStr">
         <is>
+          <t>guide.cannon.paragraph2</t>
+        </is>
+      </c>
+      <c r="B327" s="2" t="inlineStr">
+        <is>
+          <t>Moves &lt;b&gt;horizontally or vertically&lt;/b&gt; like a Chariot when not capturing. To capture, it must &lt;b&gt;jump over exactly one piece&lt;/b&gt; to reach its target. If there are zero or more than one pieces between the Cannon and the target, it cannot capture.</t>
+        </is>
+      </c>
+      <c r="C327" s="2" t="inlineStr">
+        <is>
+          <t>Đi ngang hoặc dọc giống Xe khi không bắt quân. Để bắt quân, nó phải &lt;b&gt;nhảy qua đúng một quân khác&lt;/b&gt; để đến mục tiêu. Nếu không có hoặc có nhiều hơn một quân giữa Pháo và mục tiêu, nó không thể bắt quân.</t>
+        </is>
+      </c>
+    </row>
+    <row r="328" ht="54" customHeight="1">
+      <c r="A328" s="2" t="inlineStr">
+        <is>
+          <t>guide.soldier.paragraph1</t>
+        </is>
+      </c>
+      <c r="B328" s="2" t="inlineStr">
+        <is>
+          <t>Soldier</t>
+        </is>
+      </c>
+      <c r="C328" s="2" t="inlineStr">
+        <is>
+          <t>Tốt</t>
+        </is>
+      </c>
+    </row>
+    <row r="329" ht="54" customHeight="1">
+      <c r="A329" s="2" t="inlineStr">
+        <is>
+          <t>guide.soldier.paragraph2</t>
+        </is>
+      </c>
+      <c r="B329" s="2" t="inlineStr">
+        <is>
+          <t>Moves &lt;b&gt;one step&lt;/b&gt; each turn. Before crossing the river, it can only move forward. After crossing the river, it may move &lt;b&gt;forward or sideways&lt;/b&gt;, but never backward.</t>
+        </is>
+      </c>
+      <c r="C329" s="2" t="inlineStr">
+        <is>
+          <t>Mỗi nước đi &lt;b&gt;một bước&lt;/b&gt;. Khi chưa qua sông, Tốt chỉ được tiến. Khi Tốt đã qua sông được quyền &lt;b&gt;đi tiến và đi ngang&lt;/b&gt;, không được phép lùi.</t>
+        </is>
+      </c>
+    </row>
+    <row r="330" ht="90" customHeight="1">
+      <c r="A330" s="2" t="inlineStr">
+        <is>
           <t>guide.capturing.paragraph1</t>
         </is>
       </c>
-      <c r="B327" s="2" t="inlineStr">
+      <c r="B330" s="2" t="inlineStr">
         <is>
           <t>When a piece moves to an intersection occupied by an opponent's piece, it may &lt;b&gt;capture that piece&lt;/b&gt; and occupy its position.</t>
         </is>
       </c>
-      <c r="C327" s="2" t="inlineStr">
+      <c r="C330" s="2" t="inlineStr">
         <is>
           <t>Khi một quân đi tới một giao điểm khác đã có quân đối phương đứng thì được quyền &lt;b&gt;bắt quân đó&lt;/b&gt;, đồng thời chiếm giữ vị trí quân bị bắt.</t>
         </is>
       </c>
     </row>
-    <row r="328" ht="36" customHeight="1">
-      <c r="A328" s="2" t="inlineStr">
+    <row r="331" ht="54" customHeight="1">
+      <c r="A331" s="2" t="inlineStr">
         <is>
           <t>guide.capturing.paragraph2</t>
         </is>
       </c>
-      <c r="B328" s="2" t="inlineStr">
+      <c r="B331" s="2" t="inlineStr">
         <is>
           <t>You may not capture your own pieces. You may sacrifice your own pieces to be captured by the opponent, &lt;b&gt;except for the General&lt;/b&gt;.</t>
         </is>
       </c>
-      <c r="C328" s="2" t="inlineStr">
+      <c r="C331" s="2" t="inlineStr">
         <is>
           <t>Không được bắt quân bên mình. Được phép cho đối phương bắt đầu quân mình chủ động hiến mình cho đối phương, &lt;b&gt;trừ Tướng&lt;/b&gt;.</t>
         </is>
       </c>
     </row>
-    <row r="329" ht="18" customHeight="1">
-      <c r="A329" s="2" t="inlineStr">
+    <row r="332" ht="36" customHeight="1">
+      <c r="A332" s="2" t="inlineStr">
         <is>
           <t>guide.capturing.paragraph3</t>
         </is>
       </c>
-      <c r="B329" s="2" t="inlineStr">
+      <c r="B332" s="2" t="inlineStr">
         <is>
           <t>A captured piece is removed from the board. &lt;b&gt;Chasing one piece for more than 6 consecutive moves is not allowed&lt;/b&gt;.</t>
         </is>
       </c>
-      <c r="C329" s="2" t="inlineStr">
+      <c r="C332" s="2" t="inlineStr">
         <is>
           <t>Quân bị bắt phải bị loại và bị nhấc ra khỏi bàn cờ. &lt;b&gt;Không được đuổi 1 quân quá 6 nước cờ liên tiếp&lt;/b&gt;.</t>
         </is>
       </c>
     </row>
-    <row r="330" ht="36" customHeight="1">
-      <c r="A330" s="2" t="inlineStr">
+    <row r="333" ht="18" customHeight="1">
+      <c r="A333" s="2" t="inlineStr">
         <is>
           <t>guide.check.paragraph1</t>
         </is>
       </c>
-      <c r="B330" s="2" t="inlineStr">
+      <c r="B333" s="2" t="inlineStr">
         <is>
           <t>If a player makes a move that threatens to capture the opponent's General on the next move (by the same piece or another piece), it is called a &lt;b&gt;Check&lt;/b&gt;. The checked side must respond to avoid check. Otherwise, that side loses</t>
         </is>
       </c>
-      <c r="C330" s="2" t="inlineStr">
+      <c r="C333" s="2" t="inlineStr">
         <is>
           <t>Nếu người chơi thực hiện một nước đi đe dọa bắt Tướng của đối phương ở nước đi tiếp theo (bằng chính quân cờ đó hoặc một quân cờ khác), thì đó được gọi là &lt;b&gt;Chiếu&lt;/b&gt;. Bên bị chiếu phải đáp trả để tránh bị chiếu. Nếu không sẽ bị xử thua</t>
         </is>
       </c>
     </row>
-    <row r="331" ht="36" customHeight="1">
-      <c r="A331" s="2" t="inlineStr">
+    <row r="334" ht="36" customHeight="1">
+      <c r="A334" s="2" t="inlineStr">
         <is>
           <t>guide.check.paragraph2</t>
         </is>
       </c>
-      <c r="B331" s="2" t="inlineStr">
+      <c r="B334" s="2" t="inlineStr">
         <is>
           <t>When the General is checked from any direction (including from behind), the checked side may respond in one of the following ways:</t>
         </is>
       </c>
-      <c r="C331" s="2" t="inlineStr">
+      <c r="C334" s="2" t="inlineStr">
         <is>
           <t>Tướng bị chiếu từ cả bốn hướng (bị chiếu cả từ phía sau) có thể ứng phó với nước chiếu tướng bằng một trong các cách sau:</t>
         </is>
       </c>
     </row>
-    <row r="332" ht="72" customHeight="1">
-      <c r="A332" s="2" t="inlineStr">
+    <row r="335" ht="36" customHeight="1">
+      <c r="A335" s="2" t="inlineStr">
         <is>
           <t>guide.check.paragraph3</t>
         </is>
       </c>
-      <c r="B332" s="2" t="inlineStr">
+      <c r="B335" s="2" t="inlineStr">
         <is>
           <t>Move the General to another position to escape check</t>
         </is>
       </c>
-      <c r="C332" s="2" t="inlineStr">
+      <c r="C335" s="2" t="inlineStr">
         <is>
           <t>Di chuyển tướng sang vị trí khác để tránh nước chiếu</t>
         </is>
       </c>
     </row>
-    <row r="333" ht="54" customHeight="1">
-      <c r="A333" s="2" t="inlineStr">
+    <row r="336" ht="72" customHeight="1">
+      <c r="A336" s="2" t="inlineStr">
         <is>
           <t>guide.check.paragraph4</t>
         </is>
       </c>
-      <c r="B333" s="2" t="inlineStr">
+      <c r="B336" s="2" t="inlineStr">
         <is>
           <t>Capture the checking piece</t>
         </is>
       </c>
-      <c r="C333" s="2" t="inlineStr">
+      <c r="C336" s="2" t="inlineStr">
         <is>
           <t>Bắt quân đang chiếu</t>
         </is>
       </c>
     </row>
-    <row r="334" ht="54" customHeight="1">
-      <c r="A334" s="2" t="inlineStr">
+    <row r="337" ht="54" customHeight="1">
+      <c r="A337" s="2" t="inlineStr">
         <is>
           <t>guide.check.paragraph5</t>
         </is>
       </c>
-      <c r="B334" s="2" t="inlineStr">
+      <c r="B337" s="2" t="inlineStr">
         <is>
           <t>Block the checking line with another piece to protect the General</t>
         </is>
       </c>
-      <c r="C334" s="2" t="inlineStr">
+      <c r="C337" s="2" t="inlineStr">
         <is>
           <t>Dùng quân khác cản quân chiếu, đi quân che đỡ cho tướng</t>
         </is>
       </c>
     </row>
-    <row r="335" ht="90" customHeight="1">
-      <c r="A335" s="2" t="inlineStr">
+    <row r="338" ht="54" customHeight="1">
+      <c r="A338" s="2" t="inlineStr">
         <is>
           <t>guide.check.paragraph6</t>
         </is>
       </c>
-      <c r="B335" s="2" t="inlineStr">
+      <c r="B338" s="2" t="inlineStr">
         <is>
           <t>Repeatedly checking for more than 6 consecutive moves is not allowed</t>
         </is>
       </c>
-      <c r="C335" s="2" t="inlineStr">
+      <c r="C338" s="2" t="inlineStr">
         <is>
           <t>Không được chiếu tướng quá 6 nước cờ liên tiếp</t>
         </is>
       </c>
     </row>
-    <row r="336" ht="54" customHeight="1">
-      <c r="A336" s="2" t="inlineStr">
+    <row r="339" ht="90" customHeight="1">
+      <c r="A339" s="2" t="inlineStr">
         <is>
           <t>guide.result.paragraph1</t>
         </is>
       </c>
-      <c r="B336" s="2" t="inlineStr">
+      <c r="B339" s="2" t="inlineStr">
         <is>
           <t>When one side gives Check and the other side has no legal way to protect the General, it is called a &lt;b&gt;Checkmate&lt;/b&gt;. The side that delivers Checkmate wins.</t>
         </is>
       </c>
-      <c r="C336" s="2" t="inlineStr">
+      <c r="C339" s="2" t="inlineStr">
         <is>
           <t>Khi một bên chiếu Tướng mà bên còn lại không thể làm gì để bảo vệ Tướng thì được gọi là &lt;b&gt;Chiếu Hết&lt;/b&gt;, bên thực hiện được Chiếu Hết sẽ giành chiến thắng.</t>
         </is>
       </c>
     </row>
-    <row r="337" ht="17" customHeight="1">
-      <c r="A337" s="2" t="inlineStr">
+    <row r="340" ht="54" customHeight="1">
+      <c r="A340" s="2" t="inlineStr">
         <is>
           <t>guide.result.paragraph2</t>
         </is>
       </c>
-      <c r="B337" s="2" t="inlineStr">
+      <c r="B340" s="2" t="inlineStr">
         <is>
           <t>If a player runs out of time for a single move (for example: 90s) without moving, the other side is awarded a &lt;b&gt;win&lt;/b&gt;.</t>
         </is>
       </c>
-      <c r="C337" s="2" t="inlineStr">
+      <c r="C340" s="2" t="inlineStr">
         <is>
           <t>Khi hết thời gian một nước đi (ví dụ: 90s) mà vẫn chưa di chuyển quân thì bên còn lại sẽ được &lt;b&gt;xử Thắng&lt;/b&gt;.</t>
         </is>
       </c>
     </row>
-    <row r="338" ht="17" customHeight="1">
-      <c r="A338" s="2" t="inlineStr">
+    <row r="341" ht="18" customHeight="1">
+      <c r="A341" s="2" t="inlineStr">
         <is>
           <t>guide.result.paragraph3</t>
         </is>
       </c>
-      <c r="B338" s="2" t="inlineStr">
+      <c r="B341" s="2" t="inlineStr">
         <is>
           <t>If a player runs out of total game time (for example: 5 minutes or 10 minutes), the other side is awarded a &lt;b&gt;win&lt;/b&gt;.</t>
         </is>
       </c>
-      <c r="C338" s="2" t="inlineStr">
+      <c r="C341" s="2" t="inlineStr">
         <is>
           <t>Khi một bên hết thời gian ván đấu (ví dụ: 5 phút, 10 phút) thì bên còn lại sẽ được &lt;b&gt;xử Thắng&lt;/b&gt;.</t>
         </is>
       </c>
     </row>
-    <row r="339" ht="17" customHeight="1">
-      <c r="A339" s="2" t="inlineStr">
+    <row r="342" ht="18" customHeight="1">
+      <c r="A342" s="2" t="inlineStr">
         <is>
           <t>guide.result.paragraph4</t>
         </is>
       </c>
-      <c r="B339" s="2" t="inlineStr">
+      <c r="B342" s="2" t="inlineStr">
         <is>
           <t>If both sides have no pieces that have crossed the river, the game is declared a &lt;b&gt;draw&lt;/b&gt;. If one side still has pieces across the river but runs out of time, while the other side still has time but has no pieces across the river, the game is declared a &lt;b&gt;draw&lt;/b&gt;.</t>
         </is>
       </c>
-      <c r="C339" s="2" t="inlineStr">
+      <c r="C342" s="2" t="inlineStr">
         <is>
           <t>Khi cả 2 bên đều không còn quân qua sông, ván đấu sẽ được &lt;b&gt;xử Hòa&lt;/b&gt;. Khi một bên còn quân qua sông nhưng cạn thời gian, một bên còn thời gian nhưng hết quân qua sông, ván đấu sẽ được &lt;b&gt;xử Hòa&lt;/b&gt;.</t>
         </is>
       </c>
     </row>
-    <row r="340" ht="17" customHeight="1">
-      <c r="A340" s="2" t="inlineStr">
+    <row r="343" ht="36" customHeight="1">
+      <c r="A343" s="2" t="inlineStr">
         <is>
           <t>guide.result.paragraph5</t>
         </is>
       </c>
-      <c r="B340" s="2" t="inlineStr">
+      <c r="B343" s="2" t="inlineStr">
         <is>
           <t>Within 40 moves, if there is no capture and no Soldier advances by one square, the game is declared a &lt;b&gt;draw&lt;/b&gt;.</t>
         </is>
       </c>
-      <c r="C340" s="2" t="inlineStr">
+      <c r="C343" s="2" t="inlineStr">
         <is>
           <t>Trong vòng 40 nước nếu không phát sinh nước bắt quân, Tốt không tiến 1 ô thì ván đấu sẽ được &lt;b&gt;xử Hòa&lt;/b&gt;.</t>
         </is>
       </c>
     </row>
-    <row r="341" ht="17" customHeight="1">
-      <c r="A341" s="2" t="inlineStr"/>
-      <c r="B341" s="2" t="inlineStr"/>
-      <c r="C341" s="2" t="inlineStr"/>
-    </row>
-    <row r="342" ht="17" customHeight="1">
-      <c r="A342" s="2" t="inlineStr"/>
-      <c r="B342" s="2" t="inlineStr"/>
-      <c r="C342" s="2" t="inlineStr"/>
-    </row>
-    <row r="343" ht="17" customHeight="1">
-      <c r="A343" s="2" t="inlineStr"/>
-      <c r="B343" s="2" t="inlineStr"/>
-      <c r="C343" s="2" t="inlineStr"/>
-    </row>
-    <row r="344" ht="17" customHeight="1">
-      <c r="A344" s="2" t="inlineStr"/>
-      <c r="B344" s="2" t="inlineStr"/>
-      <c r="C344" s="2" t="inlineStr"/>
-    </row>
-    <row r="345">
-      <c r="A345" t="inlineStr"/>
-      <c r="B345" t="inlineStr"/>
-      <c r="C345" t="inlineStr"/>
-    </row>
-    <row r="346">
-      <c r="A346" t="inlineStr"/>
-      <c r="B346" t="inlineStr"/>
-      <c r="C346" t="inlineStr"/>
-    </row>
-    <row r="347">
-      <c r="A347" t="inlineStr"/>
-      <c r="B347" t="inlineStr"/>
-      <c r="C347" t="inlineStr"/>
-    </row>
-    <row r="348">
-      <c r="A348" t="inlineStr"/>
-      <c r="B348" t="inlineStr"/>
-      <c r="C348" t="inlineStr"/>
-    </row>
-    <row r="349">
-      <c r="A349" t="inlineStr"/>
-      <c r="B349" t="inlineStr"/>
-      <c r="C349" t="inlineStr"/>
-    </row>
-    <row r="350">
-      <c r="A350" t="inlineStr"/>
-      <c r="B350" t="inlineStr"/>
-      <c r="C350" t="inlineStr"/>
-    </row>
-    <row r="351">
-      <c r="A351" t="inlineStr"/>
-      <c r="B351" t="inlineStr"/>
-      <c r="C351" t="inlineStr"/>
+    <row r="344" ht="18" customHeight="1">
+      <c r="A344" s="2" t="inlineStr">
+        <is>
+          <t>extra-money.lucky-wheel.title</t>
+        </is>
+      </c>
+      <c r="B344" s="2" t="inlineStr">
+        <is>
+          <t>Lucky Wheel</t>
+        </is>
+      </c>
+      <c r="C344" s="2" t="inlineStr">
+        <is>
+          <t>Vòng quay may mắn</t>
+        </is>
+      </c>
+    </row>
+    <row r="345" ht="18" customHeight="1">
+      <c r="A345" s="2" t="inlineStr">
+        <is>
+          <t>extra-money.lucky-wheel.description</t>
+        </is>
+      </c>
+      <c r="B345" s="2" t="inlineStr">
+        <is>
+          <t>Spin the wheel to earn money! Click the spin button in the middle of the wheel to try your luck.</t>
+        </is>
+      </c>
+      <c r="C345" s="2" t="inlineStr">
+        <is>
+          <t>Quay vòng để kiếm tiền! Bấm nút Quay ở giữa vòng quay để thử vận may của bạn.</t>
+        </is>
+      </c>
+    </row>
+    <row r="346" ht="36" customHeight="1">
+      <c r="A346" s="2" t="inlineStr">
+        <is>
+          <t>extra-money.lucky-wheel.spin-button</t>
+        </is>
+      </c>
+      <c r="B346" s="2" t="inlineStr">
+        <is>
+          <t>Spin</t>
+        </is>
+      </c>
+      <c r="C346" s="2" t="inlineStr">
+        <is>
+          <t>Quay</t>
+        </is>
+      </c>
+    </row>
+    <row r="347" ht="18" customHeight="1">
+      <c r="A347" s="2" t="inlineStr">
+        <is>
+          <t>extra-money.lucky-wheel.reward-placeholder</t>
+        </is>
+      </c>
+      <c r="B347" s="2" t="inlineStr">
+        <is>
+          <t>Click Spin to get started</t>
+        </is>
+      </c>
+      <c r="C347" s="2" t="inlineStr">
+        <is>
+          <t>Nhấp Quay để bắt đầu</t>
+        </is>
+      </c>
+    </row>
+    <row r="348" ht="36" customHeight="1">
+      <c r="A348" s="2" t="inlineStr">
+        <is>
+          <t>extra-money.title</t>
+        </is>
+      </c>
+      <c r="B348" s="2" t="inlineStr">
+        <is>
+          <t>Daily tasks</t>
+        </is>
+      </c>
+      <c r="C348" s="2" t="inlineStr">
+        <is>
+          <t>Tác vụ thường nhật</t>
+        </is>
+      </c>
+    </row>
+    <row r="349" ht="18" customHeight="1">
+      <c r="A349" s="2" t="inlineStr">
+        <is>
+          <t>extra-money.tab.lucky-wheel</t>
+        </is>
+      </c>
+      <c r="B349" s="2" t="inlineStr">
+        <is>
+          <t>Lucky Wheel</t>
+        </is>
+      </c>
+      <c r="C349" s="2" t="inlineStr">
+        <is>
+          <t>Vòng Quay May Mắn</t>
+        </is>
+      </c>
+    </row>
+    <row r="350" ht="18" customHeight="1">
+      <c r="A350" s="2" t="inlineStr">
+        <is>
+          <t>extra-money.tab.bonus-coin</t>
+        </is>
+      </c>
+      <c r="B350" s="2" t="inlineStr">
+        <is>
+          <t>Bonus Coin</t>
+        </is>
+      </c>
+      <c r="C350" s="2" t="inlineStr">
+        <is>
+          <t>Xu Thưởng</t>
+        </is>
+      </c>
+    </row>
+    <row r="351" ht="18" customHeight="1">
+      <c r="A351" s="2" t="inlineStr">
+        <is>
+          <t>extra-money.tab.daily-bonus</t>
+        </is>
+      </c>
+      <c r="B351" s="2" t="inlineStr">
+        <is>
+          <t>Daily Bonus</t>
+        </is>
+      </c>
+      <c r="C351" s="2" t="inlineStr">
+        <is>
+          <t>Thưởng hàng ngày</t>
+        </is>
+      </c>
+    </row>
+    <row r="352" ht="18" customHeight="1">
+      <c r="A352" s="2" t="inlineStr">
+        <is>
+          <t>extra-money.bonus-coin.subtitle</t>
+        </is>
+      </c>
+      <c r="B352" s="2" t="inlineStr">
+        <is>
+          <t>Watch a short video to earn free coin</t>
+        </is>
+      </c>
+      <c r="C352" s="2" t="inlineStr">
+        <is>
+          <t>Xem video ngắn để nhận xu miễn phí</t>
+        </is>
+      </c>
+    </row>
+    <row r="353" ht="18" customHeight="1">
+      <c r="A353" s="2" t="inlineStr">
+        <is>
+          <t>extra-money.bonus-coin.next-in</t>
+        </is>
+      </c>
+      <c r="B353" s="2" t="inlineStr">
+        <is>
+          <t>Next in:</t>
+        </is>
+      </c>
+      <c r="C353" s="2" t="inlineStr">
+        <is>
+          <t>Lượt kế tiếp:</t>
+        </is>
+      </c>
+    </row>
+    <row r="354" ht="17" customHeight="1">
+      <c r="A354" s="2" t="inlineStr">
+        <is>
+          <t>extra-money.bonus-coin.coin-unit</t>
+        </is>
+      </c>
+      <c r="B354" s="2" t="inlineStr">
+        <is>
+          <t>coin</t>
+        </is>
+      </c>
+      <c r="C354" s="2" t="inlineStr">
+        <is>
+          <t>xu</t>
+        </is>
+      </c>
+    </row>
+    <row r="355" ht="18" customHeight="1">
+      <c r="A355" s="2" t="inlineStr">
+        <is>
+          <t>extra-money.bonus-coin.watch-video</t>
+        </is>
+      </c>
+      <c r="B355" s="2" t="inlineStr">
+        <is>
+          <t>Watch video</t>
+        </is>
+      </c>
+      <c r="C355" s="2" t="inlineStr">
+        <is>
+          <t>Xem video</t>
+        </is>
+      </c>
+    </row>
+    <row r="356" ht="18" customHeight="1">
+      <c r="A356" s="2" t="inlineStr">
+        <is>
+          <t>extra-money.daily-bonus.subtitle</t>
+        </is>
+      </c>
+      <c r="B356" s="2" t="inlineStr">
+        <is>
+          <t>Login 7 days in a row to earn 4000 coin</t>
+        </is>
+      </c>
+      <c r="C356" s="2" t="inlineStr">
+        <is>
+          <t>Đăng nhập 7 ngày liên tiếp để nhận 4000 xu</t>
+        </is>
+      </c>
+    </row>
+    <row r="357" ht="18" customHeight="1">
+      <c r="A357" s="2" t="inlineStr">
+        <is>
+          <t>extra-money.daily-bonus.day</t>
+        </is>
+      </c>
+      <c r="B357" s="2" t="inlineStr">
+        <is>
+          <t>Day</t>
+        </is>
+      </c>
+      <c r="C357" s="2" t="inlineStr">
+        <is>
+          <t>Ngày</t>
+        </is>
+      </c>
+    </row>
+    <row r="358" ht="18" customHeight="1">
+      <c r="A358" s="2" t="inlineStr">
+        <is>
+          <t>profile.button.save</t>
+        </is>
+      </c>
+      <c r="B358" s="2" t="inlineStr">
+        <is>
+          <t>Save</t>
+        </is>
+      </c>
+      <c r="C358" s="2" t="inlineStr">
+        <is>
+          <t>Lưu</t>
+        </is>
+      </c>
+    </row>
+    <row r="359" ht="18" customHeight="1">
+      <c r="A359" s="2" t="inlineStr">
+        <is>
+          <t>profile.button.cancel</t>
+        </is>
+      </c>
+      <c r="B359" s="2" t="inlineStr">
+        <is>
+          <t>Cancel</t>
+        </is>
+      </c>
+      <c r="C359" s="2" t="inlineStr">
+        <is>
+          <t>Huỷ</t>
+        </is>
+      </c>
+    </row>
+    <row r="360" ht="18" customHeight="1">
+      <c r="A360" s="2" t="inlineStr"/>
+      <c r="B360" s="2" t="inlineStr"/>
+      <c r="C360" s="2" t="inlineStr"/>
+    </row>
+    <row r="361" ht="17" customHeight="1">
+      <c r="A361" s="2" t="inlineStr"/>
+      <c r="B361" s="2" t="inlineStr"/>
+      <c r="C361" s="2" t="inlineStr"/>
+    </row>
+    <row r="362" ht="17" customHeight="1">
+      <c r="A362" s="2" t="inlineStr"/>
+      <c r="B362" s="2" t="inlineStr"/>
+      <c r="C362" s="2" t="inlineStr"/>
+    </row>
+    <row r="363" ht="17" customHeight="1">
+      <c r="A363" s="2" t="inlineStr"/>
+      <c r="B363" s="2" t="inlineStr"/>
+      <c r="C363" s="2" t="inlineStr"/>
+    </row>
+    <row r="364" ht="17" customHeight="1">
+      <c r="A364" s="2" t="inlineStr"/>
+      <c r="B364" s="2" t="inlineStr"/>
+      <c r="C364" s="2" t="inlineStr"/>
+    </row>
+    <row r="365" ht="17" customHeight="1">
+      <c r="A365" s="2" t="inlineStr"/>
+      <c r="B365" s="2" t="inlineStr"/>
+      <c r="C365" s="2" t="inlineStr"/>
+    </row>
+    <row r="366" ht="17" customHeight="1">
+      <c r="A366" s="2" t="inlineStr"/>
+      <c r="B366" s="2" t="inlineStr"/>
+      <c r="C366" s="2" t="inlineStr"/>
+    </row>
+    <row r="367" ht="17" customHeight="1">
+      <c r="A367" s="2" t="inlineStr"/>
+      <c r="B367" s="2" t="inlineStr"/>
+      <c r="C367" s="2" t="inlineStr"/>
+    </row>
+    <row r="368" ht="17" customHeight="1">
+      <c r="A368" s="2" t="inlineStr"/>
+      <c r="B368" s="2" t="inlineStr"/>
+      <c r="C368" s="2" t="inlineStr"/>
+    </row>
+    <row r="369" ht="17" customHeight="1">
+      <c r="A369" s="2" t="inlineStr"/>
+      <c r="B369" s="2" t="inlineStr"/>
+      <c r="C369" s="2" t="inlineStr"/>
+    </row>
+    <row r="370" ht="17" customHeight="1">
+      <c r="A370" s="2" t="inlineStr"/>
+      <c r="B370" s="2" t="inlineStr"/>
+      <c r="C370" s="2" t="inlineStr"/>
+    </row>
+    <row r="371" ht="17" customHeight="1">
+      <c r="A371" s="2" t="inlineStr"/>
+      <c r="B371" s="2" t="inlineStr"/>
+      <c r="C371" s="2" t="inlineStr"/>
+    </row>
+    <row r="372" ht="17" customHeight="1">
+      <c r="A372" s="2" t="inlineStr"/>
+      <c r="B372" s="2" t="inlineStr"/>
+      <c r="C372" s="2" t="inlineStr"/>
+    </row>
+    <row r="373" ht="17" customHeight="1">
+      <c r="A373" s="2" t="inlineStr"/>
+      <c r="B373" s="2" t="inlineStr"/>
+      <c r="C373" s="2" t="inlineStr"/>
+    </row>
+    <row r="374" ht="17" customHeight="1">
+      <c r="A374" s="2" t="inlineStr"/>
+      <c r="B374" s="2" t="inlineStr"/>
+      <c r="C374" s="2" t="inlineStr"/>
+    </row>
+    <row r="375" ht="17" customHeight="1">
+      <c r="A375" s="2" t="inlineStr"/>
+      <c r="B375" s="2" t="inlineStr"/>
+      <c r="C375" s="2" t="inlineStr"/>
+    </row>
+    <row r="376" ht="17" customHeight="1">
+      <c r="A376" s="2" t="inlineStr"/>
+      <c r="B376" s="2" t="inlineStr"/>
+      <c r="C376" s="2" t="inlineStr"/>
+    </row>
+    <row r="377" ht="17" customHeight="1">
+      <c r="A377" s="2" t="inlineStr"/>
+      <c r="B377" s="2" t="inlineStr"/>
+      <c r="C377" s="2" t="inlineStr"/>
+    </row>
+    <row r="378" ht="17" customHeight="1">
+      <c r="A378" s="2" t="n"/>
+      <c r="B378" s="2" t="n"/>
+      <c r="C378" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
merge xiangqi and chess into one repo
</commit_message>
<xml_diff>
--- a/tools/languages.xlsx
+++ b/tools/languages.xlsx
@@ -325,7 +325,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C433"/>
+  <dimension ref="A1:C442"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -3345,2098 +3345,2098 @@
     <row r="178" ht="18" customHeight="1">
       <c r="A178" s="1" t="inlineStr">
         <is>
-          <t>create-room.messages.invalid-time-limit</t>
+          <t>create-room.messages.invalid-game-type</t>
         </is>
       </c>
       <c r="B178" s="2" t="inlineStr">
         <is>
-          <t>Invalid time limit</t>
+          <t>Invalid game type</t>
         </is>
       </c>
       <c r="C178" s="2" t="inlineStr">
         <is>
-          <t>Thời gian không hợp lệ</t>
+          <t>Loại cờ không hợp lệ</t>
         </is>
       </c>
     </row>
     <row r="179" ht="18" customHeight="1">
       <c r="A179" s="1" t="inlineStr">
         <is>
-          <t>create-room.messages.invalid-redFirst</t>
+          <t>create-room.messages.pve-not-supported</t>
         </is>
       </c>
       <c r="B179" s="2" t="inlineStr">
         <is>
-          <t>'redFirst' must be a boolean</t>
+          <t>This game does not support playing against the bot yet</t>
         </is>
       </c>
       <c r="C179" s="2" t="inlineStr">
         <is>
-          <t>'redFirst' phải là giá trị boolean</t>
+          <t>Trò chơi này chưa hỗ trợ đấu với máy</t>
         </is>
       </c>
     </row>
     <row r="180" ht="18" customHeight="1">
       <c r="A180" s="1" t="inlineStr">
         <is>
-          <t>create-room.messages.invalid-team-name</t>
+          <t>create-room.messages.invalid-time-limit</t>
         </is>
       </c>
       <c r="B180" s="2" t="inlineStr">
         <is>
-          <t>Team name must be either 'red', 'black', or null</t>
+          <t>Invalid time limit</t>
         </is>
       </c>
       <c r="C180" s="2" t="inlineStr">
         <is>
-          <t>Tên đội phải là 'red', 'black' hoặc null</t>
+          <t>Thời gian không hợp lệ</t>
         </is>
       </c>
     </row>
     <row r="181" ht="18" customHeight="1">
       <c r="A181" s="1" t="inlineStr">
         <is>
-          <t>create-room.messages.name-required</t>
+          <t>create-room.messages.invalid-redFirst</t>
         </is>
       </c>
       <c r="B181" s="2" t="inlineStr">
         <is>
-          <t>Room name (tableName) is required and must not be empty</t>
+          <t>'redFirst' must be a boolean</t>
         </is>
       </c>
       <c r="C181" s="2" t="inlineStr">
         <is>
-          <t>Tên phòng (tableName) là bắt buộc và không được để trống</t>
+          <t>'redFirst' phải là giá trị boolean</t>
         </is>
       </c>
     </row>
     <row r="182" ht="18" customHeight="1">
       <c r="A182" s="1" t="inlineStr">
         <is>
-          <t>create-room.messages.room-created</t>
+          <t>create-room.messages.invalid-team-name</t>
         </is>
       </c>
       <c r="B182" s="2" t="inlineStr">
         <is>
-          <t>Room created successfully</t>
+          <t>Team name must be either 'red', 'black', or null</t>
         </is>
       </c>
       <c r="C182" s="2" t="inlineStr">
         <is>
-          <t>Phòng được tạo thành công</t>
+          <t>Tên đội phải là 'red', 'black' hoặc null</t>
         </is>
       </c>
     </row>
     <row r="183" ht="18" customHeight="1">
       <c r="A183" s="1" t="inlineStr">
         <is>
-          <t>fetch-rooms.messages.internal-server-error</t>
+          <t>create-room.messages.name-required</t>
         </is>
       </c>
       <c r="B183" s="2" t="inlineStr">
         <is>
-          <t>Internal server error</t>
+          <t>Room name (tableName) is required and must not be empty</t>
         </is>
       </c>
       <c r="C183" s="2" t="inlineStr">
         <is>
-          <t>Lỗi máy chủ nội bộ</t>
+          <t>Tên phòng (tableName) là bắt buộc và không được để trống</t>
         </is>
       </c>
     </row>
     <row r="184" ht="18" customHeight="1">
       <c r="A184" s="1" t="inlineStr">
         <is>
-          <t>fetch-rooms.messages.invalid-status</t>
+          <t>create-room.messages.room-created</t>
         </is>
       </c>
       <c r="B184" s="2" t="inlineStr">
         <is>
-          <t>Query parameter 'status' must be an integer</t>
+          <t>Room created successfully</t>
         </is>
       </c>
       <c r="C184" s="2" t="inlineStr">
         <is>
-          <t>Tham số truy vấn 'status' phải là số nguyên</t>
+          <t>Phòng được tạo thành công</t>
         </is>
       </c>
     </row>
     <row r="185" ht="36" customHeight="1">
       <c r="A185" s="1" t="inlineStr">
         <is>
-          <t>fetch-rooms.messages.success</t>
+          <t>fetch-rooms.messages.internal-server-error</t>
         </is>
       </c>
       <c r="B185" s="2" t="inlineStr">
         <is>
-          <t>Fetch rooms successfully</t>
+          <t>Internal server error</t>
         </is>
       </c>
       <c r="C185" s="2" t="inlineStr">
         <is>
-          <t>Lấy phòng thành công</t>
+          <t>Lỗi máy chủ nội bộ</t>
         </is>
       </c>
     </row>
     <row r="186" ht="18" customHeight="1">
       <c r="A186" s="1" t="inlineStr">
         <is>
-          <t>forgot-password.messages.email-not-found</t>
+          <t>fetch-rooms.messages.invalid-status</t>
         </is>
       </c>
       <c r="B186" s="2" t="inlineStr">
         <is>
-          <t>Email does not exist</t>
+          <t>Query parameter 'status' must be an integer</t>
         </is>
       </c>
       <c r="C186" s="2" t="inlineStr">
         <is>
-          <t>Email không tồn tại</t>
+          <t>Tham số truy vấn 'status' phải là số nguyên</t>
         </is>
       </c>
     </row>
     <row r="187" ht="36" customHeight="1">
       <c r="A187" s="1" t="inlineStr">
         <is>
-          <t>forgot-password.messages.email-service-not-configured</t>
+          <t>fetch-rooms.messages.invalid-game-type</t>
         </is>
       </c>
       <c r="B187" s="2" t="inlineStr">
         <is>
-          <t>Email service is not configured</t>
+          <t>Query parameter 'gameType' is invalid</t>
         </is>
       </c>
       <c r="C187" s="2" t="inlineStr">
         <is>
-          <t>Dịch vụ email chưa được cấu hình</t>
+          <t>Tham số truy vấn 'gameType' không hợp lệ</t>
         </is>
       </c>
     </row>
     <row r="188" ht="18" customHeight="1">
       <c r="A188" s="1" t="inlineStr">
         <is>
-          <t>forgot-password.messages.internal-server-error</t>
+          <t>variant.xiangqi.name</t>
         </is>
       </c>
       <c r="B188" s="2" t="inlineStr">
         <is>
-          <t>Internal server error</t>
+          <t>Chinese Chess</t>
         </is>
       </c>
       <c r="C188" s="2" t="inlineStr">
         <is>
-          <t>Lỗi máy chủ nội bộ</t>
+          <t>Cờ Tướng</t>
         </is>
       </c>
     </row>
     <row r="189" ht="18" customHeight="1">
       <c r="A189" s="1" t="inlineStr">
         <is>
-          <t>forgot-password.messages.invalid-email-format</t>
+          <t>variant.chess.name</t>
         </is>
       </c>
       <c r="B189" s="2" t="inlineStr">
         <is>
-          <t>Invalid email format</t>
+          <t>Chess</t>
         </is>
       </c>
       <c r="C189" s="2" t="inlineStr">
         <is>
-          <t>Định dạng email không hợp lệ</t>
+          <t>Cờ Vua</t>
         </is>
       </c>
     </row>
     <row r="190" ht="18" customHeight="1">
       <c r="A190" s="1" t="inlineStr">
         <is>
-          <t>forgot-password.messages.missing-email</t>
+          <t>variant.xiangqi.team.red</t>
         </is>
       </c>
       <c r="B190" s="2" t="inlineStr">
         <is>
-          <t>Email is required</t>
+          <t>Red</t>
         </is>
       </c>
       <c r="C190" s="2" t="inlineStr">
         <is>
-          <t>Email là bắt buộc</t>
+          <t>Đỏ</t>
         </is>
       </c>
     </row>
     <row r="191" ht="18" customHeight="1">
       <c r="A191" s="1" t="inlineStr">
         <is>
-          <t>forgot-password.messages.success</t>
+          <t>variant.xiangqi.team.black</t>
         </is>
       </c>
       <c r="B191" s="2" t="inlineStr">
         <is>
-          <t>Forgot password email sent</t>
+          <t>Black</t>
         </is>
       </c>
       <c r="C191" s="2" t="inlineStr">
         <is>
-          <t>Email đặt lại mật khẩu đã được gửi</t>
+          <t>Đen</t>
         </is>
       </c>
     </row>
     <row r="192" ht="18" customHeight="1">
       <c r="A192" s="1" t="inlineStr">
         <is>
-          <t>join-room.messages.internal-server-error</t>
+          <t>variant.chess.team.white</t>
         </is>
       </c>
       <c r="B192" s="2" t="inlineStr">
         <is>
-          <t>Internal server error</t>
+          <t>White</t>
         </is>
       </c>
       <c r="C192" s="2" t="inlineStr">
         <is>
-          <t>Lỗi máy chủ nội bộ</t>
+          <t>Trắng</t>
         </is>
       </c>
     </row>
     <row r="193" ht="18" customHeight="1">
       <c r="A193" s="1" t="inlineStr">
         <is>
-          <t>join-room.messages.invalid-team</t>
+          <t>variant.chess.team.black</t>
         </is>
       </c>
       <c r="B193" s="2" t="inlineStr">
         <is>
-          <t>Field 'team' must be 'red', 'black', null, or undefined</t>
+          <t>Black</t>
         </is>
       </c>
       <c r="C193" s="2" t="inlineStr">
         <is>
-          <t>Trường 'team' phải là 'red', 'black', null hoặc không truyền</t>
+          <t>Đen</t>
         </is>
       </c>
     </row>
     <row r="194" ht="18" customHeight="1">
       <c r="A194" s="1" t="inlineStr">
         <is>
-          <t>join-room.messages.invalid-room-id</t>
+          <t>fetch-rooms.messages.success</t>
         </is>
       </c>
       <c r="B194" s="2" t="inlineStr">
         <is>
-          <t>Field 'id' is required and must be a positive integer</t>
+          <t>Fetch rooms successfully</t>
         </is>
       </c>
       <c r="C194" s="2" t="inlineStr">
         <is>
-          <t>Trường 'id' là bắt buộc và phải là số nguyên dương</t>
+          <t>Lấy phòng thành công</t>
         </is>
       </c>
     </row>
     <row r="195" ht="18" customHeight="1">
       <c r="A195" s="1" t="inlineStr">
         <is>
-          <t>join-room.messages.room-not-found</t>
+          <t>forgot-password.messages.email-not-found</t>
         </is>
       </c>
       <c r="B195" s="2" t="inlineStr">
         <is>
-          <t>Room not found</t>
+          <t>Email does not exist</t>
         </is>
       </c>
       <c r="C195" s="2" t="inlineStr">
         <is>
-          <t>Không tìm thấy phòng</t>
+          <t>Email không tồn tại</t>
         </is>
       </c>
     </row>
     <row r="196" ht="18" customHeight="1">
       <c r="A196" s="1" t="inlineStr">
         <is>
-          <t>join-room.messages.success</t>
+          <t>forgot-password.messages.email-service-not-configured</t>
         </is>
       </c>
       <c r="B196" s="2" t="inlineStr">
         <is>
-          <t>Successfully joined the room</t>
+          <t>Email service is not configured</t>
         </is>
       </c>
       <c r="C196" s="2" t="inlineStr">
         <is>
-          <t>Tham gia phòng thành công</t>
+          <t>Dịch vụ email chưa được cấu hình</t>
         </is>
       </c>
     </row>
     <row r="197" ht="18" customHeight="1">
       <c r="A197" s="1" t="inlineStr">
         <is>
-          <t>join-room.messages.team-seat-occupied</t>
+          <t>forgot-password.messages.internal-server-error</t>
         </is>
       </c>
       <c r="B197" s="2" t="inlineStr">
         <is>
-          <t>Selected team seat is already occupied</t>
+          <t>Internal server error</t>
         </is>
       </c>
       <c r="C197" s="2" t="inlineStr">
         <is>
-          <t>Vị trí đội đã chọn đã có người chơi</t>
+          <t>Lỗi máy chủ nội bộ</t>
         </is>
       </c>
     </row>
     <row r="198" ht="18" customHeight="1">
       <c r="A198" s="1" t="inlineStr">
         <is>
-          <t>kick-user.messages.cannot-kick-self</t>
+          <t>forgot-password.messages.invalid-email-format</t>
         </is>
       </c>
       <c r="B198" s="2" t="inlineStr">
         <is>
-          <t>You cannot kick yourself</t>
+          <t>Invalid email format</t>
         </is>
       </c>
       <c r="C198" s="2" t="inlineStr">
         <is>
-          <t>Bạn không thể kick chính mình</t>
+          <t>Định dạng email không hợp lệ</t>
         </is>
       </c>
     </row>
     <row r="199" ht="18" customHeight="1">
       <c r="A199" s="1" t="inlineStr">
         <is>
-          <t>kick-user.messages.forbidden</t>
+          <t>forgot-password.messages.missing-email</t>
         </is>
       </c>
       <c r="B199" s="2" t="inlineStr">
         <is>
-          <t>Only the host can kick users</t>
+          <t>Email is required</t>
         </is>
       </c>
       <c r="C199" s="2" t="inlineStr">
         <is>
-          <t>Chỉ chủ phòng mới có thể kick người dùng</t>
+          <t>Email là bắt buộc</t>
         </is>
       </c>
     </row>
     <row r="200" ht="18" customHeight="1">
       <c r="A200" s="1" t="inlineStr">
         <is>
-          <t>kick-user.messages.internal-server-error</t>
+          <t>forgot-password.messages.success</t>
         </is>
       </c>
       <c r="B200" s="2" t="inlineStr">
         <is>
-          <t>Internal server error</t>
+          <t>Forgot password email sent</t>
         </is>
       </c>
       <c r="C200" s="2" t="inlineStr">
         <is>
-          <t>Lỗi máy chủ nội bộ</t>
+          <t>Email đặt lại mật khẩu đã được gửi</t>
         </is>
       </c>
     </row>
     <row r="201" ht="18" customHeight="1">
       <c r="A201" s="1" t="inlineStr">
         <is>
-          <t>kick-user.messages.invalid-room-id</t>
+          <t>join-room.messages.internal-server-error</t>
         </is>
       </c>
       <c r="B201" s="2" t="inlineStr">
         <is>
-          <t>Field 'id' is required and must be a positive integer</t>
+          <t>Internal server error</t>
         </is>
       </c>
       <c r="C201" s="2" t="inlineStr">
         <is>
-          <t>Trường 'id' là bắt buộc và phải là số nguyên dương</t>
+          <t>Lỗi máy chủ nội bộ</t>
         </is>
       </c>
     </row>
     <row r="202" ht="18" customHeight="1">
       <c r="A202" s="1" t="inlineStr">
         <is>
-          <t>kick-user.messages.invalid-user-id</t>
+          <t>join-room.messages.invalid-team</t>
         </is>
       </c>
       <c r="B202" s="2" t="inlineStr">
         <is>
-          <t>Field 'userId' is required and must be a positive integer</t>
+          <t>Field 'team' must be 'red', 'black', null, or undefined</t>
         </is>
       </c>
       <c r="C202" s="2" t="inlineStr">
         <is>
-          <t>Trường 'userId' là bắt buộc và phải là số nguyên dương</t>
+          <t>Trường 'team' phải là 'red', 'black', null hoặc không truyền</t>
         </is>
       </c>
     </row>
     <row r="203" ht="18" customHeight="1">
       <c r="A203" s="1" t="inlineStr">
         <is>
-          <t>kick-user.messages.room-not-found</t>
+          <t>join-room.messages.invalid-room-id</t>
         </is>
       </c>
       <c r="B203" s="2" t="inlineStr">
         <is>
-          <t>Room not found</t>
+          <t>Field 'id' is required and must be a positive integer</t>
         </is>
       </c>
       <c r="C203" s="2" t="inlineStr">
         <is>
-          <t>Không tìm thấy phòng</t>
+          <t>Trường 'id' là bắt buộc và phải là số nguyên dương</t>
         </is>
       </c>
     </row>
     <row r="204" ht="18" customHeight="1">
       <c r="A204" s="1" t="inlineStr">
         <is>
-          <t>kick-user.messages.room-not-waiting</t>
+          <t>join-room.messages.room-not-found</t>
         </is>
       </c>
       <c r="B204" s="2" t="inlineStr">
         <is>
-          <t>You can only kick users while the room is waiting</t>
+          <t>Room not found</t>
         </is>
       </c>
       <c r="C204" s="2" t="inlineStr">
         <is>
-          <t>Chỉ có thể kick người dùng khi phòng đang ở trạng thái chờ</t>
+          <t>Không tìm thấy phòng</t>
         </is>
       </c>
     </row>
     <row r="205" ht="18" customHeight="1">
       <c r="A205" s="1" t="inlineStr">
         <is>
-          <t>kick-user.messages.success</t>
+          <t>join-room.messages.success</t>
         </is>
       </c>
       <c r="B205" s="2" t="inlineStr">
         <is>
-          <t>User has been kicked</t>
+          <t>Successfully joined the room</t>
         </is>
       </c>
       <c r="C205" s="2" t="inlineStr">
         <is>
-          <t>Người dùng đã bị kick</t>
+          <t>Tham gia phòng thành công</t>
         </is>
       </c>
     </row>
     <row r="206" ht="18" customHeight="1">
       <c r="A206" s="1" t="inlineStr">
         <is>
-          <t>kick-user.messages.user-not-in-room</t>
+          <t>join-room.messages.team-seat-occupied</t>
         </is>
       </c>
       <c r="B206" s="2" t="inlineStr">
         <is>
-          <t>User is not in this room</t>
+          <t>Selected team seat is already occupied</t>
         </is>
       </c>
       <c r="C206" s="2" t="inlineStr">
         <is>
-          <t>Người dùng không trong phòng này</t>
+          <t>Vị trí đội đã chọn đã có người chơi</t>
         </is>
       </c>
     </row>
     <row r="207" ht="18" customHeight="1">
       <c r="A207" s="1" t="inlineStr">
         <is>
-          <t>kick-user.messages.you-were-kicked</t>
+          <t>kick-user.messages.cannot-kick-self</t>
         </is>
       </c>
       <c r="B207" s="2" t="inlineStr">
         <is>
-          <t>You have been removed from the room by the host</t>
+          <t>You cannot kick yourself</t>
         </is>
       </c>
       <c r="C207" s="2" t="inlineStr">
         <is>
-          <t>Bạn đã bị chủ phòng đưa ra khỏi phòng</t>
+          <t>Bạn không thể kick chính mình</t>
         </is>
       </c>
     </row>
     <row r="208" ht="18" customHeight="1">
       <c r="A208" s="1" t="inlineStr">
         <is>
-          <t>leave-room.messages.internal-server-error</t>
+          <t>kick-user.messages.forbidden</t>
         </is>
       </c>
       <c r="B208" s="2" t="inlineStr">
         <is>
-          <t>Internal server error</t>
+          <t>Only the host can kick users</t>
         </is>
       </c>
       <c r="C208" s="2" t="inlineStr">
         <is>
-          <t>Lỗi máy chủ nội bộ</t>
+          <t>Chỉ chủ phòng mới có thể kick người dùng</t>
         </is>
       </c>
     </row>
     <row r="209" ht="18" customHeight="1">
       <c r="A209" s="1" t="inlineStr">
         <is>
-          <t>leave-room.messages.invalid-room-id</t>
+          <t>kick-user.messages.internal-server-error</t>
         </is>
       </c>
       <c r="B209" s="2" t="inlineStr">
         <is>
-          <t>Field 'id' is required and must be a positive integer</t>
+          <t>Internal server error</t>
         </is>
       </c>
       <c r="C209" s="2" t="inlineStr">
         <is>
-          <t>Trường 'id' là bắt buộc và phải là số nguyên dương</t>
+          <t>Lỗi máy chủ nội bộ</t>
         </is>
       </c>
     </row>
     <row r="210" ht="18" customHeight="1">
       <c r="A210" s="1" t="inlineStr">
         <is>
-          <t>leave-room.messages.player-not-in-room</t>
+          <t>kick-user.messages.invalid-room-id</t>
         </is>
       </c>
       <c r="B210" s="2" t="inlineStr">
         <is>
-          <t>Player is not in this room</t>
+          <t>Field 'id' is required and must be a positive integer</t>
         </is>
       </c>
       <c r="C210" s="2" t="inlineStr">
         <is>
-          <t>Người chơi không trong phòng này</t>
+          <t>Trường 'id' là bắt buộc và phải là số nguyên dương</t>
         </is>
       </c>
     </row>
     <row r="211" ht="36" customHeight="1">
       <c r="A211" s="1" t="inlineStr">
         <is>
-          <t>leave-room.messages.success</t>
+          <t>kick-user.messages.invalid-user-id</t>
         </is>
       </c>
       <c r="B211" s="2" t="inlineStr">
         <is>
-          <t>Leave room successfully</t>
+          <t>Field 'userId' is required and must be a positive integer</t>
         </is>
       </c>
       <c r="C211" s="2" t="inlineStr">
         <is>
-          <t>Rời phòng thành công</t>
+          <t>Trường 'userId' là bắt buộc và phải là số nguyên dương</t>
         </is>
       </c>
     </row>
     <row r="212" ht="18" customHeight="1">
       <c r="A212" s="1" t="inlineStr">
         <is>
-          <t>load-room.messages.internal-server-error</t>
+          <t>kick-user.messages.room-not-found</t>
         </is>
       </c>
       <c r="B212" s="2" t="inlineStr">
         <is>
-          <t>Internal server error</t>
+          <t>Room not found</t>
         </is>
       </c>
       <c r="C212" s="2" t="inlineStr">
         <is>
-          <t>Lỗi máy chủ nội bộ</t>
+          <t>Không tìm thấy phòng</t>
         </is>
       </c>
     </row>
     <row r="213" ht="18" customHeight="1">
       <c r="A213" s="1" t="inlineStr">
         <is>
-          <t>load-room.messages.invalid-room-id</t>
+          <t>kick-user.messages.room-not-waiting</t>
         </is>
       </c>
       <c r="B213" s="2" t="inlineStr">
         <is>
-          <t>Room ID must be a positive integer</t>
+          <t>You can only kick users while the room is waiting</t>
         </is>
       </c>
       <c r="C213" s="2" t="inlineStr">
         <is>
-          <t>ID phòng phải là số nguyên dương</t>
+          <t>Chỉ có thể kick người dùng khi phòng đang ở trạng thái chờ</t>
         </is>
       </c>
     </row>
     <row r="214" ht="18" customHeight="1">
       <c r="A214" s="1" t="inlineStr">
         <is>
-          <t>load-room.messages.room-not-found</t>
+          <t>kick-user.messages.success</t>
         </is>
       </c>
       <c r="B214" s="2" t="inlineStr">
         <is>
-          <t>Room not found</t>
+          <t>User has been kicked</t>
         </is>
       </c>
       <c r="C214" s="2" t="inlineStr">
         <is>
-          <t>Không tìm thấy phòng</t>
+          <t>Người dùng đã bị kick</t>
         </is>
       </c>
     </row>
     <row r="215" ht="18" customHeight="1">
       <c r="A215" s="1" t="inlineStr">
         <is>
-          <t>load-room.messages.success</t>
+          <t>kick-user.messages.user-not-in-room</t>
         </is>
       </c>
       <c r="B215" s="2" t="inlineStr">
         <is>
-          <t>Load room successfully</t>
+          <t>User is not in this room</t>
         </is>
       </c>
       <c r="C215" s="2" t="inlineStr">
         <is>
-          <t>Tải phòng thành công</t>
+          <t>Người dùng không trong phòng này</t>
         </is>
       </c>
     </row>
     <row r="216" ht="18" customHeight="1">
       <c r="A216" s="1" t="inlineStr">
         <is>
-          <t>google-login.messages.email-not-verified</t>
+          <t>kick-user.messages.you-were-kicked</t>
         </is>
       </c>
       <c r="B216" s="2" t="inlineStr">
         <is>
-          <t>Your Google email is not verified</t>
+          <t>You have been removed from the room by the host</t>
         </is>
       </c>
       <c r="C216" s="2" t="inlineStr">
         <is>
-          <t>Email Google của bạn chưa được xác minh</t>
+          <t>Bạn đã bị chủ phòng đưa ra khỏi phòng</t>
         </is>
       </c>
     </row>
     <row r="217" ht="18" customHeight="1">
       <c r="A217" s="1" t="inlineStr">
         <is>
-          <t>google-login.messages.failed</t>
+          <t>leave-room.messages.internal-server-error</t>
         </is>
       </c>
       <c r="B217" s="2" t="inlineStr">
         <is>
-          <t>Login failed</t>
+          <t>Internal server error</t>
         </is>
       </c>
       <c r="C217" s="2" t="inlineStr">
         <is>
-          <t>Đăng nhập không thành công</t>
+          <t>Lỗi máy chủ nội bộ</t>
         </is>
       </c>
     </row>
     <row r="218" ht="18" customHeight="1">
       <c r="A218" s="1" t="inlineStr">
         <is>
-          <t>google-login.messages.internal-server-error</t>
+          <t>leave-room.messages.invalid-room-id</t>
         </is>
       </c>
       <c r="B218" s="2" t="inlineStr">
         <is>
-          <t>Internal server error</t>
+          <t>Field 'id' is required and must be a positive integer</t>
         </is>
       </c>
       <c r="C218" s="2" t="inlineStr">
         <is>
-          <t>Lỗi máy chủ nội bộ</t>
+          <t>Trường 'id' là bắt buộc và phải là số nguyên dương</t>
         </is>
       </c>
     </row>
     <row r="219" ht="18" customHeight="1">
       <c r="A219" s="1" t="inlineStr">
         <is>
-          <t>google-login.messages.invalid-token</t>
+          <t>leave-room.messages.player-not-in-room</t>
         </is>
       </c>
       <c r="B219" s="2" t="inlineStr">
         <is>
-          <t>Invalid Google credential</t>
+          <t>Player is not in this room</t>
         </is>
       </c>
       <c r="C219" s="2" t="inlineStr">
         <is>
-          <t>Thông tin đăng nhập Google không hợp lệ</t>
+          <t>Người chơi không trong phòng này</t>
         </is>
       </c>
     </row>
     <row r="220" ht="18" customHeight="1">
       <c r="A220" s="1" t="inlineStr">
         <is>
-          <t>google-login.messages.missing-credential</t>
+          <t>leave-room.messages.success</t>
         </is>
       </c>
       <c r="B220" s="2" t="inlineStr">
         <is>
-          <t>Google credential is required</t>
+          <t>Leave room successfully</t>
         </is>
       </c>
       <c r="C220" s="2" t="inlineStr">
         <is>
-          <t>Thiếu thông tin đăng nhập Google</t>
+          <t>Rời phòng thành công</t>
         </is>
       </c>
     </row>
     <row r="221" ht="18" customHeight="1">
       <c r="A221" s="1" t="inlineStr">
         <is>
-          <t>facebook-login.messages.missing-token</t>
+          <t>load-room.messages.internal-server-error</t>
         </is>
       </c>
       <c r="B221" s="2" t="inlineStr">
         <is>
-          <t>Facebook token is required</t>
+          <t>Internal server error</t>
         </is>
       </c>
       <c r="C221" s="2" t="inlineStr">
         <is>
-          <t>Thiếu thông tin đăng nhập Facebook</t>
+          <t>Lỗi máy chủ nội bộ</t>
         </is>
       </c>
     </row>
     <row r="222" ht="18" customHeight="1">
       <c r="A222" s="1" t="inlineStr">
         <is>
-          <t>facebook-login.messages.invalid-token</t>
+          <t>load-room.messages.invalid-room-id</t>
         </is>
       </c>
       <c r="B222" s="2" t="inlineStr">
         <is>
-          <t>Invalid Facebook token</t>
+          <t>Room ID must be a positive integer</t>
         </is>
       </c>
       <c r="C222" s="2" t="inlineStr">
         <is>
-          <t>Thông tin đăng nhập Facebook không hợp lệ</t>
+          <t>ID phòng phải là số nguyên dương</t>
         </is>
       </c>
     </row>
     <row r="223" ht="18" customHeight="1">
       <c r="A223" s="1" t="inlineStr">
         <is>
-          <t>facebook-login.messages.not-linked</t>
+          <t>load-room.messages.room-not-found</t>
         </is>
       </c>
       <c r="B223" s="2" t="inlineStr">
         <is>
-          <t>This Facebook account is not linked. Log in another way and link it in Settings</t>
+          <t>Room not found</t>
         </is>
       </c>
       <c r="C223" s="2" t="inlineStr">
         <is>
-          <t>Tài khoản Facebook này chưa được liên kết. Hãy đăng nhập cách khác rồi liên kết trong Cài đặt</t>
+          <t>Không tìm thấy phòng</t>
         </is>
       </c>
     </row>
     <row r="224" ht="18" customHeight="1">
       <c r="A224" s="1" t="inlineStr">
         <is>
-          <t>facebook-login.messages.internal-server-error</t>
+          <t>load-room.messages.success</t>
         </is>
       </c>
       <c r="B224" s="2" t="inlineStr">
         <is>
-          <t>Internal server error</t>
+          <t>Load room successfully</t>
         </is>
       </c>
       <c r="C224" s="2" t="inlineStr">
         <is>
-          <t>Lỗi máy chủ nội bộ</t>
+          <t>Tải phòng thành công</t>
         </is>
       </c>
     </row>
     <row r="225" ht="18" customHeight="1">
       <c r="A225" s="1" t="inlineStr">
         <is>
-          <t>facebook-link.messages.missing-token</t>
+          <t>google-login.messages.email-not-verified</t>
         </is>
       </c>
       <c r="B225" s="2" t="inlineStr">
         <is>
-          <t>Facebook token is required</t>
+          <t>Your Google email is not verified</t>
         </is>
       </c>
       <c r="C225" s="2" t="inlineStr">
         <is>
-          <t>Thiếu thông tin đăng nhập Facebook</t>
+          <t>Email Google của bạn chưa được xác minh</t>
         </is>
       </c>
     </row>
     <row r="226" ht="18" customHeight="1">
       <c r="A226" s="1" t="inlineStr">
         <is>
-          <t>facebook-link.messages.invalid-token</t>
+          <t>google-login.messages.failed</t>
         </is>
       </c>
       <c r="B226" s="2" t="inlineStr">
         <is>
-          <t>Invalid Facebook token</t>
+          <t>Login failed</t>
         </is>
       </c>
       <c r="C226" s="2" t="inlineStr">
         <is>
-          <t>Thông tin đăng nhập Facebook không hợp lệ</t>
+          <t>Đăng nhập không thành công</t>
         </is>
       </c>
     </row>
     <row r="227" ht="18" customHeight="1">
       <c r="A227" s="1" t="inlineStr">
         <is>
-          <t>facebook-link.messages.linked</t>
+          <t>google-login.messages.internal-server-error</t>
         </is>
       </c>
       <c r="B227" s="2" t="inlineStr">
         <is>
-          <t>Facebook linked successfully</t>
+          <t>Internal server error</t>
         </is>
       </c>
       <c r="C227" s="2" t="inlineStr">
         <is>
-          <t>Đã liên kết Facebook</t>
+          <t>Lỗi máy chủ nội bộ</t>
         </is>
       </c>
     </row>
     <row r="228" ht="18" customHeight="1">
       <c r="A228" s="1" t="inlineStr">
         <is>
-          <t>facebook-link.messages.already-linked</t>
+          <t>google-login.messages.invalid-token</t>
         </is>
       </c>
       <c r="B228" s="2" t="inlineStr">
         <is>
-          <t>This Facebook account is already linked to your account</t>
+          <t>Invalid Google credential</t>
         </is>
       </c>
       <c r="C228" s="2" t="inlineStr">
         <is>
-          <t>Tài khoản Facebook này đã được liên kết với bạn</t>
+          <t>Thông tin đăng nhập Google không hợp lệ</t>
         </is>
       </c>
     </row>
     <row r="229" ht="18" customHeight="1">
       <c r="A229" s="1" t="inlineStr">
         <is>
-          <t>facebook-link.messages.linked-to-other</t>
+          <t>google-login.messages.missing-credential</t>
         </is>
       </c>
       <c r="B229" s="2" t="inlineStr">
         <is>
-          <t>This Facebook account is already linked to another account</t>
+          <t>Google credential is required</t>
         </is>
       </c>
       <c r="C229" s="2" t="inlineStr">
         <is>
-          <t>Tài khoản Facebook này đã được liên kết với tài khoản khác</t>
+          <t>Thiếu thông tin đăng nhập Google</t>
         </is>
       </c>
     </row>
     <row r="230" ht="18" customHeight="1">
       <c r="A230" s="1" t="inlineStr">
         <is>
-          <t>facebook-link.messages.already-has-facebook</t>
+          <t>facebook-login.messages.missing-token</t>
         </is>
       </c>
       <c r="B230" s="2" t="inlineStr">
         <is>
-          <t>You already linked a different Facebook account</t>
+          <t>Facebook token is required</t>
         </is>
       </c>
       <c r="C230" s="2" t="inlineStr">
         <is>
-          <t>Bạn đã liên kết một tài khoản Facebook khác</t>
+          <t>Thiếu thông tin đăng nhập Facebook</t>
         </is>
       </c>
     </row>
     <row r="231" ht="18" customHeight="1">
       <c r="A231" s="1" t="inlineStr">
         <is>
-          <t>facebook-link.messages.unlinked</t>
+          <t>facebook-login.messages.invalid-token</t>
         </is>
       </c>
       <c r="B231" s="2" t="inlineStr">
         <is>
-          <t>Facebook unlinked</t>
+          <t>Invalid Facebook token</t>
         </is>
       </c>
       <c r="C231" s="2" t="inlineStr">
         <is>
-          <t>Đã huỷ liên kết Facebook</t>
+          <t>Thông tin đăng nhập Facebook không hợp lệ</t>
         </is>
       </c>
     </row>
     <row r="232" ht="18" customHeight="1">
       <c r="A232" s="1" t="inlineStr">
         <is>
-          <t>facebook-link.messages.internal-server-error</t>
+          <t>facebook-login.messages.not-linked</t>
         </is>
       </c>
       <c r="B232" s="2" t="inlineStr">
         <is>
-          <t>Internal server error</t>
+          <t>This Facebook account is not linked. Log in another way and link it in Settings</t>
         </is>
       </c>
       <c r="C232" s="2" t="inlineStr">
         <is>
-          <t>Lỗi máy chủ nội bộ</t>
+          <t>Tài khoản Facebook này chưa được liên kết. Hãy đăng nhập cách khác rồi liên kết trong Cài đặt</t>
         </is>
       </c>
     </row>
     <row r="233" ht="18" customHeight="1">
       <c r="A233" s="1" t="inlineStr">
         <is>
-          <t>logout.messages.already-inactive</t>
+          <t>facebook-login.messages.internal-server-error</t>
         </is>
       </c>
       <c r="B233" s="2" t="inlineStr">
         <is>
-          <t>Session already inactive</t>
+          <t>Internal server error</t>
         </is>
       </c>
       <c r="C233" s="2" t="inlineStr">
         <is>
-          <t>Phiên đã ngưng hoạt động</t>
+          <t>Lỗi máy chủ nội bộ</t>
         </is>
       </c>
     </row>
     <row r="234" ht="18" customHeight="1">
       <c r="A234" s="1" t="inlineStr">
         <is>
-          <t>logout.messages.internal-server-error</t>
+          <t>facebook-link.messages.missing-token</t>
         </is>
       </c>
       <c r="B234" s="2" t="inlineStr">
         <is>
-          <t>Internal server error</t>
+          <t>Facebook token is required</t>
         </is>
       </c>
       <c r="C234" s="2" t="inlineStr">
         <is>
-          <t>Lỗi máy chủ nội bộ</t>
+          <t>Thiếu thông tin đăng nhập Facebook</t>
         </is>
       </c>
     </row>
     <row r="235" ht="18" customHeight="1">
       <c r="A235" s="1" t="inlineStr">
         <is>
-          <t>logout.messages.success</t>
+          <t>facebook-link.messages.invalid-token</t>
         </is>
       </c>
       <c r="B235" s="2" t="inlineStr">
         <is>
-          <t>Logout successful</t>
+          <t>Invalid Facebook token</t>
         </is>
       </c>
       <c r="C235" s="2" t="inlineStr">
         <is>
-          <t>Đăng xuất thành công</t>
+          <t>Thông tin đăng nhập Facebook không hợp lệ</t>
         </is>
       </c>
     </row>
     <row r="236" ht="18" customHeight="1">
       <c r="A236" s="1" t="inlineStr">
         <is>
-          <t>refresh-token.messages.missing-refresh-token</t>
+          <t>facebook-link.messages.linked</t>
         </is>
       </c>
       <c r="B236" s="2" t="inlineStr">
         <is>
-          <t>Missing refresh token cookie</t>
+          <t>Facebook linked successfully</t>
         </is>
       </c>
       <c r="C236" s="2" t="inlineStr">
         <is>
-          <t>Thiếu cookie token làm mới</t>
+          <t>Đã liên kết Facebook</t>
         </is>
       </c>
     </row>
     <row r="237" ht="18" customHeight="1">
       <c r="A237" s="1" t="inlineStr">
         <is>
-          <t>refresh-token.messages.mismatch-or-expired</t>
+          <t>facebook-link.messages.already-linked</t>
         </is>
       </c>
       <c r="B237" s="2" t="inlineStr">
         <is>
-          <t>Refresh token mismatch or expired</t>
+          <t>This Facebook account is already linked to your account</t>
         </is>
       </c>
       <c r="C237" s="2" t="inlineStr">
         <is>
-          <t>Thiếu refresh token hoặc đã hết hạn</t>
+          <t>Tài khoản Facebook này đã được liên kết với bạn</t>
         </is>
       </c>
     </row>
     <row r="238" ht="18" customHeight="1">
       <c r="A238" s="1" t="inlineStr">
         <is>
-          <t>refresh-token.messages.success</t>
+          <t>facebook-link.messages.linked-to-other</t>
         </is>
       </c>
       <c r="B238" s="2" t="inlineStr">
         <is>
-          <t>Token refreshed</t>
+          <t>This Facebook account is already linked to another account</t>
         </is>
       </c>
       <c r="C238" s="2" t="inlineStr">
         <is>
-          <t>Token đã làm mới</t>
+          <t>Tài khoản Facebook này đã được liên kết với tài khoản khác</t>
         </is>
       </c>
     </row>
     <row r="239" ht="18" customHeight="1">
       <c r="A239" s="1" t="inlineStr">
         <is>
-          <t>register.messages.email-exists</t>
+          <t>facebook-link.messages.already-has-facebook</t>
         </is>
       </c>
       <c r="B239" s="2" t="inlineStr">
         <is>
-          <t>Email already exists</t>
+          <t>You already linked a different Facebook account</t>
         </is>
       </c>
       <c r="C239" s="2" t="inlineStr">
         <is>
-          <t>Email đã tồn tại</t>
+          <t>Bạn đã liên kết một tài khoản Facebook khác</t>
         </is>
       </c>
     </row>
     <row r="240" ht="18" customHeight="1">
       <c r="A240" s="1" t="inlineStr">
         <is>
-          <t>register.messages.internal-server-error</t>
+          <t>facebook-link.messages.unlinked</t>
         </is>
       </c>
       <c r="B240" s="2" t="inlineStr">
         <is>
-          <t>Internal server error</t>
+          <t>Facebook unlinked</t>
         </is>
       </c>
       <c r="C240" s="2" t="inlineStr">
         <is>
-          <t>Lỗi máy chủ nội bộ</t>
+          <t>Đã huỷ liên kết Facebook</t>
         </is>
       </c>
     </row>
     <row r="241" ht="18" customHeight="1">
       <c r="A241" s="1" t="inlineStr">
         <is>
-          <t>register.messages.missing-fields</t>
+          <t>facebook-link.messages.internal-server-error</t>
         </is>
       </c>
       <c r="B241" s="2" t="inlineStr">
         <is>
-          <t>Username, password, gender, displayName and email are required</t>
+          <t>Internal server error</t>
         </is>
       </c>
       <c r="C241" s="2" t="inlineStr">
         <is>
-          <t>Tên người dùng, mật khẩu, giới tính, tên hiển thị và email là bắt buộc</t>
+          <t>Lỗi máy chủ nội bộ</t>
         </is>
       </c>
     </row>
     <row r="242" ht="18" customHeight="1">
       <c r="A242" s="1" t="inlineStr">
         <is>
-          <t>register.messages.success</t>
+          <t>logout.messages.already-inactive</t>
         </is>
       </c>
       <c r="B242" s="2" t="inlineStr">
         <is>
-          <t>User created successfully</t>
+          <t>Session already inactive</t>
         </is>
       </c>
       <c r="C242" s="2" t="inlineStr">
         <is>
-          <t>Người dùng được tạo thành công</t>
+          <t>Phiên đã ngưng hoạt động</t>
         </is>
       </c>
     </row>
     <row r="243" ht="18" customHeight="1">
       <c r="A243" s="1" t="inlineStr">
         <is>
-          <t>register.messages.username-exists</t>
+          <t>logout.messages.internal-server-error</t>
         </is>
       </c>
       <c r="B243" s="2" t="inlineStr">
         <is>
-          <t>Username already exists</t>
+          <t>Internal server error</t>
         </is>
       </c>
       <c r="C243" s="2" t="inlineStr">
         <is>
-          <t>Tên người dùng đã tồn tại</t>
+          <t>Lỗi máy chủ nội bộ</t>
         </is>
       </c>
     </row>
     <row r="244" ht="18" customHeight="1">
       <c r="A244" s="1" t="inlineStr">
         <is>
-          <t>reset-password.messages.internal-server-error</t>
+          <t>logout.messages.success</t>
         </is>
       </c>
       <c r="B244" s="2" t="inlineStr">
         <is>
-          <t>Internal server error</t>
+          <t>Logout successful</t>
         </is>
       </c>
       <c r="C244" s="2" t="inlineStr">
         <is>
-          <t>Lỗi máy chủ nội bộ</t>
+          <t>Đăng xuất thành công</t>
         </is>
       </c>
     </row>
     <row r="245" ht="18" customHeight="1">
       <c r="A245" s="1" t="inlineStr">
         <is>
-          <t>reset-password.messages.invalid-or-expired-token</t>
+          <t>refresh-token.messages.missing-refresh-token</t>
         </is>
       </c>
       <c r="B245" s="2" t="inlineStr">
         <is>
-          <t>Invalid or expired reset password token</t>
+          <t>Missing refresh token cookie</t>
         </is>
       </c>
       <c r="C245" s="2" t="inlineStr">
         <is>
-          <t>Token đặt lại mật khẩu không hợp lệ hoặc đã hết hạn</t>
+          <t>Thiếu cookie token làm mới</t>
         </is>
       </c>
     </row>
     <row r="246" ht="18" customHeight="1">
       <c r="A246" s="1" t="inlineStr">
         <is>
-          <t>reset-password.messages.invalid-user-id</t>
+          <t>refresh-token.messages.mismatch-or-expired</t>
         </is>
       </c>
       <c r="B246" s="2" t="inlineStr">
         <is>
-          <t>Invalid user id</t>
+          <t>Refresh token mismatch or expired</t>
         </is>
       </c>
       <c r="C246" s="2" t="inlineStr">
         <is>
-          <t>ID người dùng không hợp lệ</t>
+          <t>Thiếu refresh token hoặc đã hết hạn</t>
         </is>
       </c>
     </row>
     <row r="247" ht="18" customHeight="1">
       <c r="A247" s="1" t="inlineStr">
         <is>
-          <t>reset-password.messages.missing-id-or-token</t>
+          <t>refresh-token.messages.success</t>
         </is>
       </c>
       <c r="B247" s="2" t="inlineStr">
         <is>
-          <t>ID and token are required</t>
+          <t>Token refreshed</t>
         </is>
       </c>
       <c r="C247" s="2" t="inlineStr">
         <is>
-          <t>ID và token là bắt buộc</t>
+          <t>Token đã làm mới</t>
         </is>
       </c>
     </row>
     <row r="248" ht="18" customHeight="1">
       <c r="A248" s="1" t="inlineStr">
         <is>
-          <t>reset-password.messages.missing-userId-or-password</t>
+          <t>register.messages.email-exists</t>
         </is>
       </c>
       <c r="B248" s="2" t="inlineStr">
         <is>
-          <t>UserId and password are required</t>
+          <t>Email already exists</t>
         </is>
       </c>
       <c r="C248" s="2" t="inlineStr">
         <is>
-          <t>UserId và mật khẩu là bắt buộc</t>
+          <t>Email đã tồn tại</t>
         </is>
       </c>
     </row>
     <row r="249" ht="18" customHeight="1">
       <c r="A249" s="1" t="inlineStr">
         <is>
-          <t>reset-password.messages.token-valid</t>
+          <t>register.messages.internal-server-error</t>
         </is>
       </c>
       <c r="B249" s="2" t="inlineStr">
         <is>
-          <t>Reset password token is valid</t>
+          <t>Internal server error</t>
         </is>
       </c>
       <c r="C249" s="2" t="inlineStr">
         <is>
-          <t>Token đặt lại mật khẩu hợp lệ</t>
+          <t>Lỗi máy chủ nội bộ</t>
         </is>
       </c>
     </row>
     <row r="250" ht="18" customHeight="1">
       <c r="A250" s="1" t="inlineStr">
         <is>
-          <t>reset-password.messages.user-not-found</t>
+          <t>register.messages.missing-fields</t>
         </is>
       </c>
       <c r="B250" s="2" t="inlineStr">
         <is>
-          <t>User not found</t>
+          <t>Username, password, gender, displayName and email are required</t>
         </is>
       </c>
       <c r="C250" s="2" t="inlineStr">
         <is>
-          <t>Không tìm thấy người dùng</t>
+          <t>Tên người dùng, mật khẩu, giới tính, tên hiển thị và email là bắt buộc</t>
         </is>
       </c>
     </row>
     <row r="251" ht="18" customHeight="1">
       <c r="A251" s="1" t="inlineStr">
         <is>
-          <t>room.actions.start-room</t>
+          <t>register.messages.success</t>
         </is>
       </c>
       <c r="B251" s="2" t="inlineStr">
         <is>
-          <t>Start room</t>
+          <t>User created successfully</t>
         </is>
       </c>
       <c r="C251" s="2" t="inlineStr">
         <is>
-          <t>Bắt đầu chơi</t>
+          <t>Người dùng được tạo thành công</t>
         </is>
       </c>
     </row>
     <row r="252" ht="18" customHeight="1">
       <c r="A252" s="1" t="inlineStr">
         <is>
-          <t>room.actions.challenge</t>
+          <t>register.messages.username-exists</t>
         </is>
       </c>
       <c r="B252" s="2" t="inlineStr">
         <is>
-          <t>Challenge</t>
+          <t>Username already exists</t>
         </is>
       </c>
       <c r="C252" s="2" t="inlineStr">
         <is>
-          <t>Vào chơi</t>
+          <t>Tên người dùng đã tồn tại</t>
         </is>
       </c>
     </row>
     <row r="253" ht="18" customHeight="1">
       <c r="A253" s="1" t="inlineStr">
         <is>
-          <t>room.actions.leave-seat</t>
+          <t>reset-password.messages.internal-server-error</t>
         </is>
       </c>
       <c r="B253" s="2" t="inlineStr">
         <is>
-          <t>Leave seat</t>
+          <t>Internal server error</t>
         </is>
       </c>
       <c r="C253" s="2" t="inlineStr">
         <is>
-          <t>Ra xem</t>
+          <t>Lỗi máy chủ nội bộ</t>
         </is>
       </c>
     </row>
     <row r="254" ht="18" customHeight="1">
       <c r="A254" s="1" t="inlineStr">
         <is>
-          <t>room.actions.undo</t>
+          <t>reset-password.messages.invalid-or-expired-token</t>
         </is>
       </c>
       <c r="B254" s="2" t="inlineStr">
         <is>
-          <t>Undo</t>
+          <t>Invalid or expired reset password token</t>
         </is>
       </c>
       <c r="C254" s="2" t="inlineStr">
         <is>
-          <t>Hoán tác</t>
+          <t>Token đặt lại mật khẩu không hợp lệ hoặc đã hết hạn</t>
         </is>
       </c>
     </row>
     <row r="255" ht="18" customHeight="1">
       <c r="A255" s="1" t="inlineStr">
         <is>
-          <t>room.actions.surrender</t>
+          <t>reset-password.messages.invalid-user-id</t>
         </is>
       </c>
       <c r="B255" s="2" t="inlineStr">
         <is>
-          <t>Surrender</t>
+          <t>Invalid user id</t>
         </is>
       </c>
       <c r="C255" s="2" t="inlineStr">
         <is>
-          <t>Đầu hàng</t>
+          <t>ID người dùng không hợp lệ</t>
         </is>
       </c>
     </row>
     <row r="256" ht="18" customHeight="1">
       <c r="A256" s="1" t="inlineStr">
         <is>
-          <t>room.actions.draw</t>
+          <t>reset-password.messages.missing-id-or-token</t>
         </is>
       </c>
       <c r="B256" s="2" t="inlineStr">
         <is>
-          <t>Draw</t>
+          <t>ID and token are required</t>
         </is>
       </c>
       <c r="C256" s="2" t="inlineStr">
         <is>
-          <t>Hòa</t>
+          <t>ID và token là bắt buộc</t>
         </is>
       </c>
     </row>
     <row r="257" ht="18" customHeight="1">
       <c r="A257" s="1" t="inlineStr">
         <is>
-          <t>room.actions.back-home</t>
+          <t>reset-password.messages.missing-userId-or-password</t>
         </is>
       </c>
       <c r="B257" s="2" t="inlineStr">
         <is>
-          <t>Back to home</t>
+          <t>UserId and password are required</t>
         </is>
       </c>
       <c r="C257" s="2" t="inlineStr">
         <is>
-          <t>Thoát phòng</t>
+          <t>UserId và mật khẩu là bắt buộc</t>
         </is>
       </c>
     </row>
     <row r="258" ht="18" customHeight="1">
       <c r="A258" s="1" t="inlineStr">
         <is>
-          <t>room.actions.flip-board</t>
+          <t>reset-password.messages.token-valid</t>
         </is>
       </c>
       <c r="B258" s="2" t="inlineStr">
         <is>
-          <t>Flip board</t>
+          <t>Reset password token is valid</t>
         </is>
       </c>
       <c r="C258" s="2" t="inlineStr">
         <is>
-          <t>Đảo chiều bàn cờ</t>
+          <t>Token đặt lại mật khẩu hợp lệ</t>
         </is>
       </c>
     </row>
     <row r="259" ht="18" customHeight="1">
       <c r="A259" s="1" t="inlineStr">
         <is>
-          <t>room.actions.accept-draw</t>
+          <t>reset-password.messages.user-not-found</t>
         </is>
       </c>
       <c r="B259" s="2" t="inlineStr">
         <is>
-          <t>Accept</t>
+          <t>User not found</t>
         </is>
       </c>
       <c r="C259" s="2" t="inlineStr">
         <is>
-          <t>Chấp nhận</t>
+          <t>Không tìm thấy người dùng</t>
         </is>
       </c>
     </row>
     <row r="260" ht="36" customHeight="1">
       <c r="A260" s="1" t="inlineStr">
         <is>
-          <t>room.actions.reject-draw</t>
+          <t>room.actions.start-room</t>
         </is>
       </c>
       <c r="B260" s="2" t="inlineStr">
         <is>
-          <t>Reject</t>
+          <t>Start room</t>
         </is>
       </c>
       <c r="C260" s="2" t="inlineStr">
         <is>
-          <t>Từ chối</t>
+          <t>Bắt đầu chơi</t>
         </is>
       </c>
     </row>
     <row r="261" ht="36" customHeight="1">
       <c r="A261" s="1" t="inlineStr">
         <is>
-          <t>room.actions.send-pm</t>
+          <t>room.actions.challenge</t>
         </is>
       </c>
       <c r="B261" s="2" t="inlineStr">
         <is>
-          <t>Send PM</t>
+          <t>Challenge</t>
         </is>
       </c>
       <c r="C261" s="2" t="inlineStr">
         <is>
-          <t>Chat</t>
+          <t>Vào chơi</t>
         </is>
       </c>
     </row>
     <row r="262" ht="18" customHeight="1">
       <c r="A262" s="1" t="inlineStr">
         <is>
-          <t>room.actions.view-history</t>
+          <t>room.actions.leave-seat</t>
         </is>
       </c>
       <c r="B262" s="2" t="inlineStr">
         <is>
-          <t>History</t>
+          <t>Leave seat</t>
         </is>
       </c>
       <c r="C262" s="2" t="inlineStr">
         <is>
-          <t>Lịch sử</t>
+          <t>Ra xem</t>
         </is>
       </c>
     </row>
     <row r="263" ht="18" customHeight="1">
       <c r="A263" s="1" t="inlineStr">
         <is>
-          <t>room.actions.kick</t>
+          <t>room.actions.undo</t>
         </is>
       </c>
       <c r="B263" s="2" t="inlineStr">
         <is>
-          <t>Kick</t>
+          <t>Undo</t>
         </is>
       </c>
       <c r="C263" s="2" t="inlineStr">
         <is>
-          <t>Kick</t>
+          <t>Hoán tác</t>
         </is>
       </c>
     </row>
     <row r="264" ht="18" customHeight="1">
       <c r="A264" s="1" t="inlineStr">
         <is>
-          <t>room.actions.back-to-room</t>
+          <t>room.actions.surrender</t>
         </is>
       </c>
       <c r="B264" s="2" t="inlineStr">
         <is>
-          <t>Back to room</t>
+          <t>Surrender</t>
         </is>
       </c>
       <c r="C264" s="2" t="inlineStr">
         <is>
-          <t>Quay lại phòng chơi</t>
+          <t>Đầu hàng</t>
         </is>
       </c>
     </row>
     <row r="265" ht="17" customHeight="1">
       <c r="A265" s="1" t="inlineStr">
         <is>
-          <t>room.actions.chat</t>
+          <t>room.actions.draw</t>
         </is>
       </c>
       <c r="B265" s="1" t="inlineStr">
         <is>
-          <t>Room chat</t>
+          <t>Draw</t>
         </is>
       </c>
       <c r="C265" s="1" t="inlineStr">
         <is>
-          <t>Phòng chat</t>
+          <t>Hòa</t>
         </is>
       </c>
     </row>
     <row r="266" ht="18" customHeight="1">
       <c r="A266" s="2" t="inlineStr">
         <is>
-          <t>room.messages.draw-accepted</t>
+          <t>room.actions.back-home</t>
         </is>
       </c>
       <c r="B266" s="2" t="inlineStr">
         <is>
-          <t>Opponent accepted the draw</t>
+          <t>Back to home</t>
         </is>
       </c>
       <c r="C266" s="2" t="inlineStr">
         <is>
-          <t>Đối phương đã đồng ý hòa</t>
+          <t>Thoát phòng</t>
         </is>
       </c>
     </row>
     <row r="267" ht="18" customHeight="1">
       <c r="A267" s="2" t="inlineStr">
         <is>
-          <t>room.messages.draw-rejected</t>
+          <t>room.actions.flip-board</t>
         </is>
       </c>
       <c r="B267" s="2" t="inlineStr">
         <is>
-          <t>Opponent rejected the draw</t>
+          <t>Flip board</t>
         </is>
       </c>
       <c r="C267" s="2" t="inlineStr">
         <is>
-          <t>Đối phương từ chối hòa</t>
+          <t>Đảo chiều bàn cờ</t>
         </is>
       </c>
     </row>
     <row r="268" ht="18" customHeight="1">
       <c r="A268" s="2" t="inlineStr">
         <is>
-          <t>room.messages.opponent-surrendered</t>
+          <t>room.actions.accept-draw</t>
         </is>
       </c>
       <c r="B268" s="2" t="inlineStr">
         <is>
-          <t>Opponent surrendered! You won!</t>
+          <t>Accept</t>
         </is>
       </c>
       <c r="C268" s="2" t="inlineStr">
         <is>
-          <t>Đối phương đã đầu hàng! Bạn thắng!</t>
+          <t>Chấp nhận</t>
         </is>
       </c>
     </row>
     <row r="269" ht="18" customHeight="1">
       <c r="A269" s="2" t="inlineStr">
         <is>
-          <t>room.messages.confirm-leave</t>
+          <t>room.actions.reject-draw</t>
         </is>
       </c>
       <c r="B269" s="2" t="inlineStr">
         <is>
-          <t>Are you sure you want to leave room?</t>
+          <t>Reject</t>
         </is>
       </c>
       <c r="C269" s="2" t="inlineStr">
         <is>
-          <t>Bạn có chắc muốn rời bàn chơi?</t>
+          <t>Từ chối</t>
         </is>
       </c>
     </row>
     <row r="270" ht="18" customHeight="1">
       <c r="A270" s="2" t="inlineStr">
         <is>
-          <t>room.messages.confirm-surrender</t>
+          <t>room.actions.send-pm</t>
         </is>
       </c>
       <c r="B270" s="2" t="inlineStr">
         <is>
-          <t>Are you sure you want to surrender?</t>
+          <t>Send PM</t>
         </is>
       </c>
       <c r="C270" s="2" t="inlineStr">
         <is>
-          <t>Bạn có chắc chắn muốn đầu hàng không?</t>
+          <t>Chat</t>
         </is>
       </c>
     </row>
     <row r="271" ht="36" customHeight="1">
       <c r="A271" s="2" t="inlineStr">
         <is>
-          <t>room.messages.confirm-draw</t>
+          <t>room.actions.view-history</t>
         </is>
       </c>
       <c r="B271" s="2" t="inlineStr">
         <is>
-          <t>Are you sure you want to draw?</t>
+          <t>History</t>
         </is>
       </c>
       <c r="C271" s="2" t="inlineStr">
         <is>
-          <t>Bạn có chắc chắn muốn hòa không?</t>
+          <t>Lịch sử</t>
         </is>
       </c>
     </row>
     <row r="272" ht="36" customHeight="1">
       <c r="A272" s="2" t="inlineStr">
         <is>
-          <t>room.messages.confirm-accept-draw</t>
+          <t>room.actions.kick</t>
         </is>
       </c>
       <c r="B272" s="2" t="inlineStr">
         <is>
-          <t>Opponent has proposed a draw. Do you accept?</t>
+          <t>Kick</t>
         </is>
       </c>
       <c r="C272" s="2" t="inlineStr">
         <is>
-          <t>Đối phương đã chủ hòa, bạn có đồng ý không?</t>
+          <t>Kick</t>
         </is>
       </c>
     </row>
     <row r="273" ht="18" customHeight="1">
       <c r="A273" s="2" t="inlineStr">
         <is>
-          <t>room.messages.insufficient-amount</t>
+          <t>room.actions.back-to-room</t>
         </is>
       </c>
       <c r="B273" s="2" t="inlineStr">
         <is>
-          <t>You do not have enough balance to join this room</t>
+          <t>Back to room</t>
         </is>
       </c>
       <c r="C273" s="2" t="inlineStr">
         <is>
-          <t>Bạn không đủ tiền để tham gia bàn chơi này</t>
+          <t>Quay lại phòng chơi</t>
         </is>
       </c>
     </row>
     <row r="274" ht="18" customHeight="1">
       <c r="A274" s="1" t="inlineStr">
         <is>
-          <t>room.messages.will-leave-current-room</t>
+          <t>room.actions.chat</t>
         </is>
       </c>
       <c r="B274" s="2" t="inlineStr">
         <is>
-          <t>You are currently in another room. Joining this room will remove you from the current room</t>
+          <t>Room chat</t>
         </is>
       </c>
       <c r="C274" s="2" t="inlineStr">
         <is>
-          <t>Bạn đang ở trong một phòng khác. Tham gia phòng này sẽ loại bạn ra khỏi phòng hiện tại</t>
+          <t>Phòng chat</t>
         </is>
       </c>
     </row>
     <row r="275" ht="18" customHeight="1">
       <c r="A275" s="1" t="inlineStr">
         <is>
-          <t>room.messages.all-seats-occupied</t>
+          <t>room.messages.draw-accepted</t>
         </is>
       </c>
       <c r="B275" s="2" t="inlineStr">
         <is>
-          <t>All player seats are occupied</t>
+          <t>Opponent accepted the draw</t>
         </is>
       </c>
       <c r="C275" s="2" t="inlineStr">
         <is>
-          <t>Tất cả ghế chơi đã được chiếm</t>
+          <t>Đối phương đã đồng ý hòa</t>
         </is>
       </c>
     </row>
     <row r="276" ht="18" customHeight="1">
       <c r="A276" s="1" t="inlineStr">
         <is>
-          <t>room.messages.game-ended</t>
+          <t>room.messages.draw-rejected</t>
         </is>
       </c>
       <c r="B276" s="2" t="inlineStr">
         <is>
-          <t>Game ended</t>
+          <t>Opponent rejected the draw</t>
         </is>
       </c>
       <c r="C276" s="2" t="inlineStr">
         <is>
-          <t>Ván đấu đã kết thúc</t>
+          <t>Đối phương từ chối hòa</t>
         </is>
       </c>
     </row>
     <row r="277" ht="18" customHeight="1">
       <c r="A277" s="1" t="inlineStr">
         <is>
-          <t>room.messages.you-win</t>
+          <t>room.messages.opponent-surrendered</t>
         </is>
       </c>
       <c r="B277" s="2" t="inlineStr">
         <is>
-          <t>You win</t>
+          <t>Opponent surrendered! You won!</t>
         </is>
       </c>
       <c r="C277" s="2" t="inlineStr">
         <is>
-          <t>Bạn đã chiến thắng</t>
+          <t>Đối phương đã đầu hàng! Bạn thắng!</t>
         </is>
       </c>
     </row>
     <row r="278" ht="18" customHeight="1">
       <c r="A278" s="1" t="inlineStr">
         <is>
-          <t>room.messages.you-lose</t>
+          <t>room.messages.confirm-leave</t>
         </is>
       </c>
       <c r="B278" s="2" t="inlineStr">
         <is>
-          <t>You lose</t>
+          <t>Are you sure you want to leave room?</t>
         </is>
       </c>
       <c r="C278" s="2" t="inlineStr">
         <is>
-          <t>Bạn đã thua</t>
+          <t>Bạn có chắc muốn rời bàn chơi?</t>
         </is>
       </c>
     </row>
     <row r="279" ht="18" customHeight="1">
       <c r="A279" s="1" t="inlineStr">
         <is>
-          <t>room.messages.back-to-room</t>
+          <t>room.messages.confirm-surrender</t>
         </is>
       </c>
       <c r="B279" s="2" t="inlineStr">
         <is>
-          <t>Back to room</t>
+          <t>Are you sure you want to surrender?</t>
         </is>
       </c>
       <c r="C279" s="2" t="inlineStr">
         <is>
-          <t>Quay lại phòng</t>
+          <t>Bạn có chắc chắn muốn đầu hàng không?</t>
         </is>
       </c>
     </row>
     <row r="280" ht="18" customHeight="1">
       <c r="A280" s="1" t="inlineStr">
         <is>
-          <t>room.messages.auto-back-countdown</t>
+          <t>room.messages.confirm-draw</t>
         </is>
       </c>
       <c r="B280" s="2" t="inlineStr">
         <is>
-          <t>{0}. Press the back button to return to the room. You will be automatically returned in {1}s</t>
+          <t>Are you sure you want to draw?</t>
         </is>
       </c>
       <c r="C280" s="2" t="inlineStr">
         <is>
-          <t>{0}. Bấm nút quay lại để quay lại room. Bạn sẽ tự động quay lại trong {1}s</t>
+          <t>Bạn có chắc chắn muốn hòa không?</t>
         </is>
       </c>
     </row>
     <row r="281" ht="18" customHeight="1">
       <c r="A281" s="1" t="inlineStr">
         <is>
-          <t>room.notifications.joined</t>
+          <t>room.messages.confirm-accept-draw</t>
         </is>
       </c>
       <c r="B281" s="2" t="inlineStr">
         <is>
-          <t>{0} joined the room</t>
+          <t>Opponent has proposed a draw. Do you accept?</t>
         </is>
       </c>
       <c r="C281" s="2" t="inlineStr">
         <is>
-          <t>{0} đã vào phòng</t>
+          <t>Đối phương đã chủ hòa, bạn có đồng ý không?</t>
         </is>
       </c>
     </row>
     <row r="282" ht="18" customHeight="1">
       <c r="A282" s="1" t="inlineStr">
         <is>
-          <t>room.notifications.left</t>
+          <t>room.messages.insufficient-amount</t>
         </is>
       </c>
       <c r="B282" s="2" t="inlineStr">
         <is>
-          <t>{0} left the room</t>
+          <t>You do not have enough balance to join this room</t>
         </is>
       </c>
       <c r="C282" s="2" t="inlineStr">
         <is>
-          <t>{0} đã rời phòng</t>
+          <t>Bạn không đủ tiền để tham gia bàn chơi này</t>
         </is>
       </c>
     </row>
     <row r="283" ht="18" customHeight="1">
       <c r="A283" s="1" t="inlineStr">
         <is>
-          <t>room.settings.title</t>
+          <t>room.messages.will-leave-current-room</t>
         </is>
       </c>
       <c r="B283" s="2" t="inlineStr">
         <is>
-          <t>Room Settings</t>
+          <t>You are currently in another room. Joining this room will remove you from the current room</t>
         </is>
       </c>
       <c r="C283" s="2" t="inlineStr">
         <is>
-          <t>Cài đặt phòng</t>
+          <t>Bạn đang ở trong một phòng khác. Tham gia phòng này sẽ loại bạn ra khỏi phòng hiện tại</t>
         </is>
       </c>
     </row>
     <row r="284" ht="18" customHeight="1">
       <c r="A284" s="1" t="inlineStr">
         <is>
-          <t>room.settings.room-name</t>
+          <t>room.messages.all-seats-occupied</t>
         </is>
       </c>
       <c r="B284" s="2" t="inlineStr">
         <is>
-          <t>Room name</t>
+          <t>All player seats are occupied</t>
         </is>
       </c>
       <c r="C284" s="2" t="inlineStr">
         <is>
-          <t>Tên phòng</t>
+          <t>Tất cả ghế chơi đã được chiếm</t>
         </is>
       </c>
     </row>
     <row r="285" ht="18" customHeight="1">
       <c r="A285" s="1" t="inlineStr">
         <is>
-          <t>room.settings.players</t>
+          <t>room.messages.game-ended</t>
         </is>
       </c>
       <c r="B285" s="2" t="inlineStr">
         <is>
-          <t>Spectators</t>
+          <t>Game ended</t>
         </is>
       </c>
       <c r="C285" s="2" t="inlineStr">
         <is>
-          <t>Người xem</t>
+          <t>Ván đấu đã kết thúc</t>
         </is>
       </c>
     </row>
     <row r="286" ht="18" customHeight="1">
       <c r="A286" s="1" t="inlineStr">
         <is>
-          <t>room.settings.save</t>
+          <t>room.messages.you-win</t>
         </is>
       </c>
       <c r="B286" s="2" t="inlineStr">
         <is>
-          <t>Save</t>
+          <t>You win</t>
         </is>
       </c>
       <c r="C286" s="2" t="inlineStr">
         <is>
-          <t>Lưu</t>
+          <t>Bạn đã chiến thắng</t>
         </is>
       </c>
     </row>
     <row r="287" ht="18" customHeight="1">
       <c r="A287" s="1" t="inlineStr">
         <is>
-          <t>room-invite.messages.title</t>
+          <t>room.messages.you-lose</t>
         </is>
       </c>
       <c r="B287" s="2" t="inlineStr">
         <is>
-          <t>Room Invitation</t>
+          <t>You lose</t>
         </is>
       </c>
       <c r="C287" s="2" t="inlineStr">
         <is>
-          <t>Lời mời vào phòng</t>
+          <t>Bạn đã thua</t>
         </is>
       </c>
     </row>
     <row r="288" ht="18" customHeight="1">
       <c r="A288" s="1" t="inlineStr">
         <is>
-          <t>start-game.messages.success</t>
+          <t>room.messages.back-to-room</t>
         </is>
       </c>
       <c r="B288" s="2" t="inlineStr">
         <is>
-          <t>Game started successfully</t>
+          <t>Back to room</t>
         </is>
       </c>
       <c r="C288" s="2" t="inlineStr">
         <is>
-          <t>Bắt đầu trò chơi thành công</t>
+          <t>Quay lại phòng</t>
         </is>
       </c>
     </row>
     <row r="289" ht="18" customHeight="1">
       <c r="A289" s="1" t="inlineStr">
         <is>
-          <t>start-game.messages.internal-server-error</t>
+          <t>room.messages.auto-back-countdown</t>
         </is>
       </c>
       <c r="B289" s="2" t="inlineStr">
         <is>
-          <t>Internal server error while starting game</t>
+          <t>{0}. Press the back button to return to the room. You will be automatically returned in {1}s</t>
         </is>
       </c>
       <c r="C289" s="2" t="inlineStr">
         <is>
-          <t>Lỗi máy chủ nội bộ khi bắt đầu trò chơi</t>
+          <t>{0}. Bấm nút quay lại để quay lại room. Bạn sẽ tự động quay lại trong {1}s</t>
         </is>
       </c>
     </row>
     <row r="290" ht="18" customHeight="1">
       <c r="A290" s="1" t="inlineStr">
         <is>
-          <t>start-game.messages.invalid-room-id</t>
+          <t>room.notifications.joined</t>
         </is>
       </c>
       <c r="B290" s="2" t="inlineStr">
         <is>
-          <t>Field 'id' is required and must be a positive integer</t>
+          <t>{0} joined the room</t>
         </is>
       </c>
       <c r="C290" s="2" t="inlineStr">
         <is>
-          <t>Trường 'id' là bắt buộc và phải là số nguyên dương</t>
+          <t>{0} đã vào phòng</t>
         </is>
       </c>
     </row>
     <row r="291" ht="18" customHeight="1">
       <c r="A291" s="1" t="inlineStr">
         <is>
-          <t>start-game.messages.invalid-difficulty</t>
+          <t>room.notifications.left</t>
         </is>
       </c>
       <c r="B291" s="2" t="inlineStr">
         <is>
-          <t>Bot difficulty must be between 1 and 5</t>
+          <t>{0} left the room</t>
         </is>
       </c>
       <c r="C291" s="2" t="inlineStr">
         <is>
-          <t>Độ khó của bot phải từ 1 đến 5</t>
+          <t>{0} đã rời phòng</t>
         </is>
       </c>
     </row>
     <row r="292" ht="18" customHeight="1">
       <c r="A292" s="1" t="inlineStr">
         <is>
-          <t>start-game.messages.room-not-found</t>
+          <t>room.settings.title</t>
         </is>
       </c>
       <c r="B292" s="2" t="inlineStr">
         <is>
-          <t>Room not found</t>
+          <t>Room Settings</t>
         </is>
       </c>
       <c r="C292" s="2" t="inlineStr">
         <is>
-          <t>Không tìm thấy phòng</t>
+          <t>Cài đặt phòng</t>
         </is>
       </c>
     </row>
     <row r="293" ht="18" customHeight="1">
       <c r="A293" s="1" t="inlineStr">
         <is>
-          <t>start-game.messages.forbidden</t>
+          <t>room.settings.room-name</t>
         </is>
       </c>
       <c r="B293" s="2" t="inlineStr">
         <is>
-          <t>Only the room host can start the game</t>
+          <t>Room name</t>
         </is>
       </c>
       <c r="C293" s="2" t="inlineStr">
         <is>
-          <t>Chỉ chủ phòng mới có thể bắt đầu trò chơi</t>
+          <t>Tên phòng</t>
         </is>
       </c>
     </row>
     <row r="294" ht="18" customHeight="1">
       <c r="A294" s="1" t="inlineStr">
         <is>
-          <t>start-game.messages.insufficient-amount</t>
+          <t>room.settings.players</t>
         </is>
       </c>
       <c r="B294" s="2" t="inlineStr">
         <is>
-          <t>You do not have enough balance to start a game with this bet</t>
+          <t>Spectators</t>
         </is>
       </c>
       <c r="C294" s="2" t="inlineStr">
         <is>
-          <t>Bạn không còn đủ amount để start room</t>
+          <t>Người xem</t>
         </is>
       </c>
     </row>
     <row r="295" ht="18" customHeight="1">
       <c r="A295" s="1" t="inlineStr">
         <is>
-          <t>start-game.messages.requester-must-pick-team</t>
+          <t>room.settings.save</t>
         </is>
       </c>
       <c r="B295" s="2" t="inlineStr">
         <is>
-          <t>You must select a team before starting a game with bot</t>
+          <t>Save</t>
         </is>
       </c>
       <c r="C295" s="2" t="inlineStr">
         <is>
-          <t>Bạn phải chọn team trước khi bắt đầu trò chơi với bot</t>
+          <t>Lưu</t>
         </is>
       </c>
     </row>
     <row r="296" ht="18" customHeight="1">
       <c r="A296" s="1" t="inlineStr">
         <is>
-          <t>update-room.messages.success</t>
+          <t>room-invite.messages.title</t>
         </is>
       </c>
       <c r="B296" s="2" t="inlineStr">
         <is>
-          <t>Room updated successfully</t>
+          <t>Room Invitation</t>
         </is>
       </c>
       <c r="C296" s="2" t="inlineStr">
         <is>
-          <t>Cập nhật phòng thành công</t>
+          <t>Lời mời vào phòng</t>
         </is>
       </c>
     </row>
     <row r="297" ht="18" customHeight="1">
       <c r="A297" s="1" t="inlineStr">
         <is>
-          <t>update-room.messages.internal-server-error</t>
+          <t>start-game.messages.success</t>
         </is>
       </c>
       <c r="B297" s="2" t="inlineStr">
         <is>
-          <t>Internal server error</t>
+          <t>Game started successfully</t>
         </is>
       </c>
       <c r="C297" s="2" t="inlineStr">
         <is>
-          <t>Lỗi máy chủ nội bộ</t>
+          <t>Bắt đầu trò chơi thành công</t>
         </is>
       </c>
     </row>
     <row r="298" ht="18" customHeight="1">
       <c r="A298" s="1" t="inlineStr">
         <is>
-          <t>update-room.messages.invalid-room-id</t>
+          <t>start-game.messages.internal-server-error</t>
         </is>
       </c>
       <c r="B298" s="2" t="inlineStr">
         <is>
-          <t>Invalid room ID</t>
+          <t>Internal server error while starting game</t>
         </is>
       </c>
       <c r="C298" s="2" t="inlineStr">
         <is>
-          <t>ID phòng không hợp lệ</t>
+          <t>Lỗi máy chủ nội bộ khi bắt đầu trò chơi</t>
         </is>
       </c>
     </row>
     <row r="299" ht="18" customHeight="1">
       <c r="A299" s="1" t="inlineStr">
         <is>
-          <t>update-room.messages.invalid-time-limit</t>
+          <t>start-game.messages.invalid-room-id</t>
         </is>
       </c>
       <c r="B299" s="2" t="inlineStr">
         <is>
-          <t>Invalid time limit</t>
+          <t>Field 'id' is required and must be a positive integer</t>
         </is>
       </c>
       <c r="C299" s="2" t="inlineStr">
         <is>
-          <t>Thời gian không hợp lệ</t>
+          <t>Trường 'id' là bắt buộc và phải là số nguyên dương</t>
         </is>
       </c>
     </row>
     <row r="300" ht="18" customHeight="1">
       <c r="A300" s="1" t="inlineStr">
         <is>
-          <t>update-room.messages.name-required</t>
+          <t>start-game.messages.invalid-difficulty</t>
         </is>
       </c>
       <c r="B300" s="2" t="inlineStr">
         <is>
-          <t>Room name is required</t>
+          <t>Bot difficulty must be between 1 and 5</t>
         </is>
       </c>
       <c r="C300" s="2" t="inlineStr">
         <is>
-          <t>Tên phòng không được để trống</t>
+          <t>Độ khó của bot phải từ 1 đến 5</t>
         </is>
       </c>
     </row>
     <row r="301" ht="18" customHeight="1">
       <c r="A301" s="1" t="inlineStr">
         <is>
-          <t>update-room.messages.room-not-found</t>
+          <t>start-game.messages.room-not-found</t>
         </is>
       </c>
       <c r="B301" s="2" t="inlineStr">
@@ -5453,874 +5453,874 @@
     <row r="302" ht="18" customHeight="1">
       <c r="A302" s="1" t="inlineStr">
         <is>
-          <t>update-room.messages.forbidden</t>
+          <t>start-game.messages.forbidden</t>
         </is>
       </c>
       <c r="B302" s="2" t="inlineStr">
         <is>
-          <t>You are not the host of this room</t>
+          <t>Only the room host can start the game</t>
         </is>
       </c>
       <c r="C302" s="2" t="inlineStr">
         <is>
-          <t>Bạn không phải chủ phòng</t>
+          <t>Chỉ chủ phòng mới có thể bắt đầu trò chơi</t>
         </is>
       </c>
     </row>
     <row r="303" ht="18" customHeight="1">
       <c r="A303" s="1" t="inlineStr">
         <is>
-          <t>draw-game.messages.invalid-game-id</t>
+          <t>start-game.messages.insufficient-amount</t>
         </is>
       </c>
       <c r="B303" s="2" t="inlineStr">
         <is>
-          <t>Invalid game ID</t>
+          <t>You do not have enough balance to start a game with this bet</t>
         </is>
       </c>
       <c r="C303" s="2" t="inlineStr">
         <is>
-          <t>ID trò chơi không hợp lệ</t>
+          <t>Bạn không còn đủ amount để start room</t>
         </is>
       </c>
     </row>
     <row r="304" ht="18" customHeight="1">
       <c r="A304" s="1" t="inlineStr">
         <is>
-          <t>draw-game.messages.game-not-found</t>
+          <t>start-game.messages.requester-must-pick-team</t>
         </is>
       </c>
       <c r="B304" s="2" t="inlineStr">
         <is>
-          <t>Game not found</t>
+          <t>You must select a team before starting a game with bot</t>
         </is>
       </c>
       <c r="C304" s="2" t="inlineStr">
         <is>
-          <t>Không tìm thấy trò chơi</t>
+          <t>Bạn phải chọn team trước khi bắt đầu trò chơi với bot</t>
         </is>
       </c>
     </row>
     <row r="305" ht="18" customHeight="1">
       <c r="A305" s="1" t="inlineStr">
         <is>
-          <t>draw-game.messages.forbidden</t>
+          <t>update-room.messages.success</t>
         </is>
       </c>
       <c r="B305" s="2" t="inlineStr">
         <is>
-          <t>You are not in this room</t>
+          <t>Room updated successfully</t>
         </is>
       </c>
       <c r="C305" s="2" t="inlineStr">
         <is>
-          <t>Bạn không có trong phòng này</t>
+          <t>Cập nhật phòng thành công</t>
         </is>
       </c>
     </row>
     <row r="306" ht="90" customHeight="1">
       <c r="A306" s="1" t="inlineStr">
         <is>
-          <t>draw-game.messages.game-history-not-found</t>
+          <t>update-room.messages.internal-server-error</t>
         </is>
       </c>
       <c r="B306" s="2" t="inlineStr">
         <is>
-          <t>Game history not found</t>
+          <t>Internal server error</t>
         </is>
       </c>
       <c r="C306" s="2" t="inlineStr">
         <is>
-          <t>Không tìm thấy lịch sử trò chơi</t>
+          <t>Lỗi máy chủ nội bộ</t>
         </is>
       </c>
     </row>
     <row r="307" ht="90" customHeight="1">
       <c r="A307" s="1" t="inlineStr">
         <is>
-          <t>draw-game.messages.game-already-finished</t>
+          <t>update-room.messages.invalid-room-id</t>
         </is>
       </c>
       <c r="B307" s="2" t="inlineStr">
         <is>
-          <t>Game is already finished</t>
+          <t>Invalid room ID</t>
         </is>
       </c>
       <c r="C307" s="2" t="inlineStr">
         <is>
-          <t>Trò chơi đã kết thúc</t>
+          <t>ID phòng không hợp lệ</t>
         </is>
       </c>
     </row>
     <row r="308" ht="18" customHeight="1">
       <c r="A308" s="1" t="inlineStr">
         <is>
-          <t>draw-game.messages.success</t>
+          <t>update-room.messages.invalid-time-limit</t>
         </is>
       </c>
       <c r="B308" s="2" t="inlineStr">
         <is>
-          <t>Draw game successfully</t>
+          <t>Invalid time limit</t>
         </is>
       </c>
       <c r="C308" s="2" t="inlineStr">
         <is>
-          <t>Hòa cờ thành công</t>
+          <t>Thời gian không hợp lệ</t>
         </is>
       </c>
     </row>
     <row r="309" ht="18" customHeight="1">
       <c r="A309" s="1" t="inlineStr">
         <is>
-          <t>draw-game.messages.internal-server-error</t>
+          <t>update-room.messages.name-required</t>
         </is>
       </c>
       <c r="B309" s="2" t="inlineStr">
         <is>
-          <t>Internal server error</t>
+          <t>Room name is required</t>
         </is>
       </c>
       <c r="C309" s="2" t="inlineStr">
         <is>
-          <t>Lỗi máy chủ nội bộ</t>
+          <t>Tên phòng không được để trống</t>
         </is>
       </c>
     </row>
     <row r="310" ht="18" customHeight="1">
       <c r="A310" s="1" t="inlineStr">
         <is>
-          <t>surrender.messages.game-already-finished</t>
+          <t>update-room.messages.room-not-found</t>
         </is>
       </c>
       <c r="B310" s="2" t="inlineStr">
         <is>
-          <t>Game is already finished</t>
+          <t>Room not found</t>
         </is>
       </c>
       <c r="C310" s="2" t="inlineStr">
         <is>
-          <t>Trò chơi đã kết thúc</t>
+          <t>Không tìm thấy phòng</t>
         </is>
       </c>
     </row>
     <row r="311" ht="18" customHeight="1">
       <c r="A311" s="2" t="inlineStr">
         <is>
-          <t>surrender.messages.game-history-not-found</t>
+          <t>update-room.messages.forbidden</t>
         </is>
       </c>
       <c r="B311" s="2" t="inlineStr">
         <is>
-          <t>Game history not found</t>
+          <t>You are not the host of this room</t>
         </is>
       </c>
       <c r="C311" s="2" t="inlineStr">
         <is>
-          <t>Không tìm thấy lịch sử trò chơi</t>
+          <t>Bạn không phải chủ phòng</t>
         </is>
       </c>
     </row>
     <row r="312" ht="18" customHeight="1">
       <c r="A312" s="2" t="inlineStr">
         <is>
-          <t>surrender.messages.game-not-found</t>
+          <t>draw-game.messages.invalid-game-id</t>
         </is>
       </c>
       <c r="B312" s="2" t="inlineStr">
         <is>
-          <t>Game not found</t>
+          <t>Invalid game ID</t>
         </is>
       </c>
       <c r="C312" s="2" t="inlineStr">
         <is>
-          <t>Không tìm thấy trò chơi</t>
+          <t>ID trò chơi không hợp lệ</t>
         </is>
       </c>
     </row>
     <row r="313" ht="18" customHeight="1">
       <c r="A313" s="2" t="inlineStr">
         <is>
-          <t>surrender.messages.internal-server-error</t>
+          <t>draw-game.messages.game-not-found</t>
         </is>
       </c>
       <c r="B313" s="2" t="inlineStr">
         <is>
-          <t>Internal server error</t>
+          <t>Game not found</t>
         </is>
       </c>
       <c r="C313" s="2" t="inlineStr">
         <is>
-          <t>Lỗi máy chủ nội bộ</t>
+          <t>Không tìm thấy trò chơi</t>
         </is>
       </c>
     </row>
     <row r="314" ht="18" customHeight="1">
       <c r="A314" s="2" t="inlineStr">
         <is>
-          <t>surrender.messages.invalid-game-id</t>
+          <t>draw-game.messages.forbidden</t>
         </is>
       </c>
       <c r="B314" s="2" t="inlineStr">
         <is>
-          <t>Invalid game ID</t>
+          <t>You are not in this room</t>
         </is>
       </c>
       <c r="C314" s="2" t="inlineStr">
         <is>
-          <t>ID trò chơi không hợp lệ</t>
+          <t>Bạn không có trong phòng này</t>
         </is>
       </c>
     </row>
     <row r="315" ht="54" customHeight="1">
       <c r="A315" s="2" t="inlineStr">
         <is>
-          <t>surrender.messages.invalid-surrender-player</t>
+          <t>draw-game.messages.game-history-not-found</t>
         </is>
       </c>
       <c r="B315" s="2" t="inlineStr">
         <is>
-          <t>You are not a player in this game</t>
+          <t>Game history not found</t>
         </is>
       </c>
       <c r="C315" s="2" t="inlineStr">
         <is>
-          <t>Bạn không phải là người chơi trong trò chơi này</t>
+          <t>Không tìm thấy lịch sử trò chơi</t>
         </is>
       </c>
     </row>
     <row r="316" ht="18" customHeight="1">
       <c r="A316" s="2" t="inlineStr">
         <is>
-          <t>surrender.messages.opponent-not-found</t>
+          <t>draw-game.messages.game-already-finished</t>
         </is>
       </c>
       <c r="B316" s="2" t="inlineStr">
         <is>
-          <t>Opponent not found</t>
+          <t>Game is already finished</t>
         </is>
       </c>
       <c r="C316" s="2" t="inlineStr">
         <is>
-          <t>Không tìm thấy đối thủ</t>
+          <t>Trò chơi đã kết thúc</t>
         </is>
       </c>
     </row>
     <row r="317" ht="90" customHeight="1">
       <c r="A317" s="2" t="inlineStr">
         <is>
-          <t>surrender.messages.success</t>
+          <t>draw-game.messages.success</t>
         </is>
       </c>
       <c r="B317" s="2" t="inlineStr">
         <is>
-          <t>Surrendered</t>
+          <t>Draw game successfully</t>
         </is>
       </c>
       <c r="C317" s="2" t="inlineStr">
         <is>
-          <t>Đã đầu hàng</t>
+          <t>Hòa cờ thành công</t>
         </is>
       </c>
     </row>
     <row r="318" ht="18" customHeight="1">
       <c r="A318" s="2" t="inlineStr">
         <is>
-          <t>undo.messages.invalid-game-id</t>
+          <t>draw-game.messages.internal-server-error</t>
         </is>
       </c>
       <c r="B318" s="2" t="inlineStr">
         <is>
-          <t>Invalid game ID</t>
+          <t>Internal server error</t>
         </is>
       </c>
       <c r="C318" s="2" t="inlineStr">
         <is>
-          <t>ID trò chơi không hợp lệ</t>
+          <t>Lỗi máy chủ nội bộ</t>
         </is>
       </c>
     </row>
     <row r="319" ht="36" customHeight="1">
       <c r="A319" s="2" t="inlineStr">
         <is>
-          <t>undo.messages.unauthorized</t>
+          <t>surrender.messages.game-already-finished</t>
         </is>
       </c>
       <c r="B319" s="2" t="inlineStr">
         <is>
-          <t>Unauthorized</t>
+          <t>Game is already finished</t>
         </is>
       </c>
       <c r="C319" s="2" t="inlineStr">
         <is>
-          <t>Không được phép truy cập</t>
+          <t>Trò chơi đã kết thúc</t>
         </is>
       </c>
     </row>
     <row r="320" ht="18" customHeight="1">
       <c r="A320" s="2" t="inlineStr">
         <is>
-          <t>undo.messages.game-not-found</t>
+          <t>surrender.messages.game-history-not-found</t>
         </is>
       </c>
       <c r="B320" s="2" t="inlineStr">
         <is>
-          <t>Game not found</t>
+          <t>Game history not found</t>
         </is>
       </c>
       <c r="C320" s="2" t="inlineStr">
         <is>
-          <t>Không tìm thấy trò chơi</t>
+          <t>Không tìm thấy lịch sử trò chơi</t>
         </is>
       </c>
     </row>
     <row r="321" ht="72" customHeight="1">
       <c r="A321" s="2" t="inlineStr">
         <is>
-          <t>undo.messages.not-in-game</t>
+          <t>surrender.messages.game-not-found</t>
         </is>
       </c>
       <c r="B321" s="2" t="inlineStr">
         <is>
-          <t>You are not part of this game</t>
+          <t>Game not found</t>
         </is>
       </c>
       <c r="C321" s="2" t="inlineStr">
         <is>
-          <t>Bạn không phải là người chơi trong trò chơi này</t>
+          <t>Không tìm thấy trò chơi</t>
         </is>
       </c>
     </row>
     <row r="322" ht="18" customHeight="1">
       <c r="A322" s="2" t="inlineStr">
         <is>
-          <t>undo.messages.not-in-room</t>
+          <t>surrender.messages.internal-server-error</t>
         </is>
       </c>
       <c r="B322" s="2" t="inlineStr">
         <is>
-          <t>You are not in this room</t>
+          <t>Internal server error</t>
         </is>
       </c>
       <c r="C322" s="2" t="inlineStr">
         <is>
-          <t>Bạn không trong phòng này</t>
+          <t>Lỗi máy chủ nội bộ</t>
         </is>
       </c>
     </row>
     <row r="323" ht="54" customHeight="1">
       <c r="A323" s="2" t="inlineStr">
         <is>
-          <t>undo.messages.spectator-cannot-undo</t>
+          <t>surrender.messages.invalid-game-id</t>
         </is>
       </c>
       <c r="B323" s="2" t="inlineStr">
         <is>
-          <t>Spectators cannot undo moves</t>
+          <t>Invalid game ID</t>
         </is>
       </c>
       <c r="C323" s="2" t="inlineStr">
         <is>
-          <t>Người xem không thể hoàn tác nước đi</t>
+          <t>ID trò chơi không hợp lệ</t>
         </is>
       </c>
     </row>
     <row r="324" ht="18" customHeight="1">
       <c r="A324" s="2" t="inlineStr">
         <is>
-          <t>undo.messages.no-moves</t>
+          <t>surrender.messages.invalid-surrender-player</t>
         </is>
       </c>
       <c r="B324" s="2" t="inlineStr">
         <is>
-          <t>No moves to undo</t>
+          <t>You are not a player in this game</t>
         </is>
       </c>
       <c r="C324" s="2" t="inlineStr">
         <is>
-          <t>Không có nước đi để hoàn tác</t>
+          <t>Bạn không phải là người chơi trong trò chơi này</t>
         </is>
       </c>
     </row>
     <row r="325" ht="72" customHeight="1">
       <c r="A325" s="2" t="inlineStr">
         <is>
-          <t>undo.messages.delete-failed</t>
+          <t>surrender.messages.opponent-not-found</t>
         </is>
       </c>
       <c r="B325" s="2" t="inlineStr">
         <is>
-          <t>Failed to undo move</t>
+          <t>Opponent not found</t>
         </is>
       </c>
       <c r="C325" s="2" t="inlineStr">
         <is>
-          <t>Không thể hoàn tác nước đi</t>
+          <t>Không tìm thấy đối thủ</t>
         </is>
       </c>
     </row>
     <row r="326" ht="18" customHeight="1">
       <c r="A326" s="2" t="inlineStr">
         <is>
-          <t>undo.messages.undo-limit-exceeded</t>
+          <t>surrender.messages.success</t>
         </is>
       </c>
       <c r="B326" s="2" t="inlineStr">
         <is>
-          <t>Maximum 3 undo per game exceeded</t>
+          <t>Surrendered</t>
         </is>
       </c>
       <c r="C326" s="2" t="inlineStr">
         <is>
-          <t>Đã đạt tối đa 3 lần hoàn tác trong trò chơi</t>
+          <t>Đã đầu hàng</t>
         </is>
       </c>
     </row>
     <row r="327" ht="90" customHeight="1">
       <c r="A327" s="2" t="inlineStr">
         <is>
-          <t>undo.messages.success</t>
+          <t>undo.messages.invalid-game-id</t>
         </is>
       </c>
       <c r="B327" s="2" t="inlineStr">
         <is>
-          <t>Move undone successfully</t>
+          <t>Invalid game ID</t>
         </is>
       </c>
       <c r="C327" s="2" t="inlineStr">
         <is>
-          <t>Hoàn tác nước đi thành công</t>
+          <t>ID trò chơi không hợp lệ</t>
         </is>
       </c>
     </row>
     <row r="328" ht="18" customHeight="1">
       <c r="A328" s="2" t="inlineStr">
         <is>
-          <t>undo.messages.internal-server-error</t>
+          <t>undo.messages.unauthorized</t>
         </is>
       </c>
       <c r="B328" s="2" t="inlineStr">
         <is>
-          <t>Internal server error</t>
+          <t>Unauthorized</t>
         </is>
       </c>
       <c r="C328" s="2" t="inlineStr">
         <is>
-          <t>Lỗi máy chủ nội bộ</t>
+          <t>Không được phép truy cập</t>
         </is>
       </c>
     </row>
     <row r="329" ht="72" customHeight="1">
       <c r="A329" s="2" t="inlineStr">
         <is>
-          <t>player-history.messages.invalid-user-id</t>
+          <t>undo.messages.game-not-found</t>
         </is>
       </c>
       <c r="B329" s="2" t="inlineStr">
         <is>
-          <t>Invalid user ID</t>
+          <t>Game not found</t>
         </is>
       </c>
       <c r="C329" s="2" t="inlineStr">
         <is>
-          <t>ID người dùng không hợp lệ</t>
+          <t>Không tìm thấy trò chơi</t>
         </is>
       </c>
     </row>
     <row r="330" ht="54" customHeight="1">
       <c r="A330" s="2" t="inlineStr">
         <is>
-          <t>player-history.messages.success</t>
+          <t>undo.messages.not-in-game</t>
         </is>
       </c>
       <c r="B330" s="2" t="inlineStr">
         <is>
-          <t>Fetch game history successfully</t>
+          <t>You are not part of this game</t>
         </is>
       </c>
       <c r="C330" s="2" t="inlineStr">
         <is>
-          <t>Lấy lịch sử trò chơi thành công</t>
+          <t>Bạn không phải là người chơi trong trò chơi này</t>
         </is>
       </c>
     </row>
     <row r="331" ht="54" customHeight="1">
       <c r="A331" s="2" t="inlineStr">
         <is>
-          <t>validate-token.messages.success</t>
+          <t>undo.messages.not-in-room</t>
         </is>
       </c>
       <c r="B331" s="2" t="inlineStr">
         <is>
-          <t>Token is valid</t>
+          <t>You are not in this room</t>
         </is>
       </c>
       <c r="C331" s="2" t="inlineStr">
         <is>
-          <t>Token hợp lệ</t>
+          <t>Bạn không trong phòng này</t>
         </is>
       </c>
     </row>
     <row r="332" ht="54" customHeight="1">
       <c r="A332" s="2" t="inlineStr">
         <is>
-          <t>guide.section.objective</t>
+          <t>undo.messages.spectator-cannot-undo</t>
         </is>
       </c>
       <c r="B332" s="2" t="inlineStr">
         <is>
-          <t>Objective of the game</t>
+          <t>Spectators cannot undo moves</t>
         </is>
       </c>
       <c r="C332" s="2" t="inlineStr">
         <is>
-          <t>Mục tiêu của trò chơi</t>
+          <t>Người xem không thể hoàn tác nước đi</t>
         </is>
       </c>
     </row>
     <row r="333" ht="90" customHeight="1">
       <c r="A333" s="2" t="inlineStr">
         <is>
-          <t>guide.section.pieces</t>
+          <t>undo.messages.no-moves</t>
         </is>
       </c>
       <c r="B333" s="2" t="inlineStr">
         <is>
-          <t>Pieces</t>
+          <t>No moves to undo</t>
         </is>
       </c>
       <c r="C333" s="2" t="inlineStr">
         <is>
-          <t>Quân cờ</t>
+          <t>Không có nước đi để hoàn tác</t>
         </is>
       </c>
     </row>
     <row r="334" ht="54" customHeight="1">
       <c r="A334" s="2" t="inlineStr">
         <is>
-          <t>guide.section.moving-pieces</t>
+          <t>undo.messages.delete-failed</t>
         </is>
       </c>
       <c r="B334" s="2" t="inlineStr">
         <is>
-          <t>Moving pieces</t>
+          <t>Failed to undo move</t>
         </is>
       </c>
       <c r="C334" s="2" t="inlineStr">
         <is>
-          <t>Đi quân</t>
+          <t>Không thể hoàn tác nước đi</t>
         </is>
       </c>
     </row>
     <row r="335" ht="36" customHeight="1">
       <c r="A335" s="2" t="inlineStr">
         <is>
-          <t>guide.section.capturing</t>
+          <t>undo.messages.undo-limit-exceeded</t>
         </is>
       </c>
       <c r="B335" s="2" t="inlineStr">
         <is>
-          <t>Capturing</t>
+          <t>Maximum 3 undo per game exceeded</t>
         </is>
       </c>
       <c r="C335" s="2" t="inlineStr">
         <is>
-          <t>Bắt quân</t>
+          <t>Đã đạt tối đa 3 lần hoàn tác trong trò chơi</t>
         </is>
       </c>
     </row>
     <row r="336" ht="18" customHeight="1">
       <c r="A336" s="2" t="inlineStr">
         <is>
-          <t>guide.section.check</t>
+          <t>undo.messages.success</t>
         </is>
       </c>
       <c r="B336" s="2" t="inlineStr">
         <is>
-          <t>Check</t>
+          <t>Move undone successfully</t>
         </is>
       </c>
       <c r="C336" s="2" t="inlineStr">
         <is>
-          <t>Chiếu tướng</t>
+          <t>Hoàn tác nước đi thành công</t>
         </is>
       </c>
     </row>
     <row r="337" ht="36" customHeight="1">
       <c r="A337" s="2" t="inlineStr">
         <is>
-          <t>guide.section.result</t>
+          <t>undo.messages.internal-server-error</t>
         </is>
       </c>
       <c r="B337" s="2" t="inlineStr">
         <is>
-          <t>Result</t>
+          <t>Internal server error</t>
         </is>
       </c>
       <c r="C337" s="2" t="inlineStr">
         <is>
-          <t>Kết quả</t>
+          <t>Lỗi máy chủ nội bộ</t>
         </is>
       </c>
     </row>
     <row r="338" ht="36" customHeight="1">
       <c r="A338" s="2" t="inlineStr">
         <is>
-          <t>guide.table.piece</t>
+          <t>player-history.messages.invalid-user-id</t>
         </is>
       </c>
       <c r="B338" s="2" t="inlineStr">
         <is>
-          <t>Piece</t>
+          <t>Invalid user ID</t>
         </is>
       </c>
       <c r="C338" s="2" t="inlineStr">
         <is>
-          <t>Quân</t>
+          <t>ID người dùng không hợp lệ</t>
         </is>
       </c>
     </row>
     <row r="339" ht="72" customHeight="1">
       <c r="A339" s="2" t="inlineStr">
         <is>
-          <t>guide.table.symbol</t>
+          <t>player-history.messages.success</t>
         </is>
       </c>
       <c r="B339" s="2" t="inlineStr">
         <is>
-          <t>Symbol</t>
+          <t>Fetch game history successfully</t>
         </is>
       </c>
       <c r="C339" s="2" t="inlineStr">
         <is>
-          <t>Ký hiệu</t>
+          <t>Lấy lịch sử trò chơi thành công</t>
         </is>
       </c>
     </row>
     <row r="340" ht="54" customHeight="1">
       <c r="A340" s="2" t="inlineStr">
         <is>
-          <t>guide.table.quantity</t>
+          <t>validate-token.messages.success</t>
         </is>
       </c>
       <c r="B340" s="2" t="inlineStr">
         <is>
-          <t>Quantity</t>
+          <t>Token is valid</t>
         </is>
       </c>
       <c r="C340" s="2" t="inlineStr">
         <is>
-          <t>Số lượng</t>
+          <t>Token hợp lệ</t>
         </is>
       </c>
     </row>
     <row r="341" ht="54" customHeight="1">
       <c r="A341" s="2" t="inlineStr">
         <is>
-          <t>guide.objective.paragraph1</t>
+          <t>guide.section.objective</t>
         </is>
       </c>
       <c r="B341" s="2" t="inlineStr">
         <is>
-          <t>A match is played between two players: one controls the Red pieces, and the other controls the Black pieces. The objective of each player is to use their pieces on the board to &lt;b&gt;checkmate&lt;/b&gt; the opponent's General, and win the game.</t>
+          <t>Objective of the game</t>
         </is>
       </c>
       <c r="C341" s="2" t="inlineStr">
         <is>
-          <t>Ván cờ được tiến hành giữa 2 đấu thủ, một người cầm Quân Đỏ, một người cầm Quân Đen. Mục đích của mỗi đấu thủ là tìm mọi cách sử dụng các quân trên bàn cờ để &lt;b&gt;chiếu bí Tướng&lt;/b&gt; của đối phương, giành thắng lợi.</t>
+          <t>Mục tiêu của trò chơi</t>
         </is>
       </c>
     </row>
     <row r="342" ht="90" customHeight="1">
       <c r="A342" s="2" t="inlineStr">
         <is>
-          <t>guide.pieces.paragraph1</t>
+          <t>guide.section.pieces</t>
         </is>
       </c>
       <c r="B342" s="2" t="inlineStr">
         <is>
-          <t>At the start of each game, there must be 32 pieces in total, consisting of &lt;b&gt;7 piece types&lt;/b&gt; split evenly between both sides: 16 Red pieces and 16 Black pieces. The 7 piece types with their symbols and quantities are as follows:</t>
+          <t>Pieces</t>
         </is>
       </c>
       <c r="C342" s="2" t="inlineStr">
         <is>
-          <t>Mỗi ván cờ lúc bắt đầu phải có đủ 32 quân, gồm 7 loại chia đều cho mỗi bên gồm 16 quân Đỏ và 16 quân Đen. &lt;b&gt;7 loại quân&lt;/b&gt; có ký hiệu và số lượng như sau:</t>
+          <t>Quân cờ</t>
         </is>
       </c>
     </row>
     <row r="343" ht="54" customHeight="1">
       <c r="A343" s="2" t="inlineStr">
         <is>
-          <t>guide.piece.general</t>
+          <t>guide.section.moving-pieces</t>
         </is>
       </c>
       <c r="B343" s="2" t="inlineStr">
         <is>
-          <t>General</t>
+          <t>Moving pieces</t>
         </is>
       </c>
       <c r="C343" s="2" t="inlineStr">
         <is>
-          <t>Tướng</t>
+          <t>Đi quân</t>
         </is>
       </c>
     </row>
     <row r="344" ht="18" customHeight="1">
       <c r="A344" s="2" t="inlineStr">
         <is>
-          <t>guide.piece.advisor</t>
+          <t>guide.section.capturing</t>
         </is>
       </c>
       <c r="B344" s="2" t="inlineStr">
         <is>
-          <t>Advisor</t>
+          <t>Capturing</t>
         </is>
       </c>
       <c r="C344" s="2" t="inlineStr">
         <is>
-          <t>Sĩ</t>
+          <t>Bắt quân</t>
         </is>
       </c>
     </row>
     <row r="345" ht="18" customHeight="1">
       <c r="A345" s="2" t="inlineStr">
         <is>
-          <t>guide.piece.elephant</t>
+          <t>guide.section.check</t>
         </is>
       </c>
       <c r="B345" s="2" t="inlineStr">
         <is>
-          <t>Elephant</t>
+          <t>Check</t>
         </is>
       </c>
       <c r="C345" s="2" t="inlineStr">
         <is>
-          <t>Tượng</t>
+          <t>Chiếu tướng</t>
         </is>
       </c>
     </row>
     <row r="346" ht="36" customHeight="1">
       <c r="A346" s="2" t="inlineStr">
         <is>
-          <t>guide.piece.chariot</t>
+          <t>guide.section.result</t>
         </is>
       </c>
       <c r="B346" s="2" t="inlineStr">
         <is>
-          <t>Chariot</t>
+          <t>Result</t>
         </is>
       </c>
       <c r="C346" s="2" t="inlineStr">
         <is>
-          <t>Xe</t>
+          <t>Kết quả</t>
         </is>
       </c>
     </row>
     <row r="347" ht="18" customHeight="1">
       <c r="A347" s="2" t="inlineStr">
         <is>
-          <t>guide.piece.horse</t>
+          <t>guide.table.piece</t>
         </is>
       </c>
       <c r="B347" s="2" t="inlineStr">
         <is>
-          <t>Horse</t>
+          <t>Piece</t>
         </is>
       </c>
       <c r="C347" s="2" t="inlineStr">
         <is>
-          <t>Mã</t>
+          <t>Quân</t>
         </is>
       </c>
     </row>
     <row r="348" ht="18" customHeight="1">
       <c r="A348" s="2" t="inlineStr">
         <is>
-          <t>guide.piece.cannon</t>
+          <t>guide.table.symbol</t>
         </is>
       </c>
       <c r="B348" s="2" t="inlineStr">
         <is>
-          <t>Cannon</t>
+          <t>Symbol</t>
         </is>
       </c>
       <c r="C348" s="2" t="inlineStr">
         <is>
-          <t>Pháo</t>
+          <t>Ký hiệu</t>
         </is>
       </c>
     </row>
     <row r="349" ht="36" customHeight="1">
       <c r="A349" s="2" t="inlineStr">
         <is>
-          <t>guide.piece.soldier</t>
+          <t>guide.table.quantity</t>
         </is>
       </c>
       <c r="B349" s="2" t="inlineStr">
         <is>
-          <t>Soldier</t>
+          <t>Quantity</t>
         </is>
       </c>
       <c r="C349" s="2" t="inlineStr">
         <is>
-          <t>Tốt</t>
+          <t>Số lượng</t>
         </is>
       </c>
     </row>
     <row r="350" ht="18" customHeight="1">
       <c r="A350" s="2" t="inlineStr">
         <is>
-          <t>guide.moving-pieces.paragraph1</t>
+          <t>guide.objective.paragraph1</t>
         </is>
       </c>
       <c r="B350" s="2" t="inlineStr">
         <is>
-          <t>On each turn, each side may move only one of its own pieces according to the rules. The movement rules are as follows:</t>
+          <t>A match is played between two players: one controls the Red pieces, and the other controls the Black pieces. The objective of each player is to use their pieces on the board to &lt;b&gt;checkmate&lt;/b&gt; the opponent's General, and win the game.</t>
         </is>
       </c>
       <c r="C350" s="2" t="inlineStr">
         <is>
-          <t>Mỗi nước đi, mỗi bên chỉ được di chuyển quân của mình theo đúng quy định. Quy định di chuyển của các quân như sau:</t>
+          <t>Ván cờ được tiến hành giữa 2 đấu thủ, một người cầm Quân Đỏ, một người cầm Quân Đen. Mục đích của mỗi đấu thủ là tìm mọi cách sử dụng các quân trên bàn cờ để &lt;b&gt;chiếu bí Tướng&lt;/b&gt; của đối phương, giành thắng lợi.</t>
         </is>
       </c>
     </row>
     <row r="351" ht="36" customHeight="1">
       <c r="A351" s="2" t="inlineStr">
         <is>
-          <t>guide.general.paragraph1</t>
+          <t>guide.pieces.paragraph1</t>
         </is>
       </c>
       <c r="B351" s="2" t="inlineStr">
         <is>
-          <t>General</t>
+          <t>At the start of each game, there must be 32 pieces in total, consisting of &lt;b&gt;7 piece types&lt;/b&gt; split evenly between both sides: 16 Red pieces and 16 Black pieces. The 7 piece types with their symbols and quantities are as follows:</t>
         </is>
       </c>
       <c r="C351" s="2" t="inlineStr">
         <is>
-          <t>Tướng</t>
+          <t>Mỗi ván cờ lúc bắt đầu phải có đủ 32 quân, gồm 7 loại chia đều cho mỗi bên gồm 16 quân Đỏ và 16 quân Đen. &lt;b&gt;7 loại quân&lt;/b&gt; có ký hiệu và số lượng như sau:</t>
         </is>
       </c>
     </row>
     <row r="352" ht="18" customHeight="1">
       <c r="A352" s="2" t="inlineStr">
         <is>
-          <t>guide.general.paragraph2</t>
+          <t>guide.piece.general</t>
         </is>
       </c>
       <c r="B352" s="2" t="inlineStr">
         <is>
-          <t>Moves one step &lt;b&gt;horizontally or vertically&lt;/b&gt; within the palace. The two Generals may not face each other directly on the same file. If they are facing each other, there must be at least one piece of either side placed between them.</t>
+          <t>General</t>
         </is>
       </c>
       <c r="C352" s="2" t="inlineStr">
         <is>
-          <t>Mỗi nước được đi một bước &lt;b&gt;ngang hoặc dọc&lt;/b&gt; tùy ý trong cung Tướng. Hai tướng của 2 bên không được đối mặt nhau trực tiếp trên cùng một đường thẳng. Nếu đối mặt, bắt buộc phải có quân của bất kỳ bên nào đứng che mặt.</t>
+          <t>Tướng</t>
         </is>
       </c>
     </row>
     <row r="353" ht="18" customHeight="1">
       <c r="A353" s="2" t="inlineStr">
         <is>
-          <t>guide.advisor.paragraph1</t>
+          <t>guide.piece.advisor</t>
         </is>
       </c>
       <c r="B353" s="2" t="inlineStr">
@@ -6337,1084 +6337,1192 @@
     <row r="354" ht="18" customHeight="1">
       <c r="A354" s="2" t="inlineStr">
         <is>
-          <t>guide.advisor.paragraph2</t>
+          <t>guide.piece.elephant</t>
         </is>
       </c>
       <c r="B354" s="2" t="inlineStr">
         <is>
-          <t>Moves one step &lt;b&gt;diagonally&lt;/b&gt; within the palace.</t>
+          <t>Elephant</t>
         </is>
       </c>
       <c r="C354" s="2" t="inlineStr">
         <is>
-          <t>Mỗi nước &lt;b&gt;đi chéo một bước&lt;/b&gt; trong cung Tướng.</t>
+          <t>Tượng</t>
         </is>
       </c>
     </row>
     <row r="355" ht="18" customHeight="1">
       <c r="A355" s="2" t="inlineStr">
         <is>
-          <t>guide.elephant.paragraph1</t>
+          <t>guide.piece.chariot</t>
         </is>
       </c>
       <c r="B355" s="2" t="inlineStr">
         <is>
-          <t>Elephant</t>
+          <t>Chariot</t>
         </is>
       </c>
       <c r="C355" s="2" t="inlineStr">
         <is>
-          <t>Tượng</t>
+          <t>Xe</t>
         </is>
       </c>
     </row>
     <row r="356" ht="18" customHeight="1">
       <c r="A356" s="2" t="inlineStr">
         <is>
-          <t>guide.elephant.paragraph2</t>
+          <t>guide.piece.horse</t>
         </is>
       </c>
       <c r="B356" s="2" t="inlineStr">
         <is>
-          <t>Moves &lt;b&gt;two steps diagonally&lt;/b&gt; on its own side of the board and may not cross the river. If there is another piece on the midpoint of that diagonal path, the Elephant is blocked and cannot move.</t>
+          <t>Horse</t>
         </is>
       </c>
       <c r="C356" s="2" t="inlineStr">
         <is>
-          <t>Mỗi nước &lt;b&gt;đi chéo hai bước&lt;/b&gt; tại trận địa bên mình, không được qua sông. Nếu ở giữa đường chéo đó có quân khác đứng thì quân Tượng bị cản, không đi được.</t>
+          <t>Mã</t>
         </is>
       </c>
     </row>
     <row r="357" ht="17" customHeight="1">
       <c r="A357" s="2" t="inlineStr">
         <is>
-          <t>guide.chariot.paragraph1</t>
+          <t>guide.piece.cannon</t>
         </is>
       </c>
       <c r="B357" s="2" t="inlineStr">
         <is>
-          <t>Chariot</t>
+          <t>Cannon</t>
         </is>
       </c>
       <c r="C357" s="2" t="inlineStr">
         <is>
-          <t>Xe</t>
+          <t>Pháo</t>
         </is>
       </c>
     </row>
     <row r="358" ht="18" customHeight="1">
       <c r="A358" s="2" t="inlineStr">
         <is>
-          <t>guide.chariot.paragraph2</t>
+          <t>guide.piece.soldier</t>
         </is>
       </c>
       <c r="B358" s="2" t="inlineStr">
         <is>
-          <t>Moves &lt;b&gt;horizontally or vertically&lt;/b&gt; with no limit on distance, as long as no piece blocks the path.</t>
+          <t>Soldier</t>
         </is>
       </c>
       <c r="C358" s="2" t="inlineStr">
         <is>
-          <t>Mỗi nước được &lt;b&gt;đi dọc hoặc đi ngang&lt;/b&gt;, không hạn chế số bước đi nếu không có quân khác cản đường.</t>
+          <t>Tốt</t>
         </is>
       </c>
     </row>
     <row r="359" ht="18" customHeight="1">
       <c r="A359" s="2" t="inlineStr">
         <is>
-          <t>guide.horse.paragraph1</t>
+          <t>guide.moving-pieces.paragraph1</t>
         </is>
       </c>
       <c r="B359" s="2" t="inlineStr">
         <is>
-          <t>Horse</t>
+          <t>On each turn, each side may move only one of its own pieces according to the rules. The movement rules are as follows:</t>
         </is>
       </c>
       <c r="C359" s="2" t="inlineStr">
         <is>
-          <t>Mã</t>
+          <t>Mỗi nước đi, mỗi bên chỉ được di chuyển quân của mình theo đúng quy định. Quy định di chuyển của các quân như sau:</t>
         </is>
       </c>
     </row>
     <row r="360" ht="18" customHeight="1">
       <c r="A360" s="2" t="inlineStr">
         <is>
-          <t>guide.horse.paragraph2</t>
+          <t>guide.general.paragraph1</t>
         </is>
       </c>
       <c r="B360" s="2" t="inlineStr">
         <is>
-          <t>Moves in an &lt;b&gt;L-shape&lt;/b&gt; (one step orthogonally then one step diagonally outward). If the adjacent orthogonal point is occupied by any piece, the Horse is blocked and cannot move.</t>
+          <t>General</t>
         </is>
       </c>
       <c r="C360" s="2" t="inlineStr">
         <is>
-          <t>Đi theo &lt;b&gt;đường chéo hình chữ nhật&lt;/b&gt; của hai ô vuông liền nhau. Nếu giao điểm liền kề bước thẳng dọc ngang có một quân khác đứng thì Mã bị cản, không đi được.</t>
+          <t>Tướng</t>
         </is>
       </c>
     </row>
     <row r="361" ht="18" customHeight="1">
       <c r="A361" s="2" t="inlineStr">
         <is>
-          <t>guide.cannon.paragraph1</t>
+          <t>guide.general.paragraph2</t>
         </is>
       </c>
       <c r="B361" s="2" t="inlineStr">
         <is>
-          <t>Cannon</t>
+          <t>Moves one step &lt;b&gt;horizontally or vertically&lt;/b&gt; within the palace. The two Generals may not face each other directly on the same file. If they are facing each other, there must be at least one piece of either side placed between them.</t>
         </is>
       </c>
       <c r="C361" s="2" t="inlineStr">
         <is>
-          <t>Pháo</t>
+          <t>Mỗi nước được đi một bước &lt;b&gt;ngang hoặc dọc&lt;/b&gt; tùy ý trong cung Tướng. Hai tướng của 2 bên không được đối mặt nhau trực tiếp trên cùng một đường thẳng. Nếu đối mặt, bắt buộc phải có quân của bất kỳ bên nào đứng che mặt.</t>
         </is>
       </c>
     </row>
     <row r="362" ht="18" customHeight="1">
       <c r="A362" s="2" t="inlineStr">
         <is>
-          <t>guide.cannon.paragraph2</t>
+          <t>guide.advisor.paragraph1</t>
         </is>
       </c>
       <c r="B362" s="2" t="inlineStr">
         <is>
-          <t>Moves &lt;b&gt;horizontally or vertically&lt;/b&gt; like a Chariot when not capturing. To capture, it must &lt;b&gt;jump over exactly one piece&lt;/b&gt; to reach its target. If there are zero or more than one pieces between the Cannon and the target, it cannot capture.</t>
+          <t>Advisor</t>
         </is>
       </c>
       <c r="C362" s="2" t="inlineStr">
         <is>
-          <t>Đi ngang hoặc dọc giống Xe khi không bắt quân. Để bắt quân, nó phải &lt;b&gt;nhảy qua đúng một quân khác&lt;/b&gt; để đến mục tiêu. Nếu không có hoặc có nhiều hơn một quân giữa Pháo và mục tiêu, nó không thể bắt quân.</t>
+          <t>Sĩ</t>
         </is>
       </c>
     </row>
     <row r="363" ht="18" customHeight="1">
       <c r="A363" s="2" t="inlineStr">
         <is>
-          <t>guide.soldier.paragraph1</t>
+          <t>guide.advisor.paragraph2</t>
         </is>
       </c>
       <c r="B363" s="2" t="inlineStr">
         <is>
-          <t>Soldier</t>
+          <t>Moves one step &lt;b&gt;diagonally&lt;/b&gt; within the palace.</t>
         </is>
       </c>
       <c r="C363" s="2" t="inlineStr">
         <is>
-          <t>Tốt</t>
+          <t>Mỗi nước &lt;b&gt;đi chéo một bước&lt;/b&gt; trong cung Tướng.</t>
         </is>
       </c>
     </row>
     <row r="364" ht="17" customHeight="1">
       <c r="A364" s="2" t="inlineStr">
         <is>
-          <t>guide.soldier.paragraph2</t>
+          <t>guide.elephant.paragraph1</t>
         </is>
       </c>
       <c r="B364" s="2" t="inlineStr">
         <is>
-          <t>Moves &lt;b&gt;one step&lt;/b&gt; each turn. Before crossing the river, it can only move forward. After crossing the river, it may move &lt;b&gt;forward or sideways&lt;/b&gt;, but never backward.</t>
+          <t>Elephant</t>
         </is>
       </c>
       <c r="C364" s="2" t="inlineStr">
         <is>
-          <t>Mỗi nước đi &lt;b&gt;một bước&lt;/b&gt;. Khi chưa qua sông, Tốt chỉ được tiến. Khi Tốt đã qua sông được quyền &lt;b&gt;đi tiến và đi ngang&lt;/b&gt;, không được phép lùi.</t>
+          <t>Tượng</t>
         </is>
       </c>
     </row>
     <row r="365" ht="17" customHeight="1">
       <c r="A365" s="2" t="inlineStr">
         <is>
-          <t>guide.capturing.paragraph1</t>
+          <t>guide.elephant.paragraph2</t>
         </is>
       </c>
       <c r="B365" s="2" t="inlineStr">
         <is>
-          <t>When a piece moves to an intersection occupied by an opponent's piece, it may &lt;b&gt;capture that piece&lt;/b&gt; and occupy its position.</t>
+          <t>Moves &lt;b&gt;two steps diagonally&lt;/b&gt; on its own side of the board and may not cross the river. If there is another piece on the midpoint of that diagonal path, the Elephant is blocked and cannot move.</t>
         </is>
       </c>
       <c r="C365" s="2" t="inlineStr">
         <is>
-          <t>Khi một quân đi tới một giao điểm khác đã có quân đối phương đứng thì được quyền &lt;b&gt;bắt quân đó&lt;/b&gt;, đồng thời chiếm giữ vị trí quân bị bắt.</t>
+          <t>Mỗi nước &lt;b&gt;đi chéo hai bước&lt;/b&gt; tại trận địa bên mình, không được qua sông. Nếu ở giữa đường chéo đó có quân khác đứng thì quân Tượng bị cản, không đi được.</t>
         </is>
       </c>
     </row>
     <row r="366" ht="17" customHeight="1">
       <c r="A366" s="2" t="inlineStr">
         <is>
-          <t>guide.capturing.paragraph2</t>
+          <t>guide.chariot.paragraph1</t>
         </is>
       </c>
       <c r="B366" s="2" t="inlineStr">
         <is>
-          <t>You may not capture your own pieces. You may sacrifice your own pieces to be captured by the opponent, &lt;b&gt;except for the General&lt;/b&gt;.</t>
+          <t>Chariot</t>
         </is>
       </c>
       <c r="C366" s="2" t="inlineStr">
         <is>
-          <t>Không được bắt quân bên mình. Được phép cho đối phương bắt đầu quân mình chủ động hiến mình cho đối phương, &lt;b&gt;trừ Tướng&lt;/b&gt;.</t>
+          <t>Xe</t>
         </is>
       </c>
     </row>
     <row r="367" ht="17" customHeight="1">
       <c r="A367" s="2" t="inlineStr">
         <is>
-          <t>guide.capturing.paragraph3</t>
+          <t>guide.chariot.paragraph2</t>
         </is>
       </c>
       <c r="B367" s="2" t="inlineStr">
         <is>
-          <t>A captured piece is removed from the board. &lt;b&gt;Chasing one piece for more than 6 consecutive moves is not allowed&lt;/b&gt;.</t>
+          <t>Moves &lt;b&gt;horizontally or vertically&lt;/b&gt; with no limit on distance, as long as no piece blocks the path.</t>
         </is>
       </c>
       <c r="C367" s="2" t="inlineStr">
         <is>
-          <t>Quân bị bắt phải bị loại và bị nhấc ra khỏi bàn cờ. &lt;b&gt;Không được đuổi 1 quân quá 6 nước cờ liên tiếp&lt;/b&gt;.</t>
+          <t>Mỗi nước được &lt;b&gt;đi dọc hoặc đi ngang&lt;/b&gt;, không hạn chế số bước đi nếu không có quân khác cản đường.</t>
         </is>
       </c>
     </row>
     <row r="368" ht="17" customHeight="1">
       <c r="A368" s="2" t="inlineStr">
         <is>
-          <t>guide.check.paragraph1</t>
+          <t>guide.horse.paragraph1</t>
         </is>
       </c>
       <c r="B368" s="2" t="inlineStr">
         <is>
-          <t>If a player makes a move that threatens to capture the opponent's General on the next move (by the same piece or another piece), it is called a &lt;b&gt;Check&lt;/b&gt;. The checked side must respond to avoid check. Otherwise, that side loses</t>
+          <t>Horse</t>
         </is>
       </c>
       <c r="C368" s="2" t="inlineStr">
         <is>
-          <t>Nếu người chơi thực hiện một nước đi đe dọa bắt Tướng của đối phương ở nước đi tiếp theo (bằng chính quân cờ đó hoặc một quân cờ khác), thì đó được gọi là &lt;b&gt;Chiếu&lt;/b&gt;. Bên bị chiếu phải đáp trả để tránh bị chiếu. Nếu không sẽ bị xử thua</t>
+          <t>Mã</t>
         </is>
       </c>
     </row>
     <row r="369" ht="17" customHeight="1">
       <c r="A369" s="2" t="inlineStr">
         <is>
-          <t>guide.check.paragraph2</t>
+          <t>guide.horse.paragraph2</t>
         </is>
       </c>
       <c r="B369" s="2" t="inlineStr">
         <is>
-          <t>When the General is checked from any direction (including from behind), the checked side may respond in one of the following ways:</t>
+          <t>Moves in an &lt;b&gt;L-shape&lt;/b&gt; (one step orthogonally then one step diagonally outward). If the adjacent orthogonal point is occupied by any piece, the Horse is blocked and cannot move.</t>
         </is>
       </c>
       <c r="C369" s="2" t="inlineStr">
         <is>
-          <t>Tướng bị chiếu từ cả bốn hướng (bị chiếu cả từ phía sau) có thể ứng phó với nước chiếu tướng bằng một trong các cách sau:</t>
+          <t>Đi theo &lt;b&gt;đường chéo hình chữ nhật&lt;/b&gt; của hai ô vuông liền nhau. Nếu giao điểm liền kề bước thẳng dọc ngang có một quân khác đứng thì Mã bị cản, không đi được.</t>
         </is>
       </c>
     </row>
     <row r="370" ht="17" customHeight="1">
       <c r="A370" s="2" t="inlineStr">
         <is>
-          <t>guide.check.paragraph3</t>
+          <t>guide.cannon.paragraph1</t>
         </is>
       </c>
       <c r="B370" s="2" t="inlineStr">
         <is>
-          <t>Move the General to another position to escape check</t>
+          <t>Cannon</t>
         </is>
       </c>
       <c r="C370" s="2" t="inlineStr">
         <is>
-          <t>Di chuyển tướng sang vị trí khác để tránh nước chiếu</t>
+          <t>Pháo</t>
         </is>
       </c>
     </row>
     <row r="371" ht="17" customHeight="1">
       <c r="A371" s="2" t="inlineStr">
         <is>
-          <t>guide.check.paragraph4</t>
+          <t>guide.cannon.paragraph2</t>
         </is>
       </c>
       <c r="B371" s="2" t="inlineStr">
         <is>
-          <t>Capture the checking piece</t>
+          <t>Moves &lt;b&gt;horizontally or vertically&lt;/b&gt; like a Chariot when not capturing. To capture, it must &lt;b&gt;jump over exactly one piece&lt;/b&gt; to reach its target. If there are zero or more than one pieces between the Cannon and the target, it cannot capture.</t>
         </is>
       </c>
       <c r="C371" s="2" t="inlineStr">
         <is>
-          <t>Bắt quân đang chiếu</t>
+          <t>Đi ngang hoặc dọc giống Xe khi không bắt quân. Để bắt quân, nó phải &lt;b&gt;nhảy qua đúng một quân khác&lt;/b&gt; để đến mục tiêu. Nếu không có hoặc có nhiều hơn một quân giữa Pháo và mục tiêu, nó không thể bắt quân.</t>
         </is>
       </c>
     </row>
     <row r="372" ht="17" customHeight="1">
       <c r="A372" s="2" t="inlineStr">
         <is>
-          <t>guide.check.paragraph5</t>
+          <t>guide.soldier.paragraph1</t>
         </is>
       </c>
       <c r="B372" s="2" t="inlineStr">
         <is>
-          <t>Block the checking line with another piece to protect the General</t>
+          <t>Soldier</t>
         </is>
       </c>
       <c r="C372" s="2" t="inlineStr">
         <is>
-          <t>Dùng quân khác cản quân chiếu, đi quân che đỡ cho tướng</t>
+          <t>Tốt</t>
         </is>
       </c>
     </row>
     <row r="373" ht="17" customHeight="1">
       <c r="A373" s="2" t="inlineStr">
         <is>
-          <t>guide.check.paragraph6</t>
+          <t>guide.soldier.paragraph2</t>
         </is>
       </c>
       <c r="B373" s="2" t="inlineStr">
         <is>
-          <t>Repeatedly checking for more than 6 consecutive moves is not allowed</t>
+          <t>Moves &lt;b&gt;one step&lt;/b&gt; each turn. Before crossing the river, it can only move forward. After crossing the river, it may move &lt;b&gt;forward or sideways&lt;/b&gt;, but never backward.</t>
         </is>
       </c>
       <c r="C373" s="2" t="inlineStr">
         <is>
-          <t>Không được chiếu tướng quá 6 nước cờ liên tiếp</t>
+          <t>Mỗi nước đi &lt;b&gt;một bước&lt;/b&gt;. Khi chưa qua sông, Tốt chỉ được tiến. Khi Tốt đã qua sông được quyền &lt;b&gt;đi tiến và đi ngang&lt;/b&gt;, không được phép lùi.</t>
         </is>
       </c>
     </row>
     <row r="374" ht="17" customHeight="1">
       <c r="A374" s="2" t="inlineStr">
         <is>
-          <t>guide.result.paragraph1</t>
+          <t>guide.capturing.paragraph1</t>
         </is>
       </c>
       <c r="B374" s="2" t="inlineStr">
         <is>
-          <t>When one side gives Check and the other side has no legal way to protect the General, it is called a &lt;b&gt;Checkmate&lt;/b&gt;. The side that delivers Checkmate wins.</t>
+          <t>When a piece moves to an intersection occupied by an opponent's piece, it may &lt;b&gt;capture that piece&lt;/b&gt; and occupy its position.</t>
         </is>
       </c>
       <c r="C374" s="2" t="inlineStr">
         <is>
-          <t>Khi một bên chiếu Tướng mà bên còn lại không thể làm gì để bảo vệ Tướng thì được gọi là &lt;b&gt;Chiếu Hết&lt;/b&gt;, bên thực hiện được Chiếu Hết sẽ giành chiến thắng.</t>
+          <t>Khi một quân đi tới một giao điểm khác đã có quân đối phương đứng thì được quyền &lt;b&gt;bắt quân đó&lt;/b&gt;, đồng thời chiếm giữ vị trí quân bị bắt.</t>
         </is>
       </c>
     </row>
     <row r="375" ht="17" customHeight="1">
       <c r="A375" s="2" t="inlineStr">
         <is>
-          <t>guide.result.paragraph2</t>
+          <t>guide.capturing.paragraph2</t>
         </is>
       </c>
       <c r="B375" s="2" t="inlineStr">
         <is>
-          <t>If a player runs out of time for a single move (for example: 90s) without moving, the other side is awarded a &lt;b&gt;win&lt;/b&gt;.</t>
+          <t>You may not capture your own pieces. You may sacrifice your own pieces to be captured by the opponent, &lt;b&gt;except for the General&lt;/b&gt;.</t>
         </is>
       </c>
       <c r="C375" s="2" t="inlineStr">
         <is>
-          <t>Khi hết thời gian một nước đi (ví dụ: 90s) mà vẫn chưa di chuyển quân thì bên còn lại sẽ được &lt;b&gt;xử Thắng&lt;/b&gt;.</t>
+          <t>Không được bắt quân bên mình. Được phép cho đối phương bắt đầu quân mình chủ động hiến mình cho đối phương, &lt;b&gt;trừ Tướng&lt;/b&gt;.</t>
         </is>
       </c>
     </row>
     <row r="376" ht="17" customHeight="1">
       <c r="A376" s="2" t="inlineStr">
         <is>
-          <t>guide.result.paragraph3</t>
+          <t>guide.capturing.paragraph3</t>
         </is>
       </c>
       <c r="B376" s="2" t="inlineStr">
         <is>
-          <t>If a player runs out of total game time (for example: 5 minutes or 10 minutes), the other side is awarded a &lt;b&gt;win&lt;/b&gt;.</t>
+          <t>A captured piece is removed from the board. &lt;b&gt;Chasing one piece for more than 6 consecutive moves is not allowed&lt;/b&gt;.</t>
         </is>
       </c>
       <c r="C376" s="2" t="inlineStr">
         <is>
-          <t>Khi một bên hết thời gian ván đấu (ví dụ: 5 phút, 10 phút) thì bên còn lại sẽ được &lt;b&gt;xử Thắng&lt;/b&gt;.</t>
+          <t>Quân bị bắt phải bị loại và bị nhấc ra khỏi bàn cờ. &lt;b&gt;Không được đuổi 1 quân quá 6 nước cờ liên tiếp&lt;/b&gt;.</t>
         </is>
       </c>
     </row>
     <row r="377" ht="17" customHeight="1">
       <c r="A377" s="2" t="inlineStr">
         <is>
-          <t>guide.result.paragraph4</t>
+          <t>guide.check.paragraph1</t>
         </is>
       </c>
       <c r="B377" s="2" t="inlineStr">
         <is>
-          <t>If both sides have no pieces that have crossed the river, the game is declared a &lt;b&gt;draw&lt;/b&gt;. If one side still has pieces across the river but runs out of time, while the other side still has time but has no pieces across the river, the game is declared a &lt;b&gt;draw&lt;/b&gt;.</t>
+          <t>If a player makes a move that threatens to capture the opponent's General on the next move (by the same piece or another piece), it is called a &lt;b&gt;Check&lt;/b&gt;. The checked side must respond to avoid check. Otherwise, that side loses</t>
         </is>
       </c>
       <c r="C377" s="2" t="inlineStr">
         <is>
-          <t>Khi cả 2 bên đều không còn quân qua sông, ván đấu sẽ được &lt;b&gt;xử Hòa&lt;/b&gt;. Khi một bên còn quân qua sông nhưng cạn thời gian, một bên còn thời gian nhưng hết quân qua sông, ván đấu sẽ được &lt;b&gt;xử Hòa&lt;/b&gt;.</t>
+          <t>Nếu người chơi thực hiện một nước đi đe dọa bắt Tướng của đối phương ở nước đi tiếp theo (bằng chính quân cờ đó hoặc một quân cờ khác), thì đó được gọi là &lt;b&gt;Chiếu&lt;/b&gt;. Bên bị chiếu phải đáp trả để tránh bị chiếu. Nếu không sẽ bị xử thua</t>
         </is>
       </c>
     </row>
     <row r="378" ht="17" customHeight="1">
       <c r="A378" s="2" t="inlineStr">
         <is>
-          <t>guide.result.paragraph5</t>
+          <t>guide.check.paragraph2</t>
         </is>
       </c>
       <c r="B378" s="2" t="inlineStr">
         <is>
-          <t>Within 40 moves, if there is no capture and no Soldier advances by one square, the game is declared a &lt;b&gt;draw&lt;/b&gt;.</t>
+          <t>When the General is checked from any direction (including from behind), the checked side may respond in one of the following ways:</t>
         </is>
       </c>
       <c r="C378" s="2" t="inlineStr">
         <is>
-          <t>Trong vòng 40 nước nếu không phát sinh nước bắt quân, Tốt không tiến 1 ô thì ván đấu sẽ được &lt;b&gt;xử Hòa&lt;/b&gt;.</t>
+          <t>Tướng bị chiếu từ cả bốn hướng (bị chiếu cả từ phía sau) có thể ứng phó với nước chiếu tướng bằng một trong các cách sau:</t>
         </is>
       </c>
     </row>
     <row r="379" ht="17" customHeight="1">
       <c r="A379" s="2" t="inlineStr">
         <is>
-          <t>extra-money.title</t>
+          <t>guide.check.paragraph3</t>
         </is>
       </c>
       <c r="B379" s="2" t="inlineStr">
         <is>
-          <t>Daily tasks</t>
+          <t>Move the General to another position to escape check</t>
         </is>
       </c>
       <c r="C379" s="2" t="inlineStr">
         <is>
-          <t>Kiếm tiền</t>
+          <t>Di chuyển tướng sang vị trí khác để tránh nước chiếu</t>
         </is>
       </c>
     </row>
     <row r="380" ht="17" customHeight="1">
       <c r="A380" s="2" t="inlineStr">
         <is>
-          <t>extra-money.tab.lucky-wheel</t>
+          <t>guide.check.paragraph4</t>
         </is>
       </c>
       <c r="B380" s="2" t="inlineStr">
         <is>
-          <t>Lucky Wheel</t>
+          <t>Capture the checking piece</t>
         </is>
       </c>
       <c r="C380" s="2" t="inlineStr">
         <is>
-          <t>Vòng Quay May Mắn</t>
+          <t>Bắt quân đang chiếu</t>
         </is>
       </c>
     </row>
     <row r="381" ht="17" customHeight="1">
       <c r="A381" s="2" t="inlineStr">
         <is>
-          <t>extra-money.tab.bonus-coin</t>
+          <t>guide.check.paragraph5</t>
         </is>
       </c>
       <c r="B381" s="2" t="inlineStr">
         <is>
-          <t>Bonus Coin</t>
+          <t>Block the checking line with another piece to protect the General</t>
         </is>
       </c>
       <c r="C381" s="2" t="inlineStr">
         <is>
-          <t>Xu Thưởng</t>
+          <t>Dùng quân khác cản quân chiếu, đi quân che đỡ cho tướng</t>
         </is>
       </c>
     </row>
     <row r="382">
       <c r="A382" t="inlineStr">
         <is>
-          <t>extra-money.tab.daily-bonus</t>
+          <t>guide.check.paragraph6</t>
         </is>
       </c>
       <c r="B382" t="inlineStr">
         <is>
-          <t>Daily Bonus</t>
+          <t>Repeatedly checking for more than 6 consecutive moves is not allowed</t>
         </is>
       </c>
       <c r="C382" t="inlineStr">
         <is>
-          <t>Thưởng hàng ngày</t>
+          <t>Không được chiếu tướng quá 6 nước cờ liên tiếp</t>
         </is>
       </c>
     </row>
     <row r="383">
       <c r="A383" t="inlineStr">
         <is>
-          <t>extra-money.bonus-coin.subtitle</t>
+          <t>guide.result.paragraph1</t>
         </is>
       </c>
       <c r="B383" t="inlineStr">
         <is>
-          <t>Watch a short video to earn free coin</t>
+          <t>When one side gives Check and the other side has no legal way to protect the General, it is called a &lt;b&gt;Checkmate&lt;/b&gt;. The side that delivers Checkmate wins.</t>
         </is>
       </c>
       <c r="C383" t="inlineStr">
         <is>
-          <t>Xem video ngắn để nhận xu miễn phí</t>
+          <t>Khi một bên chiếu Tướng mà bên còn lại không thể làm gì để bảo vệ Tướng thì được gọi là &lt;b&gt;Chiếu Hết&lt;/b&gt;, bên thực hiện được Chiếu Hết sẽ giành chiến thắng.</t>
         </is>
       </c>
     </row>
     <row r="384">
       <c r="A384" t="inlineStr">
         <is>
-          <t>extra-money.bonus-coin.next-in</t>
+          <t>guide.result.paragraph2</t>
         </is>
       </c>
       <c r="B384" t="inlineStr">
         <is>
-          <t>Next in:</t>
+          <t>If a player runs out of time for a single move (for example: 90s) without moving, the other side is awarded a &lt;b&gt;win&lt;/b&gt;.</t>
         </is>
       </c>
       <c r="C384" t="inlineStr">
         <is>
-          <t>Lượt kế tiếp:</t>
+          <t>Khi hết thời gian một nước đi (ví dụ: 90s) mà vẫn chưa di chuyển quân thì bên còn lại sẽ được &lt;b&gt;xử Thắng&lt;/b&gt;.</t>
         </is>
       </c>
     </row>
     <row r="385">
       <c r="A385" t="inlineStr">
         <is>
-          <t>extra-money.bonus-coin.collect</t>
+          <t>guide.result.paragraph3</t>
         </is>
       </c>
       <c r="B385" t="inlineStr">
         <is>
-          <t>Collect</t>
+          <t>If a player runs out of total game time (for example: 5 minutes or 10 minutes), the other side is awarded a &lt;b&gt;win&lt;/b&gt;.</t>
         </is>
       </c>
       <c r="C385" t="inlineStr">
         <is>
-          <t>Thu thập</t>
+          <t>Khi một bên hết thời gian ván đấu (ví dụ: 5 phút, 10 phút) thì bên còn lại sẽ được &lt;b&gt;xử Thắng&lt;/b&gt;.</t>
         </is>
       </c>
     </row>
     <row r="386">
       <c r="A386" t="inlineStr">
         <is>
-          <t>extra-money.bonus-coin.watch-video</t>
+          <t>guide.result.paragraph4</t>
         </is>
       </c>
       <c r="B386" t="inlineStr">
         <is>
-          <t>Watch video</t>
+          <t>If both sides have no pieces that have crossed the river, the game is declared a &lt;b&gt;draw&lt;/b&gt;. If one side still has pieces across the river but runs out of time, while the other side still has time but has no pieces across the river, the game is declared a &lt;b&gt;draw&lt;/b&gt;.</t>
         </is>
       </c>
       <c r="C386" t="inlineStr">
         <is>
-          <t>Xem video</t>
+          <t>Khi cả 2 bên đều không còn quân qua sông, ván đấu sẽ được &lt;b&gt;xử Hòa&lt;/b&gt;. Khi một bên còn quân qua sông nhưng cạn thời gian, một bên còn thời gian nhưng hết quân qua sông, ván đấu sẽ được &lt;b&gt;xử Hòa&lt;/b&gt;.</t>
         </is>
       </c>
     </row>
     <row r="387">
       <c r="A387" t="inlineStr">
         <is>
-          <t>extra-money.daily-bonus.subtitle</t>
+          <t>guide.result.paragraph5</t>
         </is>
       </c>
       <c r="B387" t="inlineStr">
         <is>
-          <t>Login 7 days in a row to earn 4000 coin</t>
+          <t>Within 40 moves, if there is no capture and no Soldier advances by one square, the game is declared a &lt;b&gt;draw&lt;/b&gt;.</t>
         </is>
       </c>
       <c r="C387" t="inlineStr">
         <is>
-          <t>Đăng nhập 7 ngày liên tiếp để nhận 4000 xu</t>
+          <t>Trong vòng 40 nước nếu không phát sinh nước bắt quân, Tốt không tiến 1 ô thì ván đấu sẽ được &lt;b&gt;xử Hòa&lt;/b&gt;.</t>
         </is>
       </c>
     </row>
     <row r="388">
       <c r="A388" t="inlineStr">
         <is>
-          <t>extra-money.daily-bonus.day</t>
+          <t>extra-money.title</t>
         </is>
       </c>
       <c r="B388" t="inlineStr">
         <is>
-          <t>Day</t>
+          <t>Daily tasks</t>
         </is>
       </c>
       <c r="C388" t="inlineStr">
         <is>
-          <t>Ngày</t>
+          <t>Kiếm tiền</t>
         </is>
       </c>
     </row>
     <row r="389">
       <c r="A389" t="inlineStr">
         <is>
-          <t>extra-money.reward-ad.loading</t>
+          <t>extra-money.tab.lucky-wheel</t>
         </is>
       </c>
       <c r="B389" t="inlineStr">
         <is>
-          <t>Loading ad...</t>
+          <t>Lucky Wheel</t>
         </is>
       </c>
       <c r="C389" t="inlineStr">
         <is>
-          <t>Đang tải quảng cáo...</t>
+          <t>Vòng Quay May Mắn</t>
         </is>
       </c>
     </row>
     <row r="390">
       <c r="A390" t="inlineStr">
         <is>
-          <t>extra-money.reward-ad.error</t>
+          <t>extra-money.tab.bonus-coin</t>
         </is>
       </c>
       <c r="B390" t="inlineStr">
         <is>
-          <t>Could not load the ad. Please try again.</t>
+          <t>Bonus Coin</t>
         </is>
       </c>
       <c r="C390" t="inlineStr">
         <is>
-          <t>Không tải được quảng cáo. Vui lòng thử lại.</t>
+          <t>Xu Thưởng</t>
         </is>
       </c>
     </row>
     <row r="391">
       <c r="A391" t="inlineStr">
         <is>
-          <t>extra-money.reward-ad.retry</t>
+          <t>extra-money.tab.daily-bonus</t>
         </is>
       </c>
       <c r="B391" t="inlineStr">
         <is>
-          <t>Try again</t>
+          <t>Daily Bonus</t>
         </is>
       </c>
       <c r="C391" t="inlineStr">
         <is>
-          <t>Thử lại</t>
+          <t>Thưởng hàng ngày</t>
         </is>
       </c>
     </row>
     <row r="392">
       <c r="A392" t="inlineStr">
         <is>
-          <t>extra-money.reward-ad.close</t>
+          <t>extra-money.bonus-coin.subtitle</t>
         </is>
       </c>
       <c r="B392" t="inlineStr">
         <is>
-          <t>Close</t>
+          <t>Watch a short video to earn free coin</t>
         </is>
       </c>
       <c r="C392" t="inlineStr">
         <is>
-          <t>Đóng</t>
+          <t>Xem video ngắn để nhận xu miễn phí</t>
         </is>
       </c>
     </row>
     <row r="393">
       <c r="A393" t="inlineStr">
         <is>
-          <t>profile.button.save</t>
+          <t>extra-money.bonus-coin.next-in</t>
         </is>
       </c>
       <c r="B393" t="inlineStr">
         <is>
-          <t>Save</t>
+          <t>Next in:</t>
         </is>
       </c>
       <c r="C393" t="inlineStr">
         <is>
-          <t>Lưu</t>
+          <t>Lượt kế tiếp:</t>
         </is>
       </c>
     </row>
     <row r="394">
       <c r="A394" t="inlineStr">
         <is>
-          <t>profile.button.cancel</t>
+          <t>extra-money.bonus-coin.collect</t>
         </is>
       </c>
       <c r="B394" t="inlineStr">
         <is>
-          <t>Cancel</t>
+          <t>Collect</t>
         </is>
       </c>
       <c r="C394" t="inlineStr">
         <is>
-          <t>Huỷ</t>
+          <t>Thu thập</t>
         </is>
       </c>
     </row>
     <row r="395">
       <c r="A395" t="inlineStr">
         <is>
-          <t>change-password.title</t>
+          <t>extra-money.bonus-coin.watch-video</t>
         </is>
       </c>
       <c r="B395" t="inlineStr">
         <is>
-          <t>Change password</t>
+          <t>Watch video</t>
         </is>
       </c>
       <c r="C395" t="inlineStr">
         <is>
-          <t>Đổi mật khẩu</t>
+          <t>Xem video</t>
         </is>
       </c>
     </row>
     <row r="396">
       <c r="A396" t="inlineStr">
         <is>
-          <t>change-password.current.label</t>
+          <t>extra-money.daily-bonus.subtitle</t>
         </is>
       </c>
       <c r="B396" t="inlineStr">
         <is>
-          <t>Current password</t>
+          <t>Login 7 days in a row to earn 4000 coin</t>
         </is>
       </c>
       <c r="C396" t="inlineStr">
         <is>
-          <t>Mật khẩu hiện tại</t>
+          <t>Đăng nhập 7 ngày liên tiếp để nhận 4000 xu</t>
         </is>
       </c>
     </row>
     <row r="397">
       <c r="A397" t="inlineStr">
         <is>
-          <t>change-password.current.placeholder</t>
+          <t>extra-money.daily-bonus.day</t>
         </is>
       </c>
       <c r="B397" t="inlineStr">
         <is>
-          <t>Enter current password</t>
+          <t>Day</t>
         </is>
       </c>
       <c r="C397" t="inlineStr">
         <is>
-          <t>Nhập mật khẩu hiện tại</t>
+          <t>Ngày</t>
         </is>
       </c>
     </row>
     <row r="398">
       <c r="A398" t="inlineStr">
         <is>
-          <t>change-password.new.label</t>
+          <t>extra-money.reward-ad.loading</t>
         </is>
       </c>
       <c r="B398" t="inlineStr">
         <is>
-          <t>New password</t>
+          <t>Loading ad...</t>
         </is>
       </c>
       <c r="C398" t="inlineStr">
         <is>
-          <t>Mật khẩu mới</t>
+          <t>Đang tải quảng cáo...</t>
         </is>
       </c>
     </row>
     <row r="399">
       <c r="A399" t="inlineStr">
         <is>
-          <t>change-password.new.placeholder</t>
+          <t>extra-money.reward-ad.error</t>
         </is>
       </c>
       <c r="B399" t="inlineStr">
         <is>
-          <t>Enter new password</t>
+          <t>Could not load the ad. Please try again.</t>
         </is>
       </c>
       <c r="C399" t="inlineStr">
         <is>
-          <t>Nhập mật khẩu mới</t>
+          <t>Không tải được quảng cáo. Vui lòng thử lại.</t>
         </is>
       </c>
     </row>
     <row r="400">
       <c r="A400" t="inlineStr">
         <is>
-          <t>change-password.confirm.label</t>
+          <t>extra-money.reward-ad.retry</t>
         </is>
       </c>
       <c r="B400" t="inlineStr">
         <is>
-          <t>Confirm new password</t>
+          <t>Try again</t>
         </is>
       </c>
       <c r="C400" t="inlineStr">
         <is>
-          <t>Xác nhận mật khẩu mới</t>
+          <t>Thử lại</t>
         </is>
       </c>
     </row>
     <row r="401">
       <c r="A401" t="inlineStr">
         <is>
-          <t>change-password.confirm.placeholder</t>
+          <t>extra-money.reward-ad.close</t>
         </is>
       </c>
       <c r="B401" t="inlineStr">
         <is>
-          <t>Re-enter new password</t>
+          <t>Close</t>
         </is>
       </c>
       <c r="C401" t="inlineStr">
         <is>
-          <t>Nhập lại mật khẩu mới</t>
+          <t>Đóng</t>
         </is>
       </c>
     </row>
     <row r="402">
       <c r="A402" t="inlineStr">
         <is>
-          <t>change-password.confirm.mismatch</t>
+          <t>profile.button.save</t>
         </is>
       </c>
       <c r="B402" t="inlineStr">
         <is>
-          <t>Passwords do not match</t>
+          <t>Save</t>
         </is>
       </c>
       <c r="C402" t="inlineStr">
         <is>
-          <t>Mật khẩu xác nhận không khớp</t>
+          <t>Lưu</t>
         </is>
       </c>
     </row>
     <row r="403">
       <c r="A403" t="inlineStr">
         <is>
-          <t>change-password.show</t>
+          <t>profile.button.cancel</t>
         </is>
       </c>
       <c r="B403" t="inlineStr">
         <is>
-          <t>Show password</t>
+          <t>Cancel</t>
         </is>
       </c>
       <c r="C403" t="inlineStr">
         <is>
-          <t>Hiện mật khẩu</t>
+          <t>Huỷ</t>
         </is>
       </c>
     </row>
     <row r="404">
       <c r="A404" t="inlineStr">
         <is>
-          <t>change-password.hide</t>
+          <t>change-password.title</t>
         </is>
       </c>
       <c r="B404" t="inlineStr">
         <is>
-          <t>Hide password</t>
+          <t>Change password</t>
         </is>
       </c>
       <c r="C404" t="inlineStr">
         <is>
-          <t>Ẩn mật khẩu</t>
+          <t>Đổi mật khẩu</t>
         </is>
       </c>
     </row>
     <row r="405">
       <c r="A405" t="inlineStr">
         <is>
-          <t>change-password.submit</t>
+          <t>change-password.current.label</t>
         </is>
       </c>
       <c r="B405" t="inlineStr">
         <is>
-          <t>Change password</t>
+          <t>Current password</t>
         </is>
       </c>
       <c r="C405" t="inlineStr">
         <is>
-          <t>Đổi mật khẩu</t>
+          <t>Mật khẩu hiện tại</t>
         </is>
       </c>
     </row>
     <row r="406">
       <c r="A406" t="inlineStr">
         <is>
-          <t>change-password.submitting</t>
+          <t>change-password.current.placeholder</t>
         </is>
       </c>
       <c r="B406" t="inlineStr">
         <is>
-          <t>Changing...</t>
+          <t>Enter current password</t>
         </is>
       </c>
       <c r="C406" t="inlineStr">
         <is>
-          <t>Đang đổi...</t>
+          <t>Nhập mật khẩu hiện tại</t>
         </is>
       </c>
     </row>
     <row r="407">
       <c r="A407" t="inlineStr">
         <is>
-          <t>change-password.messages.success</t>
+          <t>change-password.new.label</t>
         </is>
       </c>
       <c r="B407" t="inlineStr">
         <is>
-          <t>Password changed successfully</t>
+          <t>New password</t>
         </is>
       </c>
       <c r="C407" t="inlineStr">
         <is>
-          <t>Đổi mật khẩu thành công</t>
+          <t>Mật khẩu mới</t>
         </is>
       </c>
     </row>
     <row r="408">
       <c r="A408" t="inlineStr">
         <is>
-          <t>change-password.messages.missing-fields</t>
+          <t>change-password.new.placeholder</t>
         </is>
       </c>
       <c r="B408" t="inlineStr">
         <is>
-          <t>Please fill in all fields</t>
+          <t>Enter new password</t>
         </is>
       </c>
       <c r="C408" t="inlineStr">
         <is>
-          <t>Vui lòng nhập đầy đủ thông tin</t>
+          <t>Nhập mật khẩu mới</t>
         </is>
       </c>
     </row>
     <row r="409">
       <c r="A409" t="inlineStr">
         <is>
-          <t>change-password.messages.weak-password</t>
+          <t>change-password.confirm.label</t>
         </is>
       </c>
       <c r="B409" t="inlineStr">
         <is>
-          <t>New password does not meet the requirements</t>
+          <t>Confirm new password</t>
         </is>
       </c>
       <c r="C409" t="inlineStr">
         <is>
-          <t>Mật khẩu mới không đạt yêu cầu</t>
+          <t>Xác nhận mật khẩu mới</t>
         </is>
       </c>
     </row>
     <row r="410">
       <c r="A410" t="inlineStr">
         <is>
-          <t>change-password.messages.same-as-current</t>
+          <t>change-password.confirm.placeholder</t>
         </is>
       </c>
       <c r="B410" t="inlineStr">
         <is>
-          <t>New password must be different from the current one</t>
+          <t>Re-enter new password</t>
         </is>
       </c>
       <c r="C410" t="inlineStr">
         <is>
-          <t>Mật khẩu mới phải khác mật khẩu hiện tại</t>
+          <t>Nhập lại mật khẩu mới</t>
         </is>
       </c>
     </row>
     <row r="411">
       <c r="A411" t="inlineStr">
         <is>
-          <t>change-password.messages.incorrect-current-password</t>
+          <t>change-password.confirm.mismatch</t>
         </is>
       </c>
       <c r="B411" t="inlineStr">
         <is>
-          <t>Current password is incorrect</t>
+          <t>Passwords do not match</t>
         </is>
       </c>
       <c r="C411" t="inlineStr">
         <is>
-          <t>Mật khẩu hiện tại không đúng</t>
+          <t>Mật khẩu xác nhận không khớp</t>
         </is>
       </c>
     </row>
     <row r="412">
       <c r="A412" t="inlineStr">
         <is>
-          <t>change-password.messages.user-not-found</t>
+          <t>change-password.show</t>
         </is>
       </c>
       <c r="B412" t="inlineStr">
         <is>
-          <t>User not found</t>
+          <t>Show password</t>
         </is>
       </c>
       <c r="C412" t="inlineStr">
         <is>
-          <t>Không tìm thấy người dùng</t>
+          <t>Hiện mật khẩu</t>
         </is>
       </c>
     </row>
     <row r="413">
       <c r="A413" t="inlineStr">
         <is>
-          <t>change-password.messages.unauthorized</t>
+          <t>change-password.hide</t>
         </is>
       </c>
       <c r="B413" t="inlineStr">
         <is>
-          <t>Session expired. Please sign in again.</t>
+          <t>Hide password</t>
         </is>
       </c>
       <c r="C413" t="inlineStr">
         <is>
-          <t>Phiên đăng nhập đã hết hạn. Vui lòng đăng nhập lại.</t>
+          <t>Ẩn mật khẩu</t>
         </is>
       </c>
     </row>
     <row r="414">
       <c r="A414" t="inlineStr">
         <is>
+          <t>change-password.submit</t>
+        </is>
+      </c>
+      <c r="B414" t="inlineStr">
+        <is>
+          <t>Change password</t>
+        </is>
+      </c>
+      <c r="C414" t="inlineStr">
+        <is>
+          <t>Đổi mật khẩu</t>
+        </is>
+      </c>
+    </row>
+    <row r="415">
+      <c r="A415" t="inlineStr">
+        <is>
+          <t>change-password.submitting</t>
+        </is>
+      </c>
+      <c r="B415" t="inlineStr">
+        <is>
+          <t>Changing...</t>
+        </is>
+      </c>
+      <c r="C415" t="inlineStr">
+        <is>
+          <t>Đang đổi...</t>
+        </is>
+      </c>
+    </row>
+    <row r="416">
+      <c r="A416" t="inlineStr">
+        <is>
+          <t>change-password.messages.success</t>
+        </is>
+      </c>
+      <c r="B416" t="inlineStr">
+        <is>
+          <t>Password changed successfully</t>
+        </is>
+      </c>
+      <c r="C416" t="inlineStr">
+        <is>
+          <t>Đổi mật khẩu thành công</t>
+        </is>
+      </c>
+    </row>
+    <row r="417">
+      <c r="A417" t="inlineStr">
+        <is>
+          <t>change-password.messages.missing-fields</t>
+        </is>
+      </c>
+      <c r="B417" t="inlineStr">
+        <is>
+          <t>Please fill in all fields</t>
+        </is>
+      </c>
+      <c r="C417" t="inlineStr">
+        <is>
+          <t>Vui lòng nhập đầy đủ thông tin</t>
+        </is>
+      </c>
+    </row>
+    <row r="418">
+      <c r="A418" t="inlineStr">
+        <is>
+          <t>change-password.messages.weak-password</t>
+        </is>
+      </c>
+      <c r="B418" t="inlineStr">
+        <is>
+          <t>New password does not meet the requirements</t>
+        </is>
+      </c>
+      <c r="C418" t="inlineStr">
+        <is>
+          <t>Mật khẩu mới không đạt yêu cầu</t>
+        </is>
+      </c>
+    </row>
+    <row r="419">
+      <c r="A419" t="inlineStr">
+        <is>
+          <t>change-password.messages.same-as-current</t>
+        </is>
+      </c>
+      <c r="B419" t="inlineStr">
+        <is>
+          <t>New password must be different from the current one</t>
+        </is>
+      </c>
+      <c r="C419" t="inlineStr">
+        <is>
+          <t>Mật khẩu mới phải khác mật khẩu hiện tại</t>
+        </is>
+      </c>
+    </row>
+    <row r="420">
+      <c r="A420" t="inlineStr">
+        <is>
+          <t>change-password.messages.incorrect-current-password</t>
+        </is>
+      </c>
+      <c r="B420" t="inlineStr">
+        <is>
+          <t>Current password is incorrect</t>
+        </is>
+      </c>
+      <c r="C420" t="inlineStr">
+        <is>
+          <t>Mật khẩu hiện tại không đúng</t>
+        </is>
+      </c>
+    </row>
+    <row r="421">
+      <c r="A421" t="inlineStr">
+        <is>
+          <t>change-password.messages.user-not-found</t>
+        </is>
+      </c>
+      <c r="B421" t="inlineStr">
+        <is>
+          <t>User not found</t>
+        </is>
+      </c>
+      <c r="C421" t="inlineStr">
+        <is>
+          <t>Không tìm thấy người dùng</t>
+        </is>
+      </c>
+    </row>
+    <row r="422">
+      <c r="A422" t="inlineStr">
+        <is>
+          <t>change-password.messages.unauthorized</t>
+        </is>
+      </c>
+      <c r="B422" t="inlineStr">
+        <is>
+          <t>Session expired. Please sign in again.</t>
+        </is>
+      </c>
+      <c r="C422" t="inlineStr">
+        <is>
+          <t>Phiên đăng nhập đã hết hạn. Vui lòng đăng nhập lại.</t>
+        </is>
+      </c>
+    </row>
+    <row r="423">
+      <c r="A423" t="inlineStr">
+        <is>
           <t>change-password.messages.internal-server-error</t>
         </is>
       </c>
-      <c r="B414" t="inlineStr">
+      <c r="B423" t="inlineStr">
         <is>
           <t>Something went wrong. Please try again.</t>
         </is>
       </c>
-      <c r="C414" t="inlineStr">
+      <c r="C423" t="inlineStr">
         <is>
           <t>Đã có lỗi xảy ra. Vui lòng thử lại.</t>
         </is>
       </c>
-    </row>
-    <row r="415">
-      <c r="A415" t="inlineStr"/>
-      <c r="B415" t="inlineStr"/>
-      <c r="C415" t="inlineStr"/>
-    </row>
-    <row r="416">
-      <c r="A416" t="inlineStr"/>
-      <c r="B416" t="inlineStr"/>
-      <c r="C416" t="inlineStr"/>
-    </row>
-    <row r="417">
-      <c r="A417" t="inlineStr"/>
-      <c r="B417" t="inlineStr"/>
-      <c r="C417" t="inlineStr"/>
-    </row>
-    <row r="418">
-      <c r="A418" t="inlineStr"/>
-      <c r="B418" t="inlineStr"/>
-      <c r="C418" t="inlineStr"/>
-    </row>
-    <row r="419">
-      <c r="A419" t="inlineStr"/>
-      <c r="B419" t="inlineStr"/>
-      <c r="C419" t="inlineStr"/>
-    </row>
-    <row r="420">
-      <c r="A420" t="inlineStr"/>
-      <c r="B420" t="inlineStr"/>
-      <c r="C420" t="inlineStr"/>
-    </row>
-    <row r="421">
-      <c r="A421" t="inlineStr"/>
-      <c r="B421" t="inlineStr"/>
-      <c r="C421" t="inlineStr"/>
-    </row>
-    <row r="422">
-      <c r="A422" t="inlineStr"/>
-      <c r="B422" t="inlineStr"/>
-      <c r="C422" t="inlineStr"/>
-    </row>
-    <row r="423">
-      <c r="A423" t="inlineStr"/>
-      <c r="B423" t="inlineStr"/>
-      <c r="C423" t="inlineStr"/>
     </row>
     <row r="424">
       <c r="A424" t="inlineStr"/>
@@ -7465,6 +7573,51 @@
       <c r="A433" t="inlineStr"/>
       <c r="B433" t="inlineStr"/>
       <c r="C433" t="inlineStr"/>
+    </row>
+    <row r="434">
+      <c r="A434" t="inlineStr"/>
+      <c r="B434" t="inlineStr"/>
+      <c r="C434" t="inlineStr"/>
+    </row>
+    <row r="435">
+      <c r="A435" t="inlineStr"/>
+      <c r="B435" t="inlineStr"/>
+      <c r="C435" t="inlineStr"/>
+    </row>
+    <row r="436">
+      <c r="A436" t="inlineStr"/>
+      <c r="B436" t="inlineStr"/>
+      <c r="C436" t="inlineStr"/>
+    </row>
+    <row r="437">
+      <c r="A437" t="inlineStr"/>
+      <c r="B437" t="inlineStr"/>
+      <c r="C437" t="inlineStr"/>
+    </row>
+    <row r="438">
+      <c r="A438" t="inlineStr"/>
+      <c r="B438" t="inlineStr"/>
+      <c r="C438" t="inlineStr"/>
+    </row>
+    <row r="439">
+      <c r="A439" t="inlineStr"/>
+      <c r="B439" t="inlineStr"/>
+      <c r="C439" t="inlineStr"/>
+    </row>
+    <row r="440">
+      <c r="A440" t="inlineStr"/>
+      <c r="B440" t="inlineStr"/>
+      <c r="C440" t="inlineStr"/>
+    </row>
+    <row r="441">
+      <c r="A441" t="inlineStr"/>
+      <c r="B441" t="inlineStr"/>
+      <c r="C441" t="inlineStr"/>
+    </row>
+    <row r="442">
+      <c r="A442" t="inlineStr"/>
+      <c r="B442" t="inlineStr"/>
+      <c r="C442" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
highlight in all moves and disable undo in pvp game
</commit_message>
<xml_diff>
--- a/tools/languages.xlsx
+++ b/tools/languages.xlsx
@@ -325,7 +325,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C433"/>
+  <dimension ref="A1:C434"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -5810,1571 +5810,1583 @@
     <row r="323" ht="54" customHeight="1">
       <c r="A323" s="2" t="inlineStr">
         <is>
-          <t>undo.messages.spectator-cannot-undo</t>
+          <t>undo.messages.pve-only</t>
         </is>
       </c>
       <c r="B323" s="2" t="inlineStr">
         <is>
-          <t>Spectators cannot undo moves</t>
+          <t>Undo is only available in PvE rooms</t>
         </is>
       </c>
       <c r="C323" s="2" t="inlineStr">
         <is>
-          <t>Người xem không thể hoàn tác nước đi</t>
+          <t>Hoàn tác chỉ khả dụng trong phòng PvE</t>
         </is>
       </c>
     </row>
     <row r="324" ht="18" customHeight="1">
       <c r="A324" s="2" t="inlineStr">
         <is>
-          <t>undo.messages.no-moves</t>
+          <t>undo.messages.spectator-cannot-undo</t>
         </is>
       </c>
       <c r="B324" s="2" t="inlineStr">
         <is>
-          <t>No moves to undo</t>
+          <t>Spectators cannot undo moves</t>
         </is>
       </c>
       <c r="C324" s="2" t="inlineStr">
         <is>
-          <t>Không có nước đi để hoàn tác</t>
+          <t>Người xem không thể hoàn tác nước đi</t>
         </is>
       </c>
     </row>
     <row r="325" ht="72" customHeight="1">
       <c r="A325" s="2" t="inlineStr">
         <is>
-          <t>undo.messages.delete-failed</t>
+          <t>undo.messages.no-moves</t>
         </is>
       </c>
       <c r="B325" s="2" t="inlineStr">
         <is>
-          <t>Failed to undo move</t>
+          <t>No moves to undo</t>
         </is>
       </c>
       <c r="C325" s="2" t="inlineStr">
         <is>
-          <t>Không thể hoàn tác nước đi</t>
+          <t>Không có nước đi để hoàn tác</t>
         </is>
       </c>
     </row>
     <row r="326" ht="18" customHeight="1">
       <c r="A326" s="2" t="inlineStr">
         <is>
-          <t>undo.messages.undo-limit-exceeded</t>
+          <t>undo.messages.delete-failed</t>
         </is>
       </c>
       <c r="B326" s="2" t="inlineStr">
         <is>
-          <t>Maximum 3 undo per game exceeded</t>
+          <t>Failed to undo move</t>
         </is>
       </c>
       <c r="C326" s="2" t="inlineStr">
         <is>
-          <t>Đã đạt tối đa 3 lần hoàn tác trong trò chơi</t>
+          <t>Không thể hoàn tác nước đi</t>
         </is>
       </c>
     </row>
     <row r="327" ht="90" customHeight="1">
       <c r="A327" s="2" t="inlineStr">
         <is>
-          <t>undo.messages.success</t>
+          <t>undo.messages.undo-limit-exceeded</t>
         </is>
       </c>
       <c r="B327" s="2" t="inlineStr">
         <is>
-          <t>Move undone successfully</t>
+          <t>Maximum 3 undo per game exceeded</t>
         </is>
       </c>
       <c r="C327" s="2" t="inlineStr">
         <is>
-          <t>Hoàn tác nước đi thành công</t>
+          <t>Đã đạt tối đa 3 lần hoàn tác trong trò chơi</t>
         </is>
       </c>
     </row>
     <row r="328" ht="18" customHeight="1">
       <c r="A328" s="2" t="inlineStr">
         <is>
-          <t>undo.messages.internal-server-error</t>
+          <t>undo.messages.success</t>
         </is>
       </c>
       <c r="B328" s="2" t="inlineStr">
         <is>
-          <t>Internal server error</t>
+          <t>Move undone successfully</t>
         </is>
       </c>
       <c r="C328" s="2" t="inlineStr">
         <is>
-          <t>Lỗi máy chủ nội bộ</t>
+          <t>Hoàn tác nước đi thành công</t>
         </is>
       </c>
     </row>
     <row r="329" ht="72" customHeight="1">
       <c r="A329" s="2" t="inlineStr">
         <is>
-          <t>player-history.messages.invalid-user-id</t>
+          <t>undo.messages.internal-server-error</t>
         </is>
       </c>
       <c r="B329" s="2" t="inlineStr">
         <is>
-          <t>Invalid user ID</t>
+          <t>Internal server error</t>
         </is>
       </c>
       <c r="C329" s="2" t="inlineStr">
         <is>
-          <t>ID người dùng không hợp lệ</t>
+          <t>Lỗi máy chủ nội bộ</t>
         </is>
       </c>
     </row>
     <row r="330" ht="54" customHeight="1">
       <c r="A330" s="2" t="inlineStr">
         <is>
-          <t>player-history.messages.success</t>
+          <t>player-history.messages.invalid-user-id</t>
         </is>
       </c>
       <c r="B330" s="2" t="inlineStr">
         <is>
-          <t>Fetch game history successfully</t>
+          <t>Invalid user ID</t>
         </is>
       </c>
       <c r="C330" s="2" t="inlineStr">
         <is>
-          <t>Lấy lịch sử trò chơi thành công</t>
+          <t>ID người dùng không hợp lệ</t>
         </is>
       </c>
     </row>
     <row r="331" ht="54" customHeight="1">
       <c r="A331" s="2" t="inlineStr">
         <is>
-          <t>validate-token.messages.success</t>
+          <t>player-history.messages.success</t>
         </is>
       </c>
       <c r="B331" s="2" t="inlineStr">
         <is>
-          <t>Token is valid</t>
+          <t>Fetch game history successfully</t>
         </is>
       </c>
       <c r="C331" s="2" t="inlineStr">
         <is>
-          <t>Token hợp lệ</t>
+          <t>Lấy lịch sử trò chơi thành công</t>
         </is>
       </c>
     </row>
     <row r="332" ht="54" customHeight="1">
       <c r="A332" s="2" t="inlineStr">
         <is>
-          <t>guide.section.objective</t>
+          <t>validate-token.messages.success</t>
         </is>
       </c>
       <c r="B332" s="2" t="inlineStr">
         <is>
-          <t>Objective of the game</t>
+          <t>Token is valid</t>
         </is>
       </c>
       <c r="C332" s="2" t="inlineStr">
         <is>
-          <t>Mục tiêu của trò chơi</t>
+          <t>Token hợp lệ</t>
         </is>
       </c>
     </row>
     <row r="333" ht="90" customHeight="1">
       <c r="A333" s="2" t="inlineStr">
         <is>
-          <t>guide.section.pieces</t>
+          <t>guide.section.objective</t>
         </is>
       </c>
       <c r="B333" s="2" t="inlineStr">
         <is>
-          <t>Pieces</t>
+          <t>Objective of the game</t>
         </is>
       </c>
       <c r="C333" s="2" t="inlineStr">
         <is>
-          <t>Quân cờ</t>
+          <t>Mục tiêu của trò chơi</t>
         </is>
       </c>
     </row>
     <row r="334" ht="54" customHeight="1">
       <c r="A334" s="2" t="inlineStr">
         <is>
-          <t>guide.section.moving-pieces</t>
+          <t>guide.section.pieces</t>
         </is>
       </c>
       <c r="B334" s="2" t="inlineStr">
         <is>
-          <t>Moving pieces</t>
+          <t>Pieces</t>
         </is>
       </c>
       <c r="C334" s="2" t="inlineStr">
         <is>
-          <t>Đi quân</t>
+          <t>Quân cờ</t>
         </is>
       </c>
     </row>
     <row r="335" ht="36" customHeight="1">
       <c r="A335" s="2" t="inlineStr">
         <is>
-          <t>guide.section.capturing</t>
+          <t>guide.section.moving-pieces</t>
         </is>
       </c>
       <c r="B335" s="2" t="inlineStr">
         <is>
-          <t>Capturing</t>
+          <t>Moving pieces</t>
         </is>
       </c>
       <c r="C335" s="2" t="inlineStr">
         <is>
-          <t>Bắt quân</t>
+          <t>Đi quân</t>
         </is>
       </c>
     </row>
     <row r="336" ht="18" customHeight="1">
       <c r="A336" s="2" t="inlineStr">
         <is>
-          <t>guide.section.check</t>
+          <t>guide.section.capturing</t>
         </is>
       </c>
       <c r="B336" s="2" t="inlineStr">
         <is>
-          <t>Check</t>
+          <t>Capturing</t>
         </is>
       </c>
       <c r="C336" s="2" t="inlineStr">
         <is>
-          <t>Chiếu tướng</t>
+          <t>Bắt quân</t>
         </is>
       </c>
     </row>
     <row r="337" ht="36" customHeight="1">
       <c r="A337" s="2" t="inlineStr">
         <is>
-          <t>guide.section.result</t>
+          <t>guide.section.check</t>
         </is>
       </c>
       <c r="B337" s="2" t="inlineStr">
         <is>
-          <t>Result</t>
+          <t>Check</t>
         </is>
       </c>
       <c r="C337" s="2" t="inlineStr">
         <is>
-          <t>Kết quả</t>
+          <t>Chiếu tướng</t>
         </is>
       </c>
     </row>
     <row r="338" ht="36" customHeight="1">
       <c r="A338" s="2" t="inlineStr">
         <is>
-          <t>guide.table.piece</t>
+          <t>guide.section.result</t>
         </is>
       </c>
       <c r="B338" s="2" t="inlineStr">
         <is>
-          <t>Piece</t>
+          <t>Result</t>
         </is>
       </c>
       <c r="C338" s="2" t="inlineStr">
         <is>
-          <t>Quân</t>
+          <t>Kết quả</t>
         </is>
       </c>
     </row>
     <row r="339" ht="72" customHeight="1">
       <c r="A339" s="2" t="inlineStr">
         <is>
-          <t>guide.table.symbol</t>
+          <t>guide.table.piece</t>
         </is>
       </c>
       <c r="B339" s="2" t="inlineStr">
         <is>
-          <t>Symbol</t>
+          <t>Piece</t>
         </is>
       </c>
       <c r="C339" s="2" t="inlineStr">
         <is>
-          <t>Ký hiệu</t>
+          <t>Quân</t>
         </is>
       </c>
     </row>
     <row r="340" ht="54" customHeight="1">
       <c r="A340" s="2" t="inlineStr">
         <is>
-          <t>guide.table.quantity</t>
+          <t>guide.table.symbol</t>
         </is>
       </c>
       <c r="B340" s="2" t="inlineStr">
         <is>
-          <t>Quantity</t>
+          <t>Symbol</t>
         </is>
       </c>
       <c r="C340" s="2" t="inlineStr">
         <is>
-          <t>Số lượng</t>
+          <t>Ký hiệu</t>
         </is>
       </c>
     </row>
     <row r="341" ht="54" customHeight="1">
       <c r="A341" s="2" t="inlineStr">
         <is>
-          <t>guide.objective.paragraph1</t>
+          <t>guide.table.quantity</t>
         </is>
       </c>
       <c r="B341" s="2" t="inlineStr">
         <is>
-          <t>A match is played between two players: one controls the Red pieces, and the other controls the Black pieces. The objective of each player is to use their pieces on the board to &lt;b&gt;checkmate&lt;/b&gt; the opponent's General, and win the game.</t>
+          <t>Quantity</t>
         </is>
       </c>
       <c r="C341" s="2" t="inlineStr">
         <is>
-          <t>Ván cờ được tiến hành giữa 2 đấu thủ, một người cầm Quân Đỏ, một người cầm Quân Đen. Mục đích của mỗi đấu thủ là tìm mọi cách sử dụng các quân trên bàn cờ để &lt;b&gt;chiếu bí Tướng&lt;/b&gt; của đối phương, giành thắng lợi.</t>
+          <t>Số lượng</t>
         </is>
       </c>
     </row>
     <row r="342" ht="90" customHeight="1">
       <c r="A342" s="2" t="inlineStr">
         <is>
-          <t>guide.pieces.paragraph1</t>
+          <t>guide.objective.paragraph1</t>
         </is>
       </c>
       <c r="B342" s="2" t="inlineStr">
         <is>
-          <t>At the start of each game, there must be 32 pieces in total, consisting of &lt;b&gt;7 piece types&lt;/b&gt; split evenly between both sides: 16 Red pieces and 16 Black pieces. The 7 piece types with their symbols and quantities are as follows:</t>
+          <t>A match is played between two players: one controls the Red pieces, and the other controls the Black pieces. The objective of each player is to use their pieces on the board to &lt;b&gt;checkmate&lt;/b&gt; the opponent's General, and win the game.</t>
         </is>
       </c>
       <c r="C342" s="2" t="inlineStr">
         <is>
-          <t>Mỗi ván cờ lúc bắt đầu phải có đủ 32 quân, gồm 7 loại chia đều cho mỗi bên gồm 16 quân Đỏ và 16 quân Đen. &lt;b&gt;7 loại quân&lt;/b&gt; có ký hiệu và số lượng như sau:</t>
+          <t>Ván cờ được tiến hành giữa 2 đấu thủ, một người cầm Quân Đỏ, một người cầm Quân Đen. Mục đích của mỗi đấu thủ là tìm mọi cách sử dụng các quân trên bàn cờ để &lt;b&gt;chiếu bí Tướng&lt;/b&gt; của đối phương, giành thắng lợi.</t>
         </is>
       </c>
     </row>
     <row r="343" ht="54" customHeight="1">
       <c r="A343" s="2" t="inlineStr">
         <is>
-          <t>guide.piece.general</t>
+          <t>guide.pieces.paragraph1</t>
         </is>
       </c>
       <c r="B343" s="2" t="inlineStr">
         <is>
-          <t>General</t>
+          <t>At the start of each game, there must be 32 pieces in total, consisting of &lt;b&gt;7 piece types&lt;/b&gt; split evenly between both sides: 16 Red pieces and 16 Black pieces. The 7 piece types with their symbols and quantities are as follows:</t>
         </is>
       </c>
       <c r="C343" s="2" t="inlineStr">
         <is>
-          <t>Tướng</t>
+          <t>Mỗi ván cờ lúc bắt đầu phải có đủ 32 quân, gồm 7 loại chia đều cho mỗi bên gồm 16 quân Đỏ và 16 quân Đen. &lt;b&gt;7 loại quân&lt;/b&gt; có ký hiệu và số lượng như sau:</t>
         </is>
       </c>
     </row>
     <row r="344" ht="18" customHeight="1">
       <c r="A344" s="2" t="inlineStr">
         <is>
-          <t>guide.piece.advisor</t>
+          <t>guide.piece.general</t>
         </is>
       </c>
       <c r="B344" s="2" t="inlineStr">
         <is>
-          <t>Advisor</t>
+          <t>General</t>
         </is>
       </c>
       <c r="C344" s="2" t="inlineStr">
         <is>
-          <t>Sĩ</t>
+          <t>Tướng</t>
         </is>
       </c>
     </row>
     <row r="345" ht="18" customHeight="1">
       <c r="A345" s="2" t="inlineStr">
         <is>
-          <t>guide.piece.elephant</t>
+          <t>guide.piece.advisor</t>
         </is>
       </c>
       <c r="B345" s="2" t="inlineStr">
         <is>
-          <t>Elephant</t>
+          <t>Advisor</t>
         </is>
       </c>
       <c r="C345" s="2" t="inlineStr">
         <is>
-          <t>Tượng</t>
+          <t>Sĩ</t>
         </is>
       </c>
     </row>
     <row r="346" ht="36" customHeight="1">
       <c r="A346" s="2" t="inlineStr">
         <is>
-          <t>guide.piece.chariot</t>
+          <t>guide.piece.elephant</t>
         </is>
       </c>
       <c r="B346" s="2" t="inlineStr">
         <is>
-          <t>Chariot</t>
+          <t>Elephant</t>
         </is>
       </c>
       <c r="C346" s="2" t="inlineStr">
         <is>
-          <t>Xe</t>
+          <t>Tượng</t>
         </is>
       </c>
     </row>
     <row r="347" ht="18" customHeight="1">
       <c r="A347" s="2" t="inlineStr">
         <is>
-          <t>guide.piece.horse</t>
+          <t>guide.piece.chariot</t>
         </is>
       </c>
       <c r="B347" s="2" t="inlineStr">
         <is>
-          <t>Horse</t>
+          <t>Chariot</t>
         </is>
       </c>
       <c r="C347" s="2" t="inlineStr">
         <is>
-          <t>Mã</t>
+          <t>Xe</t>
         </is>
       </c>
     </row>
     <row r="348" ht="18" customHeight="1">
       <c r="A348" s="2" t="inlineStr">
         <is>
-          <t>guide.piece.cannon</t>
+          <t>guide.piece.horse</t>
         </is>
       </c>
       <c r="B348" s="2" t="inlineStr">
         <is>
-          <t>Cannon</t>
+          <t>Horse</t>
         </is>
       </c>
       <c r="C348" s="2" t="inlineStr">
         <is>
-          <t>Pháo</t>
+          <t>Mã</t>
         </is>
       </c>
     </row>
     <row r="349" ht="36" customHeight="1">
       <c r="A349" s="2" t="inlineStr">
         <is>
-          <t>guide.piece.soldier</t>
+          <t>guide.piece.cannon</t>
         </is>
       </c>
       <c r="B349" s="2" t="inlineStr">
         <is>
-          <t>Soldier</t>
+          <t>Cannon</t>
         </is>
       </c>
       <c r="C349" s="2" t="inlineStr">
         <is>
-          <t>Tốt</t>
+          <t>Pháo</t>
         </is>
       </c>
     </row>
     <row r="350" ht="18" customHeight="1">
       <c r="A350" s="2" t="inlineStr">
         <is>
-          <t>guide.moving-pieces.paragraph1</t>
+          <t>guide.piece.soldier</t>
         </is>
       </c>
       <c r="B350" s="2" t="inlineStr">
         <is>
-          <t>On each turn, each side may move only one of its own pieces according to the rules. The movement rules are as follows:</t>
+          <t>Soldier</t>
         </is>
       </c>
       <c r="C350" s="2" t="inlineStr">
         <is>
-          <t>Mỗi nước đi, mỗi bên chỉ được di chuyển quân của mình theo đúng quy định. Quy định di chuyển của các quân như sau:</t>
+          <t>Tốt</t>
         </is>
       </c>
     </row>
     <row r="351" ht="36" customHeight="1">
       <c r="A351" s="2" t="inlineStr">
         <is>
-          <t>guide.general.paragraph1</t>
+          <t>guide.moving-pieces.paragraph1</t>
         </is>
       </c>
       <c r="B351" s="2" t="inlineStr">
         <is>
-          <t>General</t>
+          <t>On each turn, each side may move only one of its own pieces according to the rules. The movement rules are as follows:</t>
         </is>
       </c>
       <c r="C351" s="2" t="inlineStr">
         <is>
-          <t>Tướng</t>
+          <t>Mỗi nước đi, mỗi bên chỉ được di chuyển quân của mình theo đúng quy định. Quy định di chuyển của các quân như sau:</t>
         </is>
       </c>
     </row>
     <row r="352" ht="18" customHeight="1">
       <c r="A352" s="2" t="inlineStr">
         <is>
-          <t>guide.general.paragraph2</t>
+          <t>guide.general.paragraph1</t>
         </is>
       </c>
       <c r="B352" s="2" t="inlineStr">
         <is>
-          <t>Moves one step &lt;b&gt;horizontally or vertically&lt;/b&gt; within the palace. The two Generals may not face each other directly on the same file. If they are facing each other, there must be at least one piece of either side placed between them.</t>
+          <t>General</t>
         </is>
       </c>
       <c r="C352" s="2" t="inlineStr">
         <is>
-          <t>Mỗi nước được đi một bước &lt;b&gt;ngang hoặc dọc&lt;/b&gt; tùy ý trong cung Tướng. Hai tướng của 2 bên không được đối mặt nhau trực tiếp trên cùng một đường thẳng. Nếu đối mặt, bắt buộc phải có quân của bất kỳ bên nào đứng che mặt.</t>
+          <t>Tướng</t>
         </is>
       </c>
     </row>
     <row r="353" ht="18" customHeight="1">
       <c r="A353" s="2" t="inlineStr">
         <is>
-          <t>guide.advisor.paragraph1</t>
+          <t>guide.general.paragraph2</t>
         </is>
       </c>
       <c r="B353" s="2" t="inlineStr">
         <is>
-          <t>Advisor</t>
+          <t>Moves one step &lt;b&gt;horizontally or vertically&lt;/b&gt; within the palace. The two Generals may not face each other directly on the same file. If they are facing each other, there must be at least one piece of either side placed between them.</t>
         </is>
       </c>
       <c r="C353" s="2" t="inlineStr">
         <is>
-          <t>Sĩ</t>
+          <t>Mỗi nước được đi một bước &lt;b&gt;ngang hoặc dọc&lt;/b&gt; tùy ý trong cung Tướng. Hai tướng của 2 bên không được đối mặt nhau trực tiếp trên cùng một đường thẳng. Nếu đối mặt, bắt buộc phải có quân của bất kỳ bên nào đứng che mặt.</t>
         </is>
       </c>
     </row>
     <row r="354" ht="18" customHeight="1">
       <c r="A354" s="2" t="inlineStr">
         <is>
-          <t>guide.advisor.paragraph2</t>
+          <t>guide.advisor.paragraph1</t>
         </is>
       </c>
       <c r="B354" s="2" t="inlineStr">
         <is>
-          <t>Moves one step &lt;b&gt;diagonally&lt;/b&gt; within the palace.</t>
+          <t>Advisor</t>
         </is>
       </c>
       <c r="C354" s="2" t="inlineStr">
         <is>
-          <t>Mỗi nước &lt;b&gt;đi chéo một bước&lt;/b&gt; trong cung Tướng.</t>
+          <t>Sĩ</t>
         </is>
       </c>
     </row>
     <row r="355" ht="18" customHeight="1">
       <c r="A355" s="2" t="inlineStr">
         <is>
-          <t>guide.elephant.paragraph1</t>
+          <t>guide.advisor.paragraph2</t>
         </is>
       </c>
       <c r="B355" s="2" t="inlineStr">
         <is>
-          <t>Elephant</t>
+          <t>Moves one step &lt;b&gt;diagonally&lt;/b&gt; within the palace.</t>
         </is>
       </c>
       <c r="C355" s="2" t="inlineStr">
         <is>
-          <t>Tượng</t>
+          <t>Mỗi nước &lt;b&gt;đi chéo một bước&lt;/b&gt; trong cung Tướng.</t>
         </is>
       </c>
     </row>
     <row r="356" ht="18" customHeight="1">
       <c r="A356" s="2" t="inlineStr">
         <is>
-          <t>guide.elephant.paragraph2</t>
+          <t>guide.elephant.paragraph1</t>
         </is>
       </c>
       <c r="B356" s="2" t="inlineStr">
         <is>
-          <t>Moves &lt;b&gt;two steps diagonally&lt;/b&gt; on its own side of the board and may not cross the river. If there is another piece on the midpoint of that diagonal path, the Elephant is blocked and cannot move.</t>
+          <t>Elephant</t>
         </is>
       </c>
       <c r="C356" s="2" t="inlineStr">
         <is>
-          <t>Mỗi nước &lt;b&gt;đi chéo hai bước&lt;/b&gt; tại trận địa bên mình, không được qua sông. Nếu ở giữa đường chéo đó có quân khác đứng thì quân Tượng bị cản, không đi được.</t>
+          <t>Tượng</t>
         </is>
       </c>
     </row>
     <row r="357" ht="17" customHeight="1">
       <c r="A357" s="2" t="inlineStr">
         <is>
-          <t>guide.chariot.paragraph1</t>
+          <t>guide.elephant.paragraph2</t>
         </is>
       </c>
       <c r="B357" s="2" t="inlineStr">
         <is>
-          <t>Chariot</t>
+          <t>Moves &lt;b&gt;two steps diagonally&lt;/b&gt; on its own side of the board and may not cross the river. If there is another piece on the midpoint of that diagonal path, the Elephant is blocked and cannot move.</t>
         </is>
       </c>
       <c r="C357" s="2" t="inlineStr">
         <is>
-          <t>Xe</t>
+          <t>Mỗi nước &lt;b&gt;đi chéo hai bước&lt;/b&gt; tại trận địa bên mình, không được qua sông. Nếu ở giữa đường chéo đó có quân khác đứng thì quân Tượng bị cản, không đi được.</t>
         </is>
       </c>
     </row>
     <row r="358" ht="18" customHeight="1">
       <c r="A358" s="2" t="inlineStr">
         <is>
-          <t>guide.chariot.paragraph2</t>
+          <t>guide.chariot.paragraph1</t>
         </is>
       </c>
       <c r="B358" s="2" t="inlineStr">
         <is>
-          <t>Moves &lt;b&gt;horizontally or vertically&lt;/b&gt; with no limit on distance, as long as no piece blocks the path.</t>
+          <t>Chariot</t>
         </is>
       </c>
       <c r="C358" s="2" t="inlineStr">
         <is>
-          <t>Mỗi nước được &lt;b&gt;đi dọc hoặc đi ngang&lt;/b&gt;, không hạn chế số bước đi nếu không có quân khác cản đường.</t>
+          <t>Xe</t>
         </is>
       </c>
     </row>
     <row r="359" ht="18" customHeight="1">
       <c r="A359" s="2" t="inlineStr">
         <is>
-          <t>guide.horse.paragraph1</t>
+          <t>guide.chariot.paragraph2</t>
         </is>
       </c>
       <c r="B359" s="2" t="inlineStr">
         <is>
-          <t>Horse</t>
+          <t>Moves &lt;b&gt;horizontally or vertically&lt;/b&gt; with no limit on distance, as long as no piece blocks the path.</t>
         </is>
       </c>
       <c r="C359" s="2" t="inlineStr">
         <is>
-          <t>Mã</t>
+          <t>Mỗi nước được &lt;b&gt;đi dọc hoặc đi ngang&lt;/b&gt;, không hạn chế số bước đi nếu không có quân khác cản đường.</t>
         </is>
       </c>
     </row>
     <row r="360" ht="18" customHeight="1">
       <c r="A360" s="2" t="inlineStr">
         <is>
-          <t>guide.horse.paragraph2</t>
+          <t>guide.horse.paragraph1</t>
         </is>
       </c>
       <c r="B360" s="2" t="inlineStr">
         <is>
-          <t>Moves in an &lt;b&gt;L-shape&lt;/b&gt; (one step orthogonally then one step diagonally outward). If the adjacent orthogonal point is occupied by any piece, the Horse is blocked and cannot move.</t>
+          <t>Horse</t>
         </is>
       </c>
       <c r="C360" s="2" t="inlineStr">
         <is>
-          <t>Đi theo &lt;b&gt;đường chéo hình chữ nhật&lt;/b&gt; của hai ô vuông liền nhau. Nếu giao điểm liền kề bước thẳng dọc ngang có một quân khác đứng thì Mã bị cản, không đi được.</t>
+          <t>Mã</t>
         </is>
       </c>
     </row>
     <row r="361" ht="18" customHeight="1">
       <c r="A361" s="2" t="inlineStr">
         <is>
-          <t>guide.cannon.paragraph1</t>
+          <t>guide.horse.paragraph2</t>
         </is>
       </c>
       <c r="B361" s="2" t="inlineStr">
         <is>
-          <t>Cannon</t>
+          <t>Moves in an &lt;b&gt;L-shape&lt;/b&gt; (one step orthogonally then one step diagonally outward). If the adjacent orthogonal point is occupied by any piece, the Horse is blocked and cannot move.</t>
         </is>
       </c>
       <c r="C361" s="2" t="inlineStr">
         <is>
-          <t>Pháo</t>
+          <t>Đi theo &lt;b&gt;đường chéo hình chữ nhật&lt;/b&gt; của hai ô vuông liền nhau. Nếu giao điểm liền kề bước thẳng dọc ngang có một quân khác đứng thì Mã bị cản, không đi được.</t>
         </is>
       </c>
     </row>
     <row r="362" ht="18" customHeight="1">
       <c r="A362" s="2" t="inlineStr">
         <is>
-          <t>guide.cannon.paragraph2</t>
+          <t>guide.cannon.paragraph1</t>
         </is>
       </c>
       <c r="B362" s="2" t="inlineStr">
         <is>
-          <t>Moves &lt;b&gt;horizontally or vertically&lt;/b&gt; like a Chariot when not capturing. To capture, it must &lt;b&gt;jump over exactly one piece&lt;/b&gt; to reach its target. If there are zero or more than one pieces between the Cannon and the target, it cannot capture.</t>
+          <t>Cannon</t>
         </is>
       </c>
       <c r="C362" s="2" t="inlineStr">
         <is>
-          <t>Đi ngang hoặc dọc giống Xe khi không bắt quân. Để bắt quân, nó phải &lt;b&gt;nhảy qua đúng một quân khác&lt;/b&gt; để đến mục tiêu. Nếu không có hoặc có nhiều hơn một quân giữa Pháo và mục tiêu, nó không thể bắt quân.</t>
+          <t>Pháo</t>
         </is>
       </c>
     </row>
     <row r="363" ht="18" customHeight="1">
       <c r="A363" s="2" t="inlineStr">
         <is>
-          <t>guide.soldier.paragraph1</t>
+          <t>guide.cannon.paragraph2</t>
         </is>
       </c>
       <c r="B363" s="2" t="inlineStr">
         <is>
-          <t>Soldier</t>
+          <t>Moves &lt;b&gt;horizontally or vertically&lt;/b&gt; like a Chariot when not capturing. To capture, it must &lt;b&gt;jump over exactly one piece&lt;/b&gt; to reach its target. If there are zero or more than one pieces between the Cannon and the target, it cannot capture.</t>
         </is>
       </c>
       <c r="C363" s="2" t="inlineStr">
         <is>
-          <t>Tốt</t>
+          <t>Đi ngang hoặc dọc giống Xe khi không bắt quân. Để bắt quân, nó phải &lt;b&gt;nhảy qua đúng một quân khác&lt;/b&gt; để đến mục tiêu. Nếu không có hoặc có nhiều hơn một quân giữa Pháo và mục tiêu, nó không thể bắt quân.</t>
         </is>
       </c>
     </row>
     <row r="364" ht="17" customHeight="1">
       <c r="A364" s="2" t="inlineStr">
         <is>
-          <t>guide.soldier.paragraph2</t>
+          <t>guide.soldier.paragraph1</t>
         </is>
       </c>
       <c r="B364" s="2" t="inlineStr">
         <is>
-          <t>Moves &lt;b&gt;one step&lt;/b&gt; each turn. Before crossing the river, it can only move forward. After crossing the river, it may move &lt;b&gt;forward or sideways&lt;/b&gt;, but never backward.</t>
+          <t>Soldier</t>
         </is>
       </c>
       <c r="C364" s="2" t="inlineStr">
         <is>
-          <t>Mỗi nước đi &lt;b&gt;một bước&lt;/b&gt;. Khi chưa qua sông, Tốt chỉ được tiến. Khi Tốt đã qua sông được quyền &lt;b&gt;đi tiến và đi ngang&lt;/b&gt;, không được phép lùi.</t>
+          <t>Tốt</t>
         </is>
       </c>
     </row>
     <row r="365" ht="17" customHeight="1">
       <c r="A365" s="2" t="inlineStr">
         <is>
-          <t>guide.capturing.paragraph1</t>
+          <t>guide.soldier.paragraph2</t>
         </is>
       </c>
       <c r="B365" s="2" t="inlineStr">
         <is>
-          <t>When a piece moves to an intersection occupied by an opponent's piece, it may &lt;b&gt;capture that piece&lt;/b&gt; and occupy its position.</t>
+          <t>Moves &lt;b&gt;one step&lt;/b&gt; each turn. Before crossing the river, it can only move forward. After crossing the river, it may move &lt;b&gt;forward or sideways&lt;/b&gt;, but never backward.</t>
         </is>
       </c>
       <c r="C365" s="2" t="inlineStr">
         <is>
-          <t>Khi một quân đi tới một giao điểm khác đã có quân đối phương đứng thì được quyền &lt;b&gt;bắt quân đó&lt;/b&gt;, đồng thời chiếm giữ vị trí quân bị bắt.</t>
+          <t>Mỗi nước đi &lt;b&gt;một bước&lt;/b&gt;. Khi chưa qua sông, Tốt chỉ được tiến. Khi Tốt đã qua sông được quyền &lt;b&gt;đi tiến và đi ngang&lt;/b&gt;, không được phép lùi.</t>
         </is>
       </c>
     </row>
     <row r="366" ht="17" customHeight="1">
       <c r="A366" s="2" t="inlineStr">
         <is>
-          <t>guide.capturing.paragraph2</t>
+          <t>guide.capturing.paragraph1</t>
         </is>
       </c>
       <c r="B366" s="2" t="inlineStr">
         <is>
-          <t>You may not capture your own pieces. You may sacrifice your own pieces to be captured by the opponent, &lt;b&gt;except for the General&lt;/b&gt;.</t>
+          <t>When a piece moves to an intersection occupied by an opponent's piece, it may &lt;b&gt;capture that piece&lt;/b&gt; and occupy its position.</t>
         </is>
       </c>
       <c r="C366" s="2" t="inlineStr">
         <is>
-          <t>Không được bắt quân bên mình. Được phép cho đối phương bắt đầu quân mình chủ động hiến mình cho đối phương, &lt;b&gt;trừ Tướng&lt;/b&gt;.</t>
+          <t>Khi một quân đi tới một giao điểm khác đã có quân đối phương đứng thì được quyền &lt;b&gt;bắt quân đó&lt;/b&gt;, đồng thời chiếm giữ vị trí quân bị bắt.</t>
         </is>
       </c>
     </row>
     <row r="367" ht="17" customHeight="1">
       <c r="A367" s="2" t="inlineStr">
         <is>
-          <t>guide.capturing.paragraph3</t>
+          <t>guide.capturing.paragraph2</t>
         </is>
       </c>
       <c r="B367" s="2" t="inlineStr">
         <is>
-          <t>A captured piece is removed from the board. &lt;b&gt;Chasing one piece for more than 6 consecutive moves is not allowed&lt;/b&gt;.</t>
+          <t>You may not capture your own pieces. You may sacrifice your own pieces to be captured by the opponent, &lt;b&gt;except for the General&lt;/b&gt;.</t>
         </is>
       </c>
       <c r="C367" s="2" t="inlineStr">
         <is>
-          <t>Quân bị bắt phải bị loại và bị nhấc ra khỏi bàn cờ. &lt;b&gt;Không được đuổi 1 quân quá 6 nước cờ liên tiếp&lt;/b&gt;.</t>
+          <t>Không được bắt quân bên mình. Được phép cho đối phương bắt đầu quân mình chủ động hiến mình cho đối phương, &lt;b&gt;trừ Tướng&lt;/b&gt;.</t>
         </is>
       </c>
     </row>
     <row r="368" ht="17" customHeight="1">
       <c r="A368" s="2" t="inlineStr">
         <is>
-          <t>guide.check.paragraph1</t>
+          <t>guide.capturing.paragraph3</t>
         </is>
       </c>
       <c r="B368" s="2" t="inlineStr">
         <is>
-          <t>If a player makes a move that threatens to capture the opponent's General on the next move (by the same piece or another piece), it is called a &lt;b&gt;Check&lt;/b&gt;. The checked side must respond to avoid check. Otherwise, that side loses</t>
+          <t>A captured piece is removed from the board. &lt;b&gt;Chasing one piece for more than 6 consecutive moves is not allowed&lt;/b&gt;.</t>
         </is>
       </c>
       <c r="C368" s="2" t="inlineStr">
         <is>
-          <t>Nếu người chơi thực hiện một nước đi đe dọa bắt Tướng của đối phương ở nước đi tiếp theo (bằng chính quân cờ đó hoặc một quân cờ khác), thì đó được gọi là &lt;b&gt;Chiếu&lt;/b&gt;. Bên bị chiếu phải đáp trả để tránh bị chiếu. Nếu không sẽ bị xử thua</t>
+          <t>Quân bị bắt phải bị loại và bị nhấc ra khỏi bàn cờ. &lt;b&gt;Không được đuổi 1 quân quá 6 nước cờ liên tiếp&lt;/b&gt;.</t>
         </is>
       </c>
     </row>
     <row r="369" ht="17" customHeight="1">
       <c r="A369" s="2" t="inlineStr">
         <is>
-          <t>guide.check.paragraph2</t>
+          <t>guide.check.paragraph1</t>
         </is>
       </c>
       <c r="B369" s="2" t="inlineStr">
         <is>
-          <t>When the General is checked from any direction (including from behind), the checked side may respond in one of the following ways:</t>
+          <t>If a player makes a move that threatens to capture the opponent's General on the next move (by the same piece or another piece), it is called a &lt;b&gt;Check&lt;/b&gt;. The checked side must respond to avoid check. Otherwise, that side loses</t>
         </is>
       </c>
       <c r="C369" s="2" t="inlineStr">
         <is>
-          <t>Tướng bị chiếu từ cả bốn hướng (bị chiếu cả từ phía sau) có thể ứng phó với nước chiếu tướng bằng một trong các cách sau:</t>
+          <t>Nếu người chơi thực hiện một nước đi đe dọa bắt Tướng của đối phương ở nước đi tiếp theo (bằng chính quân cờ đó hoặc một quân cờ khác), thì đó được gọi là &lt;b&gt;Chiếu&lt;/b&gt;. Bên bị chiếu phải đáp trả để tránh bị chiếu. Nếu không sẽ bị xử thua</t>
         </is>
       </c>
     </row>
     <row r="370" ht="17" customHeight="1">
       <c r="A370" s="2" t="inlineStr">
         <is>
-          <t>guide.check.paragraph3</t>
+          <t>guide.check.paragraph2</t>
         </is>
       </c>
       <c r="B370" s="2" t="inlineStr">
         <is>
-          <t>Move the General to another position to escape check</t>
+          <t>When the General is checked from any direction (including from behind), the checked side may respond in one of the following ways:</t>
         </is>
       </c>
       <c r="C370" s="2" t="inlineStr">
         <is>
-          <t>Di chuyển tướng sang vị trí khác để tránh nước chiếu</t>
+          <t>Tướng bị chiếu từ cả bốn hướng (bị chiếu cả từ phía sau) có thể ứng phó với nước chiếu tướng bằng một trong các cách sau:</t>
         </is>
       </c>
     </row>
     <row r="371" ht="17" customHeight="1">
       <c r="A371" s="2" t="inlineStr">
         <is>
-          <t>guide.check.paragraph4</t>
+          <t>guide.check.paragraph3</t>
         </is>
       </c>
       <c r="B371" s="2" t="inlineStr">
         <is>
-          <t>Capture the checking piece</t>
+          <t>Move the General to another position to escape check</t>
         </is>
       </c>
       <c r="C371" s="2" t="inlineStr">
         <is>
-          <t>Bắt quân đang chiếu</t>
+          <t>Di chuyển tướng sang vị trí khác để tránh nước chiếu</t>
         </is>
       </c>
     </row>
     <row r="372" ht="17" customHeight="1">
       <c r="A372" s="2" t="inlineStr">
         <is>
-          <t>guide.check.paragraph5</t>
+          <t>guide.check.paragraph4</t>
         </is>
       </c>
       <c r="B372" s="2" t="inlineStr">
         <is>
-          <t>Block the checking line with another piece to protect the General</t>
+          <t>Capture the checking piece</t>
         </is>
       </c>
       <c r="C372" s="2" t="inlineStr">
         <is>
-          <t>Dùng quân khác cản quân chiếu, đi quân che đỡ cho tướng</t>
+          <t>Bắt quân đang chiếu</t>
         </is>
       </c>
     </row>
     <row r="373" ht="17" customHeight="1">
       <c r="A373" s="2" t="inlineStr">
         <is>
-          <t>guide.check.paragraph6</t>
+          <t>guide.check.paragraph5</t>
         </is>
       </c>
       <c r="B373" s="2" t="inlineStr">
         <is>
-          <t>Repeatedly checking for more than 6 consecutive moves is not allowed</t>
+          <t>Block the checking line with another piece to protect the General</t>
         </is>
       </c>
       <c r="C373" s="2" t="inlineStr">
         <is>
-          <t>Không được chiếu tướng quá 6 nước cờ liên tiếp</t>
+          <t>Dùng quân khác cản quân chiếu, đi quân che đỡ cho tướng</t>
         </is>
       </c>
     </row>
     <row r="374" ht="17" customHeight="1">
       <c r="A374" s="2" t="inlineStr">
         <is>
-          <t>guide.result.paragraph1</t>
+          <t>guide.check.paragraph6</t>
         </is>
       </c>
       <c r="B374" s="2" t="inlineStr">
         <is>
-          <t>When one side gives Check and the other side has no legal way to protect the General, it is called a &lt;b&gt;Checkmate&lt;/b&gt;. The side that delivers Checkmate wins.</t>
+          <t>Repeatedly checking for more than 6 consecutive moves is not allowed</t>
         </is>
       </c>
       <c r="C374" s="2" t="inlineStr">
         <is>
-          <t>Khi một bên chiếu Tướng mà bên còn lại không thể làm gì để bảo vệ Tướng thì được gọi là &lt;b&gt;Chiếu Hết&lt;/b&gt;, bên thực hiện được Chiếu Hết sẽ giành chiến thắng.</t>
+          <t>Không được chiếu tướng quá 6 nước cờ liên tiếp</t>
         </is>
       </c>
     </row>
     <row r="375" ht="17" customHeight="1">
       <c r="A375" s="2" t="inlineStr">
         <is>
-          <t>guide.result.paragraph2</t>
+          <t>guide.result.paragraph1</t>
         </is>
       </c>
       <c r="B375" s="2" t="inlineStr">
         <is>
-          <t>If a player runs out of time for a single move (for example: 90s) without moving, the other side is awarded a &lt;b&gt;win&lt;/b&gt;.</t>
+          <t>When one side gives Check and the other side has no legal way to protect the General, it is called a &lt;b&gt;Checkmate&lt;/b&gt;. The side that delivers Checkmate wins.</t>
         </is>
       </c>
       <c r="C375" s="2" t="inlineStr">
         <is>
-          <t>Khi hết thời gian một nước đi (ví dụ: 90s) mà vẫn chưa di chuyển quân thì bên còn lại sẽ được &lt;b&gt;xử Thắng&lt;/b&gt;.</t>
+          <t>Khi một bên chiếu Tướng mà bên còn lại không thể làm gì để bảo vệ Tướng thì được gọi là &lt;b&gt;Chiếu Hết&lt;/b&gt;, bên thực hiện được Chiếu Hết sẽ giành chiến thắng.</t>
         </is>
       </c>
     </row>
     <row r="376" ht="17" customHeight="1">
       <c r="A376" s="2" t="inlineStr">
         <is>
-          <t>guide.result.paragraph3</t>
+          <t>guide.result.paragraph2</t>
         </is>
       </c>
       <c r="B376" s="2" t="inlineStr">
         <is>
-          <t>If a player runs out of total game time (for example: 5 minutes or 10 minutes), the other side is awarded a &lt;b&gt;win&lt;/b&gt;.</t>
+          <t>If a player runs out of time for a single move (for example: 90s) without moving, the other side is awarded a &lt;b&gt;win&lt;/b&gt;.</t>
         </is>
       </c>
       <c r="C376" s="2" t="inlineStr">
         <is>
-          <t>Khi một bên hết thời gian ván đấu (ví dụ: 5 phút, 10 phút) thì bên còn lại sẽ được &lt;b&gt;xử Thắng&lt;/b&gt;.</t>
+          <t>Khi hết thời gian một nước đi (ví dụ: 90s) mà vẫn chưa di chuyển quân thì bên còn lại sẽ được &lt;b&gt;xử Thắng&lt;/b&gt;.</t>
         </is>
       </c>
     </row>
     <row r="377" ht="17" customHeight="1">
       <c r="A377" s="2" t="inlineStr">
         <is>
-          <t>guide.result.paragraph4</t>
+          <t>guide.result.paragraph3</t>
         </is>
       </c>
       <c r="B377" s="2" t="inlineStr">
         <is>
-          <t>If both sides have no pieces that have crossed the river, the game is declared a &lt;b&gt;draw&lt;/b&gt;. If one side still has pieces across the river but runs out of time, while the other side still has time but has no pieces across the river, the game is declared a &lt;b&gt;draw&lt;/b&gt;.</t>
+          <t>If a player runs out of total game time (for example: 5 minutes or 10 minutes), the other side is awarded a &lt;b&gt;win&lt;/b&gt;.</t>
         </is>
       </c>
       <c r="C377" s="2" t="inlineStr">
         <is>
-          <t>Khi cả 2 bên đều không còn quân qua sông, ván đấu sẽ được &lt;b&gt;xử Hòa&lt;/b&gt;. Khi một bên còn quân qua sông nhưng cạn thời gian, một bên còn thời gian nhưng hết quân qua sông, ván đấu sẽ được &lt;b&gt;xử Hòa&lt;/b&gt;.</t>
+          <t>Khi một bên hết thời gian ván đấu (ví dụ: 5 phút, 10 phút) thì bên còn lại sẽ được &lt;b&gt;xử Thắng&lt;/b&gt;.</t>
         </is>
       </c>
     </row>
     <row r="378" ht="17" customHeight="1">
       <c r="A378" s="2" t="inlineStr">
         <is>
-          <t>guide.result.paragraph5</t>
+          <t>guide.result.paragraph4</t>
         </is>
       </c>
       <c r="B378" s="2" t="inlineStr">
         <is>
-          <t>Within 40 moves, if there is no capture and no Soldier advances by one square, the game is declared a &lt;b&gt;draw&lt;/b&gt;.</t>
+          <t>If both sides have no pieces that have crossed the river, the game is declared a &lt;b&gt;draw&lt;/b&gt;. If one side still has pieces across the river but runs out of time, while the other side still has time but has no pieces across the river, the game is declared a &lt;b&gt;draw&lt;/b&gt;.</t>
         </is>
       </c>
       <c r="C378" s="2" t="inlineStr">
         <is>
-          <t>Trong vòng 40 nước nếu không phát sinh nước bắt quân, Tốt không tiến 1 ô thì ván đấu sẽ được &lt;b&gt;xử Hòa&lt;/b&gt;.</t>
+          <t>Khi cả 2 bên đều không còn quân qua sông, ván đấu sẽ được &lt;b&gt;xử Hòa&lt;/b&gt;. Khi một bên còn quân qua sông nhưng cạn thời gian, một bên còn thời gian nhưng hết quân qua sông, ván đấu sẽ được &lt;b&gt;xử Hòa&lt;/b&gt;.</t>
         </is>
       </c>
     </row>
     <row r="379" ht="17" customHeight="1">
       <c r="A379" s="2" t="inlineStr">
         <is>
-          <t>extra-money.title</t>
+          <t>guide.result.paragraph5</t>
         </is>
       </c>
       <c r="B379" s="2" t="inlineStr">
         <is>
-          <t>Daily tasks</t>
+          <t>Within 40 moves, if there is no capture and no Soldier advances by one square, the game is declared a &lt;b&gt;draw&lt;/b&gt;.</t>
         </is>
       </c>
       <c r="C379" s="2" t="inlineStr">
         <is>
-          <t>Kiếm tiền</t>
+          <t>Trong vòng 40 nước nếu không phát sinh nước bắt quân, Tốt không tiến 1 ô thì ván đấu sẽ được &lt;b&gt;xử Hòa&lt;/b&gt;.</t>
         </is>
       </c>
     </row>
     <row r="380" ht="17" customHeight="1">
       <c r="A380" s="2" t="inlineStr">
         <is>
-          <t>extra-money.tab.lucky-wheel</t>
+          <t>extra-money.title</t>
         </is>
       </c>
       <c r="B380" s="2" t="inlineStr">
         <is>
-          <t>Lucky Wheel</t>
+          <t>Daily tasks</t>
         </is>
       </c>
       <c r="C380" s="2" t="inlineStr">
         <is>
-          <t>Vòng Quay May Mắn</t>
+          <t>Kiếm tiền</t>
         </is>
       </c>
     </row>
     <row r="381" ht="17" customHeight="1">
       <c r="A381" s="2" t="inlineStr">
         <is>
-          <t>extra-money.tab.bonus-coin</t>
+          <t>extra-money.tab.lucky-wheel</t>
         </is>
       </c>
       <c r="B381" s="2" t="inlineStr">
         <is>
-          <t>Bonus Coin</t>
+          <t>Lucky Wheel</t>
         </is>
       </c>
       <c r="C381" s="2" t="inlineStr">
         <is>
-          <t>Xu Thưởng</t>
+          <t>Vòng Quay May Mắn</t>
         </is>
       </c>
     </row>
     <row r="382">
       <c r="A382" t="inlineStr">
         <is>
-          <t>extra-money.tab.daily-bonus</t>
+          <t>extra-money.tab.bonus-coin</t>
         </is>
       </c>
       <c r="B382" t="inlineStr">
         <is>
-          <t>Daily Bonus</t>
+          <t>Bonus Coin</t>
         </is>
       </c>
       <c r="C382" t="inlineStr">
         <is>
-          <t>Thưởng hàng ngày</t>
+          <t>Xu Thưởng</t>
         </is>
       </c>
     </row>
     <row r="383">
       <c r="A383" t="inlineStr">
         <is>
-          <t>extra-money.bonus-coin.subtitle</t>
+          <t>extra-money.tab.daily-bonus</t>
         </is>
       </c>
       <c r="B383" t="inlineStr">
         <is>
-          <t>Watch a short video to earn free coin</t>
+          <t>Daily Bonus</t>
         </is>
       </c>
       <c r="C383" t="inlineStr">
         <is>
-          <t>Xem video ngắn để nhận xu miễn phí</t>
+          <t>Thưởng hàng ngày</t>
         </is>
       </c>
     </row>
     <row r="384">
       <c r="A384" t="inlineStr">
         <is>
-          <t>extra-money.bonus-coin.next-in</t>
+          <t>extra-money.bonus-coin.subtitle</t>
         </is>
       </c>
       <c r="B384" t="inlineStr">
         <is>
-          <t>Next in:</t>
+          <t>Watch a short video to earn free coin</t>
         </is>
       </c>
       <c r="C384" t="inlineStr">
         <is>
-          <t>Lượt kế tiếp:</t>
+          <t>Xem video ngắn để nhận xu miễn phí</t>
         </is>
       </c>
     </row>
     <row r="385">
       <c r="A385" t="inlineStr">
         <is>
-          <t>extra-money.bonus-coin.collect</t>
+          <t>extra-money.bonus-coin.next-in</t>
         </is>
       </c>
       <c r="B385" t="inlineStr">
         <is>
-          <t>Collect</t>
+          <t>Next in:</t>
         </is>
       </c>
       <c r="C385" t="inlineStr">
         <is>
-          <t>Thu thập</t>
+          <t>Lượt kế tiếp:</t>
         </is>
       </c>
     </row>
     <row r="386">
       <c r="A386" t="inlineStr">
         <is>
-          <t>extra-money.bonus-coin.watch-video</t>
+          <t>extra-money.bonus-coin.collect</t>
         </is>
       </c>
       <c r="B386" t="inlineStr">
         <is>
-          <t>Watch video</t>
+          <t>Collect</t>
         </is>
       </c>
       <c r="C386" t="inlineStr">
         <is>
-          <t>Xem video</t>
+          <t>Thu thập</t>
         </is>
       </c>
     </row>
     <row r="387">
       <c r="A387" t="inlineStr">
         <is>
-          <t>extra-money.daily-bonus.subtitle</t>
+          <t>extra-money.bonus-coin.watch-video</t>
         </is>
       </c>
       <c r="B387" t="inlineStr">
         <is>
-          <t>Login 7 days in a row to earn 4000 coin</t>
+          <t>Watch video</t>
         </is>
       </c>
       <c r="C387" t="inlineStr">
         <is>
-          <t>Đăng nhập 7 ngày liên tiếp để nhận 4000 xu</t>
+          <t>Xem video</t>
         </is>
       </c>
     </row>
     <row r="388">
       <c r="A388" t="inlineStr">
         <is>
-          <t>extra-money.daily-bonus.day</t>
+          <t>extra-money.daily-bonus.subtitle</t>
         </is>
       </c>
       <c r="B388" t="inlineStr">
         <is>
-          <t>Day</t>
+          <t>Login 7 days in a row to earn 4000 coin</t>
         </is>
       </c>
       <c r="C388" t="inlineStr">
         <is>
-          <t>Ngày</t>
+          <t>Đăng nhập 7 ngày liên tiếp để nhận 4000 xu</t>
         </is>
       </c>
     </row>
     <row r="389">
       <c r="A389" t="inlineStr">
         <is>
-          <t>extra-money.reward-ad.loading</t>
+          <t>extra-money.daily-bonus.day</t>
         </is>
       </c>
       <c r="B389" t="inlineStr">
         <is>
-          <t>Loading ad...</t>
+          <t>Day</t>
         </is>
       </c>
       <c r="C389" t="inlineStr">
         <is>
-          <t>Đang tải quảng cáo...</t>
+          <t>Ngày</t>
         </is>
       </c>
     </row>
     <row r="390">
       <c r="A390" t="inlineStr">
         <is>
-          <t>extra-money.reward-ad.error</t>
+          <t>extra-money.reward-ad.loading</t>
         </is>
       </c>
       <c r="B390" t="inlineStr">
         <is>
-          <t>Could not load the ad. Please try again.</t>
+          <t>Loading ad...</t>
         </is>
       </c>
       <c r="C390" t="inlineStr">
         <is>
-          <t>Không tải được quảng cáo. Vui lòng thử lại.</t>
+          <t>Đang tải quảng cáo...</t>
         </is>
       </c>
     </row>
     <row r="391">
       <c r="A391" t="inlineStr">
         <is>
-          <t>extra-money.reward-ad.retry</t>
+          <t>extra-money.reward-ad.error</t>
         </is>
       </c>
       <c r="B391" t="inlineStr">
         <is>
-          <t>Try again</t>
+          <t>Could not load the ad. Please try again.</t>
         </is>
       </c>
       <c r="C391" t="inlineStr">
         <is>
-          <t>Thử lại</t>
+          <t>Không tải được quảng cáo. Vui lòng thử lại.</t>
         </is>
       </c>
     </row>
     <row r="392">
       <c r="A392" t="inlineStr">
         <is>
-          <t>extra-money.reward-ad.close</t>
+          <t>extra-money.reward-ad.retry</t>
         </is>
       </c>
       <c r="B392" t="inlineStr">
         <is>
-          <t>Close</t>
+          <t>Try again</t>
         </is>
       </c>
       <c r="C392" t="inlineStr">
         <is>
-          <t>Đóng</t>
+          <t>Thử lại</t>
         </is>
       </c>
     </row>
     <row r="393">
       <c r="A393" t="inlineStr">
         <is>
-          <t>profile.button.save</t>
+          <t>extra-money.reward-ad.close</t>
         </is>
       </c>
       <c r="B393" t="inlineStr">
         <is>
-          <t>Save</t>
+          <t>Close</t>
         </is>
       </c>
       <c r="C393" t="inlineStr">
         <is>
-          <t>Lưu</t>
+          <t>Đóng</t>
         </is>
       </c>
     </row>
     <row r="394">
       <c r="A394" t="inlineStr">
         <is>
-          <t>profile.button.cancel</t>
+          <t>profile.button.save</t>
         </is>
       </c>
       <c r="B394" t="inlineStr">
         <is>
-          <t>Cancel</t>
+          <t>Save</t>
         </is>
       </c>
       <c r="C394" t="inlineStr">
         <is>
-          <t>Huỷ</t>
+          <t>Lưu</t>
         </is>
       </c>
     </row>
     <row r="395">
       <c r="A395" t="inlineStr">
         <is>
-          <t>change-password.title</t>
+          <t>profile.button.cancel</t>
         </is>
       </c>
       <c r="B395" t="inlineStr">
         <is>
-          <t>Change password</t>
+          <t>Cancel</t>
         </is>
       </c>
       <c r="C395" t="inlineStr">
         <is>
-          <t>Đổi mật khẩu</t>
+          <t>Huỷ</t>
         </is>
       </c>
     </row>
     <row r="396">
       <c r="A396" t="inlineStr">
         <is>
-          <t>change-password.current.label</t>
+          <t>change-password.title</t>
         </is>
       </c>
       <c r="B396" t="inlineStr">
         <is>
-          <t>Current password</t>
+          <t>Change password</t>
         </is>
       </c>
       <c r="C396" t="inlineStr">
         <is>
-          <t>Mật khẩu hiện tại</t>
+          <t>Đổi mật khẩu</t>
         </is>
       </c>
     </row>
     <row r="397">
       <c r="A397" t="inlineStr">
         <is>
-          <t>change-password.current.placeholder</t>
+          <t>change-password.current.label</t>
         </is>
       </c>
       <c r="B397" t="inlineStr">
         <is>
-          <t>Enter current password</t>
+          <t>Current password</t>
         </is>
       </c>
       <c r="C397" t="inlineStr">
         <is>
-          <t>Nhập mật khẩu hiện tại</t>
+          <t>Mật khẩu hiện tại</t>
         </is>
       </c>
     </row>
     <row r="398">
       <c r="A398" t="inlineStr">
         <is>
-          <t>change-password.new.label</t>
+          <t>change-password.current.placeholder</t>
         </is>
       </c>
       <c r="B398" t="inlineStr">
         <is>
-          <t>New password</t>
+          <t>Enter current password</t>
         </is>
       </c>
       <c r="C398" t="inlineStr">
         <is>
-          <t>Mật khẩu mới</t>
+          <t>Nhập mật khẩu hiện tại</t>
         </is>
       </c>
     </row>
     <row r="399">
       <c r="A399" t="inlineStr">
         <is>
-          <t>change-password.new.placeholder</t>
+          <t>change-password.new.label</t>
         </is>
       </c>
       <c r="B399" t="inlineStr">
         <is>
-          <t>Enter new password</t>
+          <t>New password</t>
         </is>
       </c>
       <c r="C399" t="inlineStr">
         <is>
-          <t>Nhập mật khẩu mới</t>
+          <t>Mật khẩu mới</t>
         </is>
       </c>
     </row>
     <row r="400">
       <c r="A400" t="inlineStr">
         <is>
-          <t>change-password.confirm.label</t>
+          <t>change-password.new.placeholder</t>
         </is>
       </c>
       <c r="B400" t="inlineStr">
         <is>
-          <t>Confirm new password</t>
+          <t>Enter new password</t>
         </is>
       </c>
       <c r="C400" t="inlineStr">
         <is>
-          <t>Xác nhận mật khẩu mới</t>
+          <t>Nhập mật khẩu mới</t>
         </is>
       </c>
     </row>
     <row r="401">
       <c r="A401" t="inlineStr">
         <is>
-          <t>change-password.confirm.placeholder</t>
+          <t>change-password.confirm.label</t>
         </is>
       </c>
       <c r="B401" t="inlineStr">
         <is>
-          <t>Re-enter new password</t>
+          <t>Confirm new password</t>
         </is>
       </c>
       <c r="C401" t="inlineStr">
         <is>
-          <t>Nhập lại mật khẩu mới</t>
+          <t>Xác nhận mật khẩu mới</t>
         </is>
       </c>
     </row>
     <row r="402">
       <c r="A402" t="inlineStr">
         <is>
-          <t>change-password.confirm.mismatch</t>
+          <t>change-password.confirm.placeholder</t>
         </is>
       </c>
       <c r="B402" t="inlineStr">
         <is>
-          <t>Passwords do not match</t>
+          <t>Re-enter new password</t>
         </is>
       </c>
       <c r="C402" t="inlineStr">
         <is>
-          <t>Mật khẩu xác nhận không khớp</t>
+          <t>Nhập lại mật khẩu mới</t>
         </is>
       </c>
     </row>
     <row r="403">
       <c r="A403" t="inlineStr">
         <is>
-          <t>change-password.show</t>
+          <t>change-password.confirm.mismatch</t>
         </is>
       </c>
       <c r="B403" t="inlineStr">
         <is>
-          <t>Show password</t>
+          <t>Passwords do not match</t>
         </is>
       </c>
       <c r="C403" t="inlineStr">
         <is>
-          <t>Hiện mật khẩu</t>
+          <t>Mật khẩu xác nhận không khớp</t>
         </is>
       </c>
     </row>
     <row r="404">
       <c r="A404" t="inlineStr">
         <is>
-          <t>change-password.hide</t>
+          <t>change-password.show</t>
         </is>
       </c>
       <c r="B404" t="inlineStr">
         <is>
-          <t>Hide password</t>
+          <t>Show password</t>
         </is>
       </c>
       <c r="C404" t="inlineStr">
         <is>
-          <t>Ẩn mật khẩu</t>
+          <t>Hiện mật khẩu</t>
         </is>
       </c>
     </row>
     <row r="405">
       <c r="A405" t="inlineStr">
         <is>
-          <t>change-password.submit</t>
+          <t>change-password.hide</t>
         </is>
       </c>
       <c r="B405" t="inlineStr">
         <is>
-          <t>Change password</t>
+          <t>Hide password</t>
         </is>
       </c>
       <c r="C405" t="inlineStr">
         <is>
-          <t>Đổi mật khẩu</t>
+          <t>Ẩn mật khẩu</t>
         </is>
       </c>
     </row>
     <row r="406">
       <c r="A406" t="inlineStr">
         <is>
-          <t>change-password.submitting</t>
+          <t>change-password.submit</t>
         </is>
       </c>
       <c r="B406" t="inlineStr">
         <is>
-          <t>Changing...</t>
+          <t>Change password</t>
         </is>
       </c>
       <c r="C406" t="inlineStr">
         <is>
-          <t>Đang đổi...</t>
+          <t>Đổi mật khẩu</t>
         </is>
       </c>
     </row>
     <row r="407">
       <c r="A407" t="inlineStr">
         <is>
-          <t>change-password.messages.success</t>
+          <t>change-password.submitting</t>
         </is>
       </c>
       <c r="B407" t="inlineStr">
         <is>
-          <t>Password changed successfully</t>
+          <t>Changing...</t>
         </is>
       </c>
       <c r="C407" t="inlineStr">
         <is>
-          <t>Đổi mật khẩu thành công</t>
+          <t>Đang đổi...</t>
         </is>
       </c>
     </row>
     <row r="408">
       <c r="A408" t="inlineStr">
         <is>
-          <t>change-password.messages.missing-fields</t>
+          <t>change-password.messages.success</t>
         </is>
       </c>
       <c r="B408" t="inlineStr">
         <is>
-          <t>Please fill in all fields</t>
+          <t>Password changed successfully</t>
         </is>
       </c>
       <c r="C408" t="inlineStr">
         <is>
-          <t>Vui lòng nhập đầy đủ thông tin</t>
+          <t>Đổi mật khẩu thành công</t>
         </is>
       </c>
     </row>
     <row r="409">
       <c r="A409" t="inlineStr">
         <is>
-          <t>change-password.messages.weak-password</t>
+          <t>change-password.messages.missing-fields</t>
         </is>
       </c>
       <c r="B409" t="inlineStr">
         <is>
-          <t>New password does not meet the requirements</t>
+          <t>Please fill in all fields</t>
         </is>
       </c>
       <c r="C409" t="inlineStr">
         <is>
-          <t>Mật khẩu mới không đạt yêu cầu</t>
+          <t>Vui lòng nhập đầy đủ thông tin</t>
         </is>
       </c>
     </row>
     <row r="410">
       <c r="A410" t="inlineStr">
         <is>
-          <t>change-password.messages.same-as-current</t>
+          <t>change-password.messages.weak-password</t>
         </is>
       </c>
       <c r="B410" t="inlineStr">
         <is>
-          <t>New password must be different from the current one</t>
+          <t>New password does not meet the requirements</t>
         </is>
       </c>
       <c r="C410" t="inlineStr">
         <is>
-          <t>Mật khẩu mới phải khác mật khẩu hiện tại</t>
+          <t>Mật khẩu mới không đạt yêu cầu</t>
         </is>
       </c>
     </row>
     <row r="411">
       <c r="A411" t="inlineStr">
         <is>
-          <t>change-password.messages.incorrect-current-password</t>
+          <t>change-password.messages.same-as-current</t>
         </is>
       </c>
       <c r="B411" t="inlineStr">
         <is>
-          <t>Current password is incorrect</t>
+          <t>New password must be different from the current one</t>
         </is>
       </c>
       <c r="C411" t="inlineStr">
         <is>
-          <t>Mật khẩu hiện tại không đúng</t>
+          <t>Mật khẩu mới phải khác mật khẩu hiện tại</t>
         </is>
       </c>
     </row>
     <row r="412">
       <c r="A412" t="inlineStr">
         <is>
-          <t>change-password.messages.user-not-found</t>
+          <t>change-password.messages.incorrect-current-password</t>
         </is>
       </c>
       <c r="B412" t="inlineStr">
         <is>
-          <t>User not found</t>
+          <t>Current password is incorrect</t>
         </is>
       </c>
       <c r="C412" t="inlineStr">
         <is>
-          <t>Không tìm thấy người dùng</t>
+          <t>Mật khẩu hiện tại không đúng</t>
         </is>
       </c>
     </row>
     <row r="413">
       <c r="A413" t="inlineStr">
         <is>
-          <t>change-password.messages.unauthorized</t>
+          <t>change-password.messages.user-not-found</t>
         </is>
       </c>
       <c r="B413" t="inlineStr">
         <is>
-          <t>Session expired. Please sign in again.</t>
+          <t>User not found</t>
         </is>
       </c>
       <c r="C413" t="inlineStr">
         <is>
-          <t>Phiên đăng nhập đã hết hạn. Vui lòng đăng nhập lại.</t>
+          <t>Không tìm thấy người dùng</t>
         </is>
       </c>
     </row>
     <row r="414">
       <c r="A414" t="inlineStr">
         <is>
+          <t>change-password.messages.unauthorized</t>
+        </is>
+      </c>
+      <c r="B414" t="inlineStr">
+        <is>
+          <t>Session expired. Please sign in again.</t>
+        </is>
+      </c>
+      <c r="C414" t="inlineStr">
+        <is>
+          <t>Phiên đăng nhập đã hết hạn. Vui lòng đăng nhập lại.</t>
+        </is>
+      </c>
+    </row>
+    <row r="415">
+      <c r="A415" t="inlineStr">
+        <is>
           <t>change-password.messages.internal-server-error</t>
         </is>
       </c>
-      <c r="B414" t="inlineStr">
+      <c r="B415" t="inlineStr">
         <is>
           <t>Something went wrong. Please try again.</t>
         </is>
       </c>
-      <c r="C414" t="inlineStr">
+      <c r="C415" t="inlineStr">
         <is>
           <t>Đã có lỗi xảy ra. Vui lòng thử lại.</t>
         </is>
       </c>
-    </row>
-    <row r="415">
-      <c r="A415" t="inlineStr"/>
-      <c r="B415" t="inlineStr"/>
-      <c r="C415" t="inlineStr"/>
     </row>
     <row r="416">
       <c r="A416" t="inlineStr"/>
@@ -7465,6 +7477,11 @@
       <c r="A433" t="inlineStr"/>
       <c r="B433" t="inlineStr"/>
       <c r="C433" t="inlineStr"/>
+    </row>
+    <row r="434">
+      <c r="A434" t="inlineStr"/>
+      <c r="B434" t="inlineStr"/>
+      <c r="C434" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>